<commit_message>
Vuelvo atras el cambio de modelo en Italia
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -261,7 +261,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="151">
   <si>
     <t>id_country</t>
   </si>
@@ -413,13 +413,13 @@
     }</t>
   </si>
   <si>
-    <t>0.10</t>
-  </si>
-  <si>
     <t>[771, 772, 773, 774]</t>
   </si>
   <si>
     <t>SVC</t>
+  </si>
+  <si>
+    <t>4.9%</t>
   </si>
   <si>
     <t>Hasta el 20/8, le tenia miedo al doble oportunidad pero ahora ya no.</t>
@@ -473,6 +473,9 @@
   </si>
   <si>
     <t>0.7</t>
+  </si>
+  <si>
+    <t>0.10</t>
   </si>
   <si>
     <t>[591, 593, 594]</t>
@@ -1291,23 +1294,23 @@
     <xf borderId="3" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="3" fillId="0" fontId="3" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center"/>
-    </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="3" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="4" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="3" fillId="4" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="3" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -2077,7 +2080,7 @@
         <v>41</v>
       </c>
       <c r="F4" s="14">
-        <v>174.0</v>
+        <v>470.0</v>
       </c>
       <c r="G4" s="15">
         <v>30.0</v>
@@ -2085,27 +2088,25 @@
       <c r="H4" s="15">
         <v>3.0</v>
       </c>
-      <c r="I4" s="16" t="b">
-        <v>1</v>
-      </c>
-      <c r="J4" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="K4" s="28" t="s">
-        <v>42</v>
+      <c r="I4" s="15" t="b">
+        <v>0</v>
+      </c>
+      <c r="J4" s="15"/>
+      <c r="K4" s="16" t="s">
+        <v>31</v>
       </c>
       <c r="L4" s="15">
         <v>5.0</v>
       </c>
       <c r="M4" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N4" s="15"/>
       <c r="O4" s="15" t="s">
         <v>38</v>
       </c>
       <c r="P4" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q4" s="18">
         <v>35.0</v>
@@ -2127,24 +2128,24 @@
         <v>14.60463869</v>
       </c>
       <c r="W4" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="X4" s="29">
-        <v>0.0205</v>
+        <v>39</v>
+      </c>
+      <c r="X4" s="15" t="s">
+        <v>44</v>
       </c>
       <c r="Y4" s="20">
-        <v>56.36</v>
+        <v>63.09</v>
       </c>
       <c r="Z4" s="15">
         <v>112.0</v>
       </c>
       <c r="AA4" s="20">
         <f t="shared" si="1"/>
-        <v>0.5032142857</v>
+        <v>0.5633035714</v>
       </c>
       <c r="AB4" s="20">
         <f>'Data preparation'!$B$2*AA4</f>
-        <v>0.07548214286</v>
+        <v>0.08449553571</v>
       </c>
       <c r="AC4" s="21" t="s">
         <v>45</v>
@@ -2157,13 +2158,13 @@
       <c r="B5" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C5" s="30">
+      <c r="C5" s="28">
         <v>45419.0</v>
       </c>
       <c r="D5" s="12">
         <v>1536.0</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="29"/>
       <c r="F5" s="14">
         <v>808.0</v>
       </c>
@@ -2193,7 +2194,7 @@
         <v>38</v>
       </c>
       <c r="P5" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q5" s="18">
         <v>34.0</v>
@@ -2217,7 +2218,7 @@
       <c r="W5" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="X5" s="29">
+      <c r="X5" s="30">
         <v>1.39</v>
       </c>
       <c r="Y5" s="20">
@@ -2237,7 +2238,7 @@
       <c r="AC5" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="AG5" s="32"/>
+      <c r="AG5" s="31"/>
     </row>
     <row r="6" ht="41.25" customHeight="1">
       <c r="A6" s="9">
@@ -2252,7 +2253,7 @@
       <c r="D6" s="26">
         <v>1536.0</v>
       </c>
-      <c r="E6" s="33" t="s">
+      <c r="E6" s="32" t="s">
         <v>50</v>
       </c>
       <c r="F6" s="14">
@@ -2267,10 +2268,10 @@
       <c r="I6" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="J6" s="28" t="s">
+      <c r="J6" s="33" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="28"/>
+      <c r="K6" s="33"/>
       <c r="L6" s="15"/>
       <c r="M6" s="15" t="s">
         <v>52</v>
@@ -2339,7 +2340,7 @@
       <c r="D7" s="12">
         <v>1152.0</v>
       </c>
-      <c r="E7" s="31" t="s">
+      <c r="E7" s="29" t="s">
         <v>41</v>
       </c>
       <c r="F7" s="14">
@@ -2358,13 +2359,13 @@
         <v>54</v>
       </c>
       <c r="K7" s="15" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="L7" s="15">
         <v>10.0</v>
       </c>
       <c r="M7" s="15" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="N7" s="15"/>
       <c r="O7" s="15" t="s">
@@ -2395,7 +2396,7 @@
       <c r="W7" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="X7" s="29">
+      <c r="X7" s="30">
         <v>0.2515</v>
       </c>
       <c r="Y7" s="20">
@@ -2420,9 +2421,9 @@
         <v>6.0</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C8" s="30">
+        <v>57</v>
+      </c>
+      <c r="C8" s="28">
         <v>45419.0</v>
       </c>
       <c r="D8" s="12">
@@ -2451,7 +2452,7 @@
         <v>3.0</v>
       </c>
       <c r="M8" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N8" s="16"/>
       <c r="O8" s="16" t="s">
@@ -2482,7 +2483,7 @@
       <c r="W8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="X8" s="29">
+      <c r="X8" s="30">
         <v>3.0E-4</v>
       </c>
       <c r="Y8" s="20">
@@ -2652,12 +2653,12 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="47" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="48" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B2" s="44">
         <v>0.15</v>
@@ -2666,19 +2667,19 @@
     </row>
     <row r="3">
       <c r="A3" s="47" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B3" s="49">
         <f>MAX('Modelos actuales'!T3:T7)</f>
         <v>18.6475</v>
       </c>
       <c r="E3" s="48" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="47" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B4" s="48">
         <v>18.0</v>
@@ -2692,7 +2693,7 @@
       <c r="A7" s="50"/>
       <c r="B7" s="50"/>
       <c r="E7" s="51" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F7" s="36">
         <f t="shared" ref="F7:F16" si="1">REPLACE(E7,FIND(".",E7),1,",")*1</f>
@@ -2701,7 +2702,7 @@
     </row>
     <row r="8">
       <c r="E8" s="52" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F8" s="36">
         <f t="shared" si="1"/>
@@ -2710,7 +2711,7 @@
     </row>
     <row r="9">
       <c r="E9" s="51" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F9" s="36">
         <f t="shared" si="1"/>
@@ -2719,7 +2720,7 @@
     </row>
     <row r="10">
       <c r="E10" s="52" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F10" s="36">
         <f t="shared" si="1"/>
@@ -2728,7 +2729,7 @@
     </row>
     <row r="11">
       <c r="E11" s="51" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F11" s="36">
         <f t="shared" si="1"/>
@@ -2737,7 +2738,7 @@
     </row>
     <row r="12">
       <c r="E12" s="52" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F12" s="36">
         <f t="shared" si="1"/>
@@ -2746,7 +2747,7 @@
     </row>
     <row r="13">
       <c r="E13" s="51" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F13" s="36">
         <f t="shared" si="1"/>
@@ -2755,7 +2756,7 @@
     </row>
     <row r="14">
       <c r="E14" s="52" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="F14" s="36">
         <f t="shared" si="1"/>
@@ -2764,7 +2765,7 @@
     </row>
     <row r="15">
       <c r="E15" s="51" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F15" s="36">
         <f t="shared" si="1"/>
@@ -2773,7 +2774,7 @@
     </row>
     <row r="16">
       <c r="E16" s="52" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F16" s="36">
         <f t="shared" si="1"/>
@@ -2804,11 +2805,11 @@
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
       <c r="D1" s="54" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="F1" s="55"/>
       <c r="G1" s="56" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="J1" s="53"/>
       <c r="K1" s="53"/>
@@ -2816,13 +2817,13 @@
     </row>
     <row r="2">
       <c r="A2" s="57" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B2" s="57" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C2" s="57" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D2" s="58" t="s">
         <v>3</v>
@@ -2831,7 +2832,7 @@
         <v>4</v>
       </c>
       <c r="F2" s="60" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="G2" s="61" t="s">
         <v>20</v>
@@ -2843,20 +2844,20 @@
         <v>19</v>
       </c>
       <c r="J2" s="57" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="K2" s="57" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L2" s="57" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" ht="108.0" customHeight="1">
       <c r="A3" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="30">
+      <c r="B3" s="28">
         <v>45418.0</v>
       </c>
       <c r="C3" s="63"/>
@@ -2872,23 +2873,23 @@
         <v>17.31</v>
       </c>
       <c r="I3" s="68" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J3" s="69" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K3" s="70" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="L3" s="71" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" ht="108.0" customHeight="1">
       <c r="A4" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="B4" s="30">
+      <c r="B4" s="28">
         <v>45418.0</v>
       </c>
       <c r="C4" s="63"/>
@@ -2907,20 +2908,20 @@
         <v>46.72</v>
       </c>
       <c r="J4" s="69" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K4" s="70" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L4" s="74" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" ht="42.0" customHeight="1">
       <c r="A5" s="75" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="30">
+      <c r="B5" s="28">
         <v>45419.0</v>
       </c>
       <c r="C5" s="63"/>
@@ -2939,7 +2940,7 @@
         <v>16.21</v>
       </c>
       <c r="J5" s="69" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K5" s="76"/>
       <c r="L5" s="77"/>
@@ -2961,7 +2962,7 @@
       <c r="H6" s="80"/>
       <c r="I6" s="81"/>
       <c r="J6" s="69" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K6" s="76"/>
       <c r="L6" s="75" t="s">
@@ -2970,9 +2971,9 @@
     </row>
     <row r="7">
       <c r="A7" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="B7" s="30">
+        <v>57</v>
+      </c>
+      <c r="B7" s="28">
         <v>45419.0</v>
       </c>
       <c r="C7" s="63"/>
@@ -2985,11 +2986,11 @@
       <c r="H7" s="83"/>
       <c r="I7" s="83"/>
       <c r="J7" s="69" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K7" s="76"/>
       <c r="L7" s="75" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="8">
@@ -3009,7 +3010,7 @@
       <c r="H8" s="80"/>
       <c r="I8" s="81"/>
       <c r="J8" s="69" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K8" s="76"/>
       <c r="L8" s="77"/>
@@ -3022,7 +3023,7 @@
         <v>45498.0</v>
       </c>
       <c r="C9" s="84" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D9" s="82">
         <v>1152.0</v>
@@ -3041,11 +3042,11 @@
         <v>15.41</v>
       </c>
       <c r="J9" s="69" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K9" s="84"/>
       <c r="L9" s="75" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" ht="49.5" customHeight="1">
@@ -3056,7 +3057,7 @@
         <v>45498.0</v>
       </c>
       <c r="C10" s="84" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" s="82">
         <v>1152.0</v>
@@ -3075,7 +3076,7 @@
         <v>8.63</v>
       </c>
       <c r="J10" s="75" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K10" s="84"/>
       <c r="L10" s="75"/>
@@ -3088,16 +3089,16 @@
         <v>45502.0</v>
       </c>
       <c r="C11" s="84" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D11" s="82">
         <v>1728.0</v>
       </c>
       <c r="E11" s="85" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F11" s="86" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G11" s="37">
         <v>8.9</v>
@@ -3109,13 +3110,13 @@
         <v>5.5</v>
       </c>
       <c r="J11" s="75" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K11" s="84" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="L11" s="75" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" ht="73.5" customHeight="1">
@@ -3126,7 +3127,7 @@
         <v>45504.0</v>
       </c>
       <c r="C12" s="84" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D12" s="82">
         <v>1536.0</v>
@@ -3135,7 +3136,7 @@
         <v>50</v>
       </c>
       <c r="F12" s="86" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G12" s="37">
         <v>19.73</v>
@@ -3144,16 +3145,16 @@
         <v>47.88</v>
       </c>
       <c r="I12" s="38" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="J12" s="75" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K12" s="84" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="L12" s="75" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
     </row>
     <row r="13">
@@ -3167,7 +3168,7 @@
     </row>
     <row r="14">
       <c r="A14" s="94" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D14" s="88"/>
       <c r="F14" s="89"/>
@@ -10233,7 +10234,7 @@
         <v>1</v>
       </c>
       <c r="J2" s="15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K2" s="15" t="s">
         <v>31</v>
@@ -10242,12 +10243,12 @@
         <v>5.0</v>
       </c>
       <c r="M2" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N2" s="16"/>
       <c r="O2" s="16"/>
       <c r="P2" s="34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q2" s="18">
         <v>18.0</v>
@@ -10270,7 +10271,7 @@
         <v>66.1176029</v>
       </c>
       <c r="W2" s="14" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="X2" s="20">
         <v>15.0684194244387</v>
@@ -10308,7 +10309,7 @@
       <c r="F3" s="14">
         <v>300.0</v>
       </c>
-      <c r="G3" s="28">
+      <c r="G3" s="33">
         <v>30.0</v>
       </c>
       <c r="H3" s="96">
@@ -10317,7 +10318,7 @@
       <c r="I3" s="16" t="b">
         <v>0</v>
       </c>
-      <c r="J3" s="28" t="s">
+      <c r="J3" s="33" t="s">
         <v>54</v>
       </c>
       <c r="K3" s="96"/>
@@ -10325,7 +10326,7 @@
         <v>10.0</v>
       </c>
       <c r="M3" s="16" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N3" s="15" t="s">
         <v>33</v>
@@ -10462,7 +10463,7 @@
         <v>0.04863669065</v>
       </c>
       <c r="AC4" s="21" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="5" ht="31.5" customHeight="1">
@@ -10478,7 +10479,7 @@
       <c r="D5" s="12">
         <v>1536.0</v>
       </c>
-      <c r="E5" s="31"/>
+      <c r="E5" s="29"/>
       <c r="F5" s="14">
         <v>808.0</v>
       </c>
@@ -10508,7 +10509,7 @@
         <v>38</v>
       </c>
       <c r="P5" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q5" s="18">
         <v>34.0</v>
@@ -10552,7 +10553,7 @@
       <c r="AC5" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="AG5" s="32"/>
+      <c r="AG5" s="31"/>
     </row>
     <row r="6" ht="41.25" customHeight="1">
       <c r="A6" s="9">
@@ -10567,7 +10568,7 @@
       <c r="D6" s="12">
         <v>1152.0</v>
       </c>
-      <c r="E6" s="31" t="s">
+      <c r="E6" s="29" t="s">
         <v>41</v>
       </c>
       <c r="F6" s="14">
@@ -10586,20 +10587,20 @@
         <v>30</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="L6" s="15">
         <v>5.0</v>
       </c>
       <c r="M6" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N6" s="16"/>
       <c r="O6" s="16" t="s">
         <v>38</v>
       </c>
       <c r="P6" s="34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q6" s="18">
         <v>35.0</v>
@@ -10623,7 +10624,7 @@
       <c r="W6" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="X6" s="29">
+      <c r="X6" s="30">
         <v>0.047</v>
       </c>
       <c r="Y6" s="20">
@@ -10656,7 +10657,7 @@
       <c r="D7" s="12">
         <v>1152.0</v>
       </c>
-      <c r="E7" s="31" t="s">
+      <c r="E7" s="29" t="s">
         <v>41</v>
       </c>
       <c r="F7" s="14">
@@ -10675,7 +10676,7 @@
       <c r="K7" s="16"/>
       <c r="L7" s="16"/>
       <c r="M7" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N7" s="15" t="s">
         <v>33</v>
@@ -10704,9 +10705,9 @@
         <v>8.330339188</v>
       </c>
       <c r="W7" s="14" t="s">
-        <v>105</v>
-      </c>
-      <c r="X7" s="29">
+        <v>106</v>
+      </c>
+      <c r="X7" s="30">
         <v>0.3172</v>
       </c>
       <c r="Y7" s="20">
@@ -10731,7 +10732,7 @@
         <v>6.0</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C8" s="22">
         <v>45419.0</v>
@@ -10760,7 +10761,7 @@
         <v>10.0</v>
       </c>
       <c r="M8" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N8" s="16" t="s">
         <v>33</v>
@@ -10793,7 +10794,7 @@
       <c r="W8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="X8" s="29">
+      <c r="X8" s="30">
         <v>-6.0E-4</v>
       </c>
       <c r="Y8" s="20">
@@ -10826,7 +10827,7 @@
       <c r="D9" s="12">
         <v>768.0</v>
       </c>
-      <c r="E9" s="31"/>
+      <c r="E9" s="29"/>
       <c r="F9" s="14">
         <v>358.0</v>
       </c>
@@ -10840,12 +10841,12 @@
         <v>0</v>
       </c>
       <c r="J9" s="15" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="K9" s="15"/>
       <c r="L9" s="15"/>
       <c r="M9" s="15" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="N9" s="16"/>
       <c r="O9" s="15" t="s">
@@ -10877,7 +10878,7 @@
       <c r="W9" s="14">
         <v>-0.15</v>
       </c>
-      <c r="X9" s="29">
+      <c r="X9" s="30">
         <v>0.0598</v>
       </c>
       <c r="Y9" s="20">
@@ -10923,7 +10924,7 @@
       <c r="D12" s="97"/>
       <c r="E12" s="97"/>
       <c r="F12" s="97"/>
-      <c r="S12" s="32"/>
+      <c r="S12" s="31"/>
       <c r="T12" s="90"/>
       <c r="U12" s="90"/>
       <c r="AG12" s="36"/>
@@ -10948,7 +10949,7 @@
     </row>
     <row r="18">
       <c r="A18" s="101" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C18" s="97"/>
       <c r="D18" s="97"/>
@@ -11075,7 +11076,7 @@
         <v>1</v>
       </c>
       <c r="J20" s="15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K20" s="15" t="s">
         <v>31</v>
@@ -11084,12 +11085,12 @@
         <v>5.0</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="N20" s="16"/>
       <c r="O20" s="16"/>
       <c r="P20" s="34" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q20" s="18">
         <v>18.0</v>
@@ -11110,7 +11111,7 @@
         <v>17.717537506466634</v>
       </c>
       <c r="W20" s="43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="X20" s="44">
         <v>15.0684194244387</v>
@@ -11211,7 +11212,7 @@
         <v>0.048636690647482016</v>
       </c>
       <c r="AC21" s="48" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AG21" s="36"/>
     </row>
@@ -11228,30 +11229,30 @@
       <c r="D22" s="26">
         <v>1536.0</v>
       </c>
-      <c r="E22" s="33" t="s">
+      <c r="E22" s="32" t="s">
         <v>50</v>
       </c>
       <c r="F22" s="14">
         <v>559.0</v>
       </c>
-      <c r="G22" s="28">
+      <c r="G22" s="33">
         <v>30.0</v>
       </c>
-      <c r="H22" s="28">
+      <c r="H22" s="33">
         <v>3.0</v>
       </c>
       <c r="I22" s="15" t="b">
         <v>0</v>
       </c>
-      <c r="J22" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="K22" s="28" t="s">
-        <v>42</v>
+      <c r="J22" s="33" t="s">
+        <v>114</v>
+      </c>
+      <c r="K22" s="33" t="s">
+        <v>55</v>
       </c>
       <c r="L22" s="15"/>
       <c r="M22" s="15" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="N22" s="15" t="s">
         <v>33</v>
@@ -11279,7 +11280,7 @@
         <v>15.310398344542163</v>
       </c>
       <c r="W22" s="43" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="X22" s="44">
         <v>1.11</v>
@@ -11306,13 +11307,13 @@
       <c r="B23" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="C23" s="30">
+      <c r="C23" s="28">
         <v>45419.0</v>
       </c>
       <c r="D23" s="12">
         <v>1536.0</v>
       </c>
-      <c r="E23" s="31"/>
+      <c r="E23" s="29"/>
       <c r="F23" s="14">
         <v>808.0</v>
       </c>
@@ -11342,7 +11343,7 @@
         <v>38</v>
       </c>
       <c r="P23" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q23" s="18">
         <v>34.0</v>
@@ -11413,23 +11414,23 @@
         <v>1</v>
       </c>
       <c r="J24" s="15" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="K24" s="15" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="L24" s="15">
         <v>5.0</v>
       </c>
       <c r="M24" s="15" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="N24" s="16"/>
       <c r="O24" s="15" t="s">
         <v>38</v>
       </c>
       <c r="P24" s="17" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="Q24" s="18">
         <v>35.0</v>
@@ -11450,7 +11451,7 @@
         <v>11.958096223486809</v>
       </c>
       <c r="W24" s="43" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="X24" s="46">
         <v>0.047</v>
@@ -11482,7 +11483,7 @@
       <c r="D25" s="12">
         <v>1152.0</v>
       </c>
-      <c r="E25" s="31" t="s">
+      <c r="E25" s="29" t="s">
         <v>41</v>
       </c>
       <c r="F25" s="14">
@@ -11501,7 +11502,7 @@
       <c r="K25" s="16"/>
       <c r="L25" s="16"/>
       <c r="M25" s="15" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="N25" s="15" t="s">
         <v>33</v>
@@ -11529,7 +11530,7 @@
         <v>6.696844283497156</v>
       </c>
       <c r="W25" s="43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="X25" s="46">
         <v>0.3172</v>
@@ -11553,9 +11554,9 @@
         <v>6.0</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C26" s="30">
+        <v>57</v>
+      </c>
+      <c r="C26" s="28">
         <v>45419.0</v>
       </c>
       <c r="D26" s="12">
@@ -11584,7 +11585,7 @@
         <v>3.0</v>
       </c>
       <c r="M26" s="15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="N26" s="16"/>
       <c r="O26" s="16" t="s">
@@ -11645,7 +11646,7 @@
     </row>
     <row r="34">
       <c r="A34" s="101" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="W34" s="42"/>
     </row>
@@ -11738,7 +11739,7 @@
         <v>17.690894981893432</v>
       </c>
       <c r="J37" s="43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="K37" s="44">
         <v>6.11</v>
@@ -11778,7 +11779,7 @@
         <v>15.888515261251941</v>
       </c>
       <c r="J38" s="43" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="K38" s="46">
         <v>0.0259</v>
@@ -11852,7 +11853,7 @@
         <v>13.457061562338335</v>
       </c>
       <c r="J40" s="43" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="K40" s="44">
         <v>0.83</v>
@@ -11889,7 +11890,7 @@
         <v>4.319710294878428</v>
       </c>
       <c r="J41" s="43" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="K41" s="46">
         <v>0.2515</v>
@@ -12004,10 +12005,10 @@
   <sheetData>
     <row r="5">
       <c r="F5" s="104" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H5" s="105" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J5" s="55"/>
     </row>
@@ -12022,22 +12023,22 @@
         <v>2</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F6" s="106" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G6" s="107" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H6" s="108" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I6" s="109" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J6" s="110" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="7">
@@ -12047,7 +12048,7 @@
       <c r="C7" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="D7" s="30">
+      <c r="D7" s="28">
         <v>45419.0</v>
       </c>
       <c r="E7" s="17">
@@ -12057,7 +12058,7 @@
         <v>-0.16</v>
       </c>
       <c r="G7" s="17" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H7" s="113">
         <v>2304.0</v>
@@ -12087,7 +12088,7 @@
         <v>-0.34</v>
       </c>
       <c r="G8" s="17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H8" s="116">
         <v>768.0</v>
@@ -12107,7 +12108,7 @@
       <c r="C9" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="30">
+      <c r="D9" s="28">
         <v>45504.0</v>
       </c>
       <c r="E9" s="17">
@@ -12117,7 +12118,7 @@
         <v>-0.23</v>
       </c>
       <c r="G9" s="17" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H9" s="117">
         <v>1536.0</v>
@@ -12137,7 +12138,7 @@
       <c r="C10" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="D10" s="30">
+      <c r="D10" s="28">
         <v>45419.0</v>
       </c>
       <c r="E10" s="17">
@@ -12147,7 +12148,7 @@
         <v>-0.23</v>
       </c>
       <c r="G10" s="17" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H10" s="116">
         <v>1536.0</v>
@@ -12167,7 +12168,7 @@
       <c r="C11" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="D11" s="30">
+      <c r="D11" s="28">
         <v>45498.0</v>
       </c>
       <c r="E11" s="17">
@@ -12177,7 +12178,7 @@
         <v>-0.2</v>
       </c>
       <c r="G11" s="17" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H11" s="117">
         <v>1152.0</v>
@@ -12207,7 +12208,7 @@
         <v>-0.24</v>
       </c>
       <c r="G12" s="17" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H12" s="116">
         <v>1152.0</v>
@@ -12225,9 +12226,9 @@
         <v>6.0</v>
       </c>
       <c r="C13" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="D13" s="30">
+        <v>57</v>
+      </c>
+      <c r="D13" s="28">
         <v>45419.0</v>
       </c>
       <c r="E13" s="34">
@@ -12236,8 +12237,8 @@
       <c r="F13" s="112">
         <v>-0.33</v>
       </c>
-      <c r="G13" s="30" t="s">
-        <v>132</v>
+      <c r="G13" s="28" t="s">
+        <v>133</v>
       </c>
       <c r="H13" s="116">
         <v>2304.0</v>
@@ -12270,36 +12271,36 @@
   <sheetData>
     <row r="7">
       <c r="B7" s="101" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="48" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9">
       <c r="B9" s="119" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10">
       <c r="B10" s="120" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F10" s="48" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G10" s="48" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H10" s="48" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="11">
       <c r="C11" s="48" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D11" s="48">
         <v>-0.15</v>
@@ -12315,22 +12316,22 @@
         <v>#DIV/0!</v>
       </c>
       <c r="I11" s="47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="12">
       <c r="C12" s="120" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="13">
       <c r="C13" s="120" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" s="120" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F14" s="48">
         <v>2.0</v>
@@ -12345,7 +12346,7 @@
     </row>
     <row r="15">
       <c r="C15" s="48" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D15" s="48">
         <v>-0.1</v>
@@ -12353,17 +12354,17 @@
     </row>
     <row r="16">
       <c r="C16" s="120" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
     <row r="17">
       <c r="C17" s="120" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="18">
       <c r="B18" s="120" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F18" s="48">
         <v>0.0</v>
@@ -12378,7 +12379,7 @@
     </row>
     <row r="19">
       <c r="C19" s="48" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D19" s="48">
         <v>-0.15</v>
@@ -12386,17 +12387,17 @@
     </row>
     <row r="20">
       <c r="C20" s="120" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21">
       <c r="C21" s="120" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
     </row>
     <row r="25">
       <c r="B25" s="121" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="26">
@@ -12432,7 +12433,7 @@
       <c r="C27" s="34" t="s">
         <v>36</v>
       </c>
-      <c r="D27" s="30">
+      <c r="D27" s="28">
         <v>45419.0</v>
       </c>
       <c r="E27" s="11">
@@ -12459,7 +12460,7 @@
       <c r="C28" s="34" t="s">
         <v>29</v>
       </c>
-      <c r="D28" s="30">
+      <c r="D28" s="28">
         <v>45467.0</v>
       </c>
       <c r="E28" s="11">
@@ -12485,7 +12486,7 @@
       <c r="C29" s="34" t="s">
         <v>49</v>
       </c>
-      <c r="D29" s="30">
+      <c r="D29" s="28">
         <v>45504.0</v>
       </c>
       <c r="E29" s="22">
@@ -12511,7 +12512,7 @@
       <c r="C30" s="34" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="30">
+      <c r="D30" s="28">
         <v>45419.0</v>
       </c>
       <c r="E30" s="11">
@@ -12537,7 +12538,7 @@
       <c r="C31" s="34" t="s">
         <v>40</v>
       </c>
-      <c r="D31" s="30">
+      <c r="D31" s="28">
         <v>45498.0</v>
       </c>
       <c r="E31" s="22">
@@ -12563,7 +12564,7 @@
       <c r="C32" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="D32" s="30">
+      <c r="D32" s="28">
         <v>45498.0</v>
       </c>
       <c r="E32" s="11">
@@ -12587,9 +12588,9 @@
         <v>6.0</v>
       </c>
       <c r="C33" s="34" t="s">
-        <v>56</v>
-      </c>
-      <c r="D33" s="30">
+        <v>57</v>
+      </c>
+      <c r="D33" s="28">
         <v>45419.0</v>
       </c>
       <c r="E33" s="39">

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelo en SPA
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -210,7 +210,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="404" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="263">
   <si>
     <t>id_country</t>
   </si>
@@ -644,6 +644,12 @@
     <t>4.54</t>
   </si>
   <si>
+    <t>n_iteration</t>
+  </si>
+  <si>
+    <t>roi</t>
+  </si>
+  <si>
     <t>Falta entrenarlos: 1) sin rellenar formaciones antes de construir 2) Con todos l_models y no solo logistic.</t>
   </si>
   <si>
@@ -948,9 +954,6 @@
   </si>
   <si>
     <t>roi_100</t>
-  </si>
-  <si>
-    <t>roi</t>
   </si>
   <si>
     <t>roi_por_partido</t>
@@ -2036,7 +2039,9 @@
       <c r="E4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="24"/>
+      <c r="F4" s="24">
+        <v>56.3636363636363</v>
+      </c>
       <c r="G4" s="24">
         <v>161.57</v>
       </c>
@@ -2085,7 +2090,9 @@
       <c r="E5" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="24"/>
+      <c r="F5" s="24">
+        <v>57.7981651376146</v>
+      </c>
       <c r="G5" s="24">
         <v>147.288321859431</v>
       </c>
@@ -2186,7 +2193,9 @@
       <c r="E7" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="F7" s="24"/>
+      <c r="F7" s="24">
+        <v>59.2592592592592</v>
+      </c>
       <c r="G7" s="24">
         <v>197.314387756965</v>
       </c>
@@ -2230,44 +2239,44 @@
         <v>45677.0</v>
       </c>
       <c r="D8" s="23">
-        <v>112.0</v>
+        <v>1051.0</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>17</v>
       </c>
       <c r="F8" s="24">
-        <v>56.8807339449541</v>
+        <v>53.2110091743119</v>
       </c>
       <c r="G8" s="24">
-        <v>107.0</v>
+        <v>191.629402836081</v>
       </c>
       <c r="H8" s="24">
-        <f>274.34+
-1948.08+
-12.5
+        <f>301.19+
+154.98+
+109.46
 </f>
-        <v>2234.92</v>
+        <v>565.63</v>
       </c>
       <c r="I8" s="24">
         <f t="shared" si="1"/>
-        <v>20.8871028</v>
+        <v>2.95168691</v>
       </c>
       <c r="J8" s="19">
-        <v>40.0</v>
+        <v>50.0</v>
       </c>
       <c r="K8" s="19">
-        <v>70.0</v>
+        <v>15.0</v>
       </c>
       <c r="L8" s="19">
-        <v>10.0</v>
+        <v>20.0</v>
       </c>
       <c r="M8" s="19">
         <f t="shared" si="2"/>
-        <v>40</v>
+        <v>28.33333333</v>
       </c>
       <c r="N8" s="15">
         <f>M8*'Data preparation'!$C$2</f>
-        <v>12</v>
+        <v>8.5</v>
       </c>
     </row>
     <row r="9" ht="20.25" customHeight="1">
@@ -12748,7 +12757,7 @@
       </c>
       <c r="C3" s="15">
         <f>AVERAGE('Modelos actuales'!N4:N8)</f>
-        <v>12.4</v>
+        <v>11.7</v>
       </c>
       <c r="L3" s="89"/>
       <c r="P3" s="89"/>
@@ -13649,6 +13658,15 @@
       <c r="P28" s="92">
         <v>1.0</v>
       </c>
+      <c r="AA28" s="35" t="s">
+        <v>144</v>
+      </c>
+      <c r="AB28" s="35" t="s">
+        <v>145</v>
+      </c>
+      <c r="AC28" s="35" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="29">
       <c r="F29" s="29" t="s">
@@ -13670,46 +13688,144 @@
       <c r="P29" s="92">
         <v>1.0</v>
       </c>
+      <c r="AA29" s="36">
+        <v>1051.0</v>
+      </c>
+      <c r="AB29" s="35">
+        <v>207.56</v>
+      </c>
+      <c r="AC29" s="37">
+        <f t="shared" ref="AC29:AC43" si="15">VLOOKUP(AA29,$AA$48:$AB$62,2,0)</f>
+        <v>263.81</v>
+      </c>
+      <c r="AD29" s="93">
+        <f t="shared" ref="AD29:AD43" si="16">(AC29-AB29)/AB29</f>
+        <v>0.2710059742</v>
+      </c>
     </row>
     <row r="30">
       <c r="P30" s="92">
         <v>2.0</v>
       </c>
+      <c r="AA30" s="35">
+        <v>112.0</v>
+      </c>
+      <c r="AB30" s="35">
+        <v>185.35</v>
+      </c>
+      <c r="AC30" s="37">
+        <f t="shared" si="15"/>
+        <v>130.76</v>
+      </c>
+      <c r="AD30" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.2945238738</v>
+      </c>
     </row>
     <row r="31">
       <c r="P31" s="92">
         <v>0.0</v>
       </c>
+      <c r="AA31" s="35">
+        <v>752.0</v>
+      </c>
+      <c r="AB31" s="35">
+        <v>121.6</v>
+      </c>
+      <c r="AC31" s="37">
+        <f t="shared" si="15"/>
+        <v>78.68</v>
+      </c>
+      <c r="AD31" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.3529605263</v>
+      </c>
     </row>
     <row r="32">
       <c r="B32" s="47" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G32" s="95"/>
       <c r="P32" s="92">
         <v>1.0</v>
       </c>
+      <c r="AA32" s="36">
+        <v>1475.0</v>
+      </c>
+      <c r="AB32" s="35">
+        <v>120.82</v>
+      </c>
+      <c r="AC32" s="37">
+        <f t="shared" si="15"/>
+        <v>83.5</v>
+      </c>
+      <c r="AD32" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.3088892567</v>
+      </c>
     </row>
     <row r="33">
       <c r="B33" s="101" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G33" s="102"/>
       <c r="P33" s="92">
         <v>1.0</v>
       </c>
+      <c r="AA33" s="36">
+        <v>1545.0</v>
+      </c>
+      <c r="AB33" s="35">
+        <v>111.42</v>
+      </c>
+      <c r="AC33" s="37">
+        <f t="shared" si="15"/>
+        <v>101.16</v>
+      </c>
+      <c r="AD33" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.09208400646</v>
+      </c>
     </row>
     <row r="34">
       <c r="P34" s="92">
         <v>2.0</v>
       </c>
+      <c r="AA34" s="35">
+        <v>814.0</v>
+      </c>
+      <c r="AB34" s="35">
+        <v>104.32</v>
+      </c>
+      <c r="AC34" s="37">
+        <f t="shared" si="15"/>
+        <v>60.31</v>
+      </c>
+      <c r="AD34" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.421875</v>
+      </c>
     </row>
     <row r="35">
       <c r="H35" s="29" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="P35" s="92">
         <v>0.0</v>
+      </c>
+      <c r="AA35" s="36">
+        <v>1426.0</v>
+      </c>
+      <c r="AB35" s="35">
+        <v>101.23</v>
+      </c>
+      <c r="AC35" s="37">
+        <f t="shared" si="15"/>
+        <v>68.02</v>
+      </c>
+      <c r="AD35" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.3280648029</v>
       </c>
     </row>
     <row r="36">
@@ -13721,6 +13837,20 @@
       </c>
       <c r="P36" s="92">
         <v>1.0</v>
+      </c>
+      <c r="AA36" s="36">
+        <v>1447.0</v>
+      </c>
+      <c r="AB36" s="35">
+        <v>97.89</v>
+      </c>
+      <c r="AC36" s="37">
+        <f t="shared" si="15"/>
+        <v>138.76</v>
+      </c>
+      <c r="AD36" s="93">
+        <f t="shared" si="16"/>
+        <v>0.4175094494</v>
       </c>
     </row>
     <row r="37">
@@ -13740,6 +13870,20 @@
       <c r="P37" s="92">
         <v>0.0</v>
       </c>
+      <c r="AA37" s="35">
+        <v>136.0</v>
+      </c>
+      <c r="AB37" s="35">
+        <v>87.93</v>
+      </c>
+      <c r="AC37" s="37">
+        <f t="shared" si="15"/>
+        <v>58.8</v>
+      </c>
+      <c r="AD37" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.3312862504</v>
+      </c>
     </row>
     <row r="38">
       <c r="G38" s="29" t="s">
@@ -13751,13 +13895,27 @@
       <c r="P38" s="92">
         <v>2.0</v>
       </c>
+      <c r="AA38" s="36">
+        <v>1526.0</v>
+      </c>
+      <c r="AB38" s="35">
+        <v>85.82</v>
+      </c>
+      <c r="AC38" s="37">
+        <f t="shared" si="15"/>
+        <v>53.3</v>
+      </c>
+      <c r="AD38" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.3789326497</v>
+      </c>
     </row>
     <row r="39">
       <c r="C39" s="106" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D39" s="95">
-        <f t="shared" ref="D39:D221" si="15">IF(COUNTA(C39)=1,C39/1,"")</f>
+        <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
         <v>0</v>
       </c>
       <c r="G39" s="29" t="s">
@@ -13769,13 +13927,27 @@
       <c r="P39" s="92">
         <v>2.0</v>
       </c>
+      <c r="AA39" s="35">
+        <v>952.0</v>
+      </c>
+      <c r="AB39" s="35">
+        <v>78.09</v>
+      </c>
+      <c r="AC39" s="37">
+        <f t="shared" si="15"/>
+        <v>73.76</v>
+      </c>
+      <c r="AD39" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.05544884108</v>
+      </c>
     </row>
     <row r="40">
       <c r="C40" s="107" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D40" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="G40" s="29" t="s">
@@ -13787,83 +13959,151 @@
       <c r="P40" s="92">
         <v>0.0</v>
       </c>
+      <c r="AA40" s="36">
+        <v>1606.0</v>
+      </c>
+      <c r="AB40" s="35">
+        <v>77.21</v>
+      </c>
+      <c r="AC40" s="37">
+        <f t="shared" si="15"/>
+        <v>75.05</v>
+      </c>
+      <c r="AD40" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.02797565082</v>
+      </c>
     </row>
     <row r="41">
       <c r="C41" s="107" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="D41" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.36</v>
       </c>
       <c r="P41" s="92">
         <v>1.0</v>
       </c>
+      <c r="AA41" s="36">
+        <v>1164.0</v>
+      </c>
+      <c r="AB41" s="35">
+        <v>76.05</v>
+      </c>
+      <c r="AC41" s="37">
+        <f t="shared" si="15"/>
+        <v>26.27</v>
+      </c>
+      <c r="AD41" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.6545693623</v>
+      </c>
     </row>
     <row r="42">
       <c r="C42" s="107" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D42" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.25</v>
       </c>
       <c r="P42" s="92">
         <v>1.0</v>
       </c>
+      <c r="AA42" s="36">
+        <v>1448.0</v>
+      </c>
+      <c r="AB42" s="35">
+        <v>71.77</v>
+      </c>
+      <c r="AC42" s="37">
+        <f t="shared" si="15"/>
+        <v>39.69</v>
+      </c>
+      <c r="AD42" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.4469834193</v>
+      </c>
     </row>
     <row r="43">
       <c r="C43" s="107" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D43" s="95">
+        <f t="shared" si="17"/>
+        <v>0.68</v>
+      </c>
+      <c r="P43" s="92"/>
+      <c r="AA43" s="36">
+        <v>1614.0</v>
+      </c>
+      <c r="AB43" s="35">
+        <v>68.01</v>
+      </c>
+      <c r="AC43" s="37">
         <f t="shared" si="15"/>
-        <v>0.68</v>
-      </c>
-      <c r="P43" s="92"/>
+        <v>67.42</v>
+      </c>
+      <c r="AD43" s="93">
+        <f t="shared" si="16"/>
+        <v>-0.008675194824</v>
+      </c>
     </row>
     <row r="44">
       <c r="C44" s="107" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D44" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P44" s="92"/>
+      <c r="AB44" s="37">
+        <f t="shared" ref="AB44:AD44" si="18">AVERAGE(AB29:AB43)</f>
+        <v>106.338</v>
+      </c>
+      <c r="AC44" s="37">
+        <f t="shared" si="18"/>
+        <v>87.95266667</v>
+      </c>
+      <c r="AD44" s="93">
+        <f t="shared" si="18"/>
+        <v>-0.2009168941</v>
+      </c>
     </row>
     <row r="45">
       <c r="C45" s="107" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D45" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>11.25</v>
       </c>
       <c r="P45" s="92"/>
     </row>
     <row r="46">
       <c r="C46" s="107" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D46" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>9.76</v>
       </c>
       <c r="G46" s="66" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H46" s="66" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="P46" s="92"/>
     </row>
     <row r="47">
       <c r="C47" s="107" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D47" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>10.4</v>
       </c>
       <c r="G47" s="71" t="s">
@@ -13873,13 +14113,19 @@
         <v>0.376453591155815</v>
       </c>
       <c r="P47" s="92"/>
+      <c r="AA47" s="35" t="s">
+        <v>3</v>
+      </c>
+      <c r="AB47" s="35" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="48">
       <c r="C48" s="107" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D48" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>10.84</v>
       </c>
       <c r="G48" s="71" t="s">
@@ -13889,20 +14135,26 @@
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="35" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="K48" s="93">
         <f>AVERAGE(H47:H51)</f>
         <v>0.326199044</v>
       </c>
       <c r="P48" s="92"/>
+      <c r="AA48" s="35">
+        <v>136.0</v>
+      </c>
+      <c r="AB48" s="35">
+        <v>58.8</v>
+      </c>
     </row>
     <row r="49">
       <c r="C49" s="107" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D49" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.37</v>
       </c>
       <c r="G49" s="71" t="s">
@@ -13912,20 +14164,26 @@
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="35" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K49" s="93">
         <f>MEDIAN(H47:H51)</f>
         <v>0.3667873968</v>
       </c>
       <c r="P49" s="92"/>
+      <c r="AA49" s="36">
+        <v>1051.0</v>
+      </c>
+      <c r="AB49" s="35">
+        <v>263.81</v>
+      </c>
     </row>
     <row r="50">
       <c r="C50" s="107" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="D50" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>10.22</v>
       </c>
       <c r="G50" s="71" t="s">
@@ -13935,20 +14193,26 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="35" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="K50" s="93">
         <f>PERCENTILE(H47:H51,0.25)</f>
         <v>0.2474460363</v>
       </c>
       <c r="P50" s="92"/>
+      <c r="AA50" s="35">
+        <v>112.0</v>
+      </c>
+      <c r="AB50" s="35">
+        <v>130.76</v>
+      </c>
     </row>
     <row r="51">
       <c r="C51" s="107" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D51" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.79</v>
       </c>
       <c r="G51" s="71" t="s">
@@ -13958,164 +14222,236 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="35" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="K51" s="93">
         <f>PERCENTILE(H47:H51,0.75)</f>
         <v>0.3764535912</v>
       </c>
       <c r="P51" s="92"/>
+      <c r="AA51" s="36">
+        <v>1545.0</v>
+      </c>
+      <c r="AB51" s="35">
+        <v>101.16</v>
+      </c>
     </row>
     <row r="52">
       <c r="C52" s="107" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D52" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>5.44</v>
       </c>
       <c r="P52" s="92"/>
+      <c r="AA52" s="36">
+        <v>1447.0</v>
+      </c>
+      <c r="AB52" s="35">
+        <v>138.76</v>
+      </c>
     </row>
     <row r="53">
       <c r="C53" s="107" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D53" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.3</v>
       </c>
       <c r="P53" s="92"/>
+      <c r="AA53" s="36">
+        <v>1426.0</v>
+      </c>
+      <c r="AB53" s="35">
+        <v>68.02</v>
+      </c>
     </row>
     <row r="54">
       <c r="C54" s="107" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="D54" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.81</v>
       </c>
       <c r="P54" s="92"/>
+      <c r="AA54" s="36">
+        <v>1475.0</v>
+      </c>
+      <c r="AB54" s="35">
+        <v>83.5</v>
+      </c>
     </row>
     <row r="55">
       <c r="C55" s="107" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D55" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6.54</v>
       </c>
       <c r="P55" s="92"/>
+      <c r="AA55" s="36">
+        <v>1606.0</v>
+      </c>
+      <c r="AB55" s="35">
+        <v>75.05</v>
+      </c>
     </row>
     <row r="56">
       <c r="C56" s="107" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D56" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.77</v>
       </c>
       <c r="P56" s="92"/>
+      <c r="AA56" s="36">
+        <v>1614.0</v>
+      </c>
+      <c r="AB56" s="35">
+        <v>67.42</v>
+      </c>
     </row>
     <row r="57">
       <c r="C57" s="107" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D57" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6.59</v>
       </c>
       <c r="P57" s="92"/>
+      <c r="AA57" s="35">
+        <v>814.0</v>
+      </c>
+      <c r="AB57" s="35">
+        <v>60.31</v>
+      </c>
     </row>
     <row r="58">
       <c r="C58" s="107" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D58" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.77</v>
       </c>
       <c r="G58" s="109" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H58" s="110"/>
       <c r="P58" s="92"/>
+      <c r="AA58" s="35">
+        <v>752.0</v>
+      </c>
+      <c r="AB58" s="35">
+        <v>78.68</v>
+      </c>
     </row>
     <row r="59">
       <c r="C59" s="107" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D59" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6.95</v>
       </c>
       <c r="G59" s="110"/>
       <c r="H59" s="111" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="P59" s="92"/>
+      <c r="AA59" s="35">
+        <v>952.0</v>
+      </c>
+      <c r="AB59" s="35">
+        <v>73.76</v>
+      </c>
     </row>
     <row r="60">
       <c r="C60" s="107" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D60" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.11</v>
       </c>
       <c r="G60" s="110"/>
       <c r="H60" s="111" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="P60" s="92"/>
+      <c r="AA60" s="36">
+        <v>1526.0</v>
+      </c>
+      <c r="AB60" s="35">
+        <v>53.3</v>
+      </c>
     </row>
     <row r="61">
       <c r="C61" s="107" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D61" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.73</v>
       </c>
       <c r="G61" s="110"/>
       <c r="H61" s="111" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="P61" s="92"/>
+      <c r="AA61" s="36">
+        <v>1448.0</v>
+      </c>
+      <c r="AB61" s="35">
+        <v>39.69</v>
+      </c>
     </row>
     <row r="62">
       <c r="C62" s="107" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D62" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.8</v>
       </c>
       <c r="G62" s="110"/>
       <c r="H62" s="111" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="P62" s="92"/>
+      <c r="AA62" s="36">
+        <v>1164.0</v>
+      </c>
+      <c r="AB62" s="35">
+        <v>26.27</v>
+      </c>
     </row>
     <row r="63">
       <c r="C63" s="107" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D63" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>5.1</v>
       </c>
       <c r="G63" s="110"/>
       <c r="H63" s="111" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="P63" s="92"/>
     </row>
     <row r="64">
       <c r="C64" s="107" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D64" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>5.36</v>
       </c>
       <c r="P64" s="92"/>
@@ -14125,37 +14461,37 @@
         <v>122</v>
       </c>
       <c r="D65" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.68</v>
       </c>
       <c r="P65" s="92"/>
     </row>
     <row r="66">
       <c r="C66" s="107" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="D66" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.73</v>
       </c>
       <c r="P66" s="92"/>
     </row>
     <row r="67">
       <c r="C67" s="107" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D67" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.56</v>
       </c>
       <c r="P67" s="92"/>
     </row>
     <row r="68">
       <c r="C68" s="107" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D68" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.46</v>
       </c>
       <c r="P68" s="92"/>
@@ -14165,27 +14501,27 @@
         <v>102</v>
       </c>
       <c r="D69" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.67</v>
       </c>
       <c r="P69" s="92"/>
     </row>
     <row r="70">
       <c r="C70" s="107" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D70" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.59</v>
       </c>
       <c r="P70" s="92"/>
     </row>
     <row r="71">
       <c r="C71" s="107" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D71" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.55</v>
       </c>
       <c r="F71" s="112"/>
@@ -14193,330 +14529,330 @@
     </row>
     <row r="72">
       <c r="C72" s="107" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D72" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.5</v>
       </c>
       <c r="P72" s="92"/>
     </row>
     <row r="73">
       <c r="C73" s="107" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D73" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.73</v>
       </c>
       <c r="P73" s="92"/>
     </row>
     <row r="74">
       <c r="C74" s="107" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D74" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.68</v>
       </c>
       <c r="P74" s="92"/>
     </row>
     <row r="75">
       <c r="C75" s="107" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D75" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.89</v>
       </c>
       <c r="P75" s="92"/>
     </row>
     <row r="76">
       <c r="C76" s="107" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D76" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.48</v>
       </c>
       <c r="P76" s="92"/>
     </row>
     <row r="77">
       <c r="C77" s="107" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D77" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.32</v>
       </c>
       <c r="P77" s="92"/>
     </row>
     <row r="78">
       <c r="C78" s="107" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D78" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.7</v>
       </c>
       <c r="P78" s="113"/>
     </row>
     <row r="79">
       <c r="C79" s="107" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D79" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.85</v>
       </c>
       <c r="P79" s="113"/>
     </row>
     <row r="80">
       <c r="C80" s="107" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D80" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.66</v>
       </c>
       <c r="P80" s="113"/>
     </row>
     <row r="81">
       <c r="C81" s="107" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D81" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.38</v>
       </c>
       <c r="P81" s="113"/>
     </row>
     <row r="82">
       <c r="C82" s="107" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D82" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.46</v>
       </c>
       <c r="P82" s="113"/>
     </row>
     <row r="83">
       <c r="C83" s="107" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D83" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.26</v>
       </c>
       <c r="P83" s="113"/>
     </row>
     <row r="84">
       <c r="C84" s="107" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D84" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.96</v>
       </c>
       <c r="P84" s="113"/>
     </row>
     <row r="85">
       <c r="C85" s="107" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D85" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6.1</v>
       </c>
       <c r="P85" s="113"/>
     </row>
     <row r="86">
       <c r="C86" s="107" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D86" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6</v>
       </c>
       <c r="P86" s="113"/>
     </row>
     <row r="87">
       <c r="C87" s="107" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D87" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6.42</v>
       </c>
       <c r="P87" s="113"/>
     </row>
     <row r="88">
       <c r="C88" s="107" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D88" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.62</v>
       </c>
       <c r="P88" s="113"/>
     </row>
     <row r="89">
       <c r="C89" s="107" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D89" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.03</v>
       </c>
       <c r="P89" s="113"/>
     </row>
     <row r="90">
       <c r="C90" s="107" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D90" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.51</v>
       </c>
       <c r="P90" s="113"/>
     </row>
     <row r="91">
       <c r="C91" s="107" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D91" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.4</v>
       </c>
       <c r="P91" s="113"/>
     </row>
     <row r="92">
       <c r="C92" s="107" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D92" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.59</v>
       </c>
       <c r="P92" s="113"/>
     </row>
     <row r="93">
       <c r="C93" s="107" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D93" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.61</v>
       </c>
       <c r="P93" s="113"/>
     </row>
     <row r="94">
       <c r="C94" s="107" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D94" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.6</v>
       </c>
       <c r="P94" s="113"/>
     </row>
     <row r="95">
       <c r="C95" s="107" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D95" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.05</v>
       </c>
       <c r="P95" s="113"/>
     </row>
     <row r="96">
       <c r="C96" s="107" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D96" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.04</v>
       </c>
       <c r="P96" s="113"/>
     </row>
     <row r="97">
       <c r="C97" s="107" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D97" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.18</v>
       </c>
       <c r="P97" s="113"/>
     </row>
     <row r="98">
       <c r="C98" s="107" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D98" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P98" s="113"/>
     </row>
     <row r="99">
       <c r="C99" s="107" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D99" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P99" s="113"/>
     </row>
     <row r="100">
       <c r="C100" s="107" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D100" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.25</v>
       </c>
       <c r="P100" s="113"/>
     </row>
     <row r="101">
       <c r="C101" s="107" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D101" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P101" s="113"/>
     </row>
     <row r="102">
       <c r="C102" s="107" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D102" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0</v>
       </c>
       <c r="P102" s="113"/>
     </row>
     <row r="103">
       <c r="C103" s="107" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D103" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.21</v>
       </c>
       <c r="P103" s="113"/>
     </row>
     <row r="104">
       <c r="C104" s="107" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D104" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.12</v>
       </c>
       <c r="N104" s="114"/>
@@ -14524,10 +14860,10 @@
     </row>
     <row r="105">
       <c r="C105" s="107" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D105" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>10.75</v>
       </c>
       <c r="N105" s="14"/>
@@ -14535,10 +14871,10 @@
     </row>
     <row r="106">
       <c r="C106" s="107" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D106" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>10.43</v>
       </c>
       <c r="N106" s="14"/>
@@ -14546,10 +14882,10 @@
     </row>
     <row r="107">
       <c r="C107" s="107" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D107" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>11.53</v>
       </c>
       <c r="N107" s="14"/>
@@ -14557,10 +14893,10 @@
     </row>
     <row r="108">
       <c r="C108" s="107" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D108" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>10.85</v>
       </c>
       <c r="N108" s="14"/>
@@ -14568,10 +14904,10 @@
     </row>
     <row r="109">
       <c r="C109" s="107" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D109" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>12.26</v>
       </c>
       <c r="N109" s="14"/>
@@ -14579,10 +14915,10 @@
     </row>
     <row r="110">
       <c r="C110" s="107" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D110" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>6.98</v>
       </c>
       <c r="N110" s="14"/>
@@ -14590,10 +14926,10 @@
     </row>
     <row r="111">
       <c r="C111" s="107" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D111" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.25</v>
       </c>
       <c r="N111" s="14"/>
@@ -14601,180 +14937,180 @@
     </row>
     <row r="112">
       <c r="C112" s="107" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D112" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>7.63</v>
       </c>
       <c r="P112" s="113"/>
     </row>
     <row r="113">
       <c r="C113" s="107" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D113" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>7.01</v>
       </c>
       <c r="P113" s="113"/>
     </row>
     <row r="114">
       <c r="C114" s="107" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D114" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8</v>
       </c>
       <c r="P114" s="113"/>
     </row>
     <row r="115">
       <c r="C115" s="107" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D115" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>11.16</v>
       </c>
       <c r="P115" s="113"/>
     </row>
     <row r="116">
       <c r="C116" s="107" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D116" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>7.22</v>
       </c>
       <c r="P116" s="113"/>
     </row>
     <row r="117">
       <c r="C117" s="107" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D117" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.7</v>
       </c>
       <c r="P117" s="113"/>
     </row>
     <row r="118">
       <c r="C118" s="107" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D118" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>11.55</v>
       </c>
       <c r="P118" s="113"/>
     </row>
     <row r="119">
       <c r="C119" s="107" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D119" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>11.18</v>
       </c>
       <c r="P119" s="113"/>
     </row>
     <row r="120">
       <c r="C120" s="107" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D120" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>11.69</v>
       </c>
       <c r="P120" s="113"/>
     </row>
     <row r="121">
       <c r="C121" s="107" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D121" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>4.09</v>
       </c>
       <c r="P121" s="113"/>
     </row>
     <row r="122">
       <c r="C122" s="107" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D122" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.17</v>
       </c>
       <c r="P122" s="113"/>
     </row>
     <row r="123">
       <c r="C123" s="107" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D123" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.85</v>
       </c>
       <c r="P123" s="113"/>
     </row>
     <row r="124">
       <c r="C124" s="107" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D124" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>12.66</v>
       </c>
       <c r="P124" s="113"/>
     </row>
     <row r="125">
       <c r="C125" s="107" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D125" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>12.45</v>
       </c>
       <c r="P125" s="113"/>
     </row>
     <row r="126">
       <c r="C126" s="107" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D126" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>8.98</v>
       </c>
       <c r="P126" s="113"/>
     </row>
     <row r="127">
       <c r="C127" s="107" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D127" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>3.04</v>
       </c>
       <c r="P127" s="113"/>
     </row>
     <row r="128">
       <c r="C128" s="107" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D128" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.3</v>
       </c>
       <c r="P128" s="113"/>
     </row>
     <row r="129">
       <c r="C129" s="107" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D129" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.99</v>
       </c>
       <c r="P129" s="113"/>
@@ -14784,47 +15120,47 @@
         <v>131</v>
       </c>
       <c r="D130" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>2.8</v>
       </c>
       <c r="P130" s="113"/>
     </row>
     <row r="131">
       <c r="C131" s="107" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D131" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.23</v>
       </c>
       <c r="P131" s="113"/>
     </row>
     <row r="132">
       <c r="C132" s="107" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D132" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.25</v>
       </c>
       <c r="P132" s="113"/>
     </row>
     <row r="133">
       <c r="C133" s="107" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D133" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>1.25</v>
       </c>
       <c r="P133" s="113"/>
     </row>
     <row r="134">
       <c r="C134" s="107" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D134" s="95">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v>0.8</v>
       </c>
       <c r="P134" s="113"/>
@@ -14832,7 +15168,7 @@
     <row r="135">
       <c r="C135" s="107"/>
       <c r="D135" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="P135" s="113"/>
@@ -14840,7 +15176,7 @@
     <row r="136">
       <c r="C136" s="107"/>
       <c r="D136" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="P136" s="113"/>
@@ -14848,7 +15184,7 @@
     <row r="137">
       <c r="C137" s="107"/>
       <c r="D137" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="P137" s="113"/>
@@ -14856,7 +15192,7 @@
     <row r="138">
       <c r="C138" s="107"/>
       <c r="D138" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="P138" s="113"/>
@@ -14864,7 +15200,7 @@
     <row r="139">
       <c r="C139" s="107"/>
       <c r="D139" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="P139" s="113"/>
@@ -14872,7 +15208,7 @@
     <row r="140">
       <c r="C140" s="107"/>
       <c r="D140" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H140" s="35">
@@ -14889,7 +15225,7 @@
     <row r="141">
       <c r="C141" s="107"/>
       <c r="D141" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H141" s="35">
@@ -14906,7 +15242,7 @@
     <row r="142">
       <c r="C142" s="107"/>
       <c r="D142" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H142" s="35">
@@ -14923,7 +15259,7 @@
     <row r="143">
       <c r="C143" s="107"/>
       <c r="D143" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H143" s="35">
@@ -14940,7 +15276,7 @@
     <row r="144">
       <c r="C144" s="107"/>
       <c r="D144" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H144" s="35">
@@ -14957,7 +15293,7 @@
     <row r="145">
       <c r="C145" s="107"/>
       <c r="D145" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H145" s="35">
@@ -14974,7 +15310,7 @@
     <row r="146">
       <c r="C146" s="107"/>
       <c r="D146" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H146" s="35">
@@ -14991,7 +15327,7 @@
     <row r="147">
       <c r="C147" s="107"/>
       <c r="D147" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H147" s="35">
@@ -15008,7 +15344,7 @@
     <row r="148">
       <c r="C148" s="107"/>
       <c r="D148" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H148" s="35">
@@ -15025,7 +15361,7 @@
     <row r="149">
       <c r="C149" s="107"/>
       <c r="D149" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H149" s="35">
@@ -15042,7 +15378,7 @@
     <row r="150">
       <c r="C150" s="107"/>
       <c r="D150" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H150" s="35">
@@ -15059,7 +15395,7 @@
     <row r="151">
       <c r="C151" s="107"/>
       <c r="D151" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H151" s="35">
@@ -15076,7 +15412,7 @@
     <row r="152">
       <c r="C152" s="107"/>
       <c r="D152" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H152" s="35">
@@ -15093,7 +15429,7 @@
     <row r="153">
       <c r="C153" s="107"/>
       <c r="D153" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H153" s="35">
@@ -15110,7 +15446,7 @@
     <row r="154">
       <c r="C154" s="107"/>
       <c r="D154" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H154" s="35">
@@ -15127,7 +15463,7 @@
     <row r="155">
       <c r="C155" s="107"/>
       <c r="D155" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H155" s="35">
@@ -15144,7 +15480,7 @@
     <row r="156">
       <c r="C156" s="107"/>
       <c r="D156" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H156" s="35">
@@ -15161,7 +15497,7 @@
     <row r="157">
       <c r="C157" s="107"/>
       <c r="D157" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H157" s="35">
@@ -15178,7 +15514,7 @@
     <row r="158">
       <c r="C158" s="107"/>
       <c r="D158" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H158" s="35">
@@ -15195,7 +15531,7 @@
     <row r="159">
       <c r="C159" s="107"/>
       <c r="D159" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H159" s="35">
@@ -15212,7 +15548,7 @@
     <row r="160">
       <c r="C160" s="107"/>
       <c r="D160" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H160" s="35">
@@ -15229,7 +15565,7 @@
     <row r="161">
       <c r="C161" s="107"/>
       <c r="D161" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H161" s="35">
@@ -15246,7 +15582,7 @@
     <row r="162">
       <c r="C162" s="107"/>
       <c r="D162" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H162" s="35">
@@ -15263,7 +15599,7 @@
     <row r="163">
       <c r="C163" s="107"/>
       <c r="D163" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H163" s="35">
@@ -15280,7 +15616,7 @@
     <row r="164">
       <c r="C164" s="107"/>
       <c r="D164" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H164" s="35">
@@ -15297,7 +15633,7 @@
     <row r="165">
       <c r="C165" s="107"/>
       <c r="D165" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H165" s="35">
@@ -15314,7 +15650,7 @@
     <row r="166">
       <c r="C166" s="107"/>
       <c r="D166" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H166" s="35">
@@ -15331,7 +15667,7 @@
     <row r="167">
       <c r="C167" s="107"/>
       <c r="D167" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H167" s="35">
@@ -15348,7 +15684,7 @@
     <row r="168">
       <c r="C168" s="107"/>
       <c r="D168" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H168" s="35">
@@ -15365,7 +15701,7 @@
     <row r="169">
       <c r="C169" s="107"/>
       <c r="D169" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H169" s="35">
@@ -15382,7 +15718,7 @@
     <row r="170">
       <c r="C170" s="107"/>
       <c r="D170" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H170" s="35">
@@ -15399,7 +15735,7 @@
     <row r="171">
       <c r="C171" s="107"/>
       <c r="D171" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H171" s="35">
@@ -15416,7 +15752,7 @@
     <row r="172">
       <c r="C172" s="107"/>
       <c r="D172" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H172" s="35">
@@ -15433,7 +15769,7 @@
     <row r="173">
       <c r="C173" s="107"/>
       <c r="D173" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H173" s="35">
@@ -15450,7 +15786,7 @@
     <row r="174">
       <c r="C174" s="107"/>
       <c r="D174" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H174" s="35">
@@ -15467,7 +15803,7 @@
     <row r="175">
       <c r="C175" s="107"/>
       <c r="D175" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H175" s="35">
@@ -15484,7 +15820,7 @@
     <row r="176">
       <c r="C176" s="107"/>
       <c r="D176" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H176" s="35">
@@ -15501,7 +15837,7 @@
     <row r="177">
       <c r="C177" s="107"/>
       <c r="D177" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H177" s="35">
@@ -15518,7 +15854,7 @@
     <row r="178">
       <c r="C178" s="107"/>
       <c r="D178" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H178" s="35">
@@ -15535,7 +15871,7 @@
     <row r="179">
       <c r="C179" s="107"/>
       <c r="D179" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H179" s="35">
@@ -15552,7 +15888,7 @@
     <row r="180">
       <c r="C180" s="107"/>
       <c r="D180" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H180" s="35">
@@ -15569,7 +15905,7 @@
     <row r="181">
       <c r="C181" s="107"/>
       <c r="D181" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H181" s="35">
@@ -15586,7 +15922,7 @@
     <row r="182">
       <c r="C182" s="107"/>
       <c r="D182" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H182" s="35">
@@ -15603,7 +15939,7 @@
     <row r="183">
       <c r="C183" s="107"/>
       <c r="D183" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H183" s="35">
@@ -15620,7 +15956,7 @@
     <row r="184">
       <c r="C184" s="107"/>
       <c r="D184" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H184" s="35">
@@ -15637,7 +15973,7 @@
     <row r="185">
       <c r="C185" s="107"/>
       <c r="D185" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H185" s="35">
@@ -15654,7 +15990,7 @@
     <row r="186">
       <c r="C186" s="107"/>
       <c r="D186" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H186" s="35">
@@ -15671,7 +16007,7 @@
     <row r="187">
       <c r="C187" s="107"/>
       <c r="D187" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H187" s="35">
@@ -15688,7 +16024,7 @@
     <row r="188">
       <c r="C188" s="107"/>
       <c r="D188" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H188" s="35">
@@ -15705,7 +16041,7 @@
     <row r="189">
       <c r="C189" s="107"/>
       <c r="D189" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H189" s="35">
@@ -15722,7 +16058,7 @@
     <row r="190">
       <c r="C190" s="107"/>
       <c r="D190" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H190" s="35">
@@ -15739,7 +16075,7 @@
     <row r="191">
       <c r="C191" s="107"/>
       <c r="D191" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H191" s="35">
@@ -15756,7 +16092,7 @@
     <row r="192">
       <c r="C192" s="107"/>
       <c r="D192" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H192" s="35">
@@ -15773,7 +16109,7 @@
     <row r="193">
       <c r="C193" s="107"/>
       <c r="D193" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H193" s="35">
@@ -15790,7 +16126,7 @@
     <row r="194">
       <c r="C194" s="107"/>
       <c r="D194" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H194" s="35">
@@ -15807,7 +16143,7 @@
     <row r="195">
       <c r="C195" s="107"/>
       <c r="D195" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H195" s="35">
@@ -15824,7 +16160,7 @@
     <row r="196">
       <c r="C196" s="107"/>
       <c r="D196" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H196" s="35">
@@ -15841,7 +16177,7 @@
     <row r="197">
       <c r="C197" s="107"/>
       <c r="D197" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H197" s="35">
@@ -15858,7 +16194,7 @@
     <row r="198">
       <c r="C198" s="107"/>
       <c r="D198" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H198" s="35">
@@ -15875,7 +16211,7 @@
     <row r="199">
       <c r="C199" s="107"/>
       <c r="D199" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H199" s="35">
@@ -15892,7 +16228,7 @@
     <row r="200">
       <c r="C200" s="107"/>
       <c r="D200" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H200" s="35">
@@ -15909,7 +16245,7 @@
     <row r="201">
       <c r="C201" s="107"/>
       <c r="D201" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H201" s="35">
@@ -15926,7 +16262,7 @@
     <row r="202">
       <c r="C202" s="107"/>
       <c r="D202" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H202" s="35">
@@ -15943,7 +16279,7 @@
     <row r="203">
       <c r="C203" s="107"/>
       <c r="D203" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H203" s="35">
@@ -15960,7 +16296,7 @@
     <row r="204">
       <c r="C204" s="107"/>
       <c r="D204" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H204" s="35">
@@ -15977,7 +16313,7 @@
     <row r="205">
       <c r="C205" s="107"/>
       <c r="D205" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H205" s="35">
@@ -15994,7 +16330,7 @@
     <row r="206">
       <c r="C206" s="107"/>
       <c r="D206" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H206" s="35">
@@ -16011,7 +16347,7 @@
     <row r="207">
       <c r="C207" s="107"/>
       <c r="D207" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H207" s="35">
@@ -16028,7 +16364,7 @@
     <row r="208">
       <c r="C208" s="107"/>
       <c r="D208" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H208" s="35">
@@ -16045,7 +16381,7 @@
     <row r="209">
       <c r="C209" s="107"/>
       <c r="D209" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H209" s="35">
@@ -16062,7 +16398,7 @@
     <row r="210">
       <c r="C210" s="107"/>
       <c r="D210" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H210" s="35">
@@ -16079,7 +16415,7 @@
     <row r="211">
       <c r="C211" s="107"/>
       <c r="D211" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H211" s="35">
@@ -16096,7 +16432,7 @@
     <row r="212">
       <c r="C212" s="107"/>
       <c r="D212" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H212" s="35">
@@ -16113,7 +16449,7 @@
     <row r="213">
       <c r="C213" s="107"/>
       <c r="D213" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H213" s="35">
@@ -16130,7 +16466,7 @@
     <row r="214">
       <c r="C214" s="107"/>
       <c r="D214" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H214" s="35">
@@ -16147,7 +16483,7 @@
     <row r="215">
       <c r="C215" s="107"/>
       <c r="D215" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H215" s="35">
@@ -16164,7 +16500,7 @@
     <row r="216">
       <c r="C216" s="107"/>
       <c r="D216" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H216" s="35">
@@ -16181,7 +16517,7 @@
     <row r="217">
       <c r="C217" s="107"/>
       <c r="D217" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H217" s="35">
@@ -16198,7 +16534,7 @@
     <row r="218">
       <c r="C218" s="107"/>
       <c r="D218" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H218" s="35">
@@ -16215,7 +16551,7 @@
     <row r="219">
       <c r="C219" s="107"/>
       <c r="D219" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H219" s="35">
@@ -16232,7 +16568,7 @@
     <row r="220">
       <c r="C220" s="107"/>
       <c r="D220" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H220" s="35">
@@ -16249,7 +16585,7 @@
     <row r="221">
       <c r="C221" s="107"/>
       <c r="D221" s="95" t="str">
-        <f t="shared" si="15"/>
+        <f t="shared" si="17"/>
         <v/>
       </c>
       <c r="H221" s="35">
@@ -35634,6 +35970,18 @@
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF57BB8A"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD29:AD43">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="formula" val="0"/>
+        <cfvo type="max"/>
+        <color rgb="FFE67C73"/>
         <color rgb="FFFFFFFF"/>
         <color rgb="FF57BB8A"/>
       </colorScale>
@@ -35657,14 +36005,14 @@
     <row r="1">
       <c r="A1" s="75"/>
       <c r="B1" s="117" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="C1" s="118"/>
       <c r="D1" s="118"/>
       <c r="E1" s="118"/>
       <c r="F1" s="118"/>
       <c r="G1" s="119" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="H1" s="118"/>
       <c r="I1" s="118"/>
@@ -35692,19 +36040,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="121" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C2" s="122" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D2" s="122" t="s">
-        <v>246</v>
+        <v>145</v>
       </c>
       <c r="E2" s="122" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F2" s="123" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="G2" s="121">
         <v>1.0</v>
@@ -35716,25 +36064,25 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="122" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="K2" s="124" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="L2" s="122" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M2" s="125" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="N2" s="71" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="O2" s="71" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="P2" s="71" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="Q2" s="8"/>
       <c r="R2" s="8"/>
@@ -36517,7 +36865,7 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
       <c r="G27" s="139" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -36578,7 +36926,7 @@
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
       <c r="D29" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -36600,10 +36948,10 @@
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="65" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M29" s="65" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -36739,7 +37087,7 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
       <c r="G33" s="90" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
@@ -36916,7 +37264,7 @@
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
       <c r="F38" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G38" s="142">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelos en SPA, ITA y GER
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -38,6 +38,11 @@
     <comment authorId="0" ref="I4">
       <text>
         <t xml:space="preserve">el empate...</t>
+      </text>
+    </comment>
+    <comment authorId="0" ref="J4">
+      <text>
+        <t xml:space="preserve">crece gracias a doble oportunidad. en este caso de 0.55</t>
       </text>
     </comment>
     <comment authorId="0" ref="A1">
@@ -211,7 +216,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="374" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="225">
   <si>
     <t>id_country</t>
   </si>
@@ -660,28 +665,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>1.15</t>
+    <t>1.42</t>
   </si>
   <si>
-    <t>0.00</t>
+    <t>0.99</t>
   </si>
   <si>
-    <t>9.75</t>
+    <t>9.04</t>
   </si>
   <si>
-    <t>9.37</t>
+    <t>8.68</t>
   </si>
   <si>
-    <t>9.80</t>
-  </si>
-  <si>
-    <t>7.97</t>
-  </si>
-  <si>
-    <t>8.90</t>
+    <t>9.08</t>
   </si>
   <si>
     <t>7.33</t>
+  </si>
+  <si>
+    <t>8.24</t>
+  </si>
+  <si>
+    <t>6.55</t>
   </si>
   <si>
     <t>Country</t>
@@ -690,10 +695,10 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>7.98</t>
+    <t>8.69</t>
   </si>
   <si>
-    <t>5.97</t>
+    <t>6.59</t>
   </si>
   <si>
     <t>mean</t>
@@ -711,22 +716,22 @@
     <t>p25</t>
   </si>
   <si>
-    <t>5.79</t>
+    <t>6.42</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>5.65</t>
+    <t>6.28</t>
   </si>
   <si>
-    <t>6.08</t>
+    <t>6.71</t>
   </si>
   <si>
-    <t>5.75</t>
+    <t>6.38</t>
   </si>
   <si>
-    <t>5.87</t>
+    <t>6.50</t>
   </si>
   <si>
     <t>2.08</t>
@@ -735,100 +740,100 @@
     <t>2.22</t>
   </si>
   <si>
-    <t>11.10</t>
+    <t>16.91</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
   </si>
   <si>
+    <t>1.37</t>
+  </si>
+  <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>9.12</t>
+    <t>14.23</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
+    <t>10.34</t>
+  </si>
+  <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>2.26</t>
+    <t>4.57</t>
   </si>
   <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
-    <t>11.57</t>
-  </si>
-  <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>2.10</t>
+    <t>0.69</t>
   </si>
   <si>
-    <t>2.03</t>
+    <t>1.97</t>
   </si>
   <si>
-    <t>1.25</t>
+    <t>3.71</t>
   </si>
   <si>
-    <t>1.19</t>
+    <t>2.06</t>
   </si>
   <si>
-    <t>0.01</t>
+    <t>4.48</t>
   </si>
   <si>
-    <t>0.05</t>
+    <t>3.49</t>
   </si>
   <si>
-    <t>5.01</t>
+    <t>0.10</t>
   </si>
   <si>
-    <t>5.09</t>
+    <t>0.57</t>
   </si>
   <si>
-    <t>5.00</t>
+    <t>10.77</t>
   </si>
   <si>
-    <t>11.21</t>
+    <t>10.44</t>
   </si>
   <si>
-    <t>11.06</t>
+    <t>7.80</t>
   </si>
   <si>
-    <t>12.77</t>
+    <t>8.87</t>
   </si>
   <si>
-    <t>8.80</t>
+    <t>3.11</t>
   </si>
   <si>
-    <t>9.18</t>
+    <t>7.17</t>
   </si>
   <si>
-    <t>9.74</t>
+    <t>5.37</t>
   </si>
   <si>
-    <t>5.44</t>
+    <t>11.08</t>
   </si>
   <si>
-    <t>8.59</t>
+    <t>5.78</t>
   </si>
   <si>
-    <t>6.42</t>
+    <t>9.30</t>
   </si>
   <si>
-    <t>2.94</t>
+    <t>0.35</t>
   </si>
   <si>
-    <t>3.62</t>
+    <t>1.74</t>
   </si>
   <si>
-    <t>3.72</t>
-  </si>
-  <si>
-    <t>4.85</t>
+    <t>2.19</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -1928,35 +1933,35 @@
         <v>56.3636363636363</v>
       </c>
       <c r="G4" s="24">
-        <v>161.57</v>
+        <v>215.601161375027</v>
       </c>
       <c r="H4" s="24">
-        <f>-2.18+
-2291.53+
-384.61
+        <f>71.19+
+2310.5+
+384.17
 </f>
-        <v>2673.96</v>
+        <v>2765.86</v>
       </c>
       <c r="I4" s="24">
         <f t="shared" ref="I4:I8" si="1">H4/G4</f>
-        <v>16.54985455</v>
+        <v>12.82859509</v>
       </c>
       <c r="J4" s="19">
-        <v>5.0</v>
+        <v>25.0</v>
       </c>
       <c r="K4" s="19">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="L4" s="19">
-        <v>40.0</v>
+        <v>45.0</v>
       </c>
       <c r="M4" s="24">
         <f t="shared" ref="M4:M8" si="2">AVERAGE(J4:L4)</f>
-        <v>31.66666667</v>
+        <v>38.33333333</v>
       </c>
       <c r="N4" s="15">
         <f>M4*'Data preparation'!$C$2</f>
-        <v>9.5</v>
+        <v>9.583333333</v>
       </c>
     </row>
     <row r="5">
@@ -1983,31 +1988,31 @@
       </c>
       <c r="H5" s="24">
         <f>866.5+
-335.27+
+327.23+
 114.67
 </f>
-        <v>1316.44</v>
+        <v>1308.4</v>
       </c>
       <c r="I5" s="24">
         <f t="shared" si="1"/>
-        <v>8.937843703</v>
+        <v>8.88325689</v>
       </c>
       <c r="J5" s="24">
         <v>70.0</v>
       </c>
       <c r="K5" s="24">
-        <v>40.0</v>
+        <v>45.0</v>
       </c>
       <c r="L5" s="24">
         <v>25.0</v>
       </c>
       <c r="M5" s="24">
         <f t="shared" si="2"/>
-        <v>45</v>
+        <v>46.66666667</v>
       </c>
       <c r="N5" s="15">
         <f>M5*'Data preparation'!$C$2</f>
-        <v>13.5</v>
+        <v>11.66666667</v>
       </c>
       <c r="P5" s="25"/>
     </row>
@@ -2022,44 +2027,44 @@
         <v>45680.0</v>
       </c>
       <c r="D6" s="23">
-        <v>507.0</v>
+        <v>1051.0</v>
       </c>
       <c r="E6" s="23" t="s">
         <v>17</v>
       </c>
       <c r="F6" s="24">
-        <v>56.8807339449541</v>
+        <v>62.3853211009174</v>
       </c>
       <c r="G6" s="24">
-        <v>236.14</v>
+        <v>239.456083423093</v>
       </c>
       <c r="H6" s="24">
-        <f>197670.24+
-315.6+
-8.71
+        <f>2054.41+
+8839.74+
+91.53
 </f>
-        <v>197994.55</v>
+        <v>10985.68</v>
       </c>
       <c r="I6" s="24">
         <f t="shared" si="1"/>
-        <v>838.4625646</v>
+        <v>45.87764004</v>
       </c>
       <c r="J6" s="24">
-        <v>135.0</v>
+        <v>70.0</v>
       </c>
       <c r="K6" s="24">
+        <v>70.0</v>
+      </c>
+      <c r="L6" s="24">
         <v>25.0</v>
-      </c>
-      <c r="L6" s="24">
-        <v>10.0</v>
       </c>
       <c r="M6" s="24">
         <f t="shared" si="2"/>
-        <v>56.66666667</v>
+        <v>55</v>
       </c>
       <c r="N6" s="15">
         <f>M6*'Data preparation'!$C$2</f>
-        <v>17</v>
+        <v>13.75</v>
       </c>
     </row>
     <row r="7">
@@ -2073,7 +2078,7 @@
         <v>45677.0</v>
       </c>
       <c r="D7" s="23">
-        <v>1623.0</v>
+        <v>19.0</v>
       </c>
       <c r="E7" s="23" t="s">
         <v>17</v>
@@ -2082,35 +2087,35 @@
         <v>60.0</v>
       </c>
       <c r="G7" s="24">
-        <v>146.88838482783</v>
+        <v>183.94673286652</v>
       </c>
       <c r="H7" s="24">
-        <f>-1.86+
-3963.24+
-625.47
+        <f>-16.55+
+335.32+
+3063.41
 </f>
-        <v>4586.85</v>
+        <v>3382.18</v>
       </c>
       <c r="I7" s="24">
         <f t="shared" si="1"/>
-        <v>31.2267713</v>
+        <v>18.38673592</v>
       </c>
       <c r="J7" s="19">
         <v>10.0</v>
       </c>
       <c r="K7" s="19">
+        <v>25.0</v>
+      </c>
+      <c r="L7" s="19">
         <v>70.0</v>
-      </c>
-      <c r="L7" s="19">
-        <v>45.0</v>
       </c>
       <c r="M7" s="19">
         <f t="shared" si="2"/>
-        <v>41.66666667</v>
+        <v>35</v>
       </c>
       <c r="N7" s="15">
         <f>M7*'Data preparation'!$C$2</f>
-        <v>12.5</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="8">
@@ -2124,7 +2129,7 @@
         <v>45677.0</v>
       </c>
       <c r="D8" s="23">
-        <v>1545.0</v>
+        <v>112.0</v>
       </c>
       <c r="E8" s="23" t="s">
         <v>17</v>
@@ -2133,18 +2138,18 @@
         <v>57.2727272727272</v>
       </c>
       <c r="G8" s="24">
-        <v>114.811855439534</v>
+        <v>121.438244474087</v>
       </c>
       <c r="H8" s="24">
-        <f>266.16+
+        <f>360.49+
 3511.03+
 12.5
 </f>
-        <v>3789.69</v>
+        <v>3884.02</v>
       </c>
       <c r="I8" s="24">
         <f t="shared" si="1"/>
-        <v>33.0078282</v>
+        <v>31.98349924</v>
       </c>
       <c r="J8" s="19">
         <v>45.0</v>
@@ -2161,7 +2166,7 @@
       </c>
       <c r="N8" s="15">
         <f>M8*'Data preparation'!$C$2</f>
-        <v>12.5</v>
+        <v>10.41666667</v>
       </c>
     </row>
     <row r="9" ht="20.25" customHeight="1">
@@ -11893,7 +11898,7 @@
       </c>
       <c r="N68" s="14">
         <f>L68*'Data preparation'!$C$2</f>
-        <v>9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="69">
@@ -11938,7 +11943,7 @@
       </c>
       <c r="N69" s="14">
         <f>L69*'Data preparation'!$C$2</f>
-        <v>9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="70">
@@ -11983,7 +11988,7 @@
       </c>
       <c r="N70" s="14">
         <f>L70*'Data preparation'!$C$2</f>
-        <v>7.5</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="71">
@@ -12027,7 +12032,7 @@
       </c>
       <c r="N71" s="14">
         <f>L71*'Data preparation'!$C$2</f>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="72">
@@ -12071,7 +12076,7 @@
       </c>
       <c r="N72" s="14">
         <f>L72*'Data preparation'!$C$2</f>
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="76">
@@ -12225,7 +12230,7 @@
       </c>
       <c r="R80" s="15">
         <f>P80*'Data preparation'!$C$2</f>
-        <v>9.5</v>
+        <v>7.916666667</v>
       </c>
     </row>
     <row r="81">
@@ -12280,7 +12285,7 @@
       </c>
       <c r="R81" s="61">
         <f>P81*'Data preparation'!$C$2/2</f>
-        <v>9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="82">
@@ -12335,7 +12340,7 @@
       </c>
       <c r="R82" s="61">
         <f>P82*'Data preparation'!$C$2/2</f>
-        <v>8.75</v>
+        <v>7.291666667</v>
       </c>
     </row>
     <row r="83">
@@ -12390,7 +12395,7 @@
       </c>
       <c r="R83" s="15">
         <f>P83*'Data preparation'!$C$2</f>
-        <v>10</v>
+        <v>8.333333333</v>
       </c>
     </row>
     <row r="84">
@@ -12445,7 +12450,7 @@
       </c>
       <c r="R84" s="15">
         <f>P84*'Data preparation'!$C$2</f>
-        <v>15</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="94">
@@ -12622,7 +12627,7 @@
       </c>
       <c r="U99" s="15">
         <f>T99*'Data preparation'!$C$2</f>
-        <v>9.5</v>
+        <v>7.916666667</v>
       </c>
     </row>
     <row r="100">
@@ -12683,7 +12688,7 @@
       </c>
       <c r="U100" s="61">
         <f>T100*'Data preparation'!$C$2/2</f>
-        <v>9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="101">
@@ -12744,7 +12749,7 @@
       </c>
       <c r="U101" s="61">
         <f>T101*'Data preparation'!$C$2/2</f>
-        <v>8.75</v>
+        <v>7.291666667</v>
       </c>
     </row>
     <row r="102">
@@ -12805,7 +12810,7 @@
       </c>
       <c r="U102" s="15">
         <f>T102*'Data preparation'!$C$2</f>
-        <v>13.5</v>
+        <v>11.25</v>
       </c>
     </row>
     <row r="103">
@@ -12866,7 +12871,7 @@
       </c>
       <c r="U103" s="15">
         <f>T103*'Data preparation'!$C$2</f>
-        <v>11</v>
+        <v>9.166666667</v>
       </c>
     </row>
   </sheetData>
@@ -13143,7 +13148,7 @@
         <v>84</v>
       </c>
       <c r="C2" s="19">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="L2" s="90"/>
     </row>
@@ -13154,7 +13159,7 @@
       </c>
       <c r="C3" s="15">
         <f>AVERAGE('Modelos actuales'!N4:N8)</f>
-        <v>13</v>
+        <v>10.83333333</v>
       </c>
       <c r="L3" s="90"/>
       <c r="P3" s="90"/>
@@ -14256,7 +14261,7 @@
       <c r="C37" s="34"/>
       <c r="D37" s="37">
         <f>AVERAGE(D39:D1775)</f>
-        <v>5.718823529</v>
+        <v>5.765625</v>
       </c>
       <c r="G37" s="31" t="s">
         <v>23</v>
@@ -14313,7 +14318,7 @@
       </c>
       <c r="D39" s="96">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>1.15</v>
+        <v>1.42</v>
       </c>
       <c r="G39" s="31" t="s">
         <v>25</v>
@@ -14345,7 +14350,7 @@
       </c>
       <c r="D40" s="96">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>0.99</v>
       </c>
       <c r="G40" s="31" t="s">
         <v>26</v>
@@ -14377,7 +14382,7 @@
       </c>
       <c r="D41" s="96">
         <f t="shared" si="17"/>
-        <v>9.75</v>
+        <v>9.04</v>
       </c>
       <c r="P41" s="93">
         <v>1.0</v>
@@ -14403,7 +14408,7 @@
       </c>
       <c r="D42" s="96">
         <f t="shared" si="17"/>
-        <v>9.37</v>
+        <v>8.68</v>
       </c>
       <c r="P42" s="93">
         <v>1.0</v>
@@ -14429,7 +14434,7 @@
       </c>
       <c r="D43" s="96">
         <f t="shared" si="17"/>
-        <v>9.8</v>
+        <v>9.08</v>
       </c>
       <c r="P43" s="93"/>
       <c r="AA43" s="36">
@@ -14453,7 +14458,7 @@
       </c>
       <c r="D44" s="96">
         <f t="shared" si="17"/>
-        <v>7.97</v>
+        <v>7.33</v>
       </c>
       <c r="P44" s="93"/>
       <c r="AB44" s="38">
@@ -14475,7 +14480,7 @@
       </c>
       <c r="D45" s="96">
         <f t="shared" si="17"/>
-        <v>8.9</v>
+        <v>8.24</v>
       </c>
       <c r="P45" s="93"/>
     </row>
@@ -14485,7 +14490,7 @@
       </c>
       <c r="D46" s="96">
         <f t="shared" si="17"/>
-        <v>7.33</v>
+        <v>6.55</v>
       </c>
       <c r="G46" s="67" t="s">
         <v>157</v>
@@ -14501,7 +14506,7 @@
       </c>
       <c r="D47" s="96">
         <f t="shared" si="17"/>
-        <v>7.98</v>
+        <v>8.69</v>
       </c>
       <c r="G47" s="72" t="s">
         <v>22</v>
@@ -14523,7 +14528,7 @@
       </c>
       <c r="D48" s="96">
         <f t="shared" si="17"/>
-        <v>5.97</v>
+        <v>6.59</v>
       </c>
       <c r="G48" s="72" t="s">
         <v>23</v>
@@ -14610,7 +14615,7 @@
       </c>
       <c r="D51" s="96">
         <f t="shared" si="17"/>
-        <v>5.79</v>
+        <v>6.42</v>
       </c>
       <c r="G51" s="72" t="s">
         <v>26</v>
@@ -14639,7 +14644,7 @@
       </c>
       <c r="D52" s="96">
         <f t="shared" si="17"/>
-        <v>5.65</v>
+        <v>6.28</v>
       </c>
       <c r="P52" s="93"/>
       <c r="AA52" s="36">
@@ -14655,7 +14660,7 @@
       </c>
       <c r="D53" s="96">
         <f t="shared" si="17"/>
-        <v>6.08</v>
+        <v>6.71</v>
       </c>
       <c r="P53" s="93"/>
       <c r="AA53" s="36">
@@ -14671,7 +14676,7 @@
       </c>
       <c r="D54" s="96">
         <f t="shared" si="17"/>
-        <v>5.75</v>
+        <v>6.38</v>
       </c>
       <c r="P54" s="93"/>
       <c r="AA54" s="36">
@@ -14687,7 +14692,7 @@
       </c>
       <c r="D55" s="96">
         <f t="shared" si="17"/>
-        <v>5.87</v>
+        <v>6.5</v>
       </c>
       <c r="P55" s="93"/>
       <c r="AA55" s="36">
@@ -14735,7 +14740,7 @@
       </c>
       <c r="D58" s="96">
         <f t="shared" si="17"/>
-        <v>11.1</v>
+        <v>16.91</v>
       </c>
       <c r="G58" s="109" t="s">
         <v>175</v>
@@ -14751,15 +14756,15 @@
     </row>
     <row r="59">
       <c r="C59" s="107" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="D59" s="96">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>1.37</v>
       </c>
       <c r="G59" s="110"/>
       <c r="H59" s="111" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="P59" s="93"/>
       <c r="AA59" s="32">
@@ -14771,15 +14776,15 @@
     </row>
     <row r="60">
       <c r="C60" s="107" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D60" s="96">
         <f t="shared" si="17"/>
-        <v>9.12</v>
+        <v>14.23</v>
       </c>
       <c r="G60" s="110"/>
       <c r="H60" s="111" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="P60" s="93"/>
       <c r="AA60" s="36">
@@ -14791,15 +14796,15 @@
     </row>
     <row r="61">
       <c r="C61" s="107" t="s">
-        <v>152</v>
+        <v>180</v>
       </c>
       <c r="D61" s="96">
         <f t="shared" si="17"/>
-        <v>9.37</v>
+        <v>10.34</v>
       </c>
       <c r="G61" s="110"/>
       <c r="H61" s="111" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="P61" s="93"/>
       <c r="AA61" s="36">
@@ -14811,15 +14816,15 @@
     </row>
     <row r="62">
       <c r="C62" s="107" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D62" s="96">
         <f t="shared" si="17"/>
-        <v>2.26</v>
+        <v>4.57</v>
       </c>
       <c r="G62" s="110"/>
       <c r="H62" s="111" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="P62" s="93"/>
       <c r="AA62" s="36">
@@ -14831,55 +14836,55 @@
     </row>
     <row r="63">
       <c r="C63" s="107" t="s">
-        <v>182</v>
+        <v>139</v>
       </c>
       <c r="D63" s="96">
         <f t="shared" si="17"/>
-        <v>11.57</v>
+        <v>4.73</v>
       </c>
       <c r="G63" s="110"/>
       <c r="H63" s="111" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="P63" s="93"/>
     </row>
     <row r="64">
       <c r="C64" s="107" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D64" s="96">
         <f t="shared" si="17"/>
-        <v>2.1</v>
+        <v>0.69</v>
       </c>
       <c r="P64" s="93"/>
     </row>
     <row r="65">
       <c r="C65" s="107" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="D65" s="96">
         <f t="shared" si="17"/>
-        <v>2.08</v>
+        <v>1.37</v>
       </c>
       <c r="P65" s="93"/>
     </row>
     <row r="66">
       <c r="C66" s="107" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D66" s="96">
         <f t="shared" si="17"/>
-        <v>2.03</v>
+        <v>1.97</v>
       </c>
       <c r="P66" s="93"/>
     </row>
     <row r="67">
       <c r="C67" s="107" t="s">
-        <v>186</v>
+        <v>102</v>
       </c>
       <c r="D67" s="96">
         <f t="shared" si="17"/>
-        <v>1.25</v>
+        <v>3.67</v>
       </c>
       <c r="P67" s="93"/>
     </row>
@@ -14889,218 +14894,212 @@
       </c>
       <c r="D68" s="96">
         <f t="shared" si="17"/>
-        <v>1.19</v>
+        <v>3.71</v>
       </c>
       <c r="P68" s="93"/>
     </row>
     <row r="69">
       <c r="C69" s="107" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D69" s="96">
         <f t="shared" si="17"/>
-        <v>1.25</v>
+        <v>2.06</v>
       </c>
       <c r="P69" s="93"/>
     </row>
     <row r="70">
       <c r="C70" s="107" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D70" s="96">
         <f t="shared" si="17"/>
-        <v>0.01</v>
+        <v>4.48</v>
       </c>
       <c r="P70" s="93"/>
     </row>
     <row r="71">
       <c r="C71" s="107" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D71" s="96">
         <f t="shared" si="17"/>
-        <v>0.05</v>
+        <v>3.49</v>
       </c>
       <c r="F71" s="112"/>
       <c r="P71" s="93"/>
     </row>
     <row r="72">
       <c r="C72" s="107" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="D72" s="96">
         <f t="shared" si="17"/>
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="P72" s="93"/>
     </row>
     <row r="73">
       <c r="C73" s="107" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D73" s="96">
         <f t="shared" si="17"/>
-        <v>5.01</v>
+        <v>0.57</v>
       </c>
       <c r="P73" s="93"/>
     </row>
     <row r="74">
       <c r="C74" s="107" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D74" s="96">
         <f t="shared" si="17"/>
-        <v>5.09</v>
+        <v>10.77</v>
       </c>
       <c r="P74" s="93"/>
     </row>
     <row r="75">
       <c r="C75" s="107" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D75" s="96">
         <f t="shared" si="17"/>
-        <v>5</v>
+        <v>10.44</v>
       </c>
       <c r="P75" s="93"/>
     </row>
     <row r="76">
       <c r="C76" s="107" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D76" s="96">
         <f t="shared" si="17"/>
-        <v>11.21</v>
+        <v>7.8</v>
       </c>
       <c r="P76" s="93"/>
     </row>
     <row r="77">
       <c r="C77" s="107" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D77" s="96">
         <f t="shared" si="17"/>
-        <v>11.06</v>
+        <v>8.87</v>
       </c>
       <c r="P77" s="93"/>
     </row>
     <row r="78">
       <c r="C78" s="107" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D78" s="96">
         <f t="shared" si="17"/>
-        <v>12.77</v>
+        <v>3.11</v>
       </c>
       <c r="P78" s="113"/>
     </row>
     <row r="79">
       <c r="C79" s="107" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D79" s="96">
         <f t="shared" si="17"/>
-        <v>8.8</v>
+        <v>7.17</v>
       </c>
       <c r="P79" s="113"/>
     </row>
     <row r="80">
       <c r="C80" s="107" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D80" s="96">
         <f t="shared" si="17"/>
-        <v>9.18</v>
+        <v>5.37</v>
       </c>
       <c r="P80" s="113"/>
     </row>
     <row r="81">
       <c r="C81" s="107" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D81" s="96">
         <f t="shared" si="17"/>
-        <v>9.74</v>
+        <v>11.08</v>
       </c>
       <c r="P81" s="113"/>
     </row>
     <row r="82">
       <c r="C82" s="107" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D82" s="96">
         <f t="shared" si="17"/>
-        <v>5.44</v>
+        <v>5.78</v>
       </c>
       <c r="P82" s="113"/>
     </row>
     <row r="83">
       <c r="C83" s="107" t="s">
-        <v>136</v>
+        <v>202</v>
       </c>
       <c r="D83" s="96">
         <f t="shared" si="17"/>
-        <v>7.85</v>
+        <v>9.3</v>
       </c>
       <c r="P83" s="113"/>
     </row>
     <row r="84">
       <c r="C84" s="107" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="D84" s="96">
         <f t="shared" si="17"/>
-        <v>8.59</v>
+        <v>0.35</v>
       </c>
       <c r="P84" s="113"/>
     </row>
     <row r="85">
       <c r="C85" s="107" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D85" s="96">
         <f t="shared" si="17"/>
-        <v>6.42</v>
+        <v>1.74</v>
       </c>
       <c r="P85" s="113"/>
     </row>
     <row r="86">
       <c r="C86" s="107" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="D86" s="96">
         <f t="shared" si="17"/>
-        <v>2.94</v>
+        <v>2.19</v>
       </c>
       <c r="P86" s="113"/>
     </row>
     <row r="87">
-      <c r="C87" s="107" t="s">
-        <v>203</v>
-      </c>
-      <c r="D87" s="96">
+      <c r="C87" s="107"/>
+      <c r="D87" s="96" t="str">
         <f t="shared" si="17"/>
-        <v>3.62</v>
+        <v/>
       </c>
       <c r="P87" s="113"/>
     </row>
     <row r="88">
-      <c r="C88" s="107" t="s">
-        <v>204</v>
-      </c>
-      <c r="D88" s="96">
+      <c r="C88" s="107"/>
+      <c r="D88" s="96" t="str">
         <f t="shared" si="17"/>
-        <v>3.72</v>
+        <v/>
       </c>
       <c r="P88" s="113"/>
     </row>
     <row r="89">
-      <c r="C89" s="107" t="s">
-        <v>205</v>
-      </c>
-      <c r="D89" s="96">
+      <c r="C89" s="107"/>
+      <c r="D89" s="96" t="str">
         <f t="shared" si="17"/>
-        <v>4.85</v>
+        <v/>
       </c>
       <c r="P89" s="113"/>
     </row>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelos
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -38,31 +38,6 @@
     <comment authorId="0" ref="I4">
       <text>
         <t xml:space="preserve">el empate...</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="J4">
-      <text>
-        <t xml:space="preserve">crece gracias a doble oportunidad. en este caso de 0.45</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="L6">
-      <text>
-        <t xml:space="preserve">dp 0.45</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="J7">
-      <text>
-        <t xml:space="preserve">dp 0.55</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="J8">
-      <text>
-        <t xml:space="preserve">dp 0.45</t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="L8">
-      <text>
-        <t xml:space="preserve">dp 0.7</t>
       </text>
     </comment>
     <comment authorId="0" ref="A1">
@@ -236,7 +211,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="373" uniqueCount="230">
   <si>
     <t>id_country</t>
   </si>
@@ -256,12 +231,10 @@
     <t>test_accuracy</t>
   </si>
   <si>
-    <t>G/P sin bank 
-sin ea</t>
+    <t>ROI_sin_ea</t>
   </si>
   <si>
-    <t>G/P sin bank 
-con ea</t>
+    <t>ROI_con_ea</t>
   </si>
   <si>
     <t>Multiplicador ea</t>
@@ -319,6 +292,9 @@
   </si>
   <si>
     <t>SPA</t>
+  </si>
+  <si>
+    <t>Cambiaron por: 1) sacar dp? 2) Seleccionar modelo segun todo sin bank o por que?</t>
   </si>
   <si>
     <t>deberia cambiar el modelo en: ENG y en SPA</t>
@@ -693,28 +669,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>1.40</t>
+    <t>1.87</t>
   </si>
   <si>
-    <t>0.99</t>
+    <t>0.15</t>
   </si>
   <si>
-    <t>9.03</t>
+    <t>0.10</t>
   </si>
   <si>
-    <t>8.73</t>
+    <t>0.74</t>
   </si>
   <si>
-    <t>9.07</t>
+    <t>0.42</t>
   </si>
   <si>
-    <t>7.34</t>
+    <t>7.47</t>
   </si>
   <si>
-    <t>8.24</t>
+    <t>7.63</t>
   </si>
   <si>
-    <t>6.55</t>
+    <t>8.19</t>
   </si>
   <si>
     <t>Country</t>
@@ -723,10 +699,10 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>8.66</t>
+    <t>8.59</t>
   </si>
   <si>
-    <t>6.47</t>
+    <t>6.88</t>
   </si>
   <si>
     <t>mean</t>
@@ -738,7 +714,7 @@
     <t>median</t>
   </si>
   <si>
-    <t>7.76</t>
+    <t>8.02</t>
   </si>
   <si>
     <t>p25</t>
@@ -750,13 +726,13 @@
     <t>p75</t>
   </si>
   <si>
-    <t>6.28</t>
+    <t>6.35</t>
   </si>
   <si>
-    <t>6.71</t>
+    <t>6.77</t>
   </si>
   <si>
-    <t>6.38</t>
+    <t>6.44</t>
   </si>
   <si>
     <t>6.50</t>
@@ -765,10 +741,10 @@
     <t>2.08</t>
   </si>
   <si>
-    <t>2.22</t>
+    <t>2.11</t>
   </si>
   <si>
-    <t>9.93</t>
+    <t>9.79</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
@@ -780,19 +756,19 @@
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>7.87</t>
+    <t>8.62</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
-    <t>8.12</t>
+    <t>8.96</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>1.52</t>
+    <t>1.56</t>
   </si>
   <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
@@ -804,64 +780,70 @@
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>4.13</t>
-  </si>
-  <si>
-    <t>0.44</t>
-  </si>
-  <si>
-    <t>4.02</t>
+    <t>1.65</t>
   </si>
   <si>
     <t>2.05</t>
   </si>
   <si>
-    <t>1.55</t>
+    <t>1.90</t>
   </si>
   <si>
-    <t>0.23</t>
+    <t>5.60</t>
   </si>
   <si>
-    <t>0.28</t>
+    <t>1.00</t>
   </si>
   <si>
-    <t>4.84</t>
+    <t>1.24</t>
   </si>
   <si>
-    <t>5.00</t>
+    <t>3.38</t>
   </si>
   <si>
-    <t>10.04</t>
+    <t>6.48</t>
   </si>
   <si>
-    <t>9.79</t>
+    <t>6.96</t>
   </si>
   <si>
-    <t>11.52</t>
+    <t>3.53</t>
   </si>
   <si>
-    <t>0.50</t>
+    <t>4.04</t>
   </si>
   <si>
-    <t>7.63</t>
+    <t>5.12</t>
   </si>
   <si>
-    <t>1.35</t>
+    <t>4.35</t>
   </si>
   <si>
-    <t>7.46</t>
+    <t>1.20</t>
   </si>
   <si>
-    <t>9.85</t>
+    <t>3.69</t>
   </si>
   <si>
-    <t>1.75</t>
+    <t>0.68</t>
   </si>
   <si>
-    <t>0.64</t>
+    <t>10.90</t>
   </si>
   <si>
-    <t>1.95</t>
+    <t>1.13</t>
+  </si>
+  <si>
+    <t>2.16</t>
+  </si>
+  <si>
+    <t>1.98</t>
+  </si>
+  <si>
+    <t>1.52</t>
+  </si>
+  <si>
+    <t>2.17</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -1932,7 +1914,7 @@
       <c r="O1" s="8"/>
       <c r="P1" s="9"/>
     </row>
-    <row r="2" ht="39.0" customHeight="1">
+    <row r="2" ht="39.0" hidden="1" customHeight="1">
       <c r="A2" s="10">
         <v>6.0</v>
       </c>
@@ -1975,7 +1957,7 @@
       <c r="O2" s="19"/>
       <c r="P2" s="20"/>
     </row>
-    <row r="3">
+    <row r="3" hidden="1">
       <c r="A3" s="21">
         <v>167.0</v>
       </c>
@@ -2008,26 +1990,26 @@
         <v>45679.0</v>
       </c>
       <c r="D4" s="14">
-        <v>343.0</v>
+        <v>395.0</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>15</v>
       </c>
       <c r="F4" s="15">
-        <v>55.4545454545454</v>
+        <v>56.3636363636363</v>
       </c>
       <c r="G4" s="15">
-        <v>151.075582383826</v>
+        <v>266.829530869996</v>
       </c>
       <c r="H4" s="15">
-        <v>1170.81137331263</v>
+        <v>10540.9503330339</v>
       </c>
       <c r="I4" s="16">
         <f t="shared" ref="I4:I8" si="1">H4/G4</f>
-        <v>7.749838557</v>
+        <v>39.50443678</v>
       </c>
       <c r="J4" s="17">
-        <v>45.0</v>
+        <v>10.0</v>
       </c>
       <c r="K4" s="17">
         <v>45.0</v>
@@ -2037,11 +2019,11 @@
       </c>
       <c r="M4" s="16">
         <f t="shared" ref="M4:M8" si="2">AVERAGE(J4:L4)</f>
-        <v>45</v>
+        <v>33.33333333</v>
       </c>
       <c r="N4" s="23">
         <f>M4*'Data preparation'!$C$2</f>
-        <v>11.25</v>
+        <v>8.333333333</v>
       </c>
     </row>
     <row r="5">
@@ -2064,14 +2046,14 @@
         <v>57.7981651376146</v>
       </c>
       <c r="G5" s="15">
-        <v>148.784087751072</v>
+        <v>265.483623313594</v>
       </c>
       <c r="H5" s="15">
-        <v>1017.94254308676</v>
+        <v>8764.30228233083</v>
       </c>
       <c r="I5" s="16">
         <f t="shared" si="1"/>
-        <v>6.841743351</v>
+        <v>33.01259103</v>
       </c>
       <c r="J5" s="15">
         <v>70.0</v>
@@ -2112,14 +2094,14 @@
         <v>62.3853211009174</v>
       </c>
       <c r="G6" s="15">
-        <v>223.51380979724</v>
+        <v>620.745751732881</v>
       </c>
       <c r="H6" s="29">
-        <v>1767.19401451423</v>
+        <v>235388.618048197</v>
       </c>
       <c r="I6" s="16">
         <f t="shared" si="1"/>
-        <v>7.906419814</v>
+        <v>379.2029464</v>
       </c>
       <c r="J6" s="15">
         <v>70.0</v>
@@ -2128,15 +2110,15 @@
         <v>70.0</v>
       </c>
       <c r="L6" s="15">
-        <v>25.0</v>
+        <v>10.0</v>
       </c>
       <c r="M6" s="16">
         <f t="shared" si="2"/>
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="N6" s="23">
         <f>M6*'Data preparation'!$C$2</f>
-        <v>13.75</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="7">
@@ -2150,26 +2132,26 @@
         <v>45677.0</v>
       </c>
       <c r="D7" s="14">
-        <v>1658.0</v>
+        <v>1623.0</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>15</v>
       </c>
       <c r="F7" s="15">
-        <v>59.090909090909</v>
+        <v>60.0</v>
       </c>
       <c r="G7" s="15">
-        <v>138.271334532167</v>
+        <v>259.814577663094</v>
       </c>
       <c r="H7" s="15">
-        <v>1187.20111909535</v>
+        <v>26440.0274640769</v>
       </c>
       <c r="I7" s="16">
         <f t="shared" si="1"/>
-        <v>8.586024884</v>
+        <v>101.7649883</v>
       </c>
       <c r="J7" s="17">
-        <v>25.0</v>
+        <v>10.0</v>
       </c>
       <c r="K7" s="17">
         <v>70.0</v>
@@ -2179,11 +2161,11 @@
       </c>
       <c r="M7" s="24">
         <f t="shared" si="2"/>
-        <v>46.66666667</v>
+        <v>41.66666667</v>
       </c>
       <c r="N7" s="23">
         <f>M7*'Data preparation'!$C$2</f>
-        <v>11.66666667</v>
+        <v>10.41666667</v>
       </c>
     </row>
     <row r="8">
@@ -2197,40 +2179,40 @@
         <v>45677.0</v>
       </c>
       <c r="D8" s="14">
-        <v>1545.0</v>
+        <v>112.0</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="15">
-        <v>54.5454545454545</v>
+        <v>57.2727272727272</v>
       </c>
       <c r="G8" s="15">
-        <v>83.1939735526323</v>
+        <v>148.175027775313</v>
       </c>
       <c r="H8" s="15">
-        <v>1139.23923226552</v>
+        <v>14775.5109669633</v>
       </c>
       <c r="I8" s="16">
         <f t="shared" si="1"/>
-        <v>13.69377112</v>
+        <v>99.7166067</v>
       </c>
       <c r="J8" s="17">
-        <v>70.0</v>
+        <v>45.0</v>
       </c>
       <c r="K8" s="17">
         <v>70.0</v>
       </c>
       <c r="L8" s="17">
-        <v>45.0</v>
+        <v>10.0</v>
       </c>
       <c r="M8" s="24">
         <f t="shared" si="2"/>
-        <v>61.66666667</v>
+        <v>41.66666667</v>
       </c>
       <c r="N8" s="23">
         <f>M8*'Data preparation'!$C$2</f>
-        <v>15.41666667</v>
+        <v>10.41666667</v>
       </c>
     </row>
     <row r="9" ht="20.25" customHeight="1">
@@ -2259,23 +2241,8 @@
       <c r="A13" s="33"/>
       <c r="F13" s="34"/>
     </row>
-    <row r="15">
-      <c r="C15" s="35"/>
-    </row>
-    <row r="16">
-      <c r="C16" s="35"/>
-    </row>
-    <row r="17">
-      <c r="C17" s="35"/>
-    </row>
-    <row r="18">
-      <c r="C18" s="35"/>
-    </row>
     <row r="19">
       <c r="C19" s="35"/>
-    </row>
-    <row r="20">
-      <c r="C20" s="35"/>
     </row>
     <row r="27">
       <c r="A27" s="33"/>
@@ -9259,6 +9226,11 @@
       <c r="E26" s="31"/>
       <c r="F26" s="31"/>
     </row>
+    <row r="30">
+      <c r="D30" s="37" t="s">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -9540,13 +9512,13 @@
     </row>
     <row r="11">
       <c r="E11" s="49" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L11" s="37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M11" s="44" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N11" s="50" t="s">
         <v>26</v>
@@ -9556,10 +9528,10 @@
     </row>
     <row r="12">
       <c r="E12" s="49" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="L12" s="37" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="M12" s="44" t="s">
         <v>24</v>
@@ -9821,12 +9793,12 @@
     </row>
     <row r="24">
       <c r="C24" s="36" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="25">
       <c r="C25" s="47" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="26">
@@ -9836,22 +9808,22 @@
     </row>
     <row r="27">
       <c r="C27" s="55" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="28">
       <c r="C28" s="53" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="34" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="36" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="L31" s="36" t="s">
         <v>25</v>
@@ -11843,7 +11815,7 @@
     </row>
     <row r="63">
       <c r="C63" s="36" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="65">
@@ -11863,19 +11835,19 @@
         <v>4</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K65" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L65" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="M65" s="65" t="s">
         <v>8</v>
@@ -12146,7 +12118,7 @@
     </row>
     <row r="76">
       <c r="C76" s="36" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="77">
@@ -12166,16 +12138,16 @@
         <v>4</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="K77" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L77" s="4" t="s">
         <v>9</v>
@@ -12520,7 +12492,7 @@
     </row>
     <row r="94">
       <c r="C94" s="37" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="96">
@@ -12543,25 +12515,25 @@
         <v>5</v>
       </c>
       <c r="I96" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K96" s="5" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="L96" s="5" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="M96" s="5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="N96" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="O96" s="5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="P96" s="65" t="s">
         <v>8</v>
@@ -13003,146 +12975,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="37" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="8"/>
       <c r="C2" s="72" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E2" s="73"/>
       <c r="F2" s="74" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H2" s="73"/>
     </row>
     <row r="3">
       <c r="B3" s="75" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C3" s="76" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D3" s="75" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E3" s="77" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F3" s="75" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G3" s="75" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H3" s="75" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="78" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C4" s="79" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D4" s="80" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E4" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F4" s="82" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G4" s="82" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H4" s="80"/>
     </row>
     <row r="5">
       <c r="B5" s="78" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C5" s="83" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D5" s="84"/>
       <c r="E5" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F5" s="85" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G5" s="86" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H5" s="80"/>
     </row>
     <row r="6">
       <c r="B6" s="78" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C6" s="79" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D6" s="80" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E6" s="81" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F6" s="80" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G6" s="80"/>
       <c r="H6" s="80"/>
     </row>
     <row r="7">
       <c r="B7" s="80" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C7" s="87" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D7" s="80"/>
       <c r="E7" s="88" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F7" s="79" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G7" s="80"/>
       <c r="H7" s="80" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="89" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C8" s="90" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D8" s="91"/>
       <c r="E8" s="89" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F8" s="92" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G8" s="93" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H8" s="91"/>
     </row>
     <row r="9">
       <c r="B9" s="21" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C9" s="94" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D9" s="95"/>
       <c r="E9" s="95"/>
@@ -13152,27 +13124,27 @@
     </row>
     <row r="10">
       <c r="B10" s="21" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C10" s="96"/>
       <c r="D10" s="95"/>
       <c r="E10" s="95"/>
       <c r="F10" s="96"/>
       <c r="G10" s="82" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H10" s="95"/>
     </row>
     <row r="11">
       <c r="B11" s="21" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C11" s="96"/>
       <c r="D11" s="95"/>
       <c r="E11" s="95"/>
       <c r="F11" s="96"/>
       <c r="G11" s="97" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H11" s="21"/>
     </row>
@@ -13210,7 +13182,7 @@
     <row r="2">
       <c r="A2" s="17"/>
       <c r="B2" s="74" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C2" s="17">
         <v>0.25</v>
@@ -13220,11 +13192,11 @@
     <row r="3">
       <c r="A3" s="17"/>
       <c r="B3" s="74" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C3" s="22">
         <f>AVERAGE('Modelos actuales'!N4:N8)</f>
-        <v>12.75</v>
+        <v>10.66666667</v>
       </c>
       <c r="L3" s="98"/>
       <c r="P3" s="98"/>
@@ -13238,44 +13210,44 @@
     <row r="5">
       <c r="A5" s="17"/>
       <c r="B5" s="98" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="L5" s="98" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="P5" s="98" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17"/>
       <c r="B6" s="37" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="F6" s="37" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="K6" s="36"/>
       <c r="L6" s="36" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="N6" s="36" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="P6" s="36" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="R6" s="36" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="V6" s="36" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="AA6" s="37" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="AB6" s="37" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -13311,7 +13283,7 @@
         <v>-0.6666666667</v>
       </c>
       <c r="AA7" s="37" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="AB7" s="43">
         <f t="shared" ref="AB7:AB16" si="4">LEFT(REPLACE(AA7,1,1,""),FIND(",", AA7)-2)/1</f>
@@ -13321,14 +13293,14 @@
     <row r="8">
       <c r="A8" s="17"/>
       <c r="B8" s="103" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C8" s="104" t="str">
         <f t="shared" ref="C8:C17" si="5">REPLACE(B8,FIND(".",B8),1,",")*1</f>
         <v>#VALUE!</v>
       </c>
       <c r="F8" s="47" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G8" s="104" t="str">
         <f t="shared" ref="G8:G27" si="6">REPLACE(F8,FIND(".",F8),1,",")*1</f>
@@ -13363,7 +13335,7 @@
         <v>-0.3157894737</v>
       </c>
       <c r="AA8" s="37" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AB8" s="43">
         <f t="shared" si="4"/>
@@ -13373,14 +13345,14 @@
     <row r="9">
       <c r="A9" s="17"/>
       <c r="B9" s="103" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C9" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F9" s="47" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G9" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13394,13 +13366,13 @@
       </c>
       <c r="K9" s="17"/>
       <c r="L9" s="99" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="M9" s="99" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="N9" s="36" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P9" s="101">
         <v>0.0</v>
@@ -13424,7 +13396,7 @@
         <v>-0.5</v>
       </c>
       <c r="AA9" s="37" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AB9" s="43">
         <f t="shared" si="4"/>
@@ -13434,14 +13406,14 @@
     <row r="10">
       <c r="A10" s="17"/>
       <c r="B10" s="105" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C10" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F10" s="47" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G10" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13478,7 +13450,7 @@
         <v>76</v>
       </c>
       <c r="AA10" s="37" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AB10" s="43">
         <f t="shared" si="4"/>
@@ -13487,14 +13459,14 @@
     </row>
     <row r="11">
       <c r="B11" s="103" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C11" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F11" s="47" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="G11" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13523,7 +13495,7 @@
         <v>0.0</v>
       </c>
       <c r="AA11" s="37" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="AB11" s="43">
         <f t="shared" si="4"/>
@@ -13532,14 +13504,14 @@
     </row>
     <row r="12">
       <c r="B12" s="105" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C12" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F12" s="47" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="G12" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13568,7 +13540,7 @@
         <v>2.0</v>
       </c>
       <c r="AA12" s="37" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="AB12" s="43">
         <f t="shared" si="4"/>
@@ -13577,14 +13549,14 @@
     </row>
     <row r="13">
       <c r="B13" s="103" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C13" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F13" s="47" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="G13" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13614,16 +13586,16 @@
       <c r="Q13" s="39"/>
       <c r="R13" s="95"/>
       <c r="S13" s="106" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="T13" s="106" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="U13" s="106" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="AA13" s="37" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="AB13" s="43">
         <f t="shared" si="4"/>
@@ -13632,14 +13604,14 @@
     </row>
     <row r="14">
       <c r="B14" s="103" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C14" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F14" s="47" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G14" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13679,7 +13651,7 @@
         <v>11.0</v>
       </c>
       <c r="AA14" s="37" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="AB14" s="43">
         <f t="shared" si="4"/>
@@ -13688,14 +13660,14 @@
     </row>
     <row r="15">
       <c r="B15" s="103" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C15" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F15" s="47" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="G15" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13735,7 +13707,7 @@
         <v>13.0</v>
       </c>
       <c r="AA15" s="37" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="AB15" s="43">
         <f t="shared" si="4"/>
@@ -13744,14 +13716,14 @@
     </row>
     <row r="16">
       <c r="B16" s="103" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C16" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F16" s="47" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G16" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13791,7 +13763,7 @@
         <v>12.0</v>
       </c>
       <c r="AA16" s="37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="AB16" s="43">
         <f t="shared" si="4"/>
@@ -13800,14 +13772,14 @@
     </row>
     <row r="17">
       <c r="B17" s="103" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C17" s="104" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F17" s="47" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G17" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13835,7 +13807,7 @@
         <v>0.0</v>
       </c>
       <c r="R17" s="106" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="S17" s="107">
         <f t="shared" ref="S17:U17" si="10">SUM(S14:S16)</f>
@@ -13852,7 +13824,7 @@
     </row>
     <row r="18">
       <c r="F18" s="47" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G18" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13883,14 +13855,14 @@
     </row>
     <row r="19">
       <c r="B19" s="36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C19" s="43" t="str">
         <f>AVERAGE(C8:C17)</f>
         <v>#VALUE!</v>
       </c>
       <c r="F19" s="47" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="G19" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13918,7 +13890,7 @@
       <c r="T19" s="19"/>
       <c r="U19" s="19"/>
       <c r="AA19" s="37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="AB19" s="43">
         <f>AVERAGE(AB7:AB16)</f>
@@ -13927,7 +13899,7 @@
     </row>
     <row r="20">
       <c r="F20" s="47" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="G20" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13946,7 +13918,7 @@
     </row>
     <row r="21">
       <c r="F21" s="47" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G21" s="104" t="str">
         <f t="shared" si="6"/>
@@ -13960,19 +13932,19 @@
       </c>
       <c r="R21" s="95"/>
       <c r="S21" s="106" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="T21" s="106" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="U21" s="106" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="22">
       <c r="C22" s="104"/>
       <c r="F22" s="47" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G22" s="104" t="str">
         <f t="shared" si="6"/>
@@ -14033,7 +14005,7 @@
     </row>
     <row r="24">
       <c r="F24" s="47" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G24" s="104" t="str">
         <f t="shared" si="6"/>
@@ -14063,7 +14035,7 @@
     </row>
     <row r="25">
       <c r="F25" s="47" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="G25" s="104" t="str">
         <f t="shared" si="6"/>
@@ -14076,7 +14048,7 @@
         <v>1.0</v>
       </c>
       <c r="R25" s="106" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="S25" s="107">
         <f t="shared" ref="S25:U25" si="14">SUM(S22:S24)</f>
@@ -14093,7 +14065,7 @@
     </row>
     <row r="26">
       <c r="F26" s="47" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G26" s="104" t="str">
         <f t="shared" si="6"/>
@@ -14126,18 +14098,18 @@
         <v>1.0</v>
       </c>
       <c r="AA28" s="37" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="AB28" s="37" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="AC28" s="37" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29">
       <c r="F29" s="36" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G29" s="43" t="str">
         <f>AVERAGE(G8:G27)</f>
@@ -14210,7 +14182,7 @@
     </row>
     <row r="32">
       <c r="B32" s="53" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="G32" s="104"/>
       <c r="P32" s="101">
@@ -14233,7 +14205,7 @@
     </row>
     <row r="33">
       <c r="B33" s="110" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="G33" s="111"/>
       <c r="P33" s="101">
@@ -14275,7 +14247,7 @@
     </row>
     <row r="35">
       <c r="H35" s="36" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P35" s="101">
         <v>0.0</v>
@@ -14326,7 +14298,7 @@
       <c r="C37" s="39"/>
       <c r="D37" s="42">
         <f>AVERAGE(D39:D1775)</f>
-        <v>5.33375</v>
+        <v>4.455625</v>
       </c>
       <c r="G37" s="36" t="s">
         <v>23</v>
@@ -14379,11 +14351,11 @@
     </row>
     <row r="39">
       <c r="C39" s="114" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="D39" s="104">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>1.4</v>
+        <v>1.87</v>
       </c>
       <c r="G39" s="36" t="s">
         <v>25</v>
@@ -14411,11 +14383,11 @@
     </row>
     <row r="40">
       <c r="C40" s="115" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D40" s="104">
         <f t="shared" si="17"/>
-        <v>0.99</v>
+        <v>0.15</v>
       </c>
       <c r="G40" s="36" t="s">
         <v>26</v>
@@ -14443,11 +14415,11 @@
     </row>
     <row r="41">
       <c r="C41" s="115" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D41" s="104">
         <f t="shared" si="17"/>
-        <v>9.03</v>
+        <v>0.1</v>
       </c>
       <c r="P41" s="101">
         <v>1.0</v>
@@ -14469,11 +14441,11 @@
     </row>
     <row r="42">
       <c r="C42" s="115" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D42" s="104">
         <f t="shared" si="17"/>
-        <v>8.73</v>
+        <v>0.74</v>
       </c>
       <c r="P42" s="101">
         <v>1.0</v>
@@ -14495,11 +14467,11 @@
     </row>
     <row r="43">
       <c r="C43" s="115" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D43" s="104">
         <f t="shared" si="17"/>
-        <v>9.07</v>
+        <v>0.42</v>
       </c>
       <c r="P43" s="101"/>
       <c r="AA43" s="41">
@@ -14519,11 +14491,11 @@
     </row>
     <row r="44">
       <c r="C44" s="115" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="D44" s="104">
         <f t="shared" si="17"/>
-        <v>7.34</v>
+        <v>7.47</v>
       </c>
       <c r="P44" s="101"/>
       <c r="AB44" s="43">
@@ -14541,37 +14513,37 @@
     </row>
     <row r="45">
       <c r="C45" s="115" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="D45" s="104">
         <f t="shared" si="17"/>
-        <v>8.24</v>
+        <v>7.63</v>
       </c>
       <c r="P45" s="101"/>
     </row>
     <row r="46">
       <c r="C46" s="115" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="D46" s="104">
         <f t="shared" si="17"/>
-        <v>6.55</v>
+        <v>8.19</v>
       </c>
       <c r="G46" s="75" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H46" s="75" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="P46" s="101"/>
     </row>
     <row r="47">
       <c r="C47" s="115" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="D47" s="104">
         <f t="shared" si="17"/>
-        <v>8.66</v>
+        <v>8.59</v>
       </c>
       <c r="G47" s="80" t="s">
         <v>22</v>
@@ -14584,16 +14556,16 @@
         <v>3</v>
       </c>
       <c r="AB47" s="37" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48">
       <c r="C48" s="115" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="D48" s="104">
         <f t="shared" si="17"/>
-        <v>6.47</v>
+        <v>6.88</v>
       </c>
       <c r="G48" s="80" t="s">
         <v>23</v>
@@ -14602,7 +14574,7 @@
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="37" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="K48" s="102">
         <f>AVERAGE(H47:H51)</f>
@@ -14618,7 +14590,7 @@
     </row>
     <row r="49">
       <c r="C49" s="115" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="D49" s="104">
         <f t="shared" si="17"/>
@@ -14631,7 +14603,7 @@
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="37" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="K49" s="102">
         <f>MEDIAN(H47:H51)</f>
@@ -14647,11 +14619,11 @@
     </row>
     <row r="50">
       <c r="C50" s="115" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D50" s="104">
         <f t="shared" si="17"/>
-        <v>7.76</v>
+        <v>8.02</v>
       </c>
       <c r="G50" s="80" t="s">
         <v>25</v>
@@ -14660,7 +14632,7 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="37" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K50" s="102">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -14676,7 +14648,7 @@
     </row>
     <row r="51">
       <c r="C51" s="115" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="D51" s="104">
         <f t="shared" si="17"/>
@@ -14689,7 +14661,7 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="37" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K51" s="102">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -14705,11 +14677,11 @@
     </row>
     <row r="52">
       <c r="C52" s="115" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D52" s="104">
         <f t="shared" si="17"/>
-        <v>6.28</v>
+        <v>6.35</v>
       </c>
       <c r="P52" s="101"/>
       <c r="AA52" s="41">
@@ -14721,11 +14693,11 @@
     </row>
     <row r="53">
       <c r="C53" s="115" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D53" s="104">
         <f t="shared" si="17"/>
-        <v>6.71</v>
+        <v>6.77</v>
       </c>
       <c r="P53" s="101"/>
       <c r="AA53" s="41">
@@ -14737,11 +14709,11 @@
     </row>
     <row r="54">
       <c r="C54" s="115" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D54" s="104">
         <f t="shared" si="17"/>
-        <v>6.38</v>
+        <v>6.44</v>
       </c>
       <c r="P54" s="101"/>
       <c r="AA54" s="41">
@@ -14753,7 +14725,7 @@
     </row>
     <row r="55">
       <c r="C55" s="115" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D55" s="104">
         <f t="shared" si="17"/>
@@ -14769,7 +14741,7 @@
     </row>
     <row r="56">
       <c r="C56" s="115" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D56" s="104">
         <f t="shared" si="17"/>
@@ -14785,11 +14757,11 @@
     </row>
     <row r="57">
       <c r="C57" s="115" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="D57" s="104">
         <f t="shared" si="17"/>
-        <v>2.22</v>
+        <v>2.11</v>
       </c>
       <c r="P57" s="101"/>
       <c r="AA57" s="37">
@@ -14801,14 +14773,14 @@
     </row>
     <row r="58">
       <c r="C58" s="115" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D58" s="104">
         <f t="shared" si="17"/>
-        <v>9.93</v>
+        <v>9.79</v>
       </c>
       <c r="G58" s="117" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H58" s="118"/>
       <c r="P58" s="101"/>
@@ -14821,7 +14793,7 @@
     </row>
     <row r="59">
       <c r="C59" s="115" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D59" s="104">
         <f t="shared" si="17"/>
@@ -14829,7 +14801,7 @@
       </c>
       <c r="G59" s="118"/>
       <c r="H59" s="119" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="P59" s="101"/>
       <c r="AA59" s="37">
@@ -14841,15 +14813,15 @@
     </row>
     <row r="60">
       <c r="C60" s="115" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="D60" s="104">
         <f t="shared" si="17"/>
-        <v>7.87</v>
+        <v>8.62</v>
       </c>
       <c r="G60" s="118"/>
       <c r="H60" s="119" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P60" s="101"/>
       <c r="AA60" s="41">
@@ -14861,15 +14833,15 @@
     </row>
     <row r="61">
       <c r="C61" s="115" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D61" s="104">
         <f t="shared" si="17"/>
-        <v>8.12</v>
+        <v>8.96</v>
       </c>
       <c r="G61" s="118"/>
       <c r="H61" s="119" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="P61" s="101"/>
       <c r="AA61" s="41">
@@ -14881,15 +14853,15 @@
     </row>
     <row r="62">
       <c r="C62" s="115" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D62" s="104">
         <f t="shared" si="17"/>
-        <v>1.52</v>
+        <v>1.56</v>
       </c>
       <c r="G62" s="118"/>
       <c r="H62" s="119" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P62" s="101"/>
       <c r="AA62" s="41">
@@ -14901,7 +14873,7 @@
     </row>
     <row r="63">
       <c r="C63" s="115" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D63" s="104">
         <f t="shared" si="17"/>
@@ -14909,238 +14881,238 @@
       </c>
       <c r="G63" s="118"/>
       <c r="H63" s="119" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="P63" s="101"/>
     </row>
     <row r="64">
       <c r="C64" s="115" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="D64" s="104">
         <f t="shared" si="17"/>
-        <v>4.13</v>
+        <v>1.65</v>
       </c>
       <c r="P64" s="101"/>
     </row>
     <row r="65">
       <c r="C65" s="115" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D65" s="104">
         <f t="shared" si="17"/>
-        <v>0.44</v>
+        <v>2.05</v>
       </c>
       <c r="P65" s="101"/>
     </row>
     <row r="66">
       <c r="C66" s="115" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D66" s="104">
         <f t="shared" si="17"/>
-        <v>4.02</v>
+        <v>1.9</v>
       </c>
       <c r="P66" s="101"/>
     </row>
     <row r="67">
       <c r="C67" s="115" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="D67" s="104">
         <f t="shared" si="17"/>
-        <v>2.05</v>
+        <v>5.6</v>
       </c>
       <c r="P67" s="101"/>
     </row>
     <row r="68">
       <c r="C68" s="115" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="D68" s="104">
         <f t="shared" si="17"/>
-        <v>1.55</v>
+        <v>1</v>
       </c>
       <c r="P68" s="101"/>
     </row>
     <row r="69">
       <c r="C69" s="115" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="D69" s="104">
         <f t="shared" si="17"/>
-        <v>0.23</v>
+        <v>1.24</v>
       </c>
       <c r="P69" s="101"/>
     </row>
     <row r="70">
       <c r="C70" s="115" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="D70" s="104">
         <f t="shared" si="17"/>
-        <v>0.44</v>
+        <v>3.38</v>
       </c>
       <c r="P70" s="101"/>
     </row>
     <row r="71">
       <c r="C71" s="115" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D71" s="104">
         <f t="shared" si="17"/>
-        <v>0.28</v>
+        <v>6.48</v>
       </c>
       <c r="F71" s="120"/>
       <c r="P71" s="101"/>
     </row>
     <row r="72">
       <c r="C72" s="115" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D72" s="104">
         <f t="shared" si="17"/>
-        <v>4.84</v>
+        <v>6.96</v>
       </c>
       <c r="P72" s="101"/>
     </row>
     <row r="73">
       <c r="C73" s="115" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D73" s="104">
         <f t="shared" si="17"/>
-        <v>5</v>
+        <v>3.53</v>
       </c>
       <c r="P73" s="101"/>
     </row>
     <row r="74">
       <c r="C74" s="115" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D74" s="104">
         <f t="shared" si="17"/>
-        <v>10.04</v>
+        <v>4.04</v>
       </c>
       <c r="P74" s="101"/>
     </row>
     <row r="75">
       <c r="C75" s="115" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D75" s="104">
         <f t="shared" si="17"/>
-        <v>9.79</v>
+        <v>5.12</v>
       </c>
       <c r="P75" s="101"/>
     </row>
     <row r="76">
       <c r="C76" s="115" t="s">
-        <v>199</v>
+        <v>171</v>
       </c>
       <c r="D76" s="104">
         <f t="shared" si="17"/>
-        <v>11.52</v>
+        <v>6.35</v>
       </c>
       <c r="P76" s="101"/>
     </row>
     <row r="77">
       <c r="C77" s="115" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D77" s="104">
         <f t="shared" si="17"/>
-        <v>0.5</v>
+        <v>4.35</v>
       </c>
       <c r="P77" s="101"/>
     </row>
     <row r="78">
       <c r="C78" s="115" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D78" s="104">
         <f t="shared" si="17"/>
-        <v>7.63</v>
+        <v>1.2</v>
       </c>
       <c r="P78" s="121"/>
     </row>
     <row r="79">
       <c r="C79" s="115" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D79" s="104">
         <f t="shared" si="17"/>
-        <v>1.35</v>
+        <v>3.69</v>
       </c>
       <c r="P79" s="121"/>
     </row>
     <row r="80">
       <c r="C80" s="115" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="D80" s="104">
         <f t="shared" si="17"/>
-        <v>7.46</v>
+        <v>0.68</v>
       </c>
       <c r="P80" s="121"/>
     </row>
     <row r="81">
       <c r="C81" s="115" t="s">
-        <v>114</v>
+        <v>205</v>
       </c>
       <c r="D81" s="104">
         <f t="shared" si="17"/>
-        <v>3.83</v>
+        <v>10.9</v>
       </c>
       <c r="P81" s="121"/>
     </row>
     <row r="82">
       <c r="C82" s="115" t="s">
-        <v>125</v>
+        <v>206</v>
       </c>
       <c r="D82" s="104">
         <f t="shared" si="17"/>
-        <v>9.33</v>
+        <v>1.13</v>
       </c>
       <c r="P82" s="121"/>
     </row>
     <row r="83">
       <c r="C83" s="115" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="D83" s="104">
         <f t="shared" si="17"/>
-        <v>9.85</v>
+        <v>2.16</v>
       </c>
       <c r="P83" s="121"/>
     </row>
     <row r="84">
       <c r="C84" s="115" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D84" s="104">
         <f t="shared" si="17"/>
-        <v>1.75</v>
+        <v>1.98</v>
       </c>
       <c r="P84" s="121"/>
     </row>
     <row r="85">
       <c r="C85" s="115" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="D85" s="104">
         <f t="shared" si="17"/>
-        <v>0.64</v>
+        <v>1.52</v>
       </c>
       <c r="P85" s="121"/>
     </row>
     <row r="86">
       <c r="C86" s="115" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="D86" s="104">
         <f t="shared" si="17"/>
-        <v>1.95</v>
+        <v>2.17</v>
       </c>
       <c r="P86" s="121"/>
     </row>
@@ -36376,14 +36348,14 @@
     <row r="1">
       <c r="A1" s="84"/>
       <c r="B1" s="125" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="C1" s="126"/>
       <c r="D1" s="126"/>
       <c r="E1" s="126"/>
       <c r="F1" s="126"/>
       <c r="G1" s="127" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="H1" s="126"/>
       <c r="I1" s="126"/>
@@ -36411,49 +36383,49 @@
         <v>3</v>
       </c>
       <c r="B2" s="129" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="C2" s="130" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="D2" s="130" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E2" s="130" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F2" s="131" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="G2" s="129">
         <v>1.0</v>
       </c>
       <c r="H2" s="130" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I2" s="130">
         <v>2.0</v>
       </c>
       <c r="J2" s="130" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="K2" s="132" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="L2" s="130" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="M2" s="133" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="N2" s="80" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="O2" s="80" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="P2" s="80" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="Q2" s="8"/>
       <c r="R2" s="8"/>
@@ -37126,7 +37098,7 @@
     </row>
     <row r="24">
       <c r="A24" s="74" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B24" s="146" t="str">
         <f t="shared" ref="B24:F24" si="4">IFERROR(AVERAGE(B3:B22),"")</f>
@@ -37236,7 +37208,7 @@
       <c r="E27" s="8"/>
       <c r="F27" s="8"/>
       <c r="G27" s="147" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="H27" s="8"/>
       <c r="I27" s="8"/>
@@ -37269,7 +37241,7 @@
         <v>1.0</v>
       </c>
       <c r="H28" s="148" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I28" s="148">
         <v>2.0</v>
@@ -37297,7 +37269,7 @@
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
       <c r="D29" s="4" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -37319,10 +37291,10 @@
       </c>
       <c r="K29" s="8"/>
       <c r="L29" s="74" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="M29" s="74" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -37458,7 +37430,7 @@
       <c r="E33" s="8"/>
       <c r="F33" s="8"/>
       <c r="G33" s="99" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="J33" s="8"/>
       <c r="K33" s="8"/>
@@ -37492,7 +37464,7 @@
         <v>1.0</v>
       </c>
       <c r="H34" s="151" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I34" s="151">
         <v>2.0</v>
@@ -37635,7 +37607,7 @@
       <c r="D38" s="8"/>
       <c r="E38" s="8"/>
       <c r="F38" s="4" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="G38" s="150">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
Data. Actualizo predicciones de FRA
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -211,7 +211,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="279">
   <si>
     <t>id_country</t>
   </si>
@@ -412,6 +412,12 @@
   </si>
   <si>
     <t>['ROI_sb_sin_ea', 'ROI_sb_con_ea', 'roi_last_25_matches_sb_sin_ea', 'roi_last_25_matches_sb_con_ea']</t>
+  </si>
+  <si>
+    <t>Hasta el sabado incluido</t>
+  </si>
+  <si>
+    <t>En el iniicio del domingo:</t>
   </si>
   <si>
     <t>]</t>
@@ -2222,32 +2228,22 @@
         <v>15</v>
       </c>
       <c r="F4" s="17"/>
-      <c r="G4" s="18">
-        <v>1301.22317033501</v>
-      </c>
-      <c r="H4" s="19">
-        <v>10.0</v>
-      </c>
-      <c r="I4" s="19">
-        <v>45.0</v>
-      </c>
-      <c r="J4" s="19">
-        <v>25.0</v>
-      </c>
-      <c r="K4" s="22">
+      <c r="G4" s="18"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="22" t="str">
         <f t="shared" ref="K4:K8" si="1">AVERAGE(H4:J4)</f>
-        <v>26.66666667</v>
-      </c>
-      <c r="L4" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L4" s="30" t="str">
         <f>K4*'Data preparation'!$C$2</f>
-        <v>6.666666667</v>
-      </c>
-      <c r="M4" s="21">
-        <v>5564.89670858036</v>
-      </c>
-      <c r="N4" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M4" s="21"/>
+      <c r="N4" s="22" t="str">
         <f t="shared" ref="N4:N8" si="2">M4/G4</f>
-        <v>4.27666586</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="5">
@@ -2261,40 +2257,28 @@
         <v>45679.0</v>
       </c>
       <c r="D5" s="16">
-        <v>1448.0</v>
+        <v>724.0</v>
       </c>
       <c r="E5" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="17">
-        <v>57.7981651376146</v>
-      </c>
-      <c r="G5" s="18">
-        <v>823.906317742065</v>
-      </c>
-      <c r="H5" s="21">
-        <v>70.0</v>
-      </c>
-      <c r="I5" s="21">
-        <v>45.0</v>
-      </c>
-      <c r="J5" s="21">
-        <v>25.0</v>
-      </c>
-      <c r="K5" s="22">
+      <c r="F5" s="17"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="22" t="str">
         <f t="shared" si="1"/>
-        <v>46.66666667</v>
-      </c>
-      <c r="L5" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L5" s="30" t="str">
         <f>K5*'Data preparation'!$C$2</f>
-        <v>11.66666667</v>
-      </c>
-      <c r="M5" s="21">
-        <v>8764.30228233083</v>
-      </c>
-      <c r="N5" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M5" s="21"/>
+      <c r="N5" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>10.63749858</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="P5" s="34"/>
     </row>
@@ -2314,35 +2298,23 @@
       <c r="E6" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="F6" s="17">
-        <v>62.3853211009174</v>
-      </c>
-      <c r="G6" s="18">
-        <v>2007.3027253796</v>
-      </c>
-      <c r="H6" s="21">
-        <v>70.0</v>
-      </c>
-      <c r="I6" s="21">
-        <v>70.0</v>
-      </c>
-      <c r="J6" s="21">
-        <v>10.0</v>
-      </c>
-      <c r="K6" s="22">
+      <c r="F6" s="17"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="22" t="str">
         <f t="shared" si="1"/>
-        <v>50</v>
-      </c>
-      <c r="L6" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L6" s="30" t="str">
         <f>K6*'Data preparation'!$C$2</f>
-        <v>12.5</v>
-      </c>
-      <c r="M6" s="35">
-        <v>235388.618048197</v>
-      </c>
-      <c r="N6" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M6" s="35"/>
+      <c r="N6" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>117.2661279</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="7">
@@ -2362,32 +2334,22 @@
         <v>15</v>
       </c>
       <c r="F7" s="17"/>
-      <c r="G7" s="18">
-        <v>759.494203200902</v>
-      </c>
-      <c r="H7" s="19">
-        <v>45.0</v>
-      </c>
-      <c r="I7" s="19">
-        <v>45.0</v>
-      </c>
-      <c r="J7" s="19">
-        <v>45.0</v>
-      </c>
-      <c r="K7" s="28">
+      <c r="G7" s="18"/>
+      <c r="H7" s="19"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="19"/>
+      <c r="K7" s="28" t="str">
         <f t="shared" si="1"/>
-        <v>45</v>
-      </c>
-      <c r="L7" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L7" s="30" t="str">
         <f>K7*'Data preparation'!$C$2</f>
-        <v>11.25</v>
-      </c>
-      <c r="M7" s="21">
-        <v>9433.02522864221</v>
-      </c>
-      <c r="N7" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M7" s="21"/>
+      <c r="N7" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>12.42014118</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="8">
@@ -2407,32 +2369,22 @@
         <v>15</v>
       </c>
       <c r="F8" s="17"/>
-      <c r="G8" s="18">
-        <v>422.057169223285</v>
-      </c>
-      <c r="H8" s="19">
-        <v>45.0</v>
-      </c>
-      <c r="I8" s="19">
-        <v>10.0</v>
-      </c>
-      <c r="J8" s="19">
-        <v>25.0</v>
-      </c>
-      <c r="K8" s="22">
+      <c r="G8" s="18"/>
+      <c r="H8" s="19"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="19"/>
+      <c r="K8" s="22" t="str">
         <f t="shared" si="1"/>
-        <v>26.66666667</v>
-      </c>
-      <c r="L8" s="30">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="L8" s="30" t="str">
         <f>K8*'Data preparation'!$C$2</f>
-        <v>6.666666667</v>
-      </c>
-      <c r="M8" s="21">
-        <v>1548.87389573756</v>
-      </c>
-      <c r="N8" s="22">
+        <v>#DIV/0!</v>
+      </c>
+      <c r="M8" s="21"/>
+      <c r="N8" s="22" t="str">
         <f t="shared" si="2"/>
-        <v>3.66982013</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="9" ht="20.25" customHeight="1">
@@ -12835,6 +12787,9 @@
     </row>
     <row r="10">
       <c r="A10" s="52"/>
+      <c r="E10" s="45" t="s">
+        <v>62</v>
+      </c>
       <c r="O10" s="46"/>
       <c r="P10" s="52"/>
       <c r="Q10" s="52"/>
@@ -12963,6 +12918,9 @@
     </row>
     <row r="18">
       <c r="A18" s="46"/>
+      <c r="E18" s="45" t="s">
+        <v>63</v>
+      </c>
       <c r="O18" s="46"/>
       <c r="P18" s="46"/>
       <c r="Q18" s="46"/>
@@ -12973,6 +12931,12 @@
     </row>
     <row r="19">
       <c r="A19" s="46"/>
+      <c r="E19" s="33" t="s">
+        <v>17</v>
+      </c>
+      <c r="F19" s="16">
+        <v>663.0</v>
+      </c>
       <c r="O19" s="46"/>
       <c r="P19" s="46"/>
       <c r="Q19" s="46"/>
@@ -12981,23 +12945,47 @@
       <c r="T19" s="34"/>
     </row>
     <row r="20">
+      <c r="E20" s="33" t="s">
+        <v>18</v>
+      </c>
+      <c r="F20" s="16">
+        <v>654.0</v>
+      </c>
       <c r="O20" s="46"/>
       <c r="Q20" s="34"/>
       <c r="S20" s="34"/>
       <c r="T20" s="34"/>
     </row>
     <row r="21">
+      <c r="E21" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="F21" s="16">
+        <v>1051.0</v>
+      </c>
       <c r="O21" s="46"/>
       <c r="P21" s="34"/>
       <c r="T21" s="34"/>
     </row>
     <row r="22">
+      <c r="E22" s="25" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="16">
+        <v>622.0</v>
+      </c>
       <c r="M22" s="52"/>
       <c r="O22" s="37"/>
       <c r="P22" s="34"/>
       <c r="T22" s="34"/>
     </row>
     <row r="23">
+      <c r="E23" s="25" t="s">
+        <v>21</v>
+      </c>
+      <c r="F23" s="16">
+        <v>1545.0</v>
+      </c>
       <c r="M23" s="52"/>
       <c r="O23" s="37"/>
       <c r="T23" s="34"/>
@@ -13042,146 +13030,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="45" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="10"/>
       <c r="C2" s="90" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E2" s="91"/>
       <c r="F2" s="92" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H2" s="91"/>
     </row>
     <row r="3">
       <c r="B3" s="93" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C3" s="94" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D3" s="93" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="E3" s="95" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F3" s="93" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G3" s="93" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H3" s="93" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="96" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C4" s="97" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D4" s="98" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="E4" s="99" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F4" s="100" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G4" s="100" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H4" s="98"/>
     </row>
     <row r="5">
       <c r="B5" s="96" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C5" s="101" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D5" s="102"/>
       <c r="E5" s="99" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F5" s="103" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G5" s="104" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H5" s="98"/>
     </row>
     <row r="6">
       <c r="B6" s="96" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C6" s="97" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D6" s="98" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="E6" s="99" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="F6" s="98" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="G6" s="98"/>
       <c r="H6" s="98"/>
     </row>
     <row r="7">
       <c r="B7" s="98" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C7" s="105" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D7" s="98"/>
       <c r="E7" s="106" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F7" s="97" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G7" s="98"/>
       <c r="H7" s="98" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="107" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C8" s="108" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D8" s="109"/>
       <c r="E8" s="107" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F8" s="110" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G8" s="111" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H8" s="109"/>
     </row>
     <row r="9">
       <c r="B9" s="25" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C9" s="112" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="D9" s="82"/>
       <c r="E9" s="82"/>
@@ -13191,27 +13179,27 @@
     </row>
     <row r="10">
       <c r="B10" s="25" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C10" s="113"/>
       <c r="D10" s="82"/>
       <c r="E10" s="82"/>
       <c r="F10" s="113"/>
       <c r="G10" s="100" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H10" s="82"/>
     </row>
     <row r="11">
       <c r="B11" s="25" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C11" s="113"/>
       <c r="D11" s="82"/>
       <c r="E11" s="82"/>
       <c r="F11" s="113"/>
       <c r="G11" s="114" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H11" s="25"/>
     </row>
@@ -13249,7 +13237,7 @@
     <row r="2">
       <c r="A2" s="19"/>
       <c r="B2" s="92" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="C2" s="19">
         <v>0.25</v>
@@ -13259,11 +13247,11 @@
     <row r="3">
       <c r="A3" s="19"/>
       <c r="B3" s="92" t="s">
-        <v>100</v>
-      </c>
-      <c r="C3" s="29">
+        <v>102</v>
+      </c>
+      <c r="C3" s="23" t="str">
         <f>AVERAGE('Modelos actuales'!L4:L8)</f>
-        <v>9.75</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="L3" s="115"/>
       <c r="P3" s="115"/>
@@ -13274,7 +13262,7 @@
       <c r="L4" s="115"/>
       <c r="P4" s="115"/>
       <c r="AE4" s="45" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="AF4" s="116">
         <f>CORREL(AE6:AE10000,AF6:AF10000)</f>
@@ -13284,50 +13272,50 @@
     <row r="5">
       <c r="A5" s="19"/>
       <c r="B5" s="115" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="L5" s="115" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="P5" s="115" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="AE5" s="45" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="AF5" s="45" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="19"/>
       <c r="B6" s="45" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F6" s="45" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="K6" s="38"/>
       <c r="L6" s="38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="N6" s="38" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="P6" s="38" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="R6" s="38" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="V6" s="38" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="AA6" s="45" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="AB6" s="45" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="AE6" s="45">
         <v>519.2</v>
@@ -13369,7 +13357,7 @@
         <v>0.5454545455</v>
       </c>
       <c r="AA7" s="45" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="AB7" s="44">
         <f t="shared" ref="AB7:AB16" si="4">LEFT(REPLACE(AA7,1,1,""),FIND(",", AA7)-2)/1</f>
@@ -13385,14 +13373,14 @@
     <row r="8">
       <c r="A8" s="19"/>
       <c r="B8" s="121" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C8" s="122" t="str">
         <f t="shared" ref="C8:C17" si="5">REPLACE(B8,FIND(".",B8),1,",")*1</f>
         <v>#VALUE!</v>
       </c>
       <c r="F8" s="50" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G8" s="122" t="str">
         <f t="shared" ref="G8:G27" si="6">REPLACE(F8,FIND(".",F8),1,",")*1</f>
@@ -13427,7 +13415,7 @@
         <v>0.5263157895</v>
       </c>
       <c r="AA8" s="45" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="AB8" s="44">
         <f t="shared" si="4"/>
@@ -13443,14 +13431,14 @@
     <row r="9">
       <c r="A9" s="19"/>
       <c r="B9" s="121" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C9" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F9" s="50" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G9" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13464,13 +13452,13 @@
       </c>
       <c r="K9" s="19"/>
       <c r="L9" s="117" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="M9" s="117" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="N9" s="38" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="P9" s="119">
         <v>1.0</v>
@@ -13494,7 +13482,7 @@
         <v>0.25</v>
       </c>
       <c r="AA9" s="45" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="AB9" s="44">
         <f t="shared" si="4"/>
@@ -13510,14 +13498,14 @@
     <row r="10">
       <c r="A10" s="19"/>
       <c r="B10" s="123" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C10" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F10" s="50" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="G10" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13554,7 +13542,7 @@
         <v>76</v>
       </c>
       <c r="AA10" s="45" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AB10" s="44">
         <f t="shared" si="4"/>
@@ -13569,14 +13557,14 @@
     </row>
     <row r="11">
       <c r="B11" s="121" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C11" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F11" s="50" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G11" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13605,7 +13593,7 @@
         <v>2.0</v>
       </c>
       <c r="AA11" s="45" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="AB11" s="44">
         <f t="shared" si="4"/>
@@ -13620,14 +13608,14 @@
     </row>
     <row r="12">
       <c r="B12" s="123" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C12" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F12" s="50" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G12" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13656,7 +13644,7 @@
         <v>1.0</v>
       </c>
       <c r="AA12" s="45" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AB12" s="44">
         <f t="shared" si="4"/>
@@ -13671,14 +13659,14 @@
     </row>
     <row r="13">
       <c r="B13" s="121" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C13" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F13" s="50" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G13" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13708,16 +13696,16 @@
       <c r="Q13" s="43"/>
       <c r="R13" s="82"/>
       <c r="S13" s="87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="T13" s="87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="U13" s="87" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AA13" s="45" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="AB13" s="44">
         <f t="shared" si="4"/>
@@ -13732,14 +13720,14 @@
     </row>
     <row r="14">
       <c r="B14" s="121" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C14" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F14" s="50" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G14" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13779,7 +13767,7 @@
         <v>11.0</v>
       </c>
       <c r="AA14" s="45" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="AB14" s="44">
         <f t="shared" si="4"/>
@@ -13794,14 +13782,14 @@
     </row>
     <row r="15">
       <c r="B15" s="121" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C15" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F15" s="50" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="G15" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13841,7 +13829,7 @@
         <v>13.0</v>
       </c>
       <c r="AA15" s="45" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="AB15" s="44">
         <f t="shared" si="4"/>
@@ -13856,14 +13844,14 @@
     </row>
     <row r="16">
       <c r="B16" s="121" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C16" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F16" s="50" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G16" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13903,7 +13891,7 @@
         <v>12.0</v>
       </c>
       <c r="AA16" s="45" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="AB16" s="44">
         <f t="shared" si="4"/>
@@ -13918,14 +13906,14 @@
     </row>
     <row r="17">
       <c r="B17" s="121" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C17" s="122" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F17" s="50" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="G17" s="122" t="str">
         <f t="shared" si="6"/>
@@ -13953,7 +13941,7 @@
         <v>1.0</v>
       </c>
       <c r="R17" s="87" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="S17" s="124">
         <f t="shared" ref="S17:U17" si="10">SUM(S14:S16)</f>
@@ -13976,7 +13964,7 @@
     </row>
     <row r="18">
       <c r="F18" s="50" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G18" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14013,14 +14001,14 @@
     </row>
     <row r="19">
       <c r="B19" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C19" s="44" t="str">
         <f>AVERAGE(C8:C17)</f>
         <v>#VALUE!</v>
       </c>
       <c r="F19" s="50" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="G19" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14048,7 +14036,7 @@
       <c r="T19" s="23"/>
       <c r="U19" s="23"/>
       <c r="AA19" s="45" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="AB19" s="44">
         <f>AVERAGE(AB7:AB16)</f>
@@ -14063,7 +14051,7 @@
     </row>
     <row r="20">
       <c r="F20" s="50" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G20" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14088,7 +14076,7 @@
     </row>
     <row r="21">
       <c r="F21" s="50" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="G21" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14102,13 +14090,13 @@
       </c>
       <c r="R21" s="82"/>
       <c r="S21" s="87" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="T21" s="87" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="U21" s="87" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="AE21" s="45">
         <v>146.62</v>
@@ -14120,7 +14108,7 @@
     <row r="22">
       <c r="C22" s="122"/>
       <c r="F22" s="50" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="G22" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14193,7 +14181,7 @@
     </row>
     <row r="24">
       <c r="F24" s="50" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="G24" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14229,7 +14217,7 @@
     </row>
     <row r="25">
       <c r="F25" s="50" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G25" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14242,7 +14230,7 @@
         <v>1.0</v>
       </c>
       <c r="R25" s="87" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="S25" s="124">
         <f t="shared" ref="S25:U25" si="14">SUM(S22:S24)</f>
@@ -14265,7 +14253,7 @@
     </row>
     <row r="26">
       <c r="F26" s="50" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="G26" s="122" t="str">
         <f t="shared" si="6"/>
@@ -14310,13 +14298,13 @@
         <v>1.0</v>
       </c>
       <c r="AA28" s="45" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="AB28" s="45" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AC28" s="45" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AE28" s="45">
         <v>106.73</v>
@@ -14327,7 +14315,7 @@
     </row>
     <row r="29">
       <c r="F29" s="38" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="G29" s="44" t="str">
         <f>AVERAGE(G8:G27)</f>
@@ -14418,7 +14406,7 @@
     </row>
     <row r="32">
       <c r="B32" s="57" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G32" s="122"/>
       <c r="P32" s="119">
@@ -14447,7 +14435,7 @@
     </row>
     <row r="33">
       <c r="B33" s="127" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="G33" s="128"/>
       <c r="P33" s="119">
@@ -14501,7 +14489,7 @@
     </row>
     <row r="35">
       <c r="H35" s="38" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="P35" s="119">
         <v>1.0</v>
@@ -14629,7 +14617,7 @@
     </row>
     <row r="39">
       <c r="C39" s="132" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D39" s="122">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
@@ -14667,7 +14655,7 @@
     </row>
     <row r="40">
       <c r="C40" s="133" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D40" s="122">
         <f t="shared" si="17"/>
@@ -14705,7 +14693,7 @@
     </row>
     <row r="41">
       <c r="C41" s="133" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="D41" s="122">
         <f t="shared" si="17"/>
@@ -14737,7 +14725,7 @@
     </row>
     <row r="42">
       <c r="C42" s="133" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="D42" s="122">
         <f t="shared" si="17"/>
@@ -14769,7 +14757,7 @@
     </row>
     <row r="43">
       <c r="C43" s="133" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D43" s="122">
         <f t="shared" si="17"/>
@@ -14801,7 +14789,7 @@
     </row>
     <row r="44">
       <c r="C44" s="133" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="D44" s="122">
         <f t="shared" si="17"/>
@@ -14831,7 +14819,7 @@
     </row>
     <row r="45">
       <c r="C45" s="133" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="D45" s="122">
         <f t="shared" si="17"/>
@@ -14849,17 +14837,17 @@
     </row>
     <row r="46">
       <c r="C46" s="133" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D46" s="122">
         <f t="shared" si="17"/>
         <v>4.55</v>
       </c>
       <c r="G46" s="93" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H46" s="93" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="P46" s="119">
         <v>0.0</v>
@@ -14873,7 +14861,7 @@
     </row>
     <row r="47">
       <c r="C47" s="133" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D47" s="122">
         <f t="shared" si="17"/>
@@ -14892,7 +14880,7 @@
         <v>3</v>
       </c>
       <c r="AB47" s="45" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AE47" s="45">
         <v>67.98</v>
@@ -14903,7 +14891,7 @@
     </row>
     <row r="48">
       <c r="C48" s="133" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D48" s="122">
         <f t="shared" si="17"/>
@@ -14916,7 +14904,7 @@
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="45" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="K48" s="120">
         <f>AVERAGE(H47:H51)</f>
@@ -14940,7 +14928,7 @@
     </row>
     <row r="49">
       <c r="C49" s="133" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="D49" s="122">
         <f t="shared" si="17"/>
@@ -14953,7 +14941,7 @@
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="45" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="K49" s="120">
         <f>MEDIAN(H47:H51)</f>
@@ -14977,7 +14965,7 @@
     </row>
     <row r="50">
       <c r="C50" s="133" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D50" s="122">
         <f t="shared" si="17"/>
@@ -14990,7 +14978,7 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="45" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="K50" s="120">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -15014,7 +15002,7 @@
     </row>
     <row r="51">
       <c r="C51" s="133" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="D51" s="122">
         <f t="shared" si="17"/>
@@ -15027,7 +15015,7 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="45" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="K51" s="120">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -15051,7 +15039,7 @@
     </row>
     <row r="52">
       <c r="C52" s="133" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D52" s="122">
         <f t="shared" si="17"/>
@@ -15075,7 +15063,7 @@
     </row>
     <row r="53">
       <c r="C53" s="133" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D53" s="122">
         <f t="shared" si="17"/>
@@ -15099,7 +15087,7 @@
     </row>
     <row r="54">
       <c r="C54" s="133" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D54" s="122">
         <f t="shared" si="17"/>
@@ -15123,7 +15111,7 @@
     </row>
     <row r="55">
       <c r="C55" s="133" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D55" s="122">
         <f t="shared" si="17"/>
@@ -15147,7 +15135,7 @@
     </row>
     <row r="56">
       <c r="C56" s="133" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D56" s="122">
         <f t="shared" si="17"/>
@@ -15171,7 +15159,7 @@
     </row>
     <row r="57">
       <c r="C57" s="133" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="D57" s="122">
         <f t="shared" si="17"/>
@@ -15195,14 +15183,14 @@
     </row>
     <row r="58">
       <c r="C58" s="133" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D58" s="122">
         <f t="shared" si="17"/>
         <v>7.8</v>
       </c>
       <c r="G58" s="135" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H58" s="136"/>
       <c r="P58" s="119">
@@ -15223,7 +15211,7 @@
     </row>
     <row r="59">
       <c r="C59" s="133" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D59" s="122">
         <f t="shared" si="17"/>
@@ -15231,7 +15219,7 @@
       </c>
       <c r="G59" s="136"/>
       <c r="H59" s="137" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="P59" s="119">
         <v>0.0</v>
@@ -15251,7 +15239,7 @@
     </row>
     <row r="60">
       <c r="C60" s="133" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D60" s="122">
         <f t="shared" si="17"/>
@@ -15259,7 +15247,7 @@
       </c>
       <c r="G60" s="136"/>
       <c r="H60" s="137" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="P60" s="119">
         <v>2.0</v>
@@ -15279,7 +15267,7 @@
     </row>
     <row r="61">
       <c r="C61" s="133" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="D61" s="122">
         <f t="shared" si="17"/>
@@ -15287,7 +15275,7 @@
       </c>
       <c r="G61" s="136"/>
       <c r="H61" s="137" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="P61" s="119">
         <v>2.0</v>
@@ -15307,7 +15295,7 @@
     </row>
     <row r="62">
       <c r="C62" s="133" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="D62" s="122">
         <f t="shared" si="17"/>
@@ -15315,7 +15303,7 @@
       </c>
       <c r="G62" s="136"/>
       <c r="H62" s="137" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="P62" s="119">
         <v>1.0</v>
@@ -15335,7 +15323,7 @@
     </row>
     <row r="63">
       <c r="C63" s="133" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D63" s="122">
         <f t="shared" si="17"/>
@@ -15343,7 +15331,7 @@
       </c>
       <c r="G63" s="136"/>
       <c r="H63" s="137" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="P63" s="119">
         <v>0.0</v>
@@ -15357,7 +15345,7 @@
     </row>
     <row r="64">
       <c r="C64" s="133" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D64" s="122">
         <f t="shared" si="17"/>
@@ -15375,7 +15363,7 @@
     </row>
     <row r="65">
       <c r="C65" s="133" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D65" s="122">
         <f t="shared" si="17"/>
@@ -15393,7 +15381,7 @@
     </row>
     <row r="66">
       <c r="C66" s="133" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D66" s="122">
         <f t="shared" si="17"/>
@@ -15411,7 +15399,7 @@
     </row>
     <row r="67">
       <c r="C67" s="133" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D67" s="122">
         <f t="shared" si="17"/>
@@ -15429,7 +15417,7 @@
     </row>
     <row r="68">
       <c r="C68" s="133" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D68" s="122">
         <f t="shared" si="17"/>
@@ -15447,7 +15435,7 @@
     </row>
     <row r="69">
       <c r="C69" s="133" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="D69" s="122">
         <f t="shared" si="17"/>
@@ -15465,7 +15453,7 @@
     </row>
     <row r="70">
       <c r="C70" s="133" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D70" s="122">
         <f t="shared" si="17"/>
@@ -15483,7 +15471,7 @@
     </row>
     <row r="71">
       <c r="C71" s="133" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="D71" s="122">
         <f t="shared" si="17"/>
@@ -15502,7 +15490,7 @@
     </row>
     <row r="72">
       <c r="C72" s="133" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D72" s="122">
         <f t="shared" si="17"/>
@@ -15520,7 +15508,7 @@
     </row>
     <row r="73">
       <c r="C73" s="133" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D73" s="122">
         <f t="shared" si="17"/>
@@ -15538,7 +15526,7 @@
     </row>
     <row r="74">
       <c r="C74" s="133" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D74" s="122">
         <f t="shared" si="17"/>
@@ -15556,7 +15544,7 @@
     </row>
     <row r="75">
       <c r="C75" s="133" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D75" s="122">
         <f t="shared" si="17"/>
@@ -15574,7 +15562,7 @@
     </row>
     <row r="76">
       <c r="C76" s="133" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D76" s="122">
         <f t="shared" si="17"/>
@@ -15592,7 +15580,7 @@
     </row>
     <row r="77">
       <c r="C77" s="133" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="D77" s="122">
         <f t="shared" si="17"/>
@@ -15610,7 +15598,7 @@
     </row>
     <row r="78">
       <c r="C78" s="133" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D78" s="122">
         <f t="shared" si="17"/>
@@ -15628,7 +15616,7 @@
     </row>
     <row r="79">
       <c r="C79" s="133" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D79" s="122">
         <f t="shared" si="17"/>
@@ -15646,7 +15634,7 @@
     </row>
     <row r="80">
       <c r="C80" s="133" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="D80" s="122">
         <f t="shared" si="17"/>
@@ -15664,7 +15652,7 @@
     </row>
     <row r="81">
       <c r="C81" s="133" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D81" s="122">
         <f t="shared" si="17"/>
@@ -15682,7 +15670,7 @@
     </row>
     <row r="82">
       <c r="C82" s="133" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="D82" s="122">
         <f t="shared" si="17"/>
@@ -15700,7 +15688,7 @@
     </row>
     <row r="83">
       <c r="C83" s="133" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D83" s="122">
         <f t="shared" si="17"/>
@@ -15718,7 +15706,7 @@
     </row>
     <row r="84">
       <c r="C84" s="133" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D84" s="122">
         <f t="shared" si="17"/>
@@ -15736,7 +15724,7 @@
     </row>
     <row r="85">
       <c r="C85" s="133" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="D85" s="122">
         <f t="shared" si="17"/>
@@ -15754,7 +15742,7 @@
     </row>
     <row r="86">
       <c r="C86" s="133" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D86" s="122">
         <f t="shared" si="17"/>
@@ -15772,7 +15760,7 @@
     </row>
     <row r="87">
       <c r="C87" s="133" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D87" s="122">
         <f t="shared" si="17"/>
@@ -15790,7 +15778,7 @@
     </row>
     <row r="88">
       <c r="C88" s="133" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D88" s="122">
         <f t="shared" si="17"/>
@@ -15808,7 +15796,7 @@
     </row>
     <row r="89">
       <c r="C89" s="133" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D89" s="122">
         <f t="shared" si="17"/>
@@ -15826,7 +15814,7 @@
     </row>
     <row r="90">
       <c r="C90" s="133" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D90" s="122">
         <f t="shared" si="17"/>
@@ -15844,7 +15832,7 @@
     </row>
     <row r="91">
       <c r="C91" s="133" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D91" s="122">
         <f t="shared" si="17"/>
@@ -15862,7 +15850,7 @@
     </row>
     <row r="92">
       <c r="C92" s="133" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D92" s="122">
         <f t="shared" si="17"/>
@@ -15880,7 +15868,7 @@
     </row>
     <row r="93">
       <c r="C93" s="133" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D93" s="122">
         <f t="shared" si="17"/>
@@ -15898,7 +15886,7 @@
     </row>
     <row r="94">
       <c r="C94" s="133" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D94" s="122">
         <f t="shared" si="17"/>
@@ -15916,7 +15904,7 @@
     </row>
     <row r="95">
       <c r="C95" s="133" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D95" s="122">
         <f t="shared" si="17"/>
@@ -15934,7 +15922,7 @@
     </row>
     <row r="96">
       <c r="C96" s="133" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="D96" s="122">
         <f t="shared" si="17"/>
@@ -15952,7 +15940,7 @@
     </row>
     <row r="97">
       <c r="C97" s="133" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D97" s="122">
         <f t="shared" si="17"/>
@@ -15970,7 +15958,7 @@
     </row>
     <row r="98">
       <c r="C98" s="133" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D98" s="122">
         <f t="shared" si="17"/>
@@ -15988,7 +15976,7 @@
     </row>
     <row r="99">
       <c r="C99" s="133" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="D99" s="122">
         <f t="shared" si="17"/>
@@ -16006,7 +15994,7 @@
     </row>
     <row r="100">
       <c r="C100" s="133" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="D100" s="122">
         <f t="shared" si="17"/>
@@ -16024,7 +16012,7 @@
     </row>
     <row r="101">
       <c r="C101" s="133" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D101" s="122">
         <f t="shared" si="17"/>
@@ -16042,7 +16030,7 @@
     </row>
     <row r="102">
       <c r="C102" s="133" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D102" s="122">
         <f t="shared" si="17"/>
@@ -16060,7 +16048,7 @@
     </row>
     <row r="103">
       <c r="C103" s="133" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D103" s="122">
         <f t="shared" si="17"/>
@@ -16078,7 +16066,7 @@
     </row>
     <row r="104">
       <c r="C104" s="133" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D104" s="122">
         <f t="shared" si="17"/>
@@ -16097,7 +16085,7 @@
     </row>
     <row r="105">
       <c r="C105" s="133" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="D105" s="122">
         <f t="shared" si="17"/>
@@ -16116,7 +16104,7 @@
     </row>
     <row r="106">
       <c r="C106" s="133" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D106" s="122">
         <f t="shared" si="17"/>
@@ -16135,7 +16123,7 @@
     </row>
     <row r="107">
       <c r="C107" s="133" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="D107" s="122">
         <f t="shared" si="17"/>
@@ -16154,7 +16142,7 @@
     </row>
     <row r="108">
       <c r="C108" s="133" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="D108" s="122">
         <f t="shared" si="17"/>
@@ -16173,7 +16161,7 @@
     </row>
     <row r="109">
       <c r="C109" s="133" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D109" s="122">
         <f t="shared" si="17"/>
@@ -16192,7 +16180,7 @@
     </row>
     <row r="110">
       <c r="C110" s="133" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D110" s="122">
         <f t="shared" si="17"/>
@@ -16211,7 +16199,7 @@
     </row>
     <row r="111">
       <c r="C111" s="133" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="D111" s="122">
         <f t="shared" si="17"/>
@@ -16230,7 +16218,7 @@
     </row>
     <row r="112">
       <c r="C112" s="133" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D112" s="122">
         <f t="shared" si="17"/>
@@ -16248,7 +16236,7 @@
     </row>
     <row r="113">
       <c r="C113" s="133" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="D113" s="122">
         <f t="shared" si="17"/>
@@ -16266,7 +16254,7 @@
     </row>
     <row r="114">
       <c r="C114" s="133" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D114" s="122">
         <f t="shared" si="17"/>
@@ -16284,7 +16272,7 @@
     </row>
     <row r="115">
       <c r="C115" s="133" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="D115" s="122">
         <f t="shared" si="17"/>
@@ -16302,7 +16290,7 @@
     </row>
     <row r="116">
       <c r="C116" s="133" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D116" s="122">
         <f t="shared" si="17"/>
@@ -16320,7 +16308,7 @@
     </row>
     <row r="117">
       <c r="C117" s="133" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D117" s="122">
         <f t="shared" si="17"/>
@@ -16336,7 +16324,7 @@
     </row>
     <row r="118">
       <c r="C118" s="133" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D118" s="122">
         <f t="shared" si="17"/>
@@ -16352,7 +16340,7 @@
     </row>
     <row r="119">
       <c r="C119" s="133" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D119" s="122">
         <f t="shared" si="17"/>
@@ -16368,7 +16356,7 @@
     </row>
     <row r="120">
       <c r="C120" s="133" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D120" s="122">
         <f t="shared" si="17"/>
@@ -16384,7 +16372,7 @@
     </row>
     <row r="121">
       <c r="C121" s="133" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D121" s="122">
         <f t="shared" si="17"/>
@@ -16400,7 +16388,7 @@
     </row>
     <row r="122">
       <c r="C122" s="133" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D122" s="122">
         <f t="shared" si="17"/>
@@ -16416,7 +16404,7 @@
     </row>
     <row r="123">
       <c r="C123" s="133" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="D123" s="122">
         <f t="shared" si="17"/>
@@ -16432,7 +16420,7 @@
     </row>
     <row r="124">
       <c r="C124" s="133" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D124" s="122">
         <f t="shared" si="17"/>
@@ -38884,14 +38872,14 @@
     <row r="1">
       <c r="A1" s="102"/>
       <c r="B1" s="143" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C1" s="144"/>
       <c r="D1" s="144"/>
       <c r="E1" s="144"/>
       <c r="F1" s="144"/>
       <c r="G1" s="145" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="H1" s="144"/>
       <c r="I1" s="144"/>
@@ -38919,49 +38907,49 @@
         <v>3</v>
       </c>
       <c r="B2" s="147" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C2" s="148" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="D2" s="148" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="E2" s="148" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="F2" s="149" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="G2" s="147">
         <v>1.0</v>
       </c>
       <c r="H2" s="148" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I2" s="148">
         <v>2.0</v>
       </c>
       <c r="J2" s="148" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="K2" s="150" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="L2" s="148" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="M2" s="151" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="N2" s="98" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="O2" s="98" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="P2" s="98" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="Q2" s="10"/>
       <c r="R2" s="10"/>
@@ -39634,7 +39622,7 @@
     </row>
     <row r="24">
       <c r="A24" s="92" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B24" s="163" t="str">
         <f t="shared" ref="B24:F24" si="4">IFERROR(AVERAGE(B3:B22),"")</f>
@@ -39744,7 +39732,7 @@
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
       <c r="G27" s="164" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="H27" s="10"/>
       <c r="I27" s="10"/>
@@ -39777,7 +39765,7 @@
         <v>1.0</v>
       </c>
       <c r="H28" s="165" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I28" s="165">
         <v>2.0</v>
@@ -39805,7 +39793,7 @@
       <c r="B29" s="10"/>
       <c r="C29" s="10"/>
       <c r="D29" s="6" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E29" s="6">
         <f>J29</f>
@@ -39827,10 +39815,10 @@
       </c>
       <c r="K29" s="10"/>
       <c r="L29" s="92" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="M29" s="92" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="O29" s="6">
         <v>1.0</v>
@@ -39966,7 +39954,7 @@
       <c r="E33" s="10"/>
       <c r="F33" s="10"/>
       <c r="G33" s="117" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="J33" s="10"/>
       <c r="K33" s="10"/>
@@ -40000,7 +39988,7 @@
         <v>1.0</v>
       </c>
       <c r="H34" s="168" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I34" s="168">
         <v>2.0</v>
@@ -40143,7 +40131,7 @@
       <c r="D38" s="10"/>
       <c r="E38" s="10"/>
       <c r="F38" s="6" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="G38" s="167">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
Corrijo path de betting strategy + actualizo datos
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -33,11 +33,6 @@
       <text>
         <t xml:space="preserve">los que mas valor tienen suelen tener un rdo mucho mas rentable que otro.
 </t>
-      </text>
-    </comment>
-    <comment authorId="0" ref="M4">
-      <text>
-        <t xml:space="preserve">el empate...</t>
       </text>
     </comment>
     <comment authorId="0" ref="A1">
@@ -211,7 +206,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="279">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="262">
   <si>
     <t>id_country</t>
   </si>
@@ -735,28 +730,25 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>2.33</t>
+    <t>0.00</t>
   </si>
   <si>
-    <t>0.08</t>
+    <t>2.39</t>
   </si>
   <si>
-    <t>0.86</t>
+    <t>0.37</t>
   </si>
   <si>
-    <t>0.23</t>
+    <t>6.63</t>
   </si>
   <si>
-    <t>8.96</t>
+    <t>6.25</t>
   </si>
   <si>
-    <t>9.16</t>
+    <t>2.45</t>
   </si>
   <si>
-    <t>9.83</t>
-  </si>
-  <si>
-    <t>4.55</t>
+    <t>1.66</t>
   </si>
   <si>
     <t>Country</t>
@@ -765,247 +757,199 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>6.78</t>
+    <t>2.82</t>
   </si>
   <si>
-    <t>5.35</t>
+    <t>1.16</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>9.07</t>
+    <t>2.34</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>9.62</t>
+    <t>5.55</t>
   </si>
   <si>
     <t>p25</t>
   </si>
   <si>
-    <t>6.23</t>
+    <t>6.52</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>6.67</t>
+    <t>9.11</t>
   </si>
   <si>
-    <t>7.71</t>
+    <t>8.92</t>
   </si>
   <si>
-    <t>7.62</t>
+    <t>5.46</t>
   </si>
   <si>
-    <t>8.13</t>
+    <t>2.49</t>
   </si>
   <si>
-    <t>7.73</t>
+    <t>4.97</t>
   </si>
   <si>
-    <t>7.80</t>
+    <t>4.98</t>
+  </si>
+  <si>
+    <t>4.46</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
   </si>
   <si>
-    <t>7.94</t>
+    <t>5.12</t>
   </si>
   <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>8.21</t>
+    <t>4.95</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
-    <t>8.04</t>
+    <t>4.85</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>7.59</t>
-  </si>
-  <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
-    <t>2.60</t>
+    <t>2.00</t>
   </si>
   <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>2.54</t>
+    <t>1.40</t>
   </si>
   <si>
-    <t>4.30</t>
+    <t>2.19</t>
   </si>
   <si>
-    <t>3.91</t>
+    <t>0.49</t>
   </si>
   <si>
-    <t>11.47</t>
+    <t>0.05</t>
   </si>
   <si>
-    <t>0.00</t>
+    <t>5.85</t>
   </si>
   <si>
-    <t>10.36</t>
+    <t>6.81</t>
+  </si>
+  <si>
+    <t>5.65</t>
+  </si>
+  <si>
+    <t>6.19</t>
+  </si>
+  <si>
+    <t>1.62</t>
+  </si>
+  <si>
+    <t>6.58</t>
+  </si>
+  <si>
+    <t>6.08</t>
+  </si>
+  <si>
+    <t>1.06</t>
+  </si>
+  <si>
+    <t>1.48</t>
+  </si>
+  <si>
+    <t>1.45</t>
+  </si>
+  <si>
+    <t>1.60</t>
+  </si>
+  <si>
+    <t>1.89</t>
+  </si>
+  <si>
+    <t>1.28</t>
+  </si>
+  <si>
+    <t>2.05</t>
+  </si>
+  <si>
+    <t>1.75</t>
+  </si>
+  <si>
+    <t>1.18</t>
+  </si>
+  <si>
+    <t>1.77</t>
+  </si>
+  <si>
+    <t>1.74</t>
+  </si>
+  <si>
+    <t>1.69</t>
+  </si>
+  <si>
+    <t>1.59</t>
+  </si>
+  <si>
+    <t>1.70</t>
+  </si>
+  <si>
+    <t>1.87</t>
+  </si>
+  <si>
+    <t>1.14</t>
+  </si>
+  <si>
+    <t>1.19</t>
+  </si>
+  <si>
+    <t>1.21</t>
+  </si>
+  <si>
+    <t>4.59</t>
   </si>
   <si>
     <t>10.91</t>
   </si>
   <si>
-    <t>1.95</t>
+    <t>9.79</t>
   </si>
   <si>
-    <t>9.68</t>
+    <t>10.92</t>
   </si>
   <si>
-    <t>9.01</t>
+    <t>13.09</t>
   </si>
   <si>
-    <t>9.76</t>
+    <t>13.14</t>
   </si>
   <si>
-    <t>7.88</t>
+    <t>10.26</t>
   </si>
   <si>
-    <t>13.76</t>
+    <t>11.82</t>
   </si>
   <si>
-    <t>13.51</t>
+    <t>10.88</t>
   </si>
   <si>
-    <t>1.98</t>
-  </si>
-  <si>
-    <t>2.45</t>
-  </si>
-  <si>
-    <t>2.28</t>
-  </si>
-  <si>
-    <t>2.29</t>
-  </si>
-  <si>
-    <t>0.10</t>
-  </si>
-  <si>
-    <t>2.55</t>
-  </si>
-  <si>
-    <t>2.18</t>
-  </si>
-  <si>
-    <t>1.16</t>
-  </si>
-  <si>
-    <t>1.49</t>
-  </si>
-  <si>
-    <t>4.05</t>
-  </si>
-  <si>
-    <t>7.19</t>
-  </si>
-  <si>
-    <t>2.16</t>
-  </si>
-  <si>
-    <t>2.46</t>
-  </si>
-  <si>
-    <t>7.75</t>
-  </si>
-  <si>
-    <t>8.36</t>
-  </si>
-  <si>
-    <t>4.22</t>
-  </si>
-  <si>
-    <t>8.00</t>
-  </si>
-  <si>
-    <t>8.33</t>
-  </si>
-  <si>
-    <t>7.89</t>
-  </si>
-  <si>
-    <t>4.83</t>
-  </si>
-  <si>
-    <t>3.08</t>
-  </si>
-  <si>
-    <t>6.35</t>
-  </si>
-  <si>
-    <t>3.42</t>
-  </si>
-  <si>
-    <t>5.68</t>
-  </si>
-  <si>
-    <t>6.46</t>
-  </si>
-  <si>
-    <t>6.97</t>
-  </si>
-  <si>
-    <t>6.55</t>
-  </si>
-  <si>
-    <t>6.13</t>
-  </si>
-  <si>
-    <t>3.44</t>
-  </si>
-  <si>
-    <t>7.03</t>
-  </si>
-  <si>
-    <t>2.22</t>
-  </si>
-  <si>
-    <t>2.49</t>
-  </si>
-  <si>
-    <t>5.89</t>
-  </si>
-  <si>
-    <t>4.85</t>
-  </si>
-  <si>
-    <t>2.86</t>
-  </si>
-  <si>
-    <t>2.62</t>
-  </si>
-  <si>
-    <t>2.98</t>
-  </si>
-  <si>
-    <t>3.00</t>
-  </si>
-  <si>
-    <t>2.85</t>
-  </si>
-  <si>
-    <t>2.93</t>
-  </si>
-  <si>
-    <t>2.99</t>
+    <t>10.81</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2144,31 +2088,32 @@
         <v>45685.0</v>
       </c>
       <c r="D2" s="14">
-        <v>40.0</v>
+        <v>616.0</v>
       </c>
       <c r="E2" s="15" t="s">
         <v>14</v>
       </c>
       <c r="F2" s="16">
-        <v>155.067930759269</v>
+        <f>5.8410821479406*100</f>
+        <v>584.1082148</v>
       </c>
       <c r="G2" s="17">
         <v>70.0</v>
       </c>
       <c r="H2" s="17">
-        <v>25.0</v>
+        <v>45.0</v>
       </c>
       <c r="I2" s="17">
-        <v>25.0</v>
+        <v>10.0</v>
       </c>
       <c r="J2" s="18"/>
       <c r="K2" s="18"/>
       <c r="L2" s="19">
-        <v>947.246174692297</v>
+        <v>31833.0939389723</v>
       </c>
       <c r="M2" s="20">
         <f>L2/F2</f>
-        <v>6.108588475</v>
+        <v>54.49862394</v>
       </c>
       <c r="N2" s="21"/>
       <c r="O2" s="22"/>
@@ -2211,7 +2156,8 @@
         <v>14</v>
       </c>
       <c r="F4" s="16">
-        <v>196.201829289439</v>
+        <f>1.95083127981317*100</f>
+        <v>195.083128</v>
       </c>
       <c r="G4" s="17">
         <v>10.0</v>
@@ -2231,11 +2177,11 @@
         <v>5</v>
       </c>
       <c r="L4" s="19">
-        <v>1933.66205998427</v>
+        <v>2031.72738744972</v>
       </c>
       <c r="M4" s="20">
         <f t="shared" ref="M4:M8" si="2">L4/F4</f>
-        <v>9.855474167</v>
+        <v>10.41467506</v>
       </c>
     </row>
     <row r="5">
@@ -2255,7 +2201,8 @@
         <v>14</v>
       </c>
       <c r="F5" s="16">
-        <v>328.964710450097</v>
+        <f>3.44623889518345*100</f>
+        <v>344.6238895</v>
       </c>
       <c r="G5" s="19">
         <v>70.0</v>
@@ -2275,11 +2222,11 @@
         <v>13.33333333</v>
       </c>
       <c r="L5" s="19">
-        <v>13260.6600418071</v>
+        <v>7144.81139954358</v>
       </c>
       <c r="M5" s="20">
         <f t="shared" si="2"/>
-        <v>40.31028138</v>
+        <v>20.73219999</v>
       </c>
       <c r="O5" s="31"/>
     </row>
@@ -2300,7 +2247,8 @@
         <v>14</v>
       </c>
       <c r="F6" s="16">
-        <v>507.622113409045</v>
+        <f>5.03501136998037*100</f>
+        <v>503.501137</v>
       </c>
       <c r="G6" s="19">
         <v>70.0</v>
@@ -2324,7 +2272,7 @@
       </c>
       <c r="M6" s="20">
         <f t="shared" si="2"/>
-        <v>144.8361095</v>
+        <v>146.0215412</v>
       </c>
     </row>
     <row r="7">
@@ -2338,13 +2286,14 @@
         <v>45677.0</v>
       </c>
       <c r="D7" s="15">
-        <v>1551.0</v>
+        <v>281.0</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>14</v>
       </c>
       <c r="F7" s="16">
-        <v>272.560347757221</v>
+        <f>2.76792853614368*100</f>
+        <v>276.7928536</v>
       </c>
       <c r="G7" s="17">
         <v>10.0</v>
@@ -2353,22 +2302,22 @@
         <v>70.0</v>
       </c>
       <c r="I7" s="17">
-        <v>45.0</v>
+        <v>70.0</v>
       </c>
       <c r="J7" s="25">
         <f t="shared" si="1"/>
-        <v>41.66666667</v>
+        <v>50</v>
       </c>
       <c r="K7" s="27">
         <f>J7*'Data preparation'!$C$2</f>
-        <v>10.41666667</v>
+        <v>12.5</v>
       </c>
       <c r="L7" s="19">
-        <v>1944.23207418205</v>
+        <v>13938.355259875</v>
       </c>
       <c r="M7" s="20">
         <f t="shared" si="2"/>
-        <v>7.133216883</v>
+        <v>50.3566298</v>
       </c>
     </row>
     <row r="8">
@@ -2388,7 +2337,8 @@
         <v>14</v>
       </c>
       <c r="F8" s="16">
-        <v>331.827702137116</v>
+        <f>4.33116583093229*100</f>
+        <v>433.1165831</v>
       </c>
       <c r="G8" s="17">
         <v>45.0</v>
@@ -2397,22 +2347,22 @@
         <v>10.0</v>
       </c>
       <c r="I8" s="17">
-        <v>10.0</v>
+        <v>25.0</v>
       </c>
       <c r="J8" s="20">
         <f t="shared" si="1"/>
-        <v>21.66666667</v>
+        <v>26.66666667</v>
       </c>
       <c r="K8" s="27">
         <f>J8*'Data preparation'!$C$2</f>
-        <v>5.416666667</v>
+        <v>6.666666667</v>
       </c>
       <c r="L8" s="19">
-        <v>2994.68938021348</v>
+        <v>5748.94662953238</v>
       </c>
       <c r="M8" s="20">
         <f t="shared" si="2"/>
-        <v>9.024832348</v>
+        <v>13.27343919</v>
       </c>
     </row>
     <row r="9" ht="20.25" customHeight="1">
@@ -13277,7 +13227,7 @@
       </c>
       <c r="C3" s="26">
         <f>AVERAGE('Modelos actuales'!K4:K8)</f>
-        <v>9.333333333</v>
+        <v>10</v>
       </c>
       <c r="L3" s="112"/>
       <c r="P3" s="112"/>
@@ -14578,7 +14528,7 @@
       <c r="C37" s="40"/>
       <c r="D37" s="127">
         <f>AVERAGE(D39:D1775)</f>
-        <v>5.495813953</v>
+        <v>4.334852941</v>
       </c>
       <c r="G37" s="35" t="s">
         <v>36</v>
@@ -14647,7 +14597,7 @@
       </c>
       <c r="D39" s="119">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>2.33</v>
+        <v>0</v>
       </c>
       <c r="G39" s="35" t="s">
         <v>28</v>
@@ -14685,7 +14635,7 @@
       </c>
       <c r="D40" s="119">
         <f t="shared" si="17"/>
-        <v>0.08</v>
+        <v>2.39</v>
       </c>
       <c r="G40" s="35" t="s">
         <v>24</v>
@@ -14723,7 +14673,7 @@
       </c>
       <c r="D41" s="119">
         <f t="shared" si="17"/>
-        <v>0.86</v>
+        <v>0.37</v>
       </c>
       <c r="P41" s="116">
         <v>0.0</v>
@@ -14751,11 +14701,11 @@
     </row>
     <row r="42">
       <c r="C42" s="130" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D42" s="119">
         <f t="shared" si="17"/>
-        <v>0.23</v>
+        <v>0</v>
       </c>
       <c r="P42" s="116">
         <v>2.0</v>
@@ -14783,11 +14733,11 @@
     </row>
     <row r="43">
       <c r="C43" s="130" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D43" s="119">
         <f t="shared" si="17"/>
-        <v>8.96</v>
+        <v>6.63</v>
       </c>
       <c r="P43" s="116">
         <v>1.0</v>
@@ -14815,11 +14765,11 @@
     </row>
     <row r="44">
       <c r="C44" s="130" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D44" s="119">
         <f t="shared" si="17"/>
-        <v>9.16</v>
+        <v>6.25</v>
       </c>
       <c r="P44" s="116">
         <v>2.0</v>
@@ -14845,11 +14795,11 @@
     </row>
     <row r="45">
       <c r="C45" s="130" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D45" s="119">
         <f t="shared" si="17"/>
-        <v>9.83</v>
+        <v>2.45</v>
       </c>
       <c r="P45" s="116">
         <v>1.0</v>
@@ -14863,17 +14813,17 @@
     </row>
     <row r="46">
       <c r="C46" s="130" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D46" s="119">
         <f t="shared" si="17"/>
-        <v>4.55</v>
+        <v>1.66</v>
       </c>
       <c r="G46" s="90" t="s">
+        <v>176</v>
+      </c>
+      <c r="H46" s="90" t="s">
         <v>177</v>
-      </c>
-      <c r="H46" s="90" t="s">
-        <v>178</v>
       </c>
       <c r="P46" s="116">
         <v>0.0</v>
@@ -14887,11 +14837,11 @@
     </row>
     <row r="47">
       <c r="C47" s="130" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D47" s="119">
         <f t="shared" si="17"/>
-        <v>6.78</v>
+        <v>2.82</v>
       </c>
       <c r="G47" s="95" t="s">
         <v>37</v>
@@ -14917,11 +14867,11 @@
     </row>
     <row r="48">
       <c r="C48" s="130" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D48" s="119">
         <f t="shared" si="17"/>
-        <v>5.35</v>
+        <v>1.16</v>
       </c>
       <c r="G48" s="95" t="s">
         <v>36</v>
@@ -14930,7 +14880,7 @@
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="42" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="K48" s="117">
         <f>AVERAGE(H47:H51)</f>
@@ -14954,11 +14904,11 @@
     </row>
     <row r="49">
       <c r="C49" s="130" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D49" s="119">
         <f t="shared" si="17"/>
-        <v>9.07</v>
+        <v>2.34</v>
       </c>
       <c r="G49" s="95" t="s">
         <v>27</v>
@@ -14967,7 +14917,7 @@
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="42" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K49" s="117">
         <f>MEDIAN(H47:H51)</f>
@@ -14991,11 +14941,11 @@
     </row>
     <row r="50">
       <c r="C50" s="130" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="D50" s="119">
         <f t="shared" si="17"/>
-        <v>9.62</v>
+        <v>5.55</v>
       </c>
       <c r="G50" s="95" t="s">
         <v>28</v>
@@ -15004,7 +14954,7 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="42" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K50" s="117">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -15028,11 +14978,11 @@
     </row>
     <row r="51">
       <c r="C51" s="130" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="D51" s="119">
         <f t="shared" si="17"/>
-        <v>6.23</v>
+        <v>6.52</v>
       </c>
       <c r="G51" s="95" t="s">
         <v>24</v>
@@ -15041,7 +14991,7 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="42" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K51" s="117">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -15065,11 +15015,11 @@
     </row>
     <row r="52">
       <c r="C52" s="130" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="D52" s="119">
         <f t="shared" si="17"/>
-        <v>6.67</v>
+        <v>9.11</v>
       </c>
       <c r="P52" s="116">
         <v>0.0</v>
@@ -15089,11 +15039,11 @@
     </row>
     <row r="53">
       <c r="C53" s="130" t="s">
-        <v>173</v>
+        <v>188</v>
       </c>
       <c r="D53" s="119">
         <f t="shared" si="17"/>
-        <v>8.96</v>
+        <v>8.92</v>
       </c>
       <c r="P53" s="116">
         <v>0.0</v>
@@ -15117,7 +15067,7 @@
       </c>
       <c r="D54" s="119">
         <f t="shared" si="17"/>
-        <v>7.71</v>
+        <v>5.46</v>
       </c>
       <c r="P54" s="116">
         <v>2.0</v>
@@ -15141,7 +15091,7 @@
       </c>
       <c r="D55" s="119">
         <f t="shared" si="17"/>
-        <v>7.62</v>
+        <v>2.49</v>
       </c>
       <c r="P55" s="116">
         <v>0.0</v>
@@ -15165,7 +15115,7 @@
       </c>
       <c r="D56" s="119">
         <f t="shared" si="17"/>
-        <v>8.13</v>
+        <v>4.97</v>
       </c>
       <c r="P56" s="116">
         <v>0.0</v>
@@ -15189,7 +15139,7 @@
       </c>
       <c r="D57" s="119">
         <f t="shared" si="17"/>
-        <v>7.73</v>
+        <v>4.98</v>
       </c>
       <c r="P57" s="116">
         <v>2.0</v>
@@ -15213,7 +15163,7 @@
       </c>
       <c r="D58" s="119">
         <f t="shared" si="17"/>
-        <v>7.8</v>
+        <v>4.46</v>
       </c>
       <c r="G58" s="132" t="s">
         <v>194</v>
@@ -15241,7 +15191,7 @@
       </c>
       <c r="D59" s="119">
         <f t="shared" si="17"/>
-        <v>7.94</v>
+        <v>5.12</v>
       </c>
       <c r="G59" s="133"/>
       <c r="H59" s="134" t="s">
@@ -15269,7 +15219,7 @@
       </c>
       <c r="D60" s="119">
         <f t="shared" si="17"/>
-        <v>8.21</v>
+        <v>4.95</v>
       </c>
       <c r="G60" s="133"/>
       <c r="H60" s="134" t="s">
@@ -15297,7 +15247,7 @@
       </c>
       <c r="D61" s="119">
         <f t="shared" si="17"/>
-        <v>8.04</v>
+        <v>4.85</v>
       </c>
       <c r="G61" s="133"/>
       <c r="H61" s="134" t="s">
@@ -15321,15 +15271,15 @@
     </row>
     <row r="62">
       <c r="C62" s="130" t="s">
-        <v>201</v>
+        <v>159</v>
       </c>
       <c r="D62" s="119">
         <f t="shared" si="17"/>
-        <v>7.59</v>
+        <v>4.73</v>
       </c>
       <c r="G62" s="133"/>
       <c r="H62" s="134" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="P62" s="116">
         <v>1.0</v>
@@ -15349,15 +15299,15 @@
     </row>
     <row r="63">
       <c r="C63" s="130" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D63" s="119">
         <f t="shared" si="17"/>
-        <v>2.6</v>
+        <v>2</v>
       </c>
       <c r="G63" s="133"/>
       <c r="H63" s="134" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="P63" s="116">
         <v>0.0</v>
@@ -15371,11 +15321,11 @@
     </row>
     <row r="64">
       <c r="C64" s="130" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D64" s="119">
         <f t="shared" si="17"/>
-        <v>2.54</v>
+        <v>1.4</v>
       </c>
       <c r="P64" s="116">
         <v>1.0</v>
@@ -15389,11 +15339,11 @@
     </row>
     <row r="65">
       <c r="C65" s="130" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D65" s="119">
         <f t="shared" si="17"/>
-        <v>4.3</v>
+        <v>2.19</v>
       </c>
       <c r="P65" s="116">
         <v>2.0</v>
@@ -15407,11 +15357,11 @@
     </row>
     <row r="66">
       <c r="C66" s="130" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D66" s="119">
         <f t="shared" si="17"/>
-        <v>3.91</v>
+        <v>0.49</v>
       </c>
       <c r="P66" s="116">
         <v>0.0</v>
@@ -15425,11 +15375,11 @@
     </row>
     <row r="67">
       <c r="C67" s="130" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D67" s="119">
         <f t="shared" si="17"/>
-        <v>11.47</v>
+        <v>0.05</v>
       </c>
       <c r="P67" s="116">
         <v>0.0</v>
@@ -15443,11 +15393,11 @@
     </row>
     <row r="68">
       <c r="C68" s="130" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D68" s="119">
         <f t="shared" si="17"/>
-        <v>0</v>
+        <v>5.85</v>
       </c>
       <c r="P68" s="116">
         <v>1.0</v>
@@ -15461,11 +15411,11 @@
     </row>
     <row r="69">
       <c r="C69" s="130" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D69" s="119">
         <f t="shared" si="17"/>
-        <v>10.36</v>
+        <v>6.81</v>
       </c>
       <c r="P69" s="116">
         <v>2.0</v>
@@ -15479,11 +15429,11 @@
     </row>
     <row r="70">
       <c r="C70" s="130" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="D70" s="119">
         <f t="shared" si="17"/>
-        <v>10.91</v>
+        <v>5.46</v>
       </c>
       <c r="P70" s="116">
         <v>1.0</v>
@@ -15497,11 +15447,11 @@
     </row>
     <row r="71">
       <c r="C71" s="130" t="s">
-        <v>212</v>
+        <v>159</v>
       </c>
       <c r="D71" s="119">
         <f t="shared" si="17"/>
-        <v>1.95</v>
+        <v>4.73</v>
       </c>
       <c r="F71" s="135"/>
       <c r="P71" s="116">
@@ -15516,11 +15466,11 @@
     </row>
     <row r="72">
       <c r="C72" s="130" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="D72" s="119">
         <f t="shared" si="17"/>
-        <v>9.68</v>
+        <v>5.65</v>
       </c>
       <c r="P72" s="116">
         <v>0.0</v>
@@ -15534,11 +15484,11 @@
     </row>
     <row r="73">
       <c r="C73" s="130" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="D73" s="119">
         <f t="shared" si="17"/>
-        <v>9.01</v>
+        <v>6.19</v>
       </c>
       <c r="P73" s="116">
         <v>1.0</v>
@@ -15552,11 +15502,11 @@
     </row>
     <row r="74">
       <c r="C74" s="130" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D74" s="119">
         <f t="shared" si="17"/>
-        <v>9.76</v>
+        <v>1.62</v>
       </c>
       <c r="P74" s="116">
         <v>0.0</v>
@@ -15570,11 +15520,11 @@
     </row>
     <row r="75">
       <c r="C75" s="130" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D75" s="119">
         <f t="shared" si="17"/>
-        <v>7.88</v>
+        <v>6.58</v>
       </c>
       <c r="P75" s="116">
         <v>1.0</v>
@@ -15588,11 +15538,11 @@
     </row>
     <row r="76">
       <c r="C76" s="130" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="D76" s="119">
         <f t="shared" si="17"/>
-        <v>13.76</v>
+        <v>6.58</v>
       </c>
       <c r="P76" s="116">
         <v>0.0</v>
@@ -15606,11 +15556,11 @@
     </row>
     <row r="77">
       <c r="C77" s="130" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="D77" s="119">
         <f t="shared" si="17"/>
-        <v>13.51</v>
+        <v>6.08</v>
       </c>
       <c r="P77" s="116">
         <v>0.0</v>
@@ -15624,11 +15574,11 @@
     </row>
     <row r="78">
       <c r="C78" s="130" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="D78" s="119">
         <f t="shared" si="17"/>
-        <v>1.98</v>
+        <v>1.06</v>
       </c>
       <c r="P78" s="116">
         <v>1.0</v>
@@ -15642,11 +15592,11 @@
     </row>
     <row r="79">
       <c r="C79" s="130" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="D79" s="119">
         <f t="shared" si="17"/>
-        <v>2.45</v>
+        <v>1.48</v>
       </c>
       <c r="P79" s="116">
         <v>2.0</v>
@@ -15660,11 +15610,11 @@
     </row>
     <row r="80">
       <c r="C80" s="130" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="D80" s="119">
         <f t="shared" si="17"/>
-        <v>2.28</v>
+        <v>1.45</v>
       </c>
       <c r="P80" s="116">
         <v>1.0</v>
@@ -15678,11 +15628,11 @@
     </row>
     <row r="81">
       <c r="C81" s="130" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="D81" s="119">
         <f t="shared" si="17"/>
-        <v>2.29</v>
+        <v>1.6</v>
       </c>
       <c r="P81" s="116">
         <v>2.0</v>
@@ -15696,11 +15646,11 @@
     </row>
     <row r="82">
       <c r="C82" s="130" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="D82" s="119">
         <f t="shared" si="17"/>
-        <v>0.1</v>
+        <v>1.89</v>
       </c>
       <c r="P82" s="116">
         <v>1.0</v>
@@ -15714,11 +15664,11 @@
     </row>
     <row r="83">
       <c r="C83" s="130" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="D83" s="119">
         <f t="shared" si="17"/>
-        <v>2.55</v>
+        <v>1.28</v>
       </c>
       <c r="P83" s="116">
         <v>0.0</v>
@@ -15732,11 +15682,11 @@
     </row>
     <row r="84">
       <c r="C84" s="130" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="D84" s="119">
         <f t="shared" si="17"/>
-        <v>2.18</v>
+        <v>2.05</v>
       </c>
       <c r="P84" s="116">
         <v>1.0</v>
@@ -15750,11 +15700,11 @@
     </row>
     <row r="85">
       <c r="C85" s="130" t="s">
-        <v>179</v>
+        <v>222</v>
       </c>
       <c r="D85" s="119">
         <f t="shared" si="17"/>
-        <v>6.78</v>
+        <v>1.75</v>
       </c>
       <c r="P85" s="116">
         <v>0.0</v>
@@ -15768,11 +15718,11 @@
     </row>
     <row r="86">
       <c r="C86" s="130" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D86" s="119">
         <f t="shared" si="17"/>
-        <v>1.16</v>
+        <v>1.18</v>
       </c>
       <c r="P86" s="116">
         <v>0.0</v>
@@ -15786,11 +15736,11 @@
     </row>
     <row r="87">
       <c r="C87" s="130" t="s">
-        <v>227</v>
+        <v>215</v>
       </c>
       <c r="D87" s="119">
         <f t="shared" si="17"/>
-        <v>1.49</v>
+        <v>1.06</v>
       </c>
       <c r="P87" s="116">
         <v>1.0</v>
@@ -15804,11 +15754,11 @@
     </row>
     <row r="88">
       <c r="C88" s="130" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="D88" s="119">
         <f t="shared" si="17"/>
-        <v>4.05</v>
+        <v>1.77</v>
       </c>
       <c r="P88" s="116">
         <v>2.0</v>
@@ -15822,11 +15772,11 @@
     </row>
     <row r="89">
       <c r="C89" s="130" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="D89" s="119">
         <f t="shared" si="17"/>
-        <v>7.19</v>
+        <v>1.74</v>
       </c>
       <c r="P89" s="116">
         <v>2.0</v>
@@ -15840,11 +15790,11 @@
     </row>
     <row r="90">
       <c r="C90" s="130" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="D90" s="119">
         <f t="shared" si="17"/>
-        <v>2.16</v>
+        <v>1.69</v>
       </c>
       <c r="P90" s="116">
         <v>1.0</v>
@@ -15858,11 +15808,11 @@
     </row>
     <row r="91">
       <c r="C91" s="130" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="D91" s="119">
         <f t="shared" si="17"/>
-        <v>2.46</v>
+        <v>1.59</v>
       </c>
       <c r="P91" s="116">
         <v>1.0</v>
@@ -15876,11 +15826,11 @@
     </row>
     <row r="92">
       <c r="C92" s="130" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="D92" s="119">
         <f t="shared" si="17"/>
-        <v>2.29</v>
+        <v>1.7</v>
       </c>
       <c r="P92" s="116">
         <v>2.0</v>
@@ -15894,11 +15844,11 @@
     </row>
     <row r="93">
       <c r="C93" s="130" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D93" s="119">
         <f t="shared" si="17"/>
-        <v>7.75</v>
+        <v>1.87</v>
       </c>
       <c r="P93" s="116">
         <v>0.0</v>
@@ -15912,11 +15862,11 @@
     </row>
     <row r="94">
       <c r="C94" s="130" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D94" s="119">
         <f t="shared" si="17"/>
-        <v>8.36</v>
+        <v>1.14</v>
       </c>
       <c r="P94" s="116">
         <v>0.0</v>
@@ -15930,11 +15880,11 @@
     </row>
     <row r="95">
       <c r="C95" s="130" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D95" s="119">
         <f t="shared" si="17"/>
-        <v>4.22</v>
+        <v>1.19</v>
       </c>
       <c r="P95" s="116">
         <v>1.0</v>
@@ -15948,11 +15898,11 @@
     </row>
     <row r="96">
       <c r="C96" s="130" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D96" s="119">
         <f t="shared" si="17"/>
-        <v>8</v>
+        <v>1.21</v>
       </c>
       <c r="P96" s="116">
         <v>2.0</v>
@@ -15966,11 +15916,11 @@
     </row>
     <row r="97">
       <c r="C97" s="130" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D97" s="119">
         <f t="shared" si="17"/>
-        <v>8.33</v>
+        <v>4.59</v>
       </c>
       <c r="P97" s="116">
         <v>0.0</v>
@@ -15984,11 +15934,11 @@
     </row>
     <row r="98">
       <c r="C98" s="130" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D98" s="119">
         <f t="shared" si="17"/>
-        <v>7.89</v>
+        <v>10.91</v>
       </c>
       <c r="P98" s="116">
         <v>2.0</v>
@@ -16002,11 +15952,11 @@
     </row>
     <row r="99">
       <c r="C99" s="130" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D99" s="119">
         <f t="shared" si="17"/>
-        <v>4.83</v>
+        <v>9.79</v>
       </c>
       <c r="P99" s="116">
         <v>2.0</v>
@@ -16020,11 +15970,11 @@
     </row>
     <row r="100">
       <c r="C100" s="130" t="s">
-        <v>190</v>
+        <v>236</v>
       </c>
       <c r="D100" s="119">
         <f t="shared" si="17"/>
-        <v>7.62</v>
+        <v>10.92</v>
       </c>
       <c r="P100" s="116">
         <v>2.0</v>
@@ -16038,11 +15988,11 @@
     </row>
     <row r="101">
       <c r="C101" s="130" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D101" s="119">
         <f t="shared" si="17"/>
-        <v>3.08</v>
+        <v>13.09</v>
       </c>
       <c r="P101" s="116">
         <v>2.0</v>
@@ -16056,11 +16006,11 @@
     </row>
     <row r="102">
       <c r="C102" s="130" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="D102" s="119">
         <f t="shared" si="17"/>
-        <v>6.35</v>
+        <v>13.14</v>
       </c>
       <c r="P102" s="116">
         <v>2.0</v>
@@ -16074,11 +16024,11 @@
     </row>
     <row r="103">
       <c r="C103" s="130" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="D103" s="119">
         <f t="shared" si="17"/>
-        <v>3.42</v>
+        <v>10.26</v>
       </c>
       <c r="P103" s="116">
         <v>1.0</v>
@@ -16092,11 +16042,11 @@
     </row>
     <row r="104">
       <c r="C104" s="130" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="D104" s="119">
         <f t="shared" si="17"/>
-        <v>5.68</v>
+        <v>11.82</v>
       </c>
       <c r="N104" s="136"/>
       <c r="P104" s="116">
@@ -16111,11 +16061,11 @@
     </row>
     <row r="105">
       <c r="C105" s="130" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="D105" s="119">
         <f t="shared" si="17"/>
-        <v>6.46</v>
+        <v>10.88</v>
       </c>
       <c r="N105" s="21"/>
       <c r="P105" s="116">
@@ -16130,11 +16080,11 @@
     </row>
     <row r="106">
       <c r="C106" s="130" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="D106" s="119">
         <f t="shared" si="17"/>
-        <v>6.97</v>
+        <v>10.81</v>
       </c>
       <c r="N106" s="21"/>
       <c r="P106" s="116">
@@ -16148,12 +16098,10 @@
       </c>
     </row>
     <row r="107">
-      <c r="C107" s="130" t="s">
-        <v>240</v>
-      </c>
-      <c r="D107" s="119">
+      <c r="C107" s="130"/>
+      <c r="D107" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>6.35</v>
+        <v/>
       </c>
       <c r="N107" s="21"/>
       <c r="P107" s="116">
@@ -16167,12 +16115,10 @@
       </c>
     </row>
     <row r="108">
-      <c r="C108" s="130" t="s">
-        <v>245</v>
-      </c>
-      <c r="D108" s="119">
+      <c r="C108" s="130"/>
+      <c r="D108" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>6.55</v>
+        <v/>
       </c>
       <c r="N108" s="21"/>
       <c r="P108" s="116">
@@ -16186,12 +16132,10 @@
       </c>
     </row>
     <row r="109">
-      <c r="C109" s="130" t="s">
-        <v>246</v>
-      </c>
-      <c r="D109" s="119">
+      <c r="C109" s="130"/>
+      <c r="D109" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>6.13</v>
+        <v/>
       </c>
       <c r="N109" s="21"/>
       <c r="P109" s="116">
@@ -16205,12 +16149,10 @@
       </c>
     </row>
     <row r="110">
-      <c r="C110" s="130" t="s">
-        <v>247</v>
-      </c>
-      <c r="D110" s="119">
+      <c r="C110" s="130"/>
+      <c r="D110" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>3.44</v>
+        <v/>
       </c>
       <c r="N110" s="21"/>
       <c r="P110" s="116">
@@ -16224,12 +16166,10 @@
       </c>
     </row>
     <row r="111">
-      <c r="C111" s="130" t="s">
-        <v>248</v>
-      </c>
-      <c r="D111" s="119">
+      <c r="C111" s="130"/>
+      <c r="D111" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>7.03</v>
+        <v/>
       </c>
       <c r="N111" s="21"/>
       <c r="P111" s="116">
@@ -16243,12 +16183,10 @@
       </c>
     </row>
     <row r="112">
-      <c r="C112" s="130" t="s">
-        <v>249</v>
-      </c>
-      <c r="D112" s="119">
+      <c r="C112" s="130"/>
+      <c r="D112" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.22</v>
+        <v/>
       </c>
       <c r="P112" s="116">
         <v>1.0</v>
@@ -16261,12 +16199,10 @@
       </c>
     </row>
     <row r="113">
-      <c r="C113" s="130" t="s">
-        <v>250</v>
-      </c>
-      <c r="D113" s="119">
+      <c r="C113" s="130"/>
+      <c r="D113" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.49</v>
+        <v/>
       </c>
       <c r="P113" s="116">
         <v>0.0</v>
@@ -16279,12 +16215,10 @@
       </c>
     </row>
     <row r="114">
-      <c r="C114" s="130" t="s">
-        <v>251</v>
-      </c>
-      <c r="D114" s="119">
+      <c r="C114" s="130"/>
+      <c r="D114" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>5.89</v>
+        <v/>
       </c>
       <c r="P114" s="116">
         <v>1.0</v>
@@ -16297,12 +16231,10 @@
       </c>
     </row>
     <row r="115">
-      <c r="C115" s="130" t="s">
-        <v>252</v>
-      </c>
-      <c r="D115" s="119">
+      <c r="C115" s="130"/>
+      <c r="D115" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>4.85</v>
+        <v/>
       </c>
       <c r="P115" s="116">
         <v>1.0</v>
@@ -16315,12 +16247,10 @@
       </c>
     </row>
     <row r="116">
-      <c r="C116" s="130" t="s">
-        <v>253</v>
-      </c>
-      <c r="D116" s="119">
+      <c r="C116" s="130"/>
+      <c r="D116" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.86</v>
+        <v/>
       </c>
       <c r="P116" s="116">
         <v>1.0</v>
@@ -16333,12 +16263,10 @@
       </c>
     </row>
     <row r="117">
-      <c r="C117" s="130" t="s">
-        <v>254</v>
-      </c>
-      <c r="D117" s="119">
+      <c r="C117" s="130"/>
+      <c r="D117" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.62</v>
+        <v/>
       </c>
       <c r="P117" s="137"/>
       <c r="AE117" s="42">
@@ -16349,12 +16277,10 @@
       </c>
     </row>
     <row r="118">
-      <c r="C118" s="130" t="s">
-        <v>255</v>
-      </c>
-      <c r="D118" s="119">
+      <c r="C118" s="130"/>
+      <c r="D118" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.98</v>
+        <v/>
       </c>
       <c r="P118" s="137"/>
       <c r="AE118" s="42">
@@ -16365,12 +16291,10 @@
       </c>
     </row>
     <row r="119">
-      <c r="C119" s="130" t="s">
-        <v>256</v>
-      </c>
-      <c r="D119" s="119">
+      <c r="C119" s="130"/>
+      <c r="D119" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="P119" s="137"/>
       <c r="AE119" s="42">
@@ -16381,12 +16305,10 @@
       </c>
     </row>
     <row r="120">
-      <c r="C120" s="130" t="s">
-        <v>257</v>
-      </c>
-      <c r="D120" s="119">
+      <c r="C120" s="130"/>
+      <c r="D120" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.85</v>
+        <v/>
       </c>
       <c r="P120" s="137"/>
       <c r="AE120" s="42">
@@ -16397,12 +16319,10 @@
       </c>
     </row>
     <row r="121">
-      <c r="C121" s="130" t="s">
-        <v>256</v>
-      </c>
-      <c r="D121" s="119">
+      <c r="C121" s="130"/>
+      <c r="D121" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="P121" s="137"/>
       <c r="AE121" s="42">
@@ -16413,12 +16333,10 @@
       </c>
     </row>
     <row r="122">
-      <c r="C122" s="130" t="s">
-        <v>258</v>
-      </c>
-      <c r="D122" s="119">
+      <c r="C122" s="130"/>
+      <c r="D122" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.93</v>
+        <v/>
       </c>
       <c r="P122" s="137"/>
       <c r="AE122" s="42">
@@ -16429,12 +16347,10 @@
       </c>
     </row>
     <row r="123">
-      <c r="C123" s="130" t="s">
-        <v>256</v>
-      </c>
-      <c r="D123" s="119">
+      <c r="C123" s="130"/>
+      <c r="D123" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>3</v>
+        <v/>
       </c>
       <c r="P123" s="137"/>
       <c r="AE123" s="42">
@@ -16445,12 +16361,10 @@
       </c>
     </row>
     <row r="124">
-      <c r="C124" s="130" t="s">
-        <v>259</v>
-      </c>
-      <c r="D124" s="119">
+      <c r="C124" s="130"/>
+      <c r="D124" s="119" t="str">
         <f t="shared" si="17"/>
-        <v>2.99</v>
+        <v/>
       </c>
       <c r="P124" s="137"/>
       <c r="AE124" s="42">
@@ -38898,14 +38812,14 @@
     <row r="1">
       <c r="A1" s="99"/>
       <c r="B1" s="140" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="C1" s="141"/>
       <c r="D1" s="141"/>
       <c r="E1" s="141"/>
       <c r="F1" s="141"/>
       <c r="G1" s="142" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="H1" s="141"/>
       <c r="I1" s="141"/>
@@ -38933,19 +38847,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="144" t="s">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="C2" s="145" t="s">
-        <v>263</v>
+        <v>246</v>
       </c>
       <c r="D2" s="145" t="s">
         <v>165</v>
       </c>
       <c r="E2" s="145" t="s">
-        <v>264</v>
+        <v>247</v>
       </c>
       <c r="F2" s="146" t="s">
-        <v>265</v>
+        <v>248</v>
       </c>
       <c r="G2" s="144">
         <v>1.0</v>
@@ -38957,25 +38871,25 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="145" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="K2" s="147" t="s">
-        <v>267</v>
+        <v>250</v>
       </c>
       <c r="L2" s="145" t="s">
-        <v>268</v>
+        <v>251</v>
       </c>
       <c r="M2" s="148" t="s">
-        <v>269</v>
+        <v>252</v>
       </c>
       <c r="N2" s="95" t="s">
-        <v>270</v>
+        <v>253</v>
       </c>
       <c r="O2" s="95" t="s">
-        <v>271</v>
+        <v>254</v>
       </c>
       <c r="P2" s="95" t="s">
-        <v>272</v>
+        <v>255</v>
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
@@ -39758,7 +39672,7 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="161" t="s">
-        <v>273</v>
+        <v>256</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -39819,7 +39733,7 @@
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="5" t="s">
-        <v>274</v>
+        <v>257</v>
       </c>
       <c r="E29" s="5">
         <f>J29</f>
@@ -39841,10 +39755,10 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="89" t="s">
-        <v>275</v>
+        <v>258</v>
       </c>
       <c r="M29" s="89" t="s">
-        <v>276</v>
+        <v>259</v>
       </c>
       <c r="O29" s="5">
         <v>1.0</v>
@@ -39980,7 +39894,7 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="114" t="s">
-        <v>277</v>
+        <v>260</v>
       </c>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
@@ -40157,7 +40071,7 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="5" t="s">
-        <v>278</v>
+        <v>261</v>
       </c>
       <c r="G38" s="164">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones x missing, cuotas y cambio de modelo en ENG y SPA.
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -260,7 +260,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="309">
   <si>
     <t>id_country</t>
   </si>
@@ -329,9 +329,6 @@
   </si>
   <si>
     <t>france</t>
-  </si>
-  <si>
-    <t>L</t>
   </si>
   <si>
     <t>germany</t>
@@ -2437,26 +2434,26 @@
         <v>45693.0</v>
       </c>
       <c r="D4" s="15">
-        <v>344.0</v>
+        <v>332.0</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>18</v>
       </c>
       <c r="F4" s="16">
-        <v>55.1767676767676</v>
+        <v>54.7438672438672</v>
       </c>
       <c r="G4" s="17">
-        <f>2.56753805471583*100</f>
-        <v>256.7538055</v>
+        <f>3.46734255670938*100</f>
+        <v>346.7342557</v>
       </c>
       <c r="H4" s="18">
         <v>10.0</v>
       </c>
       <c r="I4" s="18">
-        <v>45.0</v>
+        <v>25.0</v>
       </c>
       <c r="J4" s="18">
-        <v>25.0</v>
+        <v>10.0</v>
       </c>
       <c r="K4" s="18" t="s">
         <v>21</v>
@@ -2469,18 +2466,18 @@
       </c>
       <c r="N4" s="20">
         <f t="shared" ref="N4:N8" si="1">AVERAGE(H4:J4)</f>
-        <v>26.66666667</v>
+        <v>15</v>
       </c>
       <c r="O4" s="27">
         <f>N4*'Data preparation'!$C$2</f>
-        <v>6.666666667</v>
+        <v>3.75</v>
       </c>
       <c r="P4" s="16">
-        <v>5526.8335588928</v>
+        <v>2219.11264327355</v>
       </c>
       <c r="Q4" s="20">
         <f t="shared" ref="Q4:Q8" si="2">P4/G4</f>
-        <v>21.52580971</v>
+        <v>6.400038666</v>
       </c>
     </row>
     <row r="5">
@@ -2507,7 +2504,7 @@
         <v>139.3784085</v>
       </c>
       <c r="H5" s="16">
-        <v>70.0</v>
+        <v>45.0</v>
       </c>
       <c r="I5" s="16">
         <v>45.0</v>
@@ -2522,22 +2519,22 @@
         <v>21</v>
       </c>
       <c r="M5" s="16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="N5" s="20">
         <f t="shared" si="1"/>
-        <v>41.66666667</v>
+        <v>33.33333333</v>
       </c>
       <c r="O5" s="27">
         <f>N5*'Data preparation'!$C$2</f>
-        <v>10.41666667</v>
+        <v>8.333333333</v>
       </c>
       <c r="P5" s="16">
-        <v>4868.12878004277</v>
+        <v>2572.90077073494</v>
       </c>
       <c r="Q5" s="20">
         <f t="shared" si="2"/>
-        <v>34.92742407</v>
+        <v>18.45982314</v>
       </c>
       <c r="S5" s="31"/>
     </row>
@@ -2546,7 +2543,7 @@
         <v>59.0</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" s="13">
         <v>45693.0</v>
@@ -2565,37 +2562,37 @@
         <v>601.6323262</v>
       </c>
       <c r="H6" s="16">
-        <v>70.0</v>
+        <v>45.0</v>
       </c>
       <c r="I6" s="16">
-        <v>45.0</v>
+        <v>25.0</v>
       </c>
       <c r="J6" s="16">
         <v>10.0</v>
       </c>
       <c r="K6" s="16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L6" s="16" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="M6" s="16" t="s">
         <v>21</v>
       </c>
       <c r="N6" s="20">
         <f t="shared" si="1"/>
-        <v>41.66666667</v>
+        <v>26.66666667</v>
       </c>
       <c r="O6" s="27">
         <f>N6*'Data preparation'!$C$2</f>
-        <v>10.41666667</v>
+        <v>6.666666667</v>
       </c>
       <c r="P6" s="32">
-        <v>38220.1573794083</v>
+        <v>13978.9606210805</v>
       </c>
       <c r="Q6" s="20">
         <f t="shared" si="2"/>
-        <v>63.52743314</v>
+        <v>23.23505572</v>
       </c>
     </row>
     <row r="7">
@@ -2603,7 +2600,7 @@
         <v>77.0</v>
       </c>
       <c r="B7" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C7" s="13">
         <v>45693.0</v>
@@ -2631,7 +2628,7 @@
         <v>45.0</v>
       </c>
       <c r="K7" s="18" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L7" s="18" t="s">
         <v>21</v>
@@ -2639,7 +2636,7 @@
       <c r="M7" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="N7" s="25">
+      <c r="N7" s="20">
         <f t="shared" si="1"/>
         <v>31.66666667</v>
       </c>
@@ -2648,11 +2645,11 @@
         <v>7.916666667</v>
       </c>
       <c r="P7" s="16">
-        <v>2633.48953477897</v>
+        <v>2440.21825177097</v>
       </c>
       <c r="Q7" s="20">
         <f t="shared" si="2"/>
-        <v>11.35536811</v>
+        <v>10.52199986</v>
       </c>
     </row>
     <row r="8">
@@ -2660,13 +2657,13 @@
         <v>148.0</v>
       </c>
       <c r="B8" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C8" s="13">
         <v>45693.0</v>
       </c>
       <c r="D8" s="15">
-        <v>508.0</v>
+        <v>530.0</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>18</v>
@@ -2741,9 +2738,6 @@
     <row r="12" ht="20.25" customHeight="1"/>
     <row r="13">
       <c r="A13" s="37"/>
-    </row>
-    <row r="19">
-      <c r="C19" s="38"/>
     </row>
     <row r="27">
       <c r="A27" s="37"/>
@@ -8978,6 +8972,16 @@
       <formula>"K"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="N4:N8">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF57BB8A"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
@@ -9095,7 +9099,7 @@
         <v>59.0</v>
       </c>
       <c r="B4" s="42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" s="38">
         <v>45680.0</v>
@@ -9138,7 +9142,7 @@
         <v>77.0</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5" s="13">
         <v>45677.0</v>
@@ -9183,7 +9187,7 @@
         <v>148.0</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6" s="13">
         <v>45677.0</v>
@@ -9259,32 +9263,32 @@
     </row>
     <row r="11">
       <c r="E11" s="50" t="s">
+        <v>26</v>
+      </c>
+      <c r="L11" s="42" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="42" t="s">
+      <c r="M11" s="44" t="s">
         <v>28</v>
       </c>
-      <c r="M11" s="44" t="s">
+      <c r="N11" s="51" t="s">
         <v>29</v>
-      </c>
-      <c r="N11" s="51" t="s">
-        <v>30</v>
       </c>
       <c r="O11" s="34"/>
       <c r="P11" s="34"/>
     </row>
     <row r="12">
       <c r="E12" s="50" t="s">
+        <v>30</v>
+      </c>
+      <c r="L12" s="42" t="s">
         <v>31</v>
       </c>
-      <c r="L12" s="42" t="s">
+      <c r="M12" s="44" t="s">
         <v>32</v>
       </c>
-      <c r="M12" s="44" t="s">
+      <c r="N12" s="51" t="s">
         <v>33</v>
-      </c>
-      <c r="N12" s="51" t="s">
-        <v>34</v>
       </c>
       <c r="O12" s="34"/>
       <c r="P12" s="34"/>
@@ -9411,7 +9415,7 @@
         <v>59.0</v>
       </c>
       <c r="B18" s="42" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" s="38">
         <v>45680.0</v>
@@ -9452,7 +9456,7 @@
         <v>77.0</v>
       </c>
       <c r="B19" s="54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" s="38">
         <v>45677.0</v>
@@ -9495,7 +9499,7 @@
         <v>148.0</v>
       </c>
       <c r="B20" s="42" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" s="38">
         <v>45677.0</v>
@@ -9540,49 +9544,49 @@
     </row>
     <row r="24">
       <c r="C24" s="35" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="25">
       <c r="C25" s="47" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="26">
       <c r="C26" s="55" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="27">
       <c r="C27" s="56" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="28">
       <c r="C28" s="54" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="57" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="35" t="s">
+        <v>40</v>
+      </c>
+      <c r="L31" s="35" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q31" s="35" t="s">
         <v>41</v>
       </c>
-      <c r="L31" s="35" t="s">
-        <v>34</v>
-      </c>
-      <c r="Q31" s="35" t="s">
+      <c r="Z31" s="35" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH31" s="35" t="s">
         <v>42</v>
-      </c>
-      <c r="Z31" s="35" t="s">
-        <v>33</v>
-      </c>
-      <c r="AH31" s="35" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="32">
@@ -11562,7 +11566,7 @@
     </row>
     <row r="63">
       <c r="C63" s="35" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="65">
@@ -11582,19 +11586,19 @@
         <v>4</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I65" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J65" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J65" s="4" t="s">
+      <c r="K65" s="7" t="s">
         <v>46</v>
       </c>
-      <c r="K65" s="7" t="s">
+      <c r="L65" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="L65" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="M65" s="67" t="s">
         <v>16</v>
@@ -11735,7 +11739,7 @@
         <v>59.0</v>
       </c>
       <c r="D70" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E70" s="13">
         <v>45680.0</v>
@@ -11780,7 +11784,7 @@
         <v>77.0</v>
       </c>
       <c r="D71" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E71" s="13">
         <v>45677.0</v>
@@ -11824,7 +11828,7 @@
         <v>148.0</v>
       </c>
       <c r="D72" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E72" s="13">
         <v>45677.0</v>
@@ -11865,7 +11869,7 @@
     </row>
     <row r="76">
       <c r="C76" s="35" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="77">
@@ -11885,16 +11889,16 @@
         <v>4</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="I77" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="J77" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="J77" s="4" t="s">
+      <c r="K77" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="K77" s="7" t="s">
-        <v>47</v>
       </c>
       <c r="L77" s="4" t="s">
         <v>7</v>
@@ -12077,7 +12081,7 @@
         <v>59.0</v>
       </c>
       <c r="D82" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E82" s="13">
         <v>45680.0</v>
@@ -12132,7 +12136,7 @@
         <v>77.0</v>
       </c>
       <c r="D83" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E83" s="13">
         <v>45677.0</v>
@@ -12187,7 +12191,7 @@
         <v>148.0</v>
       </c>
       <c r="D84" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E84" s="13">
         <v>45677.0</v>
@@ -12239,7 +12243,7 @@
     </row>
     <row r="94">
       <c r="C94" s="42" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="96">
@@ -12259,28 +12263,28 @@
         <v>4</v>
       </c>
       <c r="H96" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I96" s="4" t="s">
         <v>5</v>
       </c>
       <c r="J96" s="4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="K96" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="L96" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="L96" s="7" t="s">
+      <c r="M96" s="7" t="s">
         <v>52</v>
       </c>
-      <c r="M96" s="7" t="s">
-        <v>53</v>
-      </c>
       <c r="N96" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="O96" s="7" t="s">
         <v>46</v>
-      </c>
-      <c r="O96" s="7" t="s">
-        <v>47</v>
       </c>
       <c r="P96" s="67" t="s">
         <v>16</v>
@@ -12480,7 +12484,7 @@
         <v>59.0</v>
       </c>
       <c r="D101" s="72" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E101" s="13">
         <v>45680.0</v>
@@ -12541,7 +12545,7 @@
         <v>77.0</v>
       </c>
       <c r="D102" s="72" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E102" s="13">
         <v>45677.0</v>
@@ -12602,7 +12606,7 @@
         <v>148.0</v>
       </c>
       <c r="D103" s="72" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E103" s="13">
         <v>45677.0</v>
@@ -12713,7 +12717,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="74" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B1" s="75"/>
       <c r="C1" s="75"/>
@@ -12736,54 +12740,54 @@
     <row r="2">
       <c r="A2" s="79"/>
       <c r="B2" s="80" t="s">
+        <v>54</v>
+      </c>
+      <c r="C2" s="80" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="80" t="s">
+      <c r="D2" s="81" t="s">
         <v>56</v>
       </c>
-      <c r="D2" s="81" t="s">
+      <c r="E2" s="81" t="s">
         <v>57</v>
       </c>
-      <c r="E2" s="81" t="s">
+      <c r="F2" s="80" t="s">
         <v>58</v>
-      </c>
-      <c r="F2" s="80" t="s">
-        <v>59</v>
       </c>
       <c r="G2" s="82" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="82" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="I2" s="82" t="s">
         <v>15</v>
       </c>
       <c r="J2" s="80"/>
       <c r="K2" s="80" t="s">
+        <v>60</v>
+      </c>
+      <c r="L2" s="80" t="s">
         <v>61</v>
       </c>
-      <c r="L2" s="80" t="s">
+      <c r="M2" s="83" t="s">
         <v>62</v>
       </c>
-      <c r="M2" s="83" t="s">
+      <c r="N2" s="82" t="s">
         <v>63</v>
       </c>
-      <c r="N2" s="82" t="s">
+      <c r="O2" s="82" t="s">
         <v>64</v>
       </c>
-      <c r="O2" s="82" t="s">
+      <c r="P2" s="82" t="s">
         <v>65</v>
-      </c>
-      <c r="P2" s="82" t="s">
-        <v>66</v>
       </c>
       <c r="U2" s="40"/>
       <c r="V2" s="35"/>
     </row>
     <row r="3">
       <c r="A3" s="84" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="23">
         <v>343.0</v>
@@ -12831,7 +12835,7 @@
     </row>
     <row r="4">
       <c r="A4" s="84" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B4" s="23">
         <v>1127.0</v>
@@ -12882,7 +12886,7 @@
     </row>
     <row r="5">
       <c r="A5" s="84" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B5" s="85">
         <v>1051.0</v>
@@ -12933,7 +12937,7 @@
     </row>
     <row r="6">
       <c r="A6" s="84" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="23">
         <v>622.0</v>
@@ -12981,7 +12985,7 @@
     </row>
     <row r="7">
       <c r="A7" s="84" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B7" s="23">
         <v>1447.0</v>
@@ -13041,7 +13045,7 @@
     <row r="10">
       <c r="A10" s="49"/>
       <c r="E10" s="42" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="O10" s="43"/>
       <c r="P10" s="49"/>
@@ -13086,7 +13090,7 @@
     <row r="13">
       <c r="A13" s="31"/>
       <c r="E13" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F13" s="15">
         <v>1051.0</v>
@@ -13102,7 +13106,7 @@
     <row r="14">
       <c r="A14" s="31"/>
       <c r="E14" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F14" s="15">
         <v>47.0</v>
@@ -13122,7 +13126,7 @@
       <c r="C15" s="31"/>
       <c r="D15" s="31"/>
       <c r="E15" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F15" s="15">
         <v>1447.0</v>
@@ -13172,7 +13176,7 @@
     <row r="18">
       <c r="A18" s="43"/>
       <c r="E18" s="42" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="O18" s="43"/>
       <c r="P18" s="43"/>
@@ -13211,7 +13215,7 @@
     </row>
     <row r="21">
       <c r="E21" s="23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F21" s="15">
         <v>1051.0</v>
@@ -13222,7 +13226,7 @@
     </row>
     <row r="22">
       <c r="E22" s="23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F22" s="15">
         <v>622.0</v>
@@ -13234,7 +13238,7 @@
     </row>
     <row r="23">
       <c r="E23" s="23" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F23" s="15">
         <v>1545.0</v>
@@ -13454,7 +13458,7 @@
         <v>59.0</v>
       </c>
       <c r="D37" s="72" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E37" s="13">
         <v>45680.0</v>
@@ -13499,7 +13503,7 @@
         <v>77.0</v>
       </c>
       <c r="D38" s="72" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38" s="13">
         <v>45677.0</v>
@@ -13544,7 +13548,7 @@
         <v>148.0</v>
       </c>
       <c r="D39" s="72" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E39" s="13">
         <v>45677.0</v>
@@ -13752,13 +13756,13 @@
     </row>
     <row r="9">
       <c r="B9" s="42" t="s">
+        <v>68</v>
+      </c>
+      <c r="C9" s="42" t="s">
         <v>69</v>
       </c>
-      <c r="C9" s="42" t="s">
+      <c r="D9" s="42" t="s">
         <v>70</v>
-      </c>
-      <c r="D9" s="42" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -13776,7 +13780,7 @@
         <v>-0.1658536585</v>
       </c>
       <c r="F10" s="42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11">
@@ -13794,7 +13798,7 @@
         <v>-0.15</v>
       </c>
       <c r="F11" s="42" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12">
@@ -13832,16 +13836,16 @@
     </row>
     <row r="16">
       <c r="H16" s="42" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17">
       <c r="G17" s="89"/>
       <c r="H17" s="35" t="s">
+        <v>74</v>
+      </c>
+      <c r="I17" s="35" t="s">
         <v>75</v>
-      </c>
-      <c r="I17" s="35" t="s">
-        <v>76</v>
       </c>
     </row>
     <row r="18">
@@ -13855,13 +13859,13 @@
         <v>0.85</v>
       </c>
       <c r="G18" s="90" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H18" s="42">
         <v>332.0</v>
       </c>
       <c r="I18" s="91" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="19">
@@ -13875,13 +13879,13 @@
         <v>0.81</v>
       </c>
       <c r="G19" s="90" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H19" s="42" t="s">
+        <v>77</v>
+      </c>
+      <c r="I19" s="42" t="s">
         <v>78</v>
-      </c>
-      <c r="I19" s="42" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="20">
@@ -13895,45 +13899,45 @@
         <v>0.89</v>
       </c>
       <c r="G20" s="90" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H20" s="42">
         <v>411.0</v>
       </c>
       <c r="I20" s="42" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="21">
       <c r="G21" s="90" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H21" s="42" t="s">
+        <v>80</v>
+      </c>
+      <c r="I21" s="42" t="s">
         <v>81</v>
-      </c>
-      <c r="I21" s="42" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="22">
       <c r="G22" s="90" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H22" s="42" t="s">
+        <v>82</v>
+      </c>
+      <c r="I22" s="42" t="s">
         <v>83</v>
-      </c>
-      <c r="I22" s="42" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="24">
       <c r="I24" s="42" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25">
       <c r="I25" s="42" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="26">
@@ -13954,28 +13958,28 @@
     </row>
     <row r="30">
       <c r="I30" s="35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="M30" s="34"/>
       <c r="N30" s="34"/>
     </row>
     <row r="31">
       <c r="I31" s="35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="M31" s="34"/>
       <c r="N31" s="34"/>
     </row>
     <row r="32">
       <c r="I32" s="42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M32" s="34"/>
       <c r="N32" s="34"/>
     </row>
     <row r="33">
       <c r="I33" s="42" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="M33" s="34"/>
       <c r="N33" s="34"/>
@@ -13986,7 +13990,7 @@
     </row>
     <row r="35">
       <c r="I35" s="42" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M35" s="34"/>
       <c r="N35" s="34"/>
@@ -14005,28 +14009,28 @@
     </row>
     <row r="39">
       <c r="I39" s="35" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="M39" s="34"/>
       <c r="N39" s="34"/>
     </row>
     <row r="40">
       <c r="I40" s="42" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="M40" s="34"/>
       <c r="N40" s="34"/>
     </row>
     <row r="41">
       <c r="I41" s="42" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="M41" s="34"/>
       <c r="N41" s="34"/>
     </row>
     <row r="42">
       <c r="I42" s="57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="M42" s="34"/>
       <c r="N42" s="34"/>
@@ -14037,7 +14041,7 @@
     </row>
     <row r="44">
       <c r="I44" s="35" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -14064,146 +14068,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="42" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="9"/>
       <c r="C2" s="92" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E2" s="93"/>
       <c r="F2" s="94" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="H2" s="93"/>
     </row>
     <row r="3">
       <c r="B3" s="95" t="s">
+        <v>99</v>
+      </c>
+      <c r="C3" s="96" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="96" t="s">
+      <c r="D3" s="95" t="s">
         <v>101</v>
       </c>
-      <c r="D3" s="95" t="s">
+      <c r="E3" s="97" t="s">
         <v>102</v>
       </c>
-      <c r="E3" s="97" t="s">
+      <c r="F3" s="95" t="s">
         <v>103</v>
       </c>
-      <c r="F3" s="95" t="s">
+      <c r="G3" s="95" t="s">
         <v>104</v>
       </c>
-      <c r="G3" s="95" t="s">
+      <c r="H3" s="95" t="s">
         <v>105</v>
-      </c>
-      <c r="H3" s="95" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="98" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="99" t="s">
         <v>107</v>
       </c>
-      <c r="C4" s="99" t="s">
+      <c r="D4" s="100" t="s">
         <v>108</v>
       </c>
-      <c r="D4" s="100" t="s">
+      <c r="E4" s="101" t="s">
         <v>109</v>
       </c>
-      <c r="E4" s="101" t="s">
+      <c r="F4" s="102" t="s">
         <v>110</v>
       </c>
-      <c r="F4" s="102" t="s">
+      <c r="G4" s="102" t="s">
         <v>111</v>
-      </c>
-      <c r="G4" s="102" t="s">
-        <v>112</v>
       </c>
       <c r="H4" s="100"/>
     </row>
     <row r="5">
       <c r="B5" s="98" t="s">
+        <v>112</v>
+      </c>
+      <c r="C5" s="103" t="s">
         <v>113</v>
-      </c>
-      <c r="C5" s="103" t="s">
-        <v>114</v>
       </c>
       <c r="D5" s="104"/>
       <c r="E5" s="101" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F5" s="105" t="s">
+        <v>114</v>
+      </c>
+      <c r="G5" s="106" t="s">
         <v>115</v>
-      </c>
-      <c r="G5" s="106" t="s">
-        <v>116</v>
       </c>
       <c r="H5" s="100"/>
     </row>
     <row r="6">
       <c r="B6" s="98" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="99" t="s">
+        <v>107</v>
+      </c>
+      <c r="D6" s="100" t="s">
         <v>117</v>
       </c>
-      <c r="C6" s="99" t="s">
-        <v>108</v>
-      </c>
-      <c r="D6" s="100" t="s">
+      <c r="E6" s="101" t="s">
+        <v>109</v>
+      </c>
+      <c r="F6" s="100" t="s">
         <v>118</v>
-      </c>
-      <c r="E6" s="101" t="s">
-        <v>110</v>
-      </c>
-      <c r="F6" s="100" t="s">
-        <v>119</v>
       </c>
       <c r="G6" s="100"/>
       <c r="H6" s="100"/>
     </row>
     <row r="7">
       <c r="B7" s="100" t="s">
+        <v>119</v>
+      </c>
+      <c r="C7" s="107" t="s">
         <v>120</v>
-      </c>
-      <c r="C7" s="107" t="s">
-        <v>121</v>
       </c>
       <c r="D7" s="100"/>
       <c r="E7" s="108" t="s">
+        <v>121</v>
+      </c>
+      <c r="F7" s="99" t="s">
         <v>122</v>
-      </c>
-      <c r="F7" s="99" t="s">
-        <v>123</v>
       </c>
       <c r="G7" s="100"/>
       <c r="H7" s="100" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="109" t="s">
+        <v>124</v>
+      </c>
+      <c r="C8" s="110" t="s">
         <v>125</v>
-      </c>
-      <c r="C8" s="110" t="s">
-        <v>126</v>
       </c>
       <c r="D8" s="111"/>
       <c r="E8" s="109" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" s="112" t="s">
         <v>127</v>
       </c>
-      <c r="F8" s="112" t="s">
+      <c r="G8" s="113" t="s">
         <v>128</v>
-      </c>
-      <c r="G8" s="113" t="s">
-        <v>129</v>
       </c>
       <c r="H8" s="111"/>
     </row>
     <row r="9">
       <c r="B9" s="23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C9" s="114" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D9" s="79"/>
       <c r="E9" s="79"/>
@@ -14213,27 +14217,27 @@
     </row>
     <row r="10">
       <c r="B10" s="23" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C10" s="115"/>
       <c r="D10" s="79"/>
       <c r="E10" s="79"/>
       <c r="F10" s="115"/>
       <c r="G10" s="102" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="H10" s="79"/>
     </row>
     <row r="11">
       <c r="B11" s="23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C11" s="115"/>
       <c r="D11" s="79"/>
       <c r="E11" s="79"/>
       <c r="F11" s="115"/>
       <c r="G11" s="116" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H11" s="23"/>
     </row>
@@ -14271,7 +14275,7 @@
     <row r="2">
       <c r="A2" s="18"/>
       <c r="B2" s="94" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C2" s="18">
         <v>0.25</v>
@@ -14281,11 +14285,11 @@
     <row r="3">
       <c r="A3" s="18"/>
       <c r="B3" s="94" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C3" s="26">
         <f>AVERAGE('Modelos actuales'!O4:O8)</f>
-        <v>8.666666667</v>
+        <v>6.916666667</v>
       </c>
       <c r="L3" s="117"/>
       <c r="P3" s="117"/>
@@ -14296,7 +14300,7 @@
       <c r="L4" s="117"/>
       <c r="P4" s="117"/>
       <c r="AE4" s="42" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="AF4" s="118">
         <f>CORREL(AE6:AE10000,AF6:AF10000)</f>
@@ -14306,50 +14310,50 @@
     <row r="5">
       <c r="A5" s="18"/>
       <c r="B5" s="117" t="s">
+        <v>136</v>
+      </c>
+      <c r="L5" s="117" t="s">
         <v>137</v>
       </c>
-      <c r="L5" s="117" t="s">
+      <c r="P5" s="117" t="s">
         <v>138</v>
       </c>
-      <c r="P5" s="117" t="s">
+      <c r="AE5" s="42" t="s">
         <v>139</v>
       </c>
-      <c r="AE5" s="42" t="s">
+      <c r="AF5" s="42" t="s">
         <v>140</v>
-      </c>
-      <c r="AF5" s="42" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="18"/>
       <c r="B6" s="42" t="s">
+        <v>141</v>
+      </c>
+      <c r="F6" s="42" t="s">
         <v>142</v>
-      </c>
-      <c r="F6" s="42" t="s">
-        <v>143</v>
       </c>
       <c r="K6" s="35"/>
       <c r="L6" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="N6" s="35" t="s">
         <v>144</v>
       </c>
-      <c r="N6" s="35" t="s">
+      <c r="P6" s="35" t="s">
         <v>145</v>
       </c>
-      <c r="P6" s="35" t="s">
+      <c r="R6" s="35" t="s">
         <v>146</v>
       </c>
-      <c r="R6" s="35" t="s">
+      <c r="V6" s="35" t="s">
         <v>147</v>
       </c>
-      <c r="V6" s="35" t="s">
+      <c r="AA6" s="42" t="s">
         <v>148</v>
       </c>
-      <c r="AA6" s="42" t="s">
+      <c r="AB6" s="42" t="s">
         <v>149</v>
-      </c>
-      <c r="AB6" s="42" t="s">
-        <v>150</v>
       </c>
       <c r="AE6" s="42">
         <v>519.2</v>
@@ -14391,7 +14395,7 @@
         <v>0.5454545455</v>
       </c>
       <c r="AA7" s="42" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="AB7" s="41">
         <f t="shared" ref="AB7:AB16" si="4">LEFT(REPLACE(AA7,1,1,""),FIND(",", AA7)-2)/1</f>
@@ -14407,14 +14411,14 @@
     <row r="8">
       <c r="A8" s="18"/>
       <c r="B8" s="122" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C8" s="123" t="str">
         <f t="shared" ref="C8:C17" si="5">REPLACE(B8,FIND(".",B8),1,",")*1</f>
         <v>#VALUE!</v>
       </c>
       <c r="F8" s="47" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G8" s="123" t="str">
         <f t="shared" ref="G8:G27" si="6">REPLACE(F8,FIND(".",F8),1,",")*1</f>
@@ -14449,7 +14453,7 @@
         <v>0.5263157895</v>
       </c>
       <c r="AA8" s="42" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="AB8" s="41">
         <f t="shared" si="4"/>
@@ -14465,14 +14469,14 @@
     <row r="9">
       <c r="A9" s="18"/>
       <c r="B9" s="122" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C9" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F9" s="47" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G9" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14486,13 +14490,13 @@
       </c>
       <c r="K9" s="18"/>
       <c r="L9" s="119" t="s">
+        <v>156</v>
+      </c>
+      <c r="M9" s="119" t="s">
         <v>157</v>
       </c>
-      <c r="M9" s="119" t="s">
+      <c r="N9" s="35" t="s">
         <v>158</v>
-      </c>
-      <c r="N9" s="35" t="s">
-        <v>159</v>
       </c>
       <c r="P9" s="121">
         <v>1.0</v>
@@ -14516,7 +14520,7 @@
         <v>0.25</v>
       </c>
       <c r="AA9" s="42" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="AB9" s="41">
         <f t="shared" si="4"/>
@@ -14532,14 +14536,14 @@
     <row r="10">
       <c r="A10" s="18"/>
       <c r="B10" s="124" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C10" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F10" s="47" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G10" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14576,7 +14580,7 @@
         <v>76</v>
       </c>
       <c r="AA10" s="42" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AB10" s="41">
         <f t="shared" si="4"/>
@@ -14591,14 +14595,14 @@
     </row>
     <row r="11">
       <c r="B11" s="122" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C11" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F11" s="47" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G11" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14627,7 +14631,7 @@
         <v>2.0</v>
       </c>
       <c r="AA11" s="42" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="AB11" s="41">
         <f t="shared" si="4"/>
@@ -14642,14 +14646,14 @@
     </row>
     <row r="12">
       <c r="B12" s="124" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C12" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F12" s="47" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G12" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14678,7 +14682,7 @@
         <v>1.0</v>
       </c>
       <c r="AA12" s="42" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="AB12" s="41">
         <f t="shared" si="4"/>
@@ -14693,14 +14697,14 @@
     </row>
     <row r="13">
       <c r="B13" s="122" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C13" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F13" s="47" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G13" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14730,16 +14734,16 @@
       <c r="Q13" s="40"/>
       <c r="R13" s="79"/>
       <c r="S13" s="84" t="s">
+        <v>170</v>
+      </c>
+      <c r="T13" s="84" t="s">
         <v>171</v>
       </c>
-      <c r="T13" s="84" t="s">
+      <c r="U13" s="84" t="s">
         <v>172</v>
       </c>
-      <c r="U13" s="84" t="s">
+      <c r="AA13" s="42" t="s">
         <v>173</v>
-      </c>
-      <c r="AA13" s="42" t="s">
-        <v>174</v>
       </c>
       <c r="AB13" s="41">
         <f t="shared" si="4"/>
@@ -14754,14 +14758,14 @@
     </row>
     <row r="14">
       <c r="B14" s="122" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C14" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F14" s="47" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G14" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14801,7 +14805,7 @@
         <v>11.0</v>
       </c>
       <c r="AA14" s="42" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="AB14" s="41">
         <f t="shared" si="4"/>
@@ -14816,14 +14820,14 @@
     </row>
     <row r="15">
       <c r="B15" s="122" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C15" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F15" s="47" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G15" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14863,7 +14867,7 @@
         <v>13.0</v>
       </c>
       <c r="AA15" s="42" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="AB15" s="41">
         <f t="shared" si="4"/>
@@ -14878,14 +14882,14 @@
     </row>
     <row r="16">
       <c r="B16" s="122" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C16" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F16" s="47" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="G16" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14925,7 +14929,7 @@
         <v>12.0</v>
       </c>
       <c r="AA16" s="42" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="AB16" s="41">
         <f t="shared" si="4"/>
@@ -14940,14 +14944,14 @@
     </row>
     <row r="17">
       <c r="B17" s="122" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="C17" s="123" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F17" s="47" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="G17" s="123" t="str">
         <f t="shared" si="6"/>
@@ -14975,7 +14979,7 @@
         <v>1.0</v>
       </c>
       <c r="R17" s="84" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="S17" s="125">
         <f t="shared" ref="S17:U17" si="10">SUM(S14:S16)</f>
@@ -14998,7 +15002,7 @@
     </row>
     <row r="18">
       <c r="F18" s="47" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="G18" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15035,14 +15039,14 @@
     </row>
     <row r="19">
       <c r="B19" s="35" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C19" s="41" t="str">
         <f>AVERAGE(C8:C17)</f>
         <v>#VALUE!</v>
       </c>
       <c r="F19" s="47" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="G19" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15070,7 +15074,7 @@
       <c r="T19" s="21"/>
       <c r="U19" s="21"/>
       <c r="AA19" s="42" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="AB19" s="41">
         <f>AVERAGE(AB7:AB16)</f>
@@ -15085,7 +15089,7 @@
     </row>
     <row r="20">
       <c r="F20" s="47" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G20" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15110,7 +15114,7 @@
     </row>
     <row r="21">
       <c r="F21" s="47" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G21" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15124,13 +15128,13 @@
       </c>
       <c r="R21" s="79"/>
       <c r="S21" s="84" t="s">
+        <v>170</v>
+      </c>
+      <c r="T21" s="84" t="s">
         <v>171</v>
       </c>
-      <c r="T21" s="84" t="s">
+      <c r="U21" s="84" t="s">
         <v>172</v>
-      </c>
-      <c r="U21" s="84" t="s">
-        <v>173</v>
       </c>
       <c r="AE21" s="42">
         <v>146.62</v>
@@ -15142,7 +15146,7 @@
     <row r="22">
       <c r="C22" s="123"/>
       <c r="F22" s="47" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="G22" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15215,7 +15219,7 @@
     </row>
     <row r="24">
       <c r="F24" s="47" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G24" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15251,7 +15255,7 @@
     </row>
     <row r="25">
       <c r="F25" s="47" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G25" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15264,7 +15268,7 @@
         <v>1.0</v>
       </c>
       <c r="R25" s="84" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="S25" s="125">
         <f t="shared" ref="S25:U25" si="14">SUM(S22:S24)</f>
@@ -15287,7 +15291,7 @@
     </row>
     <row r="26">
       <c r="F26" s="47" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G26" s="123" t="str">
         <f t="shared" si="6"/>
@@ -15332,13 +15336,13 @@
         <v>1.0</v>
       </c>
       <c r="AA28" s="42" t="s">
+        <v>196</v>
+      </c>
+      <c r="AB28" s="42" t="s">
         <v>197</v>
       </c>
-      <c r="AB28" s="42" t="s">
-        <v>198</v>
-      </c>
       <c r="AC28" s="42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AE28" s="42">
         <v>106.73</v>
@@ -15349,7 +15353,7 @@
     </row>
     <row r="29">
       <c r="F29" s="35" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="G29" s="41" t="str">
         <f>AVERAGE(G8:G27)</f>
@@ -15440,7 +15444,7 @@
     </row>
     <row r="32">
       <c r="B32" s="54" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G32" s="123"/>
       <c r="P32" s="121">
@@ -15469,7 +15473,7 @@
     </row>
     <row r="33">
       <c r="B33" s="128" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G33" s="129"/>
       <c r="P33" s="121">
@@ -15523,7 +15527,7 @@
     </row>
     <row r="35">
       <c r="H35" s="35" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="P35" s="121">
         <v>1.0</v>
@@ -15551,7 +15555,7 @@
     </row>
     <row r="36">
       <c r="G36" s="35" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H36" s="130">
         <v>4.555000000000001</v>
@@ -15589,7 +15593,7 @@
         <v>4.136590909</v>
       </c>
       <c r="G37" s="35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H37" s="130">
         <v>7.555294117647058</v>
@@ -15620,7 +15624,7 @@
     </row>
     <row r="38">
       <c r="G38" s="35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H38" s="132">
         <v>2.21</v>
@@ -15651,14 +15655,14 @@
     </row>
     <row r="39">
       <c r="C39" s="133" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D39" s="123">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
         <v>0</v>
       </c>
       <c r="G39" s="35" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H39" s="130">
         <v>9.938235294117648</v>
@@ -15689,14 +15693,14 @@
     </row>
     <row r="40">
       <c r="C40" s="134" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D40" s="123">
         <f t="shared" si="17"/>
         <v>1.89</v>
       </c>
       <c r="G40" s="35" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H40" s="130">
         <v>3.3411111111111107</v>
@@ -15727,7 +15731,7 @@
     </row>
     <row r="41">
       <c r="C41" s="134" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D41" s="123">
         <f t="shared" si="17"/>
@@ -15759,7 +15763,7 @@
     </row>
     <row r="42">
       <c r="C42" s="134" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D42" s="123">
         <f t="shared" si="17"/>
@@ -15791,7 +15795,7 @@
     </row>
     <row r="43">
       <c r="C43" s="134" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D43" s="123">
         <f t="shared" si="17"/>
@@ -15823,7 +15827,7 @@
     </row>
     <row r="44">
       <c r="C44" s="134" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D44" s="123">
         <f t="shared" si="17"/>
@@ -15853,7 +15857,7 @@
     </row>
     <row r="45">
       <c r="C45" s="134" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D45" s="123">
         <f t="shared" si="17"/>
@@ -15871,17 +15875,17 @@
     </row>
     <row r="46">
       <c r="C46" s="134" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D46" s="123">
         <f t="shared" si="17"/>
         <v>3.67</v>
       </c>
       <c r="G46" s="95" t="s">
+        <v>207</v>
+      </c>
+      <c r="H46" s="95" t="s">
         <v>208</v>
-      </c>
-      <c r="H46" s="95" t="s">
-        <v>209</v>
       </c>
       <c r="P46" s="121">
         <v>0.0</v>
@@ -15895,14 +15899,14 @@
     </row>
     <row r="47">
       <c r="C47" s="134" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D47" s="123">
         <f t="shared" si="17"/>
         <v>4.71</v>
       </c>
       <c r="G47" s="100" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H47" s="135">
         <v>0.376453591155815</v>
@@ -15914,7 +15918,7 @@
         <v>3</v>
       </c>
       <c r="AB47" s="42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="AE47" s="42">
         <v>67.98</v>
@@ -15925,20 +15929,20 @@
     </row>
     <row r="48">
       <c r="C48" s="134" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="D48" s="123">
         <f t="shared" si="17"/>
         <v>3.08</v>
       </c>
       <c r="G48" s="100" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H48" s="135">
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="42" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K48" s="88">
         <f>AVERAGE(H47:H51)</f>
@@ -15962,20 +15966,20 @@
     </row>
     <row r="49">
       <c r="C49" s="134" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D49" s="123">
         <f t="shared" si="17"/>
         <v>4.19</v>
       </c>
       <c r="G49" s="100" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="H49" s="135">
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="42" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K49" s="88">
         <f>MEDIAN(H47:H51)</f>
@@ -15999,20 +16003,20 @@
     </row>
     <row r="50">
       <c r="C50" s="134" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D50" s="123">
         <f t="shared" si="17"/>
         <v>4.02</v>
       </c>
       <c r="G50" s="100" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="H50" s="135">
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="42" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K50" s="88">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -16036,20 +16040,20 @@
     </row>
     <row r="51">
       <c r="C51" s="134" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D51" s="123">
         <f t="shared" si="17"/>
         <v>4.31</v>
       </c>
       <c r="G51" s="100" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H51" s="135">
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="42" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K51" s="88">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -16073,7 +16077,7 @@
     </row>
     <row r="52">
       <c r="C52" s="134" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D52" s="123">
         <f t="shared" si="17"/>
@@ -16097,7 +16101,7 @@
     </row>
     <row r="53">
       <c r="C53" s="134" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D53" s="123">
         <f t="shared" si="17"/>
@@ -16121,7 +16125,7 @@
     </row>
     <row r="54">
       <c r="C54" s="134" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D54" s="123">
         <f t="shared" si="17"/>
@@ -16145,7 +16149,7 @@
     </row>
     <row r="55">
       <c r="C55" s="134" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="D55" s="123">
         <f t="shared" si="17"/>
@@ -16169,7 +16173,7 @@
     </row>
     <row r="56">
       <c r="C56" s="134" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D56" s="123">
         <f t="shared" si="17"/>
@@ -16193,7 +16197,7 @@
     </row>
     <row r="57">
       <c r="C57" s="134" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D57" s="123">
         <f t="shared" si="17"/>
@@ -16217,14 +16221,14 @@
     </row>
     <row r="58">
       <c r="C58" s="134" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D58" s="123">
         <f t="shared" si="17"/>
         <v>3.34</v>
       </c>
       <c r="G58" s="136" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="H58" s="137"/>
       <c r="P58" s="121">
@@ -16245,7 +16249,7 @@
     </row>
     <row r="59">
       <c r="C59" s="134" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D59" s="123">
         <f t="shared" si="17"/>
@@ -16253,7 +16257,7 @@
       </c>
       <c r="G59" s="137"/>
       <c r="H59" s="138" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="P59" s="121">
         <v>0.0</v>
@@ -16273,7 +16277,7 @@
     </row>
     <row r="60">
       <c r="C60" s="134" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D60" s="123">
         <f t="shared" si="17"/>
@@ -16281,7 +16285,7 @@
       </c>
       <c r="G60" s="137"/>
       <c r="H60" s="138" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="P60" s="121">
         <v>2.0</v>
@@ -16301,7 +16305,7 @@
     </row>
     <row r="61">
       <c r="C61" s="134" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D61" s="123">
         <f t="shared" si="17"/>
@@ -16309,7 +16313,7 @@
       </c>
       <c r="G61" s="137"/>
       <c r="H61" s="138" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="P61" s="121">
         <v>2.0</v>
@@ -16329,7 +16333,7 @@
     </row>
     <row r="62">
       <c r="C62" s="134" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D62" s="123">
         <f t="shared" si="17"/>
@@ -16337,7 +16341,7 @@
       </c>
       <c r="G62" s="137"/>
       <c r="H62" s="138" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="P62" s="121">
         <v>1.0</v>
@@ -16357,7 +16361,7 @@
     </row>
     <row r="63">
       <c r="C63" s="134" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D63" s="123">
         <f t="shared" si="17"/>
@@ -16365,7 +16369,7 @@
       </c>
       <c r="G63" s="137"/>
       <c r="H63" s="138" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="P63" s="121">
         <v>0.0</v>
@@ -16379,7 +16383,7 @@
     </row>
     <row r="64">
       <c r="C64" s="134" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D64" s="123">
         <f t="shared" si="17"/>
@@ -16397,7 +16401,7 @@
     </row>
     <row r="65">
       <c r="C65" s="134" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D65" s="123">
         <f t="shared" si="17"/>
@@ -16415,7 +16419,7 @@
     </row>
     <row r="66">
       <c r="C66" s="134" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D66" s="123">
         <f t="shared" si="17"/>
@@ -16433,7 +16437,7 @@
     </row>
     <row r="67">
       <c r="C67" s="134" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="D67" s="123">
         <f t="shared" si="17"/>
@@ -16451,7 +16455,7 @@
     </row>
     <row r="68">
       <c r="C68" s="134" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="D68" s="123">
         <f t="shared" si="17"/>
@@ -16469,7 +16473,7 @@
     </row>
     <row r="69">
       <c r="C69" s="134" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="D69" s="123">
         <f t="shared" si="17"/>
@@ -16487,7 +16491,7 @@
     </row>
     <row r="70">
       <c r="C70" s="134" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="D70" s="123">
         <f t="shared" si="17"/>
@@ -16505,7 +16509,7 @@
     </row>
     <row r="71">
       <c r="C71" s="134" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D71" s="123">
         <f t="shared" si="17"/>
@@ -16524,7 +16528,7 @@
     </row>
     <row r="72">
       <c r="C72" s="134" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="D72" s="123">
         <f t="shared" si="17"/>
@@ -16542,7 +16546,7 @@
     </row>
     <row r="73">
       <c r="C73" s="134" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="D73" s="123">
         <f t="shared" si="17"/>
@@ -16560,7 +16564,7 @@
     </row>
     <row r="74">
       <c r="C74" s="134" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="D74" s="123">
         <f t="shared" si="17"/>
@@ -16578,7 +16582,7 @@
     </row>
     <row r="75">
       <c r="C75" s="134" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="D75" s="123">
         <f t="shared" si="17"/>
@@ -16596,7 +16600,7 @@
     </row>
     <row r="76">
       <c r="C76" s="134" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="D76" s="123">
         <f t="shared" si="17"/>
@@ -16614,7 +16618,7 @@
     </row>
     <row r="77">
       <c r="C77" s="134" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="D77" s="123">
         <f t="shared" si="17"/>
@@ -16632,7 +16636,7 @@
     </row>
     <row r="78">
       <c r="C78" s="134" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="D78" s="123">
         <f t="shared" si="17"/>
@@ -16650,7 +16654,7 @@
     </row>
     <row r="79">
       <c r="C79" s="134" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="D79" s="123">
         <f t="shared" si="17"/>
@@ -16668,7 +16672,7 @@
     </row>
     <row r="80">
       <c r="C80" s="134" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="D80" s="123">
         <f t="shared" si="17"/>
@@ -16686,7 +16690,7 @@
     </row>
     <row r="81">
       <c r="C81" s="134" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D81" s="123">
         <f t="shared" si="17"/>
@@ -16704,7 +16708,7 @@
     </row>
     <row r="82">
       <c r="C82" s="134" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="D82" s="123">
         <f t="shared" si="17"/>
@@ -16722,7 +16726,7 @@
     </row>
     <row r="83">
       <c r="C83" s="134" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D83" s="123">
         <f t="shared" si="17"/>
@@ -16740,7 +16744,7 @@
     </row>
     <row r="84">
       <c r="C84" s="134" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D84" s="123">
         <f t="shared" si="17"/>
@@ -16758,7 +16762,7 @@
     </row>
     <row r="85">
       <c r="C85" s="134" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="D85" s="123">
         <f t="shared" si="17"/>
@@ -16776,7 +16780,7 @@
     </row>
     <row r="86">
       <c r="C86" s="134" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="D86" s="123">
         <f t="shared" si="17"/>
@@ -16794,7 +16798,7 @@
     </row>
     <row r="87">
       <c r="C87" s="134" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="D87" s="123">
         <f t="shared" si="17"/>
@@ -16812,7 +16816,7 @@
     </row>
     <row r="88">
       <c r="C88" s="134" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D88" s="123">
         <f t="shared" si="17"/>
@@ -16830,7 +16834,7 @@
     </row>
     <row r="89">
       <c r="C89" s="134" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="D89" s="123">
         <f t="shared" si="17"/>
@@ -16848,7 +16852,7 @@
     </row>
     <row r="90">
       <c r="C90" s="134" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D90" s="123">
         <f t="shared" si="17"/>
@@ -16866,7 +16870,7 @@
     </row>
     <row r="91">
       <c r="C91" s="134" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D91" s="123">
         <f t="shared" si="17"/>
@@ -16884,7 +16888,7 @@
     </row>
     <row r="92">
       <c r="C92" s="134" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="D92" s="123">
         <f t="shared" si="17"/>
@@ -16902,7 +16906,7 @@
     </row>
     <row r="93">
       <c r="C93" s="134" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D93" s="123">
         <f t="shared" si="17"/>
@@ -16920,7 +16924,7 @@
     </row>
     <row r="94">
       <c r="C94" s="134" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="D94" s="123">
         <f t="shared" si="17"/>
@@ -16938,7 +16942,7 @@
     </row>
     <row r="95">
       <c r="C95" s="134" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="D95" s="123">
         <f t="shared" si="17"/>
@@ -16956,7 +16960,7 @@
     </row>
     <row r="96">
       <c r="C96" s="134" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="D96" s="123">
         <f t="shared" si="17"/>
@@ -16974,7 +16978,7 @@
     </row>
     <row r="97">
       <c r="C97" s="134" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D97" s="123">
         <f t="shared" si="17"/>
@@ -16992,7 +16996,7 @@
     </row>
     <row r="98">
       <c r="C98" s="134" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D98" s="123">
         <f t="shared" si="17"/>
@@ -17010,7 +17014,7 @@
     </row>
     <row r="99">
       <c r="C99" s="134" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D99" s="123">
         <f t="shared" si="17"/>
@@ -17028,7 +17032,7 @@
     </row>
     <row r="100">
       <c r="C100" s="134" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D100" s="123">
         <f t="shared" si="17"/>
@@ -17046,7 +17050,7 @@
     </row>
     <row r="101">
       <c r="C101" s="134" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D101" s="123">
         <f t="shared" si="17"/>
@@ -17064,7 +17068,7 @@
     </row>
     <row r="102">
       <c r="C102" s="134" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D102" s="123">
         <f t="shared" si="17"/>
@@ -17082,7 +17086,7 @@
     </row>
     <row r="103">
       <c r="C103" s="134" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D103" s="123">
         <f t="shared" si="17"/>
@@ -17100,7 +17104,7 @@
     </row>
     <row r="104">
       <c r="C104" s="134" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D104" s="123">
         <f t="shared" si="17"/>
@@ -17119,7 +17123,7 @@
     </row>
     <row r="105">
       <c r="C105" s="134" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D105" s="123">
         <f t="shared" si="17"/>
@@ -17138,7 +17142,7 @@
     </row>
     <row r="106">
       <c r="C106" s="134" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D106" s="123">
         <f t="shared" si="17"/>
@@ -17157,7 +17161,7 @@
     </row>
     <row r="107">
       <c r="C107" s="134" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D107" s="123">
         <f t="shared" si="17"/>
@@ -17176,7 +17180,7 @@
     </row>
     <row r="108">
       <c r="C108" s="134" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D108" s="123">
         <f t="shared" si="17"/>
@@ -17195,7 +17199,7 @@
     </row>
     <row r="109">
       <c r="C109" s="134" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="D109" s="123">
         <f t="shared" si="17"/>
@@ -17214,7 +17218,7 @@
     </row>
     <row r="110">
       <c r="C110" s="134" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D110" s="123">
         <f t="shared" si="17"/>
@@ -17233,7 +17237,7 @@
     </row>
     <row r="111">
       <c r="C111" s="134" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D111" s="123">
         <f t="shared" si="17"/>
@@ -17252,7 +17256,7 @@
     </row>
     <row r="112">
       <c r="C112" s="134" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D112" s="123">
         <f t="shared" si="17"/>
@@ -17270,7 +17274,7 @@
     </row>
     <row r="113">
       <c r="C113" s="134" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D113" s="123">
         <f t="shared" si="17"/>
@@ -17288,7 +17292,7 @@
     </row>
     <row r="114">
       <c r="C114" s="134" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D114" s="123">
         <f t="shared" si="17"/>
@@ -17306,7 +17310,7 @@
     </row>
     <row r="115">
       <c r="C115" s="134" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D115" s="123">
         <f t="shared" si="17"/>
@@ -17324,7 +17328,7 @@
     </row>
     <row r="116">
       <c r="C116" s="134" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D116" s="123">
         <f t="shared" si="17"/>
@@ -17342,7 +17346,7 @@
     </row>
     <row r="117">
       <c r="C117" s="134" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D117" s="123">
         <f t="shared" si="17"/>
@@ -17358,7 +17362,7 @@
     </row>
     <row r="118">
       <c r="C118" s="134" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D118" s="123">
         <f t="shared" si="17"/>
@@ -17374,7 +17378,7 @@
     </row>
     <row r="119">
       <c r="C119" s="134" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D119" s="123">
         <f t="shared" si="17"/>
@@ -17390,7 +17394,7 @@
     </row>
     <row r="120">
       <c r="C120" s="134" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D120" s="123">
         <f t="shared" si="17"/>
@@ -17406,7 +17410,7 @@
     </row>
     <row r="121">
       <c r="C121" s="134" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D121" s="123">
         <f t="shared" si="17"/>
@@ -17422,7 +17426,7 @@
     </row>
     <row r="122">
       <c r="C122" s="134" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D122" s="123">
         <f t="shared" si="17"/>
@@ -17438,7 +17442,7 @@
     </row>
     <row r="123">
       <c r="C123" s="134" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D123" s="123">
         <f t="shared" si="17"/>
@@ -17454,7 +17458,7 @@
     </row>
     <row r="124">
       <c r="C124" s="134" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D124" s="123">
         <f t="shared" si="17"/>
@@ -17470,7 +17474,7 @@
     </row>
     <row r="125">
       <c r="C125" s="134" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D125" s="123">
         <f t="shared" si="17"/>
@@ -17486,7 +17490,7 @@
     </row>
     <row r="126">
       <c r="C126" s="134" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="D126" s="123">
         <f t="shared" si="17"/>
@@ -39910,14 +39914,14 @@
     <row r="1">
       <c r="A1" s="104"/>
       <c r="B1" s="144" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C1" s="145"/>
       <c r="D1" s="145"/>
       <c r="E1" s="145"/>
       <c r="F1" s="145"/>
       <c r="G1" s="146" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H1" s="145"/>
       <c r="I1" s="145"/>
@@ -39945,49 +39949,49 @@
         <v>3</v>
       </c>
       <c r="B2" s="148" t="s">
+        <v>292</v>
+      </c>
+      <c r="C2" s="149" t="s">
         <v>293</v>
       </c>
-      <c r="C2" s="149" t="s">
+      <c r="D2" s="149" t="s">
+        <v>197</v>
+      </c>
+      <c r="E2" s="149" t="s">
         <v>294</v>
       </c>
-      <c r="D2" s="149" t="s">
-        <v>198</v>
-      </c>
-      <c r="E2" s="149" t="s">
+      <c r="F2" s="150" t="s">
         <v>295</v>
-      </c>
-      <c r="F2" s="150" t="s">
-        <v>296</v>
       </c>
       <c r="G2" s="148">
         <v>1.0</v>
       </c>
       <c r="H2" s="149" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I2" s="149">
         <v>2.0</v>
       </c>
       <c r="J2" s="149" t="s">
+        <v>296</v>
+      </c>
+      <c r="K2" s="151" t="s">
         <v>297</v>
       </c>
-      <c r="K2" s="151" t="s">
+      <c r="L2" s="149" t="s">
         <v>298</v>
       </c>
-      <c r="L2" s="149" t="s">
+      <c r="M2" s="152" t="s">
         <v>299</v>
       </c>
-      <c r="M2" s="152" t="s">
+      <c r="N2" s="100" t="s">
         <v>300</v>
       </c>
-      <c r="N2" s="100" t="s">
+      <c r="O2" s="100" t="s">
         <v>301</v>
       </c>
-      <c r="O2" s="100" t="s">
+      <c r="P2" s="100" t="s">
         <v>302</v>
-      </c>
-      <c r="P2" s="100" t="s">
-        <v>303</v>
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
@@ -40660,7 +40664,7 @@
     </row>
     <row r="24">
       <c r="A24" s="94" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B24" s="164" t="str">
         <f t="shared" ref="B24:F24" si="4">IFERROR(AVERAGE(B3:B22),"")</f>
@@ -40770,7 +40774,7 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="165" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -40803,7 +40807,7 @@
         <v>1.0</v>
       </c>
       <c r="H28" s="166" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I28" s="166">
         <v>2.0</v>
@@ -40831,7 +40835,7 @@
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="4" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -40853,10 +40857,10 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="94" t="s">
+        <v>305</v>
+      </c>
+      <c r="M29" s="94" t="s">
         <v>306</v>
-      </c>
-      <c r="M29" s="94" t="s">
-        <v>307</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -40992,7 +40996,7 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="119" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
@@ -41026,7 +41030,7 @@
         <v>1.0</v>
       </c>
       <c r="H34" s="169" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="I34" s="169">
         <v>2.0</v>
@@ -41169,7 +41173,7 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="G38" s="168">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
DATA. Obtengo predicciones para proximos 15 dias
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -2501,7 +2501,7 @@
         <v>45693.0</v>
       </c>
       <c r="D4" s="15">
-        <v>2240.0</v>
+        <v>145.0</v>
       </c>
       <c r="E4" s="15" t="s">
         <v>15</v>
@@ -2509,21 +2509,21 @@
       <c r="F4" s="16"/>
       <c r="G4" s="17"/>
       <c r="H4" s="18">
-        <v>25.0</v>
+        <v>5.0</v>
       </c>
       <c r="I4" s="18">
-        <v>10.0</v>
+        <v>15.0</v>
       </c>
       <c r="J4" s="18">
-        <v>45.0</v>
+        <v>15.0</v>
       </c>
       <c r="K4" s="20">
         <f t="shared" ref="K4:K8" si="1">AVERAGE(H4:J4)</f>
-        <v>26.66666667</v>
+        <v>11.66666667</v>
       </c>
       <c r="L4" s="27">
         <f>K4*'Data preparation'!$C$2</f>
-        <v>6.666666667</v>
+        <v>2.916666667</v>
       </c>
       <c r="M4" s="16"/>
       <c r="N4" s="20" t="str">
@@ -2542,7 +2542,7 @@
         <v>45693.0</v>
       </c>
       <c r="D5" s="15">
-        <v>218.0</v>
+        <v>1126.0</v>
       </c>
       <c r="E5" s="15" t="s">
         <v>15</v>
@@ -2550,21 +2550,21 @@
       <c r="F5" s="16"/>
       <c r="G5" s="17"/>
       <c r="H5" s="16">
-        <v>45.0</v>
+        <v>15.0</v>
       </c>
       <c r="I5" s="16">
-        <v>10.0</v>
+        <v>15.0</v>
       </c>
       <c r="J5" s="16">
-        <v>10.0</v>
+        <v>15.0</v>
       </c>
       <c r="K5" s="20">
         <f t="shared" si="1"/>
-        <v>21.66666667</v>
+        <v>15</v>
       </c>
       <c r="L5" s="27">
         <f>K5*'Data preparation'!$C$2</f>
-        <v>5.416666667</v>
+        <v>3.75</v>
       </c>
       <c r="M5" s="16"/>
       <c r="N5" s="20" t="str">
@@ -2584,7 +2584,7 @@
         <v>45693.0</v>
       </c>
       <c r="D6" s="15">
-        <v>447.0</v>
+        <v>1288.0</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>15</v>
@@ -2592,21 +2592,21 @@
       <c r="F6" s="16"/>
       <c r="G6" s="17"/>
       <c r="H6" s="16">
-        <v>45.0</v>
+        <v>15.0</v>
       </c>
       <c r="I6" s="16">
-        <v>45.0</v>
+        <v>15.0</v>
       </c>
       <c r="J6" s="16">
-        <v>10.0</v>
+        <v>15.0</v>
       </c>
       <c r="K6" s="20">
         <f t="shared" si="1"/>
-        <v>33.33333333</v>
+        <v>15</v>
       </c>
       <c r="L6" s="27">
         <f>K6*'Data preparation'!$C$2</f>
-        <v>8.333333333</v>
+        <v>3.75</v>
       </c>
       <c r="M6" s="32"/>
       <c r="N6" s="20" t="str">
@@ -2625,7 +2625,7 @@
         <v>45693.0</v>
       </c>
       <c r="D7" s="15">
-        <v>1157.0</v>
+        <v>1091.0</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>15</v>
@@ -2633,21 +2633,21 @@
       <c r="F7" s="16"/>
       <c r="G7" s="17"/>
       <c r="H7" s="18">
-        <v>10.0</v>
+        <v>5.0</v>
       </c>
       <c r="I7" s="18">
-        <v>45.0</v>
+        <v>15.0</v>
       </c>
       <c r="J7" s="18">
-        <v>25.0</v>
+        <v>15.0</v>
       </c>
       <c r="K7" s="20">
         <f t="shared" si="1"/>
-        <v>26.66666667</v>
+        <v>11.66666667</v>
       </c>
       <c r="L7" s="27">
         <f>K7*'Data preparation'!$C$2</f>
-        <v>6.666666667</v>
+        <v>2.916666667</v>
       </c>
       <c r="M7" s="16"/>
       <c r="N7" s="20" t="str">
@@ -2666,23 +2666,29 @@
         <v>45693.0</v>
       </c>
       <c r="D8" s="15">
-        <v>508.0</v>
+        <v>1201.0</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>15</v>
       </c>
       <c r="F8" s="16"/>
       <c r="G8" s="17"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="20" t="str">
+      <c r="H8" s="18">
+        <v>15.0</v>
+      </c>
+      <c r="I8" s="18">
+        <v>15.0</v>
+      </c>
+      <c r="J8" s="18">
+        <v>15.0</v>
+      </c>
+      <c r="K8" s="20">
         <f t="shared" si="1"/>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="L8" s="27" t="str">
+        <v>15</v>
+      </c>
+      <c r="L8" s="27">
         <f>K8*'Data preparation'!$C$2</f>
-        <v>#DIV/0!</v>
+        <v>3.75</v>
       </c>
       <c r="M8" s="16"/>
       <c r="N8" s="20" t="str">
@@ -14953,9 +14959,9 @@
       <c r="B3" s="94" t="s">
         <v>143</v>
       </c>
-      <c r="C3" s="21" t="str">
+      <c r="C3" s="26">
         <f>AVERAGE('Modelos actuales'!L4:L8)</f>
-        <v>#DIV/0!</v>
+        <v>3.416666667</v>
       </c>
       <c r="L3" s="117"/>
       <c r="P3" s="117"/>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones para proximos dias
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -261,7 +261,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="547" uniqueCount="335">
   <si>
     <t>id_country</t>
   </si>
@@ -1002,28 +1002,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>7.93</t>
+    <t>7.58</t>
   </si>
   <si>
-    <t>12.86</t>
+    <t>10.24</t>
   </si>
   <si>
-    <t>0.16</t>
+    <t>7.47</t>
   </si>
   <si>
-    <t>12.27</t>
+    <t>8.73</t>
   </si>
   <si>
-    <t>12.03</t>
+    <t>8.64</t>
   </si>
   <si>
-    <t>9.22</t>
+    <t>8.72</t>
   </si>
   <si>
-    <t>12.77</t>
+    <t>9.64</t>
   </si>
   <si>
-    <t>12.99</t>
+    <t>10.34</t>
   </si>
   <si>
     <t>Country</t>
@@ -1032,280 +1032,289 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>1.00</t>
+    <t>1.39</t>
   </si>
   <si>
-    <t>14.07</t>
+    <t>13.42</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>11.48</t>
+    <t>8.68</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>11.07</t>
+    <t>7.54</t>
   </si>
   <si>
     <t>p25</t>
   </si>
   <si>
-    <t>13.49</t>
+    <t>11.32</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>12.70</t>
+    <t>13.68</t>
   </si>
   <si>
-    <t>12.43</t>
+    <t>9.52</t>
   </si>
   <si>
-    <t>9.82</t>
+    <t>11.07</t>
   </si>
   <si>
-    <t>9.99</t>
+    <t>5.85</t>
   </si>
   <si>
-    <t>13.31</t>
+    <t>10.66</t>
   </si>
   <si>
-    <t>13.53</t>
+    <t>11.13</t>
   </si>
   <si>
-    <t>7.38</t>
+    <t>8.77</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
   </si>
   <si>
-    <t>10.44</t>
+    <t>6.66</t>
   </si>
   <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>8.92</t>
+    <t>1.06</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
-    <t>10.28</t>
+    <t>8.01</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>3.75</t>
+    <t>12.51</t>
   </si>
   <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
+    <t>7.35</t>
+  </si>
+  <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>10.15</t>
+    <t>7.00</t>
   </si>
   <si>
-    <t>2.04</t>
+    <t>7.32</t>
   </si>
   <si>
-    <t>11.54</t>
+    <t>12.88</t>
   </si>
   <si>
-    <t>7.35</t>
+    <t>1.34</t>
   </si>
   <si>
-    <t>11.49</t>
+    <t>9.67</t>
   </si>
   <si>
-    <t>0.12</t>
+    <t>1.47</t>
   </si>
   <si>
-    <t>3.87</t>
+    <t>13.17</t>
   </si>
   <si>
-    <t>2.25</t>
+    <t>1.23</t>
   </si>
   <si>
-    <t>1.52</t>
+    <t>8.34</t>
   </si>
   <si>
-    <t>10.50</t>
+    <t>8.06</t>
   </si>
   <si>
-    <t>11.30</t>
+    <t>6.29</t>
   </si>
   <si>
-    <t>4.37</t>
+    <t>9.97</t>
   </si>
   <si>
-    <t>11.20</t>
+    <t>1.44</t>
   </si>
   <si>
-    <t>5.74</t>
+    <t>9.59</t>
   </si>
   <si>
-    <t>4.72</t>
+    <t>12.78</t>
   </si>
   <si>
-    <t>4.46</t>
+    <t>12.76</t>
   </si>
   <si>
-    <t>2.26</t>
+    <t>9.88</t>
   </si>
   <si>
-    <t>9.41</t>
+    <t>14.80</t>
   </si>
   <si>
-    <t>12.35</t>
+    <t>13.66</t>
   </si>
   <si>
-    <t>5.57</t>
+    <t>12.90</t>
   </si>
   <si>
-    <t>11.16</t>
+    <t>1.46</t>
   </si>
   <si>
-    <t>9.69</t>
+    <t>13.01</t>
   </si>
   <si>
-    <t>11.21</t>
+    <t>1.55</t>
   </si>
   <si>
-    <t>9.32</t>
+    <t>10.88</t>
   </si>
   <si>
-    <t>12.79</t>
+    <t>9.70</t>
   </si>
   <si>
-    <t>9.83</t>
+    <t>14.30</t>
   </si>
   <si>
-    <t>10.65</t>
+    <t>7.41</t>
+  </si>
+  <si>
+    <t>10.62</t>
+  </si>
+  <si>
+    <t>6.11</t>
+  </si>
+  <si>
+    <t>8.03</t>
+  </si>
+  <si>
+    <t>8.22</t>
+  </si>
+  <si>
+    <t>8.46</t>
+  </si>
+  <si>
+    <t>7.64</t>
+  </si>
+  <si>
+    <t>8.62</t>
+  </si>
+  <si>
+    <t>9.37</t>
+  </si>
+  <si>
+    <t>4.91</t>
+  </si>
+  <si>
+    <t>10.05</t>
+  </si>
+  <si>
+    <t>7.02</t>
+  </si>
+  <si>
+    <t>1.12</t>
+  </si>
+  <si>
+    <t>8.65</t>
+  </si>
+  <si>
+    <t>8.08</t>
+  </si>
+  <si>
+    <t>8.54</t>
+  </si>
+  <si>
+    <t>6.46</t>
   </si>
   <si>
     <t>8.98</t>
   </si>
   <si>
-    <t>8.23</t>
+    <t>3.85</t>
   </si>
   <si>
-    <t>8.74</t>
+    <t>6.24</t>
   </si>
   <si>
-    <t>9.23</t>
+    <t>1.17</t>
+  </si>
+  <si>
+    <t>6.13</t>
+  </si>
+  <si>
+    <t>6.44</t>
+  </si>
+  <si>
+    <t>4.99</t>
+  </si>
+  <si>
+    <t>4.52</t>
+  </si>
+  <si>
+    <t>8.48</t>
+  </si>
+  <si>
+    <t>6.39</t>
   </si>
   <si>
     <t>9.74</t>
   </si>
   <si>
-    <t>6.85</t>
+    <t>7.70</t>
   </si>
   <si>
-    <t>5.70</t>
+    <t>0.80</t>
   </si>
   <si>
-    <t>6.47</t>
+    <t>9.57</t>
   </si>
   <si>
-    <t>3.43</t>
+    <t>0.71</t>
   </si>
   <si>
-    <t>0.15</t>
+    <t>4.34</t>
   </si>
   <si>
-    <t>9.39</t>
+    <t>8.09</t>
   </si>
   <si>
-    <t>0.53</t>
+    <t>6.41</t>
   </si>
   <si>
-    <t>6.69</t>
+    <t>8.83</t>
   </si>
   <si>
-    <t>0.18</t>
+    <t>4.75</t>
   </si>
   <si>
-    <t>6.92</t>
+    <t>5.68</t>
   </si>
   <si>
-    <t>5.60</t>
+    <t>9.04</t>
   </si>
   <si>
-    <t>0.28</t>
+    <t>6.89</t>
   </si>
   <si>
-    <t>1.24</t>
+    <t>4.98</t>
   </si>
   <si>
-    <t>9.44</t>
-  </si>
-  <si>
-    <t>3.11</t>
-  </si>
-  <si>
-    <t>12.90</t>
-  </si>
-  <si>
-    <t>0.77</t>
-  </si>
-  <si>
-    <t>8.33</t>
-  </si>
-  <si>
-    <t>13.99</t>
-  </si>
-  <si>
-    <t>1.03</t>
-  </si>
-  <si>
-    <t>13.48</t>
-  </si>
-  <si>
-    <t>13.88</t>
-  </si>
-  <si>
-    <t>8.68</t>
-  </si>
-  <si>
-    <t>12.29</t>
-  </si>
-  <si>
-    <t>5.54</t>
-  </si>
-  <si>
-    <t>8.36</t>
-  </si>
-  <si>
-    <t>13.42</t>
-  </si>
-  <si>
-    <t>10.20</t>
-  </si>
-  <si>
-    <t>4.56</t>
-  </si>
-  <si>
-    <t>11.70</t>
-  </si>
-  <si>
-    <t>14.03</t>
-  </si>
-  <si>
-    <t>8.15</t>
-  </si>
-  <si>
-    <t>8.46</t>
-  </si>
-  <si>
-    <t>5.83</t>
+    <t>7.92</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2570,14 +2579,14 @@
         <v>15</v>
       </c>
       <c r="M4" s="19">
-        <v>3464.10585075032</v>
+        <v>4127.12732043093</v>
       </c>
       <c r="N4" s="31">
         <f t="shared" ref="N4:N8" si="2">M4/F4</f>
-        <v>4.786722097</v>
+        <v>5.702889112</v>
       </c>
       <c r="O4" s="19">
-        <v>176.463140301466</v>
+        <v>83.2034043962739</v>
       </c>
     </row>
     <row r="5">
@@ -2642,13 +2651,13 @@
         <v>45693.0</v>
       </c>
       <c r="D6" s="15">
-        <v>111.0</v>
+        <v>732.0</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>16</v>
       </c>
       <c r="F6" s="16">
-        <v>391.688847010193</v>
+        <v>420.892675935302</v>
       </c>
       <c r="G6" s="19">
         <v>40.0</v>
@@ -2671,14 +2680,14 @@
         <v>20</v>
       </c>
       <c r="M6" s="33">
-        <v>2797.81722805449</v>
+        <v>3454.61988359074</v>
       </c>
       <c r="N6" s="31">
         <f t="shared" si="2"/>
-        <v>7.142958625</v>
+        <v>8.207840338</v>
       </c>
       <c r="O6" s="19">
-        <v>74.8994892871103</v>
+        <v>523.181373773246</v>
       </c>
     </row>
     <row r="7">
@@ -2692,13 +2701,13 @@
         <v>45693.0</v>
       </c>
       <c r="D7" s="15">
-        <v>374.0</v>
+        <v>1270.0</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>16</v>
       </c>
       <c r="F7" s="16">
-        <v>199.188159667619</v>
+        <v>196.200539201566</v>
       </c>
       <c r="G7" s="17">
         <v>30.0</v>
@@ -2721,14 +2730,14 @@
         <v>15</v>
       </c>
       <c r="M7" s="19">
-        <v>697.254148551371</v>
+        <v>659.351291524406</v>
       </c>
       <c r="N7" s="31">
         <f t="shared" si="2"/>
-        <v>3.500479897</v>
+        <v>3.360598774</v>
       </c>
       <c r="O7" s="19">
-        <v>839.09522760747</v>
+        <v>334.198925698403</v>
       </c>
     </row>
     <row r="8">
@@ -2742,16 +2751,16 @@
         <v>45693.0</v>
       </c>
       <c r="D8" s="15">
-        <v>499.0</v>
+        <v>508.0</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>16</v>
       </c>
       <c r="F8" s="16">
-        <v>195.637194025755</v>
+        <v>411.423262848422</v>
       </c>
       <c r="G8" s="17">
-        <v>20.0</v>
+        <v>30.0</v>
       </c>
       <c r="H8" s="17">
         <v>30.0</v>
@@ -2768,17 +2777,17 @@
       </c>
       <c r="L8" s="27">
         <f>G8*'Data preparation'!$C$2</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="M8" s="19">
-        <v>337.019635200559</v>
+        <v>1466.69528214825</v>
       </c>
       <c r="N8" s="31">
         <f t="shared" si="2"/>
-        <v>1.722676697</v>
+        <v>3.564930364</v>
       </c>
       <c r="O8" s="19">
-        <v>-52.9989623627844</v>
+        <v>-86.9543871782569</v>
       </c>
     </row>
     <row r="9" ht="20.25" customHeight="1">
@@ -16539,7 +16548,7 @@
       </c>
       <c r="C3" s="26">
         <f>AVERAGE('Modelos actuales'!L4:L8)</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L3" s="118"/>
       <c r="P3" s="118"/>
@@ -17840,7 +17849,7 @@
       <c r="C37" s="41"/>
       <c r="D37" s="132">
         <f>AVERAGE(D39:D1775)</f>
-        <v>8.188556701</v>
+        <v>7.867938144</v>
       </c>
       <c r="G37" s="39" t="s">
         <v>38</v>
@@ -17909,7 +17918,7 @@
       </c>
       <c r="D39" s="124">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>7.93</v>
+        <v>7.58</v>
       </c>
       <c r="G39" s="39" t="s">
         <v>30</v>
@@ -17947,7 +17956,7 @@
       </c>
       <c r="D40" s="124">
         <f t="shared" si="17"/>
-        <v>12.86</v>
+        <v>10.24</v>
       </c>
       <c r="G40" s="39" t="s">
         <v>26</v>
@@ -17985,7 +17994,7 @@
       </c>
       <c r="D41" s="124">
         <f t="shared" si="17"/>
-        <v>0.16</v>
+        <v>7.47</v>
       </c>
       <c r="P41" s="122">
         <v>0.0</v>
@@ -18017,7 +18026,7 @@
       </c>
       <c r="D42" s="124">
         <f t="shared" si="17"/>
-        <v>12.27</v>
+        <v>8.73</v>
       </c>
       <c r="P42" s="122">
         <v>2.0</v>
@@ -18049,7 +18058,7 @@
       </c>
       <c r="D43" s="124">
         <f t="shared" si="17"/>
-        <v>12.03</v>
+        <v>8.64</v>
       </c>
       <c r="P43" s="122">
         <v>1.0</v>
@@ -18081,7 +18090,7 @@
       </c>
       <c r="D44" s="124">
         <f t="shared" si="17"/>
-        <v>9.22</v>
+        <v>8.72</v>
       </c>
       <c r="P44" s="122">
         <v>2.0</v>
@@ -18111,7 +18120,7 @@
       </c>
       <c r="D45" s="124">
         <f t="shared" si="17"/>
-        <v>12.77</v>
+        <v>9.64</v>
       </c>
       <c r="P45" s="122">
         <v>1.0</v>
@@ -18129,7 +18138,7 @@
       </c>
       <c r="D46" s="124">
         <f t="shared" si="17"/>
-        <v>12.99</v>
+        <v>10.34</v>
       </c>
       <c r="G46" s="96" t="s">
         <v>219</v>
@@ -18153,7 +18162,7 @@
       </c>
       <c r="D47" s="124">
         <f t="shared" si="17"/>
-        <v>1</v>
+        <v>1.39</v>
       </c>
       <c r="G47" s="101" t="s">
         <v>39</v>
@@ -18183,7 +18192,7 @@
       </c>
       <c r="D48" s="124">
         <f t="shared" si="17"/>
-        <v>14.07</v>
+        <v>13.42</v>
       </c>
       <c r="G48" s="101" t="s">
         <v>38</v>
@@ -18220,7 +18229,7 @@
       </c>
       <c r="D49" s="124">
         <f t="shared" si="17"/>
-        <v>11.48</v>
+        <v>8.68</v>
       </c>
       <c r="G49" s="101" t="s">
         <v>29</v>
@@ -18257,7 +18266,7 @@
       </c>
       <c r="D50" s="124">
         <f t="shared" si="17"/>
-        <v>11.07</v>
+        <v>7.54</v>
       </c>
       <c r="G50" s="101" t="s">
         <v>30</v>
@@ -18294,7 +18303,7 @@
       </c>
       <c r="D51" s="124">
         <f t="shared" si="17"/>
-        <v>13.49</v>
+        <v>11.32</v>
       </c>
       <c r="G51" s="101" t="s">
         <v>26</v>
@@ -18331,7 +18340,7 @@
       </c>
       <c r="D52" s="124">
         <f t="shared" si="17"/>
-        <v>12.7</v>
+        <v>13.68</v>
       </c>
       <c r="P52" s="122">
         <v>0.0</v>
@@ -18355,7 +18364,7 @@
       </c>
       <c r="D53" s="124">
         <f t="shared" si="17"/>
-        <v>12.43</v>
+        <v>9.52</v>
       </c>
       <c r="P53" s="122">
         <v>0.0</v>
@@ -18379,7 +18388,7 @@
       </c>
       <c r="D54" s="124">
         <f t="shared" si="17"/>
-        <v>9.82</v>
+        <v>11.07</v>
       </c>
       <c r="P54" s="122">
         <v>2.0</v>
@@ -18403,7 +18412,7 @@
       </c>
       <c r="D55" s="124">
         <f t="shared" si="17"/>
-        <v>9.99</v>
+        <v>5.85</v>
       </c>
       <c r="P55" s="122">
         <v>0.0</v>
@@ -18427,7 +18436,7 @@
       </c>
       <c r="D56" s="124">
         <f t="shared" si="17"/>
-        <v>13.31</v>
+        <v>10.66</v>
       </c>
       <c r="P56" s="122">
         <v>0.0</v>
@@ -18451,7 +18460,7 @@
       </c>
       <c r="D57" s="124">
         <f t="shared" si="17"/>
-        <v>13.53</v>
+        <v>11.13</v>
       </c>
       <c r="P57" s="122">
         <v>2.0</v>
@@ -18475,7 +18484,7 @@
       </c>
       <c r="D58" s="124">
         <f t="shared" si="17"/>
-        <v>7.38</v>
+        <v>8.77</v>
       </c>
       <c r="G58" s="137" t="s">
         <v>237</v>
@@ -18503,7 +18512,7 @@
       </c>
       <c r="D59" s="124">
         <f t="shared" si="17"/>
-        <v>10.44</v>
+        <v>6.66</v>
       </c>
       <c r="G59" s="138"/>
       <c r="H59" s="139" t="s">
@@ -18531,7 +18540,7 @@
       </c>
       <c r="D60" s="124">
         <f t="shared" si="17"/>
-        <v>8.92</v>
+        <v>1.06</v>
       </c>
       <c r="G60" s="138"/>
       <c r="H60" s="139" t="s">
@@ -18559,7 +18568,7 @@
       </c>
       <c r="D61" s="124">
         <f t="shared" si="17"/>
-        <v>10.28</v>
+        <v>8.01</v>
       </c>
       <c r="G61" s="138"/>
       <c r="H61" s="139" t="s">
@@ -18587,7 +18596,7 @@
       </c>
       <c r="D62" s="124">
         <f t="shared" si="17"/>
-        <v>3.75</v>
+        <v>12.51</v>
       </c>
       <c r="G62" s="138"/>
       <c r="H62" s="139" t="s">
@@ -18611,15 +18620,15 @@
     </row>
     <row r="63">
       <c r="C63" s="135" t="s">
-        <v>216</v>
+        <v>246</v>
       </c>
       <c r="D63" s="124">
         <f t="shared" si="17"/>
-        <v>9.22</v>
+        <v>7.35</v>
       </c>
       <c r="G63" s="138"/>
       <c r="H63" s="139" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="P63" s="122">
         <v>0.0</v>
@@ -18633,11 +18642,11 @@
     </row>
     <row r="64">
       <c r="C64" s="135" t="s">
-        <v>247</v>
+        <v>238</v>
       </c>
       <c r="D64" s="124">
         <f t="shared" si="17"/>
-        <v>10.15</v>
+        <v>6.66</v>
       </c>
       <c r="P64" s="122">
         <v>1.0</v>
@@ -18655,7 +18664,7 @@
       </c>
       <c r="D65" s="124">
         <f t="shared" si="17"/>
-        <v>2.04</v>
+        <v>7</v>
       </c>
       <c r="P65" s="122">
         <v>2.0</v>
@@ -18673,7 +18682,7 @@
       </c>
       <c r="D66" s="124">
         <f t="shared" si="17"/>
-        <v>11.54</v>
+        <v>7.32</v>
       </c>
       <c r="P66" s="122">
         <v>0.0</v>
@@ -18691,7 +18700,7 @@
       </c>
       <c r="D67" s="124">
         <f t="shared" si="17"/>
-        <v>7.35</v>
+        <v>12.88</v>
       </c>
       <c r="P67" s="122">
         <v>0.0</v>
@@ -18705,11 +18714,11 @@
     </row>
     <row r="68">
       <c r="C68" s="135" t="s">
-        <v>201</v>
+        <v>251</v>
       </c>
       <c r="D68" s="124">
         <f t="shared" si="17"/>
-        <v>4.73</v>
+        <v>1.34</v>
       </c>
       <c r="P68" s="122">
         <v>1.0</v>
@@ -18723,11 +18732,11 @@
     </row>
     <row r="69">
       <c r="C69" s="135" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D69" s="124">
         <f t="shared" si="17"/>
-        <v>11.49</v>
+        <v>9.67</v>
       </c>
       <c r="P69" s="122">
         <v>2.0</v>
@@ -18741,11 +18750,11 @@
     </row>
     <row r="70">
       <c r="C70" s="135" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D70" s="124">
         <f t="shared" si="17"/>
-        <v>0.12</v>
+        <v>1.47</v>
       </c>
       <c r="P70" s="122">
         <v>1.0</v>
@@ -18759,11 +18768,11 @@
     </row>
     <row r="71">
       <c r="C71" s="135" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D71" s="124">
         <f t="shared" si="17"/>
-        <v>3.87</v>
+        <v>13.17</v>
       </c>
       <c r="F71" s="140"/>
       <c r="P71" s="122">
@@ -18778,11 +18787,11 @@
     </row>
     <row r="72">
       <c r="C72" s="135" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D72" s="124">
         <f t="shared" si="17"/>
-        <v>2.25</v>
+        <v>1.23</v>
       </c>
       <c r="P72" s="122">
         <v>0.0</v>
@@ -18796,11 +18805,11 @@
     </row>
     <row r="73">
       <c r="C73" s="135" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D73" s="124">
         <f t="shared" si="17"/>
-        <v>1.52</v>
+        <v>8.34</v>
       </c>
       <c r="P73" s="122">
         <v>1.0</v>
@@ -18814,11 +18823,11 @@
     </row>
     <row r="74">
       <c r="C74" s="135" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="D74" s="124">
         <f t="shared" si="17"/>
-        <v>10.5</v>
+        <v>8.06</v>
       </c>
       <c r="P74" s="122">
         <v>0.0</v>
@@ -18832,11 +18841,11 @@
     </row>
     <row r="75">
       <c r="C75" s="135" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D75" s="124">
         <f t="shared" si="17"/>
-        <v>11.3</v>
+        <v>6.29</v>
       </c>
       <c r="P75" s="122">
         <v>1.0</v>
@@ -18850,11 +18859,11 @@
     </row>
     <row r="76">
       <c r="C76" s="135" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D76" s="124">
         <f t="shared" si="17"/>
-        <v>4.37</v>
+        <v>9.97</v>
       </c>
       <c r="P76" s="122">
         <v>0.0</v>
@@ -18868,11 +18877,11 @@
     </row>
     <row r="77">
       <c r="C77" s="135" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D77" s="124">
         <f t="shared" si="17"/>
-        <v>11.2</v>
+        <v>1.44</v>
       </c>
       <c r="P77" s="122">
         <v>0.0</v>
@@ -18886,11 +18895,11 @@
     </row>
     <row r="78">
       <c r="C78" s="135" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="D78" s="124">
         <f t="shared" si="17"/>
-        <v>5.74</v>
+        <v>9.59</v>
       </c>
       <c r="P78" s="122">
         <v>1.0</v>
@@ -18904,11 +18913,11 @@
     </row>
     <row r="79">
       <c r="C79" s="135" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D79" s="124">
         <f t="shared" si="17"/>
-        <v>4.72</v>
+        <v>12.78</v>
       </c>
       <c r="P79" s="122">
         <v>2.0</v>
@@ -18922,11 +18931,11 @@
     </row>
     <row r="80">
       <c r="C80" s="135" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D80" s="124">
         <f t="shared" si="17"/>
-        <v>4.46</v>
+        <v>12.76</v>
       </c>
       <c r="P80" s="122">
         <v>1.0</v>
@@ -18940,11 +18949,11 @@
     </row>
     <row r="81">
       <c r="C81" s="135" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D81" s="124">
         <f t="shared" si="17"/>
-        <v>2.26</v>
+        <v>9.88</v>
       </c>
       <c r="P81" s="122">
         <v>2.0</v>
@@ -18958,11 +18967,11 @@
     </row>
     <row r="82">
       <c r="C82" s="135" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D82" s="124">
         <f t="shared" si="17"/>
-        <v>9.41</v>
+        <v>14.8</v>
       </c>
       <c r="P82" s="122">
         <v>1.0</v>
@@ -18976,11 +18985,11 @@
     </row>
     <row r="83">
       <c r="C83" s="135" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D83" s="124">
         <f t="shared" si="17"/>
-        <v>12.35</v>
+        <v>13.66</v>
       </c>
       <c r="P83" s="122">
         <v>0.0</v>
@@ -18994,11 +19003,11 @@
     </row>
     <row r="84">
       <c r="C84" s="135" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D84" s="124">
         <f t="shared" si="17"/>
-        <v>5.57</v>
+        <v>12.9</v>
       </c>
       <c r="P84" s="122">
         <v>1.0</v>
@@ -19012,11 +19021,11 @@
     </row>
     <row r="85">
       <c r="C85" s="135" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D85" s="124">
         <f t="shared" si="17"/>
-        <v>11.16</v>
+        <v>1.46</v>
       </c>
       <c r="P85" s="122">
         <v>0.0</v>
@@ -19030,11 +19039,11 @@
     </row>
     <row r="86">
       <c r="C86" s="135" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D86" s="124">
         <f t="shared" si="17"/>
-        <v>9.69</v>
+        <v>13.01</v>
       </c>
       <c r="P86" s="122">
         <v>0.0</v>
@@ -19048,11 +19057,11 @@
     </row>
     <row r="87">
       <c r="C87" s="135" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D87" s="124">
         <f t="shared" si="17"/>
-        <v>11.21</v>
+        <v>1.55</v>
       </c>
       <c r="P87" s="122">
         <v>1.0</v>
@@ -19066,11 +19075,11 @@
     </row>
     <row r="88">
       <c r="C88" s="135" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D88" s="124">
         <f t="shared" si="17"/>
-        <v>9.32</v>
+        <v>10.88</v>
       </c>
       <c r="P88" s="122">
         <v>2.0</v>
@@ -19084,11 +19093,11 @@
     </row>
     <row r="89">
       <c r="C89" s="135" t="s">
-        <v>249</v>
+        <v>272</v>
       </c>
       <c r="D89" s="124">
         <f t="shared" si="17"/>
-        <v>11.54</v>
+        <v>9.7</v>
       </c>
       <c r="P89" s="122">
         <v>2.0</v>
@@ -19102,11 +19111,11 @@
     </row>
     <row r="90">
       <c r="C90" s="135" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="D90" s="124">
         <f t="shared" si="17"/>
-        <v>12.79</v>
+        <v>14.3</v>
       </c>
       <c r="P90" s="122">
         <v>1.0</v>
@@ -19120,11 +19129,11 @@
     </row>
     <row r="91">
       <c r="C91" s="135" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D91" s="124">
         <f t="shared" si="17"/>
-        <v>9.83</v>
+        <v>7.41</v>
       </c>
       <c r="P91" s="122">
         <v>1.0</v>
@@ -19138,11 +19147,11 @@
     </row>
     <row r="92">
       <c r="C92" s="135" t="s">
-        <v>224</v>
+        <v>275</v>
       </c>
       <c r="D92" s="124">
         <f t="shared" si="17"/>
-        <v>11.48</v>
+        <v>10.62</v>
       </c>
       <c r="P92" s="122">
         <v>2.0</v>
@@ -19156,11 +19165,11 @@
     </row>
     <row r="93">
       <c r="C93" s="135" t="s">
-        <v>273</v>
+        <v>244</v>
       </c>
       <c r="D93" s="124">
         <f t="shared" si="17"/>
-        <v>10.65</v>
+        <v>12.51</v>
       </c>
       <c r="P93" s="122">
         <v>0.0</v>
@@ -19174,11 +19183,11 @@
     </row>
     <row r="94">
       <c r="C94" s="135" t="s">
-        <v>274</v>
+        <v>248</v>
       </c>
       <c r="D94" s="124">
         <f t="shared" si="17"/>
-        <v>8.98</v>
+        <v>7</v>
       </c>
       <c r="P94" s="122">
         <v>0.0</v>
@@ -19192,11 +19201,11 @@
     </row>
     <row r="95">
       <c r="C95" s="135" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D95" s="124">
         <f t="shared" si="17"/>
-        <v>8.23</v>
+        <v>6.11</v>
       </c>
       <c r="P95" s="122">
         <v>1.0</v>
@@ -19210,11 +19219,11 @@
     </row>
     <row r="96">
       <c r="C96" s="135" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="D96" s="124">
         <f t="shared" si="17"/>
-        <v>8.74</v>
+        <v>8.03</v>
       </c>
       <c r="P96" s="122">
         <v>2.0</v>
@@ -19228,11 +19237,11 @@
     </row>
     <row r="97">
       <c r="C97" s="135" t="s">
-        <v>277</v>
+        <v>217</v>
       </c>
       <c r="D97" s="124">
         <f t="shared" si="17"/>
-        <v>9.23</v>
+        <v>9.64</v>
       </c>
       <c r="P97" s="122">
         <v>0.0</v>
@@ -19250,7 +19259,7 @@
       </c>
       <c r="D98" s="124">
         <f t="shared" si="17"/>
-        <v>9.74</v>
+        <v>8.22</v>
       </c>
       <c r="P98" s="122">
         <v>2.0</v>
@@ -19264,11 +19273,11 @@
     </row>
     <row r="99">
       <c r="C99" s="135" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
       <c r="D99" s="124">
         <f t="shared" si="17"/>
-        <v>9.41</v>
+        <v>8.46</v>
       </c>
       <c r="P99" s="122">
         <v>2.0</v>
@@ -19282,11 +19291,11 @@
     </row>
     <row r="100">
       <c r="C100" s="135" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="D100" s="124">
         <f t="shared" si="17"/>
-        <v>6.85</v>
+        <v>7.64</v>
       </c>
       <c r="P100" s="122">
         <v>2.0</v>
@@ -19300,11 +19309,11 @@
     </row>
     <row r="101">
       <c r="C101" s="135" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D101" s="124">
         <f t="shared" si="17"/>
-        <v>5.7</v>
+        <v>8.62</v>
       </c>
       <c r="P101" s="122">
         <v>2.0</v>
@@ -19318,11 +19327,11 @@
     </row>
     <row r="102">
       <c r="C102" s="135" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="D102" s="124">
         <f t="shared" si="17"/>
-        <v>6.47</v>
+        <v>9.37</v>
       </c>
       <c r="P102" s="122">
         <v>2.0</v>
@@ -19336,11 +19345,11 @@
     </row>
     <row r="103">
       <c r="C103" s="135" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="D103" s="124">
         <f t="shared" si="17"/>
-        <v>3.43</v>
+        <v>4.91</v>
       </c>
       <c r="P103" s="122">
         <v>1.0</v>
@@ -19354,11 +19363,11 @@
     </row>
     <row r="104">
       <c r="C104" s="135" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="D104" s="124">
         <f t="shared" si="17"/>
-        <v>0.15</v>
+        <v>10.05</v>
       </c>
       <c r="N104" s="141"/>
       <c r="P104" s="122">
@@ -19373,11 +19382,11 @@
     </row>
     <row r="105">
       <c r="C105" s="135" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="D105" s="124">
         <f t="shared" si="17"/>
-        <v>9.39</v>
+        <v>7.02</v>
       </c>
       <c r="N105" s="21"/>
       <c r="P105" s="122">
@@ -19392,11 +19401,11 @@
     </row>
     <row r="106">
       <c r="C106" s="135" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="D106" s="124">
         <f t="shared" si="17"/>
-        <v>0.53</v>
+        <v>1.12</v>
       </c>
       <c r="N106" s="21"/>
       <c r="P106" s="122">
@@ -19411,11 +19420,11 @@
     </row>
     <row r="107">
       <c r="C107" s="135" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D107" s="124">
         <f t="shared" si="17"/>
-        <v>6.69</v>
+        <v>8.65</v>
       </c>
       <c r="N107" s="21"/>
       <c r="P107" s="122">
@@ -19430,11 +19439,11 @@
     </row>
     <row r="108">
       <c r="C108" s="135" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="D108" s="124">
         <f t="shared" si="17"/>
-        <v>0.18</v>
+        <v>8.08</v>
       </c>
       <c r="N108" s="21"/>
       <c r="P108" s="122">
@@ -19449,11 +19458,11 @@
     </row>
     <row r="109">
       <c r="C109" s="135" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="D109" s="124">
         <f t="shared" si="17"/>
-        <v>6.92</v>
+        <v>8.54</v>
       </c>
       <c r="N109" s="21"/>
       <c r="P109" s="122">
@@ -19468,11 +19477,11 @@
     </row>
     <row r="110">
       <c r="C110" s="135" t="s">
-        <v>213</v>
+        <v>290</v>
       </c>
       <c r="D110" s="124">
         <f t="shared" si="17"/>
-        <v>0.16</v>
+        <v>6.46</v>
       </c>
       <c r="N110" s="21"/>
       <c r="P110" s="122">
@@ -19487,11 +19496,11 @@
     </row>
     <row r="111">
       <c r="C111" s="135" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="D111" s="124">
         <f t="shared" si="17"/>
-        <v>5.6</v>
+        <v>8.98</v>
       </c>
       <c r="N111" s="21"/>
       <c r="P111" s="122">
@@ -19506,11 +19515,11 @@
     </row>
     <row r="112">
       <c r="C112" s="135" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D112" s="124">
         <f t="shared" si="17"/>
-        <v>0.28</v>
+        <v>3.85</v>
       </c>
       <c r="P112" s="122">
         <v>1.0</v>
@@ -19524,11 +19533,11 @@
     </row>
     <row r="113">
       <c r="C113" s="135" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="D113" s="124">
         <f t="shared" si="17"/>
-        <v>1.24</v>
+        <v>6.24</v>
       </c>
       <c r="P113" s="122">
         <v>0.0</v>
@@ -19542,11 +19551,11 @@
     </row>
     <row r="114">
       <c r="C114" s="135" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D114" s="124">
         <f t="shared" si="17"/>
-        <v>9.44</v>
+        <v>1.17</v>
       </c>
       <c r="P114" s="122">
         <v>1.0</v>
@@ -19560,11 +19569,11 @@
     </row>
     <row r="115">
       <c r="C115" s="135" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="D115" s="124">
         <f t="shared" si="17"/>
-        <v>3.11</v>
+        <v>6.13</v>
       </c>
       <c r="P115" s="122">
         <v>1.0</v>
@@ -19578,11 +19587,11 @@
     </row>
     <row r="116">
       <c r="C116" s="135" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D116" s="124">
         <f t="shared" si="17"/>
-        <v>12.9</v>
+        <v>6.44</v>
       </c>
       <c r="P116" s="122">
         <v>1.0</v>
@@ -19596,11 +19605,11 @@
     </row>
     <row r="117">
       <c r="C117" s="135" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D117" s="124">
         <f t="shared" si="17"/>
-        <v>0.77</v>
+        <v>4.99</v>
       </c>
       <c r="P117" s="142"/>
       <c r="AE117" s="43">
@@ -19612,11 +19621,11 @@
     </row>
     <row r="118">
       <c r="C118" s="135" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="D118" s="124">
         <f t="shared" si="17"/>
-        <v>8.33</v>
+        <v>4.52</v>
       </c>
       <c r="P118" s="142"/>
       <c r="AE118" s="43">
@@ -19628,11 +19637,11 @@
     </row>
     <row r="119">
       <c r="C119" s="135" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="D119" s="124">
         <f t="shared" si="17"/>
-        <v>13.99</v>
+        <v>8.48</v>
       </c>
       <c r="P119" s="142"/>
       <c r="AE119" s="43">
@@ -19644,11 +19653,11 @@
     </row>
     <row r="120">
       <c r="C120" s="135" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="D120" s="124">
         <f t="shared" si="17"/>
-        <v>1.03</v>
+        <v>6.39</v>
       </c>
       <c r="P120" s="142"/>
       <c r="AE120" s="43">
@@ -19660,11 +19669,11 @@
     </row>
     <row r="121">
       <c r="C121" s="135" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="D121" s="124">
         <f t="shared" si="17"/>
-        <v>13.48</v>
+        <v>9.74</v>
       </c>
       <c r="P121" s="142"/>
       <c r="AE121" s="43">
@@ -19676,11 +19685,11 @@
     </row>
     <row r="122">
       <c r="C122" s="135" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D122" s="124">
         <f t="shared" si="17"/>
-        <v>13.88</v>
+        <v>7.7</v>
       </c>
       <c r="P122" s="142"/>
       <c r="AE122" s="43">
@@ -19692,11 +19701,11 @@
     </row>
     <row r="123">
       <c r="C123" s="135" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="D123" s="124">
         <f t="shared" si="17"/>
-        <v>8.68</v>
+        <v>0.8</v>
       </c>
       <c r="P123" s="142"/>
       <c r="AE123" s="43">
@@ -19708,11 +19717,11 @@
     </row>
     <row r="124">
       <c r="C124" s="135" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D124" s="124">
         <f t="shared" si="17"/>
-        <v>12.29</v>
+        <v>9.57</v>
       </c>
       <c r="P124" s="142"/>
       <c r="AE124" s="43">
@@ -19724,11 +19733,11 @@
     </row>
     <row r="125">
       <c r="C125" s="135" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D125" s="124">
         <f t="shared" si="17"/>
-        <v>5.54</v>
+        <v>0.71</v>
       </c>
       <c r="P125" s="142"/>
       <c r="AE125" s="43">
@@ -19740,11 +19749,11 @@
     </row>
     <row r="126">
       <c r="C126" s="135" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D126" s="124">
         <f t="shared" si="17"/>
-        <v>8.36</v>
+        <v>4.34</v>
       </c>
       <c r="P126" s="142"/>
       <c r="AE126" s="43">
@@ -19756,11 +19765,11 @@
     </row>
     <row r="127">
       <c r="C127" s="135" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D127" s="124">
         <f t="shared" si="17"/>
-        <v>13.42</v>
+        <v>8.09</v>
       </c>
       <c r="P127" s="142"/>
       <c r="AE127" s="43">
@@ -19772,11 +19781,11 @@
     </row>
     <row r="128">
       <c r="C128" s="135" t="s">
-        <v>256</v>
+        <v>308</v>
       </c>
       <c r="D128" s="124">
         <f t="shared" si="17"/>
-        <v>10.5</v>
+        <v>6.41</v>
       </c>
       <c r="P128" s="142"/>
       <c r="AE128" s="43">
@@ -19788,11 +19797,11 @@
     </row>
     <row r="129">
       <c r="C129" s="135" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="D129" s="124">
         <f t="shared" si="17"/>
-        <v>10.2</v>
+        <v>8.83</v>
       </c>
       <c r="P129" s="142"/>
       <c r="AE129" s="43">
@@ -19804,11 +19813,11 @@
     </row>
     <row r="130">
       <c r="C130" s="135" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="D130" s="124">
         <f t="shared" si="17"/>
-        <v>4.56</v>
+        <v>4.75</v>
       </c>
       <c r="P130" s="142"/>
       <c r="AE130" s="43">
@@ -19820,11 +19829,11 @@
     </row>
     <row r="131">
       <c r="C131" s="135" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="D131" s="124">
         <f t="shared" si="17"/>
-        <v>11.7</v>
+        <v>5.68</v>
       </c>
       <c r="P131" s="142"/>
       <c r="AE131" s="43">
@@ -19836,11 +19845,11 @@
     </row>
     <row r="132">
       <c r="C132" s="135" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D132" s="124">
         <f t="shared" si="17"/>
-        <v>14.03</v>
+        <v>9.04</v>
       </c>
       <c r="P132" s="142"/>
       <c r="AE132" s="43">
@@ -19852,11 +19861,11 @@
     </row>
     <row r="133">
       <c r="C133" s="135" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="D133" s="124">
         <f t="shared" si="17"/>
-        <v>8.15</v>
+        <v>6.89</v>
       </c>
       <c r="P133" s="142"/>
       <c r="AE133" s="43">
@@ -19868,11 +19877,11 @@
     </row>
     <row r="134">
       <c r="C134" s="135" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D134" s="124">
         <f t="shared" si="17"/>
-        <v>8.46</v>
+        <v>4.98</v>
       </c>
       <c r="P134" s="142"/>
       <c r="AE134" s="43">
@@ -19884,11 +19893,11 @@
     </row>
     <row r="135">
       <c r="C135" s="135" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="D135" s="124">
         <f t="shared" si="17"/>
-        <v>5.83</v>
+        <v>7.92</v>
       </c>
       <c r="P135" s="142"/>
       <c r="AE135" s="43">
@@ -42182,14 +42191,14 @@
     <row r="1">
       <c r="A1" s="105"/>
       <c r="B1" s="145" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="C1" s="146"/>
       <c r="D1" s="146"/>
       <c r="E1" s="146"/>
       <c r="F1" s="146"/>
       <c r="G1" s="147" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="H1" s="146"/>
       <c r="I1" s="146"/>
@@ -42217,19 +42226,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="149" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="C2" s="150" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D2" s="150" t="s">
         <v>207</v>
       </c>
       <c r="E2" s="150" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="F2" s="151" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="G2" s="149">
         <v>1.0</v>
@@ -42241,25 +42250,25 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="150" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="K2" s="152" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="L2" s="150" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="M2" s="153" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="N2" s="101" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="O2" s="101" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="P2" s="101" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
@@ -43042,7 +43051,7 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="166" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -43103,7 +43112,7 @@
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="5" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="E29" s="5">
         <f>J29</f>
@@ -43125,10 +43134,10 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="95" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="M29" s="95" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="O29" s="5">
         <v>1.0</v>
@@ -43264,7 +43273,7 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="120" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
@@ -43441,7 +43450,7 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="5" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="G38" s="169">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
Cambie modelos de GER e ITA
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -276,7 +276,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="502" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="253">
   <si>
     <t>id_country</t>
   </si>
@@ -1020,148 +1020,40 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>3.15</t>
-  </si>
-  <si>
-    <t>8.59</t>
-  </si>
-  <si>
-    <t>7.45</t>
-  </si>
-  <si>
-    <t>7.35</t>
-  </si>
-  <si>
-    <t>5.71</t>
-  </si>
-  <si>
-    <t>11.26</t>
-  </si>
-  <si>
-    <t>6.84</t>
-  </si>
-  <si>
     <t>Country</t>
   </si>
   <si>
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>3.43</t>
-  </si>
-  <si>
     <t>mean</t>
-  </si>
-  <si>
-    <t>12.98</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>15.04</t>
-  </si>
-  <si>
     <t>p25</t>
-  </si>
-  <si>
-    <t>11.46</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>10.03</t>
-  </si>
-  <si>
-    <t>8.27</t>
-  </si>
-  <si>
-    <t>11.13</t>
-  </si>
-  <si>
-    <t>1.79</t>
-  </si>
-  <si>
-    <t>11.00</t>
-  </si>
-  <si>
-    <t>1.63</t>
-  </si>
-  <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
-  </si>
-  <si>
-    <t>2.84</t>
   </si>
   <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>2.19</t>
-  </si>
-  <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
-  </si>
-  <si>
-    <t>2.21</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>1.68</t>
-  </si>
-  <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
-    <t>0.84</t>
-  </si>
-  <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
-  </si>
-  <si>
-    <t>2.52</t>
-  </si>
-  <si>
-    <t>2.94</t>
-  </si>
-  <si>
-    <t>7.41</t>
-  </si>
-  <si>
-    <t>2.96</t>
-  </si>
-  <si>
-    <t>12.46</t>
-  </si>
-  <si>
-    <t>11.32</t>
-  </si>
-  <si>
-    <t>7.79</t>
-  </si>
-  <si>
-    <t>10.77</t>
-  </si>
-  <si>
-    <t>1.24</t>
-  </si>
-  <si>
-    <t>10.52</t>
-  </si>
-  <si>
-    <t>2.83</t>
-  </si>
-  <si>
-    <t>4.72</t>
-  </si>
-  <si>
-    <t>3.53</t>
-  </si>
-  <si>
-    <t>6.63</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2563,7 +2455,7 @@
         <v>45693.0</v>
       </c>
       <c r="D6" s="15">
-        <v>30.0</v>
+        <v>812.0</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>16</v>
@@ -2613,7 +2505,7 @@
         <v>45693.0</v>
       </c>
       <c r="D7" s="15">
-        <v>1271.0</v>
+        <v>1023.0</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>16</v>
@@ -17765,9 +17657,9 @@
       <c r="A37" s="41"/>
       <c r="B37" s="41"/>
       <c r="C37" s="41"/>
-      <c r="D37" s="133">
+      <c r="D37" s="133" t="str">
         <f>AVERAGE(D39:D1775)</f>
-        <v>6.51525</v>
+        <v>#DIV/0!</v>
       </c>
       <c r="G37" s="36" t="s">
         <v>39</v>
@@ -17831,12 +17723,10 @@
       </c>
     </row>
     <row r="39">
-      <c r="C39" s="135" t="s">
-        <v>212</v>
-      </c>
-      <c r="D39" s="125">
+      <c r="C39" s="135"/>
+      <c r="D39" s="125" t="str">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>3.15</v>
+        <v/>
       </c>
       <c r="G39" s="36" t="s">
         <v>31</v>
@@ -17869,12 +17759,10 @@
       </c>
     </row>
     <row r="40">
-      <c r="C40" s="136" t="s">
-        <v>213</v>
-      </c>
-      <c r="D40" s="125">
+      <c r="C40" s="136"/>
+      <c r="D40" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>8.59</v>
+        <v/>
       </c>
       <c r="G40" s="36" t="s">
         <v>27</v>
@@ -17907,12 +17795,10 @@
       </c>
     </row>
     <row r="41">
-      <c r="C41" s="136" t="s">
-        <v>214</v>
-      </c>
-      <c r="D41" s="125">
+      <c r="C41" s="136"/>
+      <c r="D41" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>7.45</v>
+        <v/>
       </c>
       <c r="P41" s="123">
         <v>0.0</v>
@@ -17939,12 +17825,10 @@
       </c>
     </row>
     <row r="42">
-      <c r="C42" s="136" t="s">
-        <v>215</v>
-      </c>
-      <c r="D42" s="125">
+      <c r="C42" s="136"/>
+      <c r="D42" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>7.35</v>
+        <v/>
       </c>
       <c r="P42" s="123">
         <v>2.0</v>
@@ -17971,12 +17855,10 @@
       </c>
     </row>
     <row r="43">
-      <c r="C43" s="136" t="s">
-        <v>216</v>
-      </c>
-      <c r="D43" s="125">
+      <c r="C43" s="136"/>
+      <c r="D43" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>5.71</v>
+        <v/>
       </c>
       <c r="P43" s="123">
         <v>1.0</v>
@@ -18003,12 +17885,10 @@
       </c>
     </row>
     <row r="44">
-      <c r="C44" s="136" t="s">
-        <v>217</v>
-      </c>
-      <c r="D44" s="125">
+      <c r="C44" s="136"/>
+      <c r="D44" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>11.26</v>
+        <v/>
       </c>
       <c r="P44" s="123">
         <v>2.0</v>
@@ -18033,12 +17913,10 @@
       </c>
     </row>
     <row r="45">
-      <c r="C45" s="136" t="s">
-        <v>218</v>
-      </c>
-      <c r="D45" s="125">
+      <c r="C45" s="136"/>
+      <c r="D45" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>6.84</v>
+        <v/>
       </c>
       <c r="P45" s="123">
         <v>1.0</v>
@@ -18051,18 +17929,16 @@
       </c>
     </row>
     <row r="46">
-      <c r="C46" s="136" t="s">
-        <v>218</v>
-      </c>
-      <c r="D46" s="125">
+      <c r="C46" s="136"/>
+      <c r="D46" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>6.84</v>
+        <v/>
       </c>
       <c r="G46" s="97" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="H46" s="97" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="P46" s="123">
         <v>0.0</v>
@@ -18075,12 +17951,10 @@
       </c>
     </row>
     <row r="47">
-      <c r="C47" s="136" t="s">
-        <v>215</v>
-      </c>
-      <c r="D47" s="125">
+      <c r="C47" s="136"/>
+      <c r="D47" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>7.35</v>
+        <v/>
       </c>
       <c r="G47" s="102" t="s">
         <v>40</v>
@@ -18105,12 +17979,10 @@
       </c>
     </row>
     <row r="48">
-      <c r="C48" s="136" t="s">
-        <v>221</v>
-      </c>
-      <c r="D48" s="125">
+      <c r="C48" s="136"/>
+      <c r="D48" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>3.43</v>
+        <v/>
       </c>
       <c r="G48" s="102" t="s">
         <v>39</v>
@@ -18119,7 +17991,7 @@
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="43" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="K48" s="89">
         <f>AVERAGE(H47:H51)</f>
@@ -18142,12 +18014,10 @@
       </c>
     </row>
     <row r="49">
-      <c r="C49" s="136" t="s">
-        <v>223</v>
-      </c>
-      <c r="D49" s="125">
+      <c r="C49" s="136"/>
+      <c r="D49" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>12.98</v>
+        <v/>
       </c>
       <c r="G49" s="102" t="s">
         <v>30</v>
@@ -18156,7 +18026,7 @@
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="43" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="K49" s="89">
         <f>MEDIAN(H47:H51)</f>
@@ -18179,12 +18049,10 @@
       </c>
     </row>
     <row r="50">
-      <c r="C50" s="136" t="s">
-        <v>225</v>
-      </c>
-      <c r="D50" s="125">
+      <c r="C50" s="136"/>
+      <c r="D50" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>15.04</v>
+        <v/>
       </c>
       <c r="G50" s="102" t="s">
         <v>31</v>
@@ -18193,7 +18061,7 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="43" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="K50" s="89">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -18216,12 +18084,10 @@
       </c>
     </row>
     <row r="51">
-      <c r="C51" s="136" t="s">
-        <v>227</v>
-      </c>
-      <c r="D51" s="125">
+      <c r="C51" s="136"/>
+      <c r="D51" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>11.46</v>
+        <v/>
       </c>
       <c r="G51" s="102" t="s">
         <v>27</v>
@@ -18230,7 +18096,7 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="43" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="K51" s="89">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -18253,12 +18119,10 @@
       </c>
     </row>
     <row r="52">
-      <c r="C52" s="136" t="s">
-        <v>229</v>
-      </c>
-      <c r="D52" s="125">
+      <c r="C52" s="136"/>
+      <c r="D52" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>10.03</v>
+        <v/>
       </c>
       <c r="P52" s="123">
         <v>0.0</v>
@@ -18277,12 +18141,10 @@
       </c>
     </row>
     <row r="53">
-      <c r="C53" s="136" t="s">
-        <v>230</v>
-      </c>
-      <c r="D53" s="125">
+      <c r="C53" s="136"/>
+      <c r="D53" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>8.27</v>
+        <v/>
       </c>
       <c r="P53" s="123">
         <v>0.0</v>
@@ -18301,12 +18163,10 @@
       </c>
     </row>
     <row r="54">
-      <c r="C54" s="136" t="s">
-        <v>230</v>
-      </c>
-      <c r="D54" s="125">
+      <c r="C54" s="136"/>
+      <c r="D54" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>8.27</v>
+        <v/>
       </c>
       <c r="P54" s="123">
         <v>2.0</v>
@@ -18325,12 +18185,10 @@
       </c>
     </row>
     <row r="55">
-      <c r="C55" s="136" t="s">
-        <v>231</v>
-      </c>
-      <c r="D55" s="125">
+      <c r="C55" s="136"/>
+      <c r="D55" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>11.13</v>
+        <v/>
       </c>
       <c r="P55" s="123">
         <v>0.0</v>
@@ -18349,12 +18207,10 @@
       </c>
     </row>
     <row r="56">
-      <c r="C56" s="136" t="s">
-        <v>232</v>
-      </c>
-      <c r="D56" s="125">
+      <c r="C56" s="136"/>
+      <c r="D56" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>1.79</v>
+        <v/>
       </c>
       <c r="P56" s="123">
         <v>0.0</v>
@@ -18373,12 +18229,10 @@
       </c>
     </row>
     <row r="57">
-      <c r="C57" s="136" t="s">
-        <v>233</v>
-      </c>
-      <c r="D57" s="125">
+      <c r="C57" s="136"/>
+      <c r="D57" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>11</v>
+        <v/>
       </c>
       <c r="P57" s="123">
         <v>2.0</v>
@@ -18397,15 +18251,13 @@
       </c>
     </row>
     <row r="58">
-      <c r="C58" s="136" t="s">
-        <v>234</v>
-      </c>
-      <c r="D58" s="125">
+      <c r="C58" s="136"/>
+      <c r="D58" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>1.63</v>
+        <v/>
       </c>
       <c r="G58" s="138" t="s">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="H58" s="139"/>
       <c r="P58" s="123">
@@ -18425,16 +18277,14 @@
       </c>
     </row>
     <row r="59">
-      <c r="C59" s="136" t="s">
-        <v>236</v>
-      </c>
-      <c r="D59" s="125">
+      <c r="C59" s="136"/>
+      <c r="D59" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.84</v>
+        <v/>
       </c>
       <c r="G59" s="139"/>
       <c r="H59" s="140" t="s">
-        <v>237</v>
+        <v>219</v>
       </c>
       <c r="P59" s="123">
         <v>0.0</v>
@@ -18453,16 +18303,14 @@
       </c>
     </row>
     <row r="60">
-      <c r="C60" s="136" t="s">
-        <v>238</v>
-      </c>
-      <c r="D60" s="125">
+      <c r="C60" s="136"/>
+      <c r="D60" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.19</v>
+        <v/>
       </c>
       <c r="G60" s="139"/>
       <c r="H60" s="140" t="s">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="P60" s="123">
         <v>2.0</v>
@@ -18481,16 +18329,14 @@
       </c>
     </row>
     <row r="61">
-      <c r="C61" s="136" t="s">
-        <v>240</v>
-      </c>
-      <c r="D61" s="125">
+      <c r="C61" s="136"/>
+      <c r="D61" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.21</v>
+        <v/>
       </c>
       <c r="G61" s="139"/>
       <c r="H61" s="140" t="s">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="P61" s="123">
         <v>2.0</v>
@@ -18509,16 +18355,14 @@
       </c>
     </row>
     <row r="62">
-      <c r="C62" s="136" t="s">
-        <v>242</v>
-      </c>
-      <c r="D62" s="125">
+      <c r="C62" s="136"/>
+      <c r="D62" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>1.68</v>
+        <v/>
       </c>
       <c r="G62" s="139"/>
       <c r="H62" s="140" t="s">
-        <v>243</v>
+        <v>222</v>
       </c>
       <c r="P62" s="123">
         <v>1.0</v>
@@ -18537,16 +18381,14 @@
       </c>
     </row>
     <row r="63">
-      <c r="C63" s="136" t="s">
-        <v>244</v>
-      </c>
-      <c r="D63" s="125">
+      <c r="C63" s="136"/>
+      <c r="D63" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>0.84</v>
+        <v/>
       </c>
       <c r="G63" s="139"/>
       <c r="H63" s="140" t="s">
-        <v>245</v>
+        <v>223</v>
       </c>
       <c r="P63" s="123">
         <v>0.0</v>
@@ -18559,12 +18401,10 @@
       </c>
     </row>
     <row r="64">
-      <c r="C64" s="136" t="s">
-        <v>246</v>
-      </c>
-      <c r="D64" s="125">
+      <c r="C64" s="136"/>
+      <c r="D64" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.52</v>
+        <v/>
       </c>
       <c r="P64" s="123">
         <v>1.0</v>
@@ -18577,12 +18417,10 @@
       </c>
     </row>
     <row r="65">
-      <c r="C65" s="136" t="s">
-        <v>247</v>
-      </c>
-      <c r="D65" s="125">
+      <c r="C65" s="136"/>
+      <c r="D65" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.94</v>
+        <v/>
       </c>
       <c r="P65" s="123">
         <v>2.0</v>
@@ -18595,12 +18433,10 @@
       </c>
     </row>
     <row r="66">
-      <c r="C66" s="136" t="s">
-        <v>248</v>
-      </c>
-      <c r="D66" s="125">
+      <c r="C66" s="136"/>
+      <c r="D66" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>7.41</v>
+        <v/>
       </c>
       <c r="P66" s="123">
         <v>0.0</v>
@@ -18613,12 +18449,10 @@
       </c>
     </row>
     <row r="67">
-      <c r="C67" s="136" t="s">
-        <v>249</v>
-      </c>
-      <c r="D67" s="125">
+      <c r="C67" s="136"/>
+      <c r="D67" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.96</v>
+        <v/>
       </c>
       <c r="P67" s="123">
         <v>0.0</v>
@@ -18631,12 +18465,10 @@
       </c>
     </row>
     <row r="68">
-      <c r="C68" s="136" t="s">
-        <v>250</v>
-      </c>
-      <c r="D68" s="125">
+      <c r="C68" s="136"/>
+      <c r="D68" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>12.46</v>
+        <v/>
       </c>
       <c r="P68" s="123">
         <v>1.0</v>
@@ -18649,12 +18481,10 @@
       </c>
     </row>
     <row r="69">
-      <c r="C69" s="136" t="s">
-        <v>251</v>
-      </c>
-      <c r="D69" s="125">
+      <c r="C69" s="136"/>
+      <c r="D69" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>11.32</v>
+        <v/>
       </c>
       <c r="P69" s="123">
         <v>2.0</v>
@@ -18667,12 +18497,10 @@
       </c>
     </row>
     <row r="70">
-      <c r="C70" s="136" t="s">
-        <v>252</v>
-      </c>
-      <c r="D70" s="125">
+      <c r="C70" s="136"/>
+      <c r="D70" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>7.79</v>
+        <v/>
       </c>
       <c r="P70" s="123">
         <v>1.0</v>
@@ -18685,12 +18513,10 @@
       </c>
     </row>
     <row r="71">
-      <c r="C71" s="136" t="s">
-        <v>253</v>
-      </c>
-      <c r="D71" s="125">
+      <c r="C71" s="136"/>
+      <c r="D71" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>10.77</v>
+        <v/>
       </c>
       <c r="F71" s="141"/>
       <c r="P71" s="123">
@@ -18704,12 +18530,10 @@
       </c>
     </row>
     <row r="72">
-      <c r="C72" s="136" t="s">
-        <v>254</v>
-      </c>
-      <c r="D72" s="125">
+      <c r="C72" s="136"/>
+      <c r="D72" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>1.24</v>
+        <v/>
       </c>
       <c r="P72" s="123">
         <v>0.0</v>
@@ -18722,12 +18546,10 @@
       </c>
     </row>
     <row r="73">
-      <c r="C73" s="136" t="s">
-        <v>255</v>
-      </c>
-      <c r="D73" s="125">
+      <c r="C73" s="136"/>
+      <c r="D73" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>10.52</v>
+        <v/>
       </c>
       <c r="P73" s="123">
         <v>1.0</v>
@@ -18740,12 +18562,10 @@
       </c>
     </row>
     <row r="74">
-      <c r="C74" s="136" t="s">
-        <v>256</v>
-      </c>
-      <c r="D74" s="125">
+      <c r="C74" s="136"/>
+      <c r="D74" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>2.83</v>
+        <v/>
       </c>
       <c r="P74" s="123">
         <v>0.0</v>
@@ -18758,12 +18578,10 @@
       </c>
     </row>
     <row r="75">
-      <c r="C75" s="136" t="s">
-        <v>257</v>
-      </c>
-      <c r="D75" s="125">
+      <c r="C75" s="136"/>
+      <c r="D75" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>4.72</v>
+        <v/>
       </c>
       <c r="P75" s="123">
         <v>1.0</v>
@@ -18776,12 +18594,10 @@
       </c>
     </row>
     <row r="76">
-      <c r="C76" s="136" t="s">
-        <v>258</v>
-      </c>
-      <c r="D76" s="125">
+      <c r="C76" s="136"/>
+      <c r="D76" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>3.53</v>
+        <v/>
       </c>
       <c r="P76" s="123">
         <v>0.0</v>
@@ -18794,12 +18610,10 @@
       </c>
     </row>
     <row r="77">
-      <c r="C77" s="136" t="s">
-        <v>188</v>
-      </c>
-      <c r="D77" s="125">
+      <c r="C77" s="136"/>
+      <c r="D77" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>3.64</v>
+        <v/>
       </c>
       <c r="P77" s="123">
         <v>0.0</v>
@@ -18812,12 +18626,10 @@
       </c>
     </row>
     <row r="78">
-      <c r="C78" s="136" t="s">
-        <v>259</v>
-      </c>
-      <c r="D78" s="125">
+      <c r="C78" s="136"/>
+      <c r="D78" s="125" t="str">
         <f t="shared" si="17"/>
-        <v>6.63</v>
+        <v/>
       </c>
       <c r="P78" s="123">
         <v>1.0</v>
@@ -41995,14 +41807,14 @@
     <row r="1">
       <c r="A1" s="106"/>
       <c r="B1" s="146" t="s">
-        <v>260</v>
+        <v>224</v>
       </c>
       <c r="C1" s="147"/>
       <c r="D1" s="147"/>
       <c r="E1" s="147"/>
       <c r="F1" s="147"/>
       <c r="G1" s="148" t="s">
-        <v>261</v>
+        <v>225</v>
       </c>
       <c r="H1" s="147"/>
       <c r="I1" s="147"/>
@@ -42034,19 +41846,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="150" t="s">
-        <v>262</v>
+        <v>226</v>
       </c>
       <c r="C2" s="151" t="s">
-        <v>263</v>
+        <v>227</v>
       </c>
       <c r="D2" s="151" t="s">
         <v>208</v>
       </c>
       <c r="E2" s="151" t="s">
-        <v>264</v>
+        <v>228</v>
       </c>
       <c r="F2" s="152" t="s">
-        <v>265</v>
+        <v>229</v>
       </c>
       <c r="G2" s="150">
         <v>1.0</v>
@@ -42058,30 +41870,30 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="151" t="s">
-        <v>266</v>
+        <v>230</v>
       </c>
       <c r="K2" s="153" t="s">
-        <v>267</v>
+        <v>231</v>
       </c>
       <c r="L2" s="151" t="s">
-        <v>268</v>
+        <v>232</v>
       </c>
       <c r="M2" s="154" t="s">
-        <v>269</v>
+        <v>233</v>
       </c>
       <c r="N2" s="102" t="s">
-        <v>270</v>
+        <v>234</v>
       </c>
       <c r="O2" s="102" t="s">
-        <v>271</v>
+        <v>235</v>
       </c>
       <c r="P2" s="102" t="s">
-        <v>272</v>
+        <v>236</v>
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
       <c r="S2" s="96" t="s">
-        <v>273</v>
+        <v>237</v>
       </c>
       <c r="T2" s="9"/>
       <c r="U2" s="9"/>
@@ -42167,7 +41979,7 @@
       <c r="Q4" s="9"/>
       <c r="R4" s="9"/>
       <c r="S4" s="160" t="s">
-        <v>274</v>
+        <v>238</v>
       </c>
       <c r="T4" s="161"/>
       <c r="Z4" s="36"/>
@@ -42203,7 +42015,7 @@
       <c r="P5" s="163"/>
       <c r="S5" s="161"/>
       <c r="T5" s="164" t="s">
-        <v>275</v>
+        <v>239</v>
       </c>
     </row>
     <row r="6">
@@ -42236,11 +42048,11 @@
       <c r="R6" s="9"/>
       <c r="S6" s="161"/>
       <c r="T6" s="164" t="s">
-        <v>276</v>
+        <v>240</v>
       </c>
       <c r="Z6" s="32"/>
       <c r="AD6" s="43" t="s">
-        <v>277</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7">
@@ -42270,7 +42082,7 @@
       <c r="O7" s="80"/>
       <c r="P7" s="165"/>
       <c r="AD7" s="164" t="s">
-        <v>278</v>
+        <v>242</v>
       </c>
       <c r="AE7" s="161"/>
     </row>
@@ -42301,11 +42113,11 @@
       <c r="O8" s="80"/>
       <c r="P8" s="165"/>
       <c r="S8" s="164" t="s">
-        <v>279</v>
+        <v>243</v>
       </c>
       <c r="AA8" s="32"/>
       <c r="AD8" s="164" t="s">
-        <v>280</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9">
@@ -42504,7 +42316,7 @@
       <c r="O15" s="80"/>
       <c r="P15" s="165"/>
       <c r="S15" s="43" t="s">
-        <v>281</v>
+        <v>245</v>
       </c>
     </row>
     <row r="16">
@@ -42617,7 +42429,7 @@
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
       <c r="S19" s="43" t="s">
-        <v>282</v>
+        <v>246</v>
       </c>
     </row>
     <row r="20">
@@ -42873,7 +42685,7 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="170" t="s">
-        <v>283</v>
+        <v>247</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -42942,7 +42754,7 @@
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="5" t="s">
-        <v>284</v>
+        <v>248</v>
       </c>
       <c r="E29" s="5">
         <f>J29</f>
@@ -42964,10 +42776,10 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="96" t="s">
-        <v>285</v>
+        <v>249</v>
       </c>
       <c r="M29" s="96" t="s">
-        <v>286</v>
+        <v>250</v>
       </c>
       <c r="O29" s="5">
         <v>1.0</v>
@@ -43119,7 +42931,7 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="121" t="s">
-        <v>287</v>
+        <v>251</v>
       </c>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
@@ -43316,7 +43128,7 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="5" t="s">
-        <v>288</v>
+        <v>252</v>
       </c>
       <c r="G38" s="173">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones por missing y cuotas
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -274,7 +274,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="623" uniqueCount="337">
   <si>
     <t>id_country</t>
   </si>
@@ -1111,28 +1111,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>4.84</t>
+    <t>5.98</t>
   </si>
   <si>
-    <t>4.18</t>
+    <t>5.82</t>
   </si>
   <si>
-    <t>4.80</t>
+    <t>4.89</t>
   </si>
   <si>
-    <t>1.64</t>
+    <t>6.59</t>
   </si>
   <si>
-    <t>1.05</t>
+    <t>8.42</t>
   </si>
   <si>
-    <t>7.12</t>
+    <t>5.34</t>
   </si>
   <si>
-    <t>10.03</t>
+    <t>7.38</t>
   </si>
   <si>
-    <t>6.64</t>
+    <t>7.95</t>
   </si>
   <si>
     <t>Country</t>
@@ -1141,151 +1141,148 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>5.40</t>
+    <t>6.06</t>
   </si>
   <si>
-    <t>5.92</t>
+    <t>0.81</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>5.90</t>
+    <t>6.46</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>10.26</t>
+    <t>10.16</t>
   </si>
   <si>
     <t>p25</t>
   </si>
   <si>
-    <t>5.99</t>
+    <t>5.08</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>9.16</t>
+    <t>6.77</t>
   </si>
   <si>
-    <t>4.86</t>
+    <t>1.08</t>
   </si>
   <si>
-    <t>6.89</t>
+    <t>8.41</t>
   </si>
   <si>
-    <t>8.85</t>
+    <t>6.84</t>
   </si>
   <si>
-    <t>8.58</t>
+    <t>5.65</t>
   </si>
   <si>
-    <t>1.18</t>
-  </si>
-  <si>
-    <t>5.60</t>
+    <t>7.16</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
   </si>
   <si>
-    <t>5.04</t>
+    <t>12.24</t>
   </si>
   <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>10.85</t>
+    <t>11.12</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
-    <t>10.58</t>
+    <t>12.96</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>8.46</t>
+    <t>11.90</t>
   </si>
   <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
-    <t>5.03</t>
+    <t>7.74</t>
   </si>
   <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>7.01</t>
+    <t>7.76</t>
   </si>
   <si>
-    <t>5.14</t>
+    <t>0.73</t>
   </si>
   <si>
-    <t>5.77</t>
+    <t>7.55</t>
   </si>
   <si>
-    <t>3.45</t>
+    <t>2.64</t>
   </si>
   <si>
-    <t>6.06</t>
+    <t>1.99</t>
   </si>
   <si>
-    <t>4.64</t>
+    <t>1.67</t>
   </si>
   <si>
-    <t>4.97</t>
+    <t>2.61</t>
   </si>
   <si>
-    <t>7.00</t>
+    <t>0.18</t>
   </si>
   <si>
-    <t>5.88</t>
+    <t>3.46</t>
   </si>
   <si>
-    <t>7.17</t>
+    <t>3.84</t>
   </si>
   <si>
-    <t>5.09</t>
+    <t>2.89</t>
   </si>
   <si>
-    <t>2.60</t>
+    <t>2.34</t>
   </si>
   <si>
-    <t>3.13</t>
+    <t>1.36</t>
   </si>
   <si>
-    <t>6.29</t>
+    <t>4.88</t>
   </si>
   <si>
-    <t>6.34</t>
+    <t>2.42</t>
   </si>
   <si>
-    <t>4.99</t>
+    <t>0.53</t>
   </si>
   <si>
-    <t>10.60</t>
+    <t>7.18</t>
   </si>
   <si>
-    <t>12.21</t>
+    <t>6.82</t>
   </si>
   <si>
-    <t>0.67</t>
+    <t>3.14</t>
   </si>
   <si>
-    <t>7.92</t>
+    <t>0.43</t>
   </si>
   <si>
-    <t>6.02</t>
+    <t>4.34</t>
   </si>
   <si>
-    <t>7.88</t>
+    <t>5.16</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2795,7 +2792,7 @@
         <v>45720.0</v>
       </c>
       <c r="D7" s="15">
-        <v>2516.0</v>
+        <v>2114.0</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>16</v>
@@ -2804,7 +2801,7 @@
         <v>0.707906165804836</v>
       </c>
       <c r="G7" s="17">
-        <v>20.0</v>
+        <v>40.0</v>
       </c>
       <c r="H7" s="18"/>
       <c r="I7" s="18"/>
@@ -2812,7 +2809,7 @@
       <c r="K7" s="20"/>
       <c r="L7" s="26">
         <f>G7*'Data preparation'!$C$2</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="M7" s="17">
         <v>2.431963389625</v>
@@ -17749,7 +17746,7 @@
       </c>
       <c r="C3" s="25">
         <f>AVERAGE('Modelos actuales'!L4:L8)</f>
-        <v>9</v>
+        <v>9.6</v>
       </c>
       <c r="L3" s="123"/>
       <c r="P3" s="123"/>
@@ -19050,7 +19047,7 @@
       <c r="C37" s="43"/>
       <c r="D37" s="137">
         <f>AVERAGE(D39:D1775)</f>
-        <v>6.178541667</v>
+        <v>5.356041667</v>
       </c>
       <c r="G37" s="36" t="s">
         <v>71</v>
@@ -19119,7 +19116,7 @@
       </c>
       <c r="D39" s="129">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>4.84</v>
+        <v>5.98</v>
       </c>
       <c r="G39" s="36" t="s">
         <v>63</v>
@@ -19157,7 +19154,7 @@
       </c>
       <c r="D40" s="129">
         <f t="shared" si="17"/>
-        <v>4.18</v>
+        <v>5.82</v>
       </c>
       <c r="G40" s="36" t="s">
         <v>59</v>
@@ -19195,7 +19192,7 @@
       </c>
       <c r="D41" s="129">
         <f t="shared" si="17"/>
-        <v>4.8</v>
+        <v>4.89</v>
       </c>
       <c r="P41" s="127">
         <v>0.0</v>
@@ -19227,7 +19224,7 @@
       </c>
       <c r="D42" s="129">
         <f t="shared" si="17"/>
-        <v>1.64</v>
+        <v>6.59</v>
       </c>
       <c r="P42" s="127">
         <v>2.0</v>
@@ -19259,7 +19256,7 @@
       </c>
       <c r="D43" s="129">
         <f t="shared" si="17"/>
-        <v>1.05</v>
+        <v>8.42</v>
       </c>
       <c r="P43" s="127">
         <v>1.0</v>
@@ -19291,7 +19288,7 @@
       </c>
       <c r="D44" s="129">
         <f t="shared" si="17"/>
-        <v>7.12</v>
+        <v>5.34</v>
       </c>
       <c r="P44" s="127">
         <v>2.0</v>
@@ -19321,7 +19318,7 @@
       </c>
       <c r="D45" s="129">
         <f t="shared" si="17"/>
-        <v>10.03</v>
+        <v>7.38</v>
       </c>
       <c r="P45" s="127">
         <v>1.0</v>
@@ -19339,7 +19336,7 @@
       </c>
       <c r="D46" s="129">
         <f t="shared" si="17"/>
-        <v>6.64</v>
+        <v>7.95</v>
       </c>
       <c r="G46" s="101" t="s">
         <v>251</v>
@@ -19363,7 +19360,7 @@
       </c>
       <c r="D47" s="129">
         <f t="shared" si="17"/>
-        <v>5.4</v>
+        <v>6.06</v>
       </c>
       <c r="G47" s="106" t="s">
         <v>72</v>
@@ -19393,7 +19390,7 @@
       </c>
       <c r="D48" s="129">
         <f t="shared" si="17"/>
-        <v>5.92</v>
+        <v>0.81</v>
       </c>
       <c r="G48" s="106" t="s">
         <v>71</v>
@@ -19430,7 +19427,7 @@
       </c>
       <c r="D49" s="129">
         <f t="shared" si="17"/>
-        <v>5.9</v>
+        <v>6.46</v>
       </c>
       <c r="G49" s="106" t="s">
         <v>62</v>
@@ -19467,7 +19464,7 @@
       </c>
       <c r="D50" s="129">
         <f t="shared" si="17"/>
-        <v>10.26</v>
+        <v>10.16</v>
       </c>
       <c r="G50" s="106" t="s">
         <v>63</v>
@@ -19504,7 +19501,7 @@
       </c>
       <c r="D51" s="129">
         <f t="shared" si="17"/>
-        <v>5.99</v>
+        <v>5.08</v>
       </c>
       <c r="G51" s="106" t="s">
         <v>59</v>
@@ -19541,7 +19538,7 @@
       </c>
       <c r="D52" s="129">
         <f t="shared" si="17"/>
-        <v>9.16</v>
+        <v>6.77</v>
       </c>
       <c r="P52" s="127">
         <v>0.0</v>
@@ -19561,11 +19558,11 @@
     </row>
     <row r="53">
       <c r="C53" s="140" t="s">
-        <v>263</v>
+        <v>244</v>
       </c>
       <c r="D53" s="129">
         <f t="shared" si="17"/>
-        <v>4.86</v>
+        <v>5.82</v>
       </c>
       <c r="P53" s="127">
         <v>0.0</v>
@@ -19585,11 +19582,11 @@
     </row>
     <row r="54">
       <c r="C54" s="140" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="D54" s="129">
         <f t="shared" si="17"/>
-        <v>6.89</v>
+        <v>1.08</v>
       </c>
       <c r="P54" s="127">
         <v>2.0</v>
@@ -19609,11 +19606,11 @@
     </row>
     <row r="55">
       <c r="C55" s="140" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="D55" s="129">
         <f t="shared" si="17"/>
-        <v>8.85</v>
+        <v>8.41</v>
       </c>
       <c r="P55" s="127">
         <v>0.0</v>
@@ -19633,11 +19630,11 @@
     </row>
     <row r="56">
       <c r="C56" s="140" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="D56" s="129">
         <f t="shared" si="17"/>
-        <v>8.58</v>
+        <v>6.84</v>
       </c>
       <c r="P56" s="127">
         <v>0.0</v>
@@ -19657,11 +19654,11 @@
     </row>
     <row r="57">
       <c r="C57" s="140" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D57" s="129">
         <f t="shared" si="17"/>
-        <v>1.18</v>
+        <v>5.65</v>
       </c>
       <c r="P57" s="127">
         <v>2.0</v>
@@ -19681,14 +19678,14 @@
     </row>
     <row r="58">
       <c r="C58" s="140" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D58" s="129">
         <f t="shared" si="17"/>
-        <v>5.6</v>
+        <v>7.16</v>
       </c>
       <c r="G58" s="142" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H58" s="143"/>
       <c r="P58" s="127">
@@ -19709,15 +19706,15 @@
     </row>
     <row r="59">
       <c r="C59" s="140" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D59" s="129">
         <f t="shared" si="17"/>
-        <v>5.04</v>
+        <v>12.24</v>
       </c>
       <c r="G59" s="143"/>
       <c r="H59" s="144" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="P59" s="127">
         <v>0.0</v>
@@ -19737,15 +19734,15 @@
     </row>
     <row r="60">
       <c r="C60" s="140" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D60" s="129">
         <f t="shared" si="17"/>
-        <v>10.85</v>
+        <v>11.12</v>
       </c>
       <c r="G60" s="143"/>
       <c r="H60" s="144" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="P60" s="127">
         <v>2.0</v>
@@ -19765,15 +19762,15 @@
     </row>
     <row r="61">
       <c r="C61" s="140" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="D61" s="129">
         <f t="shared" si="17"/>
-        <v>10.58</v>
+        <v>12.96</v>
       </c>
       <c r="G61" s="143"/>
       <c r="H61" s="144" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="P61" s="127">
         <v>2.0</v>
@@ -19793,15 +19790,15 @@
     </row>
     <row r="62">
       <c r="C62" s="140" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D62" s="129">
         <f t="shared" si="17"/>
-        <v>8.46</v>
+        <v>11.9</v>
       </c>
       <c r="G62" s="143"/>
       <c r="H62" s="144" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="P62" s="127">
         <v>1.0</v>
@@ -19821,15 +19818,15 @@
     </row>
     <row r="63">
       <c r="C63" s="140" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D63" s="129">
         <f t="shared" si="17"/>
-        <v>5.03</v>
+        <v>7.74</v>
       </c>
       <c r="G63" s="143"/>
       <c r="H63" s="144" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="P63" s="127">
         <v>0.0</v>
@@ -19843,11 +19840,11 @@
     </row>
     <row r="64">
       <c r="C64" s="140" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D64" s="129">
         <f t="shared" si="17"/>
-        <v>7.01</v>
+        <v>7.76</v>
       </c>
       <c r="P64" s="127">
         <v>1.0</v>
@@ -19861,11 +19858,11 @@
     </row>
     <row r="65">
       <c r="C65" s="140" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D65" s="129">
         <f t="shared" si="17"/>
-        <v>5.14</v>
+        <v>0.73</v>
       </c>
       <c r="P65" s="127">
         <v>2.0</v>
@@ -19879,11 +19876,11 @@
     </row>
     <row r="66">
       <c r="C66" s="140" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D66" s="129">
         <f t="shared" si="17"/>
-        <v>5.77</v>
+        <v>7.55</v>
       </c>
       <c r="P66" s="127">
         <v>0.0</v>
@@ -19897,11 +19894,11 @@
     </row>
     <row r="67">
       <c r="C67" s="140" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D67" s="129">
         <f t="shared" si="17"/>
-        <v>3.45</v>
+        <v>2.64</v>
       </c>
       <c r="P67" s="127">
         <v>0.0</v>
@@ -19915,11 +19912,11 @@
     </row>
     <row r="68">
       <c r="C68" s="140" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D68" s="129">
         <f t="shared" si="17"/>
-        <v>6.06</v>
+        <v>1.99</v>
       </c>
       <c r="P68" s="127">
         <v>1.0</v>
@@ -19933,11 +19930,11 @@
     </row>
     <row r="69">
       <c r="C69" s="140" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D69" s="129">
         <f t="shared" si="17"/>
-        <v>4.64</v>
+        <v>1.67</v>
       </c>
       <c r="P69" s="127">
         <v>2.0</v>
@@ -19951,11 +19948,11 @@
     </row>
     <row r="70">
       <c r="C70" s="140" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D70" s="129">
         <f t="shared" si="17"/>
-        <v>4.97</v>
+        <v>2.61</v>
       </c>
       <c r="P70" s="127">
         <v>1.0</v>
@@ -19969,11 +19966,11 @@
     </row>
     <row r="71">
       <c r="C71" s="140" t="s">
-        <v>264</v>
+        <v>286</v>
       </c>
       <c r="D71" s="129">
         <f t="shared" si="17"/>
-        <v>6.89</v>
+        <v>0.18</v>
       </c>
       <c r="F71" s="145"/>
       <c r="P71" s="127">
@@ -19992,7 +19989,7 @@
       </c>
       <c r="D72" s="129">
         <f t="shared" si="17"/>
-        <v>7</v>
+        <v>3.46</v>
       </c>
       <c r="P72" s="127">
         <v>0.0</v>
@@ -20010,7 +20007,7 @@
       </c>
       <c r="D73" s="129">
         <f t="shared" si="17"/>
-        <v>5.88</v>
+        <v>3.84</v>
       </c>
       <c r="P73" s="127">
         <v>1.0</v>
@@ -20028,7 +20025,7 @@
       </c>
       <c r="D74" s="129">
         <f t="shared" si="17"/>
-        <v>7.17</v>
+        <v>2.89</v>
       </c>
       <c r="P74" s="127">
         <v>0.0</v>
@@ -20046,7 +20043,7 @@
       </c>
       <c r="D75" s="129">
         <f t="shared" si="17"/>
-        <v>5.09</v>
+        <v>2.34</v>
       </c>
       <c r="P75" s="127">
         <v>1.0</v>
@@ -20064,7 +20061,7 @@
       </c>
       <c r="D76" s="129">
         <f t="shared" si="17"/>
-        <v>2.6</v>
+        <v>1.36</v>
       </c>
       <c r="P76" s="127">
         <v>0.0</v>
@@ -20078,11 +20075,11 @@
     </row>
     <row r="77">
       <c r="C77" s="140" t="s">
-        <v>292</v>
+        <v>238</v>
       </c>
       <c r="D77" s="129">
         <f t="shared" si="17"/>
-        <v>3.13</v>
+        <v>4.54</v>
       </c>
       <c r="P77" s="127">
         <v>0.0</v>
@@ -20096,11 +20093,11 @@
     </row>
     <row r="78">
       <c r="C78" s="140" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D78" s="129">
         <f t="shared" si="17"/>
-        <v>6.29</v>
+        <v>4.88</v>
       </c>
       <c r="P78" s="127">
         <v>1.0</v>
@@ -20114,11 +20111,11 @@
     </row>
     <row r="79">
       <c r="C79" s="140" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D79" s="129">
         <f t="shared" si="17"/>
-        <v>6.34</v>
+        <v>2.42</v>
       </c>
       <c r="P79" s="127">
         <v>2.0</v>
@@ -20132,11 +20129,11 @@
     </row>
     <row r="80">
       <c r="C80" s="140" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D80" s="129">
         <f t="shared" si="17"/>
-        <v>4.99</v>
+        <v>0.53</v>
       </c>
       <c r="P80" s="127">
         <v>1.0</v>
@@ -20150,11 +20147,11 @@
     </row>
     <row r="81">
       <c r="C81" s="140" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D81" s="129">
         <f t="shared" si="17"/>
-        <v>10.6</v>
+        <v>7.18</v>
       </c>
       <c r="P81" s="127">
         <v>2.0</v>
@@ -20168,11 +20165,11 @@
     </row>
     <row r="82">
       <c r="C82" s="140" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D82" s="129">
         <f t="shared" si="17"/>
-        <v>12.21</v>
+        <v>6.82</v>
       </c>
       <c r="P82" s="127">
         <v>1.0</v>
@@ -20186,11 +20183,11 @@
     </row>
     <row r="83">
       <c r="C83" s="140" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D83" s="129">
         <f t="shared" si="17"/>
-        <v>0.67</v>
+        <v>3.14</v>
       </c>
       <c r="P83" s="127">
         <v>0.0</v>
@@ -20204,11 +20201,11 @@
     </row>
     <row r="84">
       <c r="C84" s="140" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D84" s="129">
         <f t="shared" si="17"/>
-        <v>7.92</v>
+        <v>0.43</v>
       </c>
       <c r="P84" s="127">
         <v>1.0</v>
@@ -20222,11 +20219,11 @@
     </row>
     <row r="85">
       <c r="C85" s="140" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D85" s="129">
         <f t="shared" si="17"/>
-        <v>6.02</v>
+        <v>4.34</v>
       </c>
       <c r="P85" s="127">
         <v>0.0</v>
@@ -20240,11 +20237,11 @@
     </row>
     <row r="86">
       <c r="C86" s="140" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D86" s="129">
         <f t="shared" si="17"/>
-        <v>7.88</v>
+        <v>5.16</v>
       </c>
       <c r="P86" s="127">
         <v>0.0</v>
@@ -43294,14 +43291,14 @@
     <row r="1">
       <c r="A1" s="110"/>
       <c r="B1" s="150" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C1" s="151"/>
       <c r="D1" s="151"/>
       <c r="E1" s="151"/>
       <c r="F1" s="151"/>
       <c r="G1" s="152" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="H1" s="151"/>
       <c r="I1" s="151"/>
@@ -43335,19 +43332,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="154" t="s">
+        <v>303</v>
+      </c>
+      <c r="C2" s="155" t="s">
         <v>304</v>
-      </c>
-      <c r="C2" s="155" t="s">
-        <v>305</v>
       </c>
       <c r="D2" s="155" t="s">
         <v>43</v>
       </c>
       <c r="E2" s="155" t="s">
+        <v>305</v>
+      </c>
+      <c r="F2" s="156" t="s">
         <v>306</v>
-      </c>
-      <c r="F2" s="156" t="s">
-        <v>307</v>
       </c>
       <c r="G2" s="154">
         <v>1.0</v>
@@ -43359,30 +43356,30 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="155" t="s">
+        <v>307</v>
+      </c>
+      <c r="K2" s="157" t="s">
         <v>308</v>
       </c>
-      <c r="K2" s="157" t="s">
+      <c r="L2" s="155" t="s">
         <v>309</v>
       </c>
-      <c r="L2" s="155" t="s">
+      <c r="M2" s="158" t="s">
         <v>310</v>
       </c>
-      <c r="M2" s="158" t="s">
+      <c r="N2" s="106" t="s">
         <v>311</v>
       </c>
-      <c r="N2" s="106" t="s">
+      <c r="O2" s="106" t="s">
         <v>312</v>
       </c>
-      <c r="O2" s="106" t="s">
+      <c r="P2" s="106" t="s">
         <v>313</v>
-      </c>
-      <c r="P2" s="106" t="s">
-        <v>314</v>
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
       <c r="S2" s="100" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="T2" s="9"/>
       <c r="U2" s="9"/>
@@ -43472,7 +43469,7 @@
       <c r="Q4" s="9"/>
       <c r="R4" s="9"/>
       <c r="S4" s="164" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="T4" s="165"/>
       <c r="Z4" s="36"/>
@@ -43508,7 +43505,7 @@
       <c r="P5" s="167"/>
       <c r="S5" s="165"/>
       <c r="T5" s="168" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="6">
@@ -43541,11 +43538,11 @@
       <c r="R6" s="9"/>
       <c r="S6" s="165"/>
       <c r="T6" s="168" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="Z6" s="42"/>
       <c r="AD6" s="37" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="7">
@@ -43575,7 +43572,7 @@
       <c r="O7" s="84"/>
       <c r="P7" s="169"/>
       <c r="AD7" s="168" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="AE7" s="165"/>
       <c r="AF7" s="165"/>
@@ -43608,11 +43605,11 @@
       <c r="O8" s="84"/>
       <c r="P8" s="169"/>
       <c r="S8" s="168" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="AA8" s="42"/>
       <c r="AD8" s="168" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="9">
@@ -43811,7 +43808,7 @@
       <c r="O15" s="84"/>
       <c r="P15" s="169"/>
       <c r="S15" s="37" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="16">
@@ -43924,7 +43921,7 @@
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
       <c r="S19" s="37" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20">
@@ -44208,7 +44205,7 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="174" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -44293,7 +44290,7 @@
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="E29" s="5">
         <f>J29</f>
@@ -44315,10 +44312,10 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="100" t="s">
+        <v>326</v>
+      </c>
+      <c r="M29" s="100" t="s">
         <v>327</v>
-      </c>
-      <c r="M29" s="100" t="s">
-        <v>328</v>
       </c>
       <c r="O29" s="5">
         <v>1.0</v>
@@ -44418,7 +44415,7 @@
       </c>
       <c r="R31" s="9"/>
       <c r="S31" s="100" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
@@ -44480,7 +44477,7 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="125" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
@@ -44494,10 +44491,10 @@
       <c r="P33" s="9"/>
       <c r="R33" s="9"/>
       <c r="T33" s="45" t="s">
+        <v>330</v>
+      </c>
+      <c r="W33" s="37" t="s">
         <v>331</v>
-      </c>
-      <c r="W33" s="37" t="s">
-        <v>332</v>
       </c>
       <c r="AA33" s="36"/>
       <c r="AD33" s="9"/>
@@ -44540,7 +44537,7 @@
         <v>1626.0</v>
       </c>
       <c r="U34" s="97" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="W34" s="37">
         <v>5193.0</v>
@@ -44585,7 +44582,7 @@
         <v>4176.0</v>
       </c>
       <c r="U35" s="97" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="W35" s="37">
         <v>4863.0</v>
@@ -44683,7 +44680,7 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="G38" s="177">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>
@@ -44885,7 +44882,7 @@
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
       <c r="T45" s="168" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="AD45" s="9"/>
       <c r="AE45" s="9"/>
@@ -45681,10 +45678,10 @@
       <c r="R62" s="9"/>
       <c r="S62" s="9"/>
       <c r="U62" s="37" t="s">
+        <v>335</v>
+      </c>
+      <c r="V62" s="37" t="s">
         <v>336</v>
-      </c>
-      <c r="V62" s="37" t="s">
-        <v>337</v>
       </c>
       <c r="AC62" s="9"/>
       <c r="AD62" s="9"/>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones x cambio de modelos
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -268,7 +268,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="339">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="627" uniqueCount="341">
   <si>
     <t>id_country</t>
   </si>
@@ -1042,25 +1042,31 @@
     <t>3.32</t>
   </si>
   <si>
-    <t>4.13</t>
+    <t>7.32</t>
   </si>
   <si>
-    <t>5.38</t>
+    <t>6.99</t>
   </si>
   <si>
-    <t>7.54</t>
+    <t>0.87</t>
   </si>
   <si>
-    <t>6.69</t>
+    <t>7.21</t>
   </si>
   <si>
-    <t>0.89</t>
+    <t>13.31</t>
   </si>
   <si>
-    <t>0.93</t>
+    <t>13.63</t>
   </si>
   <si>
-    <t>0.90</t>
+    <t>10.44</t>
+  </si>
+  <si>
+    <t>0.15</t>
+  </si>
+  <si>
+    <t>1.28</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2800,7 +2806,7 @@
         <v>45720.0</v>
       </c>
       <c r="D7" s="29">
-        <v>1444.0</v>
+        <v>2114.0</v>
       </c>
       <c r="E7" s="15" t="s">
         <v>15</v>
@@ -2808,7 +2814,7 @@
       <c r="F7" s="30"/>
       <c r="G7" s="17"/>
       <c r="H7" s="18">
-        <v>40.0</v>
+        <v>120.0</v>
       </c>
       <c r="I7" s="18">
         <v>80.0</v>
@@ -2818,11 +2824,11 @@
       </c>
       <c r="K7" s="20">
         <f t="shared" si="1"/>
-        <v>53.33333333</v>
+        <v>80</v>
       </c>
       <c r="L7" s="26">
         <f>K7*'Data preparation'!$C$2</f>
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="M7" s="17"/>
       <c r="N7" s="31" t="str">
@@ -2842,7 +2848,7 @@
         <v>45720.0</v>
       </c>
       <c r="D8" s="29">
-        <v>3461.0</v>
+        <v>870.0</v>
       </c>
       <c r="E8" s="15" t="s">
         <v>15</v>
@@ -2850,7 +2856,7 @@
       <c r="F8" s="30"/>
       <c r="G8" s="17"/>
       <c r="H8" s="18">
-        <v>60.0</v>
+        <v>120.0</v>
       </c>
       <c r="I8" s="18">
         <v>120.0</v>
@@ -2860,11 +2866,11 @@
       </c>
       <c r="K8" s="20">
         <f t="shared" si="1"/>
-        <v>63.33333333</v>
+        <v>83.33333333</v>
       </c>
       <c r="L8" s="26">
         <f>K8*'Data preparation'!$C$2</f>
-        <v>9.5</v>
+        <v>12.5</v>
       </c>
       <c r="M8" s="17"/>
       <c r="N8" s="31" t="str">
@@ -15118,7 +15124,7 @@
       </c>
       <c r="C3" s="25">
         <f>AVERAGE('Modelos actuales'!L4:L8)</f>
-        <v>9.5</v>
+        <v>10.9</v>
       </c>
       <c r="L3" s="97"/>
       <c r="P3" s="97"/>
@@ -16419,7 +16425,7 @@
       <c r="C37" s="43"/>
       <c r="D37" s="112">
         <f>AVERAGE(D39:D1775)</f>
-        <v>5.199130435</v>
+        <v>5.647826087</v>
       </c>
       <c r="G37" s="38" t="s">
         <v>37</v>
@@ -17415,7 +17421,7 @@
       </c>
       <c r="D75" s="103">
         <f t="shared" si="17"/>
-        <v>4.13</v>
+        <v>7.32</v>
       </c>
       <c r="P75" s="101">
         <v>1.0</v>
@@ -17433,7 +17439,7 @@
       </c>
       <c r="D76" s="103">
         <f t="shared" si="17"/>
-        <v>5.38</v>
+        <v>6.99</v>
       </c>
       <c r="P76" s="101">
         <v>0.0</v>
@@ -17451,7 +17457,7 @@
       </c>
       <c r="D77" s="103">
         <f t="shared" si="17"/>
-        <v>7.54</v>
+        <v>0.87</v>
       </c>
       <c r="P77" s="101">
         <v>0.0</v>
@@ -17465,11 +17471,11 @@
     </row>
     <row r="78">
       <c r="C78" s="115" t="s">
-        <v>161</v>
+        <v>225</v>
       </c>
       <c r="D78" s="103">
         <f t="shared" si="17"/>
-        <v>7.85</v>
+        <v>7.21</v>
       </c>
       <c r="P78" s="101">
         <v>1.0</v>
@@ -17483,11 +17489,11 @@
     </row>
     <row r="79">
       <c r="C79" s="115" t="s">
-        <v>217</v>
+        <v>226</v>
       </c>
       <c r="D79" s="103">
         <f t="shared" si="17"/>
-        <v>6.21</v>
+        <v>13.31</v>
       </c>
       <c r="P79" s="101">
         <v>2.0</v>
@@ -17501,11 +17507,11 @@
     </row>
     <row r="80">
       <c r="C80" s="115" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D80" s="103">
         <f t="shared" si="17"/>
-        <v>6.69</v>
+        <v>13.63</v>
       </c>
       <c r="P80" s="101">
         <v>1.0</v>
@@ -17519,11 +17525,11 @@
     </row>
     <row r="81">
       <c r="C81" s="115" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D81" s="103">
         <f t="shared" si="17"/>
-        <v>0.89</v>
+        <v>10.44</v>
       </c>
       <c r="P81" s="101">
         <v>2.0</v>
@@ -17537,11 +17543,11 @@
     </row>
     <row r="82">
       <c r="C82" s="115" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D82" s="103">
         <f t="shared" si="17"/>
-        <v>0.89</v>
+        <v>0.15</v>
       </c>
       <c r="P82" s="101">
         <v>1.0</v>
@@ -17555,11 +17561,11 @@
     </row>
     <row r="83">
       <c r="C83" s="115" t="s">
-        <v>227</v>
+        <v>187</v>
       </c>
       <c r="D83" s="103">
         <f t="shared" si="17"/>
-        <v>0.93</v>
+        <v>0.85</v>
       </c>
       <c r="P83" s="101">
         <v>0.0</v>
@@ -17573,11 +17579,11 @@
     </row>
     <row r="84">
       <c r="C84" s="115" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D84" s="103">
         <f t="shared" si="17"/>
-        <v>0.9</v>
+        <v>1.28</v>
       </c>
       <c r="P84" s="101">
         <v>1.0</v>
@@ -40659,14 +40665,14 @@
     <row r="1">
       <c r="A1" s="127"/>
       <c r="B1" s="128" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C1" s="129"/>
       <c r="D1" s="129"/>
       <c r="E1" s="129"/>
       <c r="F1" s="129"/>
       <c r="G1" s="130" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H1" s="129"/>
       <c r="I1" s="129"/>
@@ -40700,19 +40706,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="132" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C2" s="133" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D2" s="133" t="s">
         <v>170</v>
       </c>
       <c r="E2" s="133" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F2" s="134" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="G2" s="132">
         <v>1.0</v>
@@ -40724,30 +40730,30 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="133" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="K2" s="135" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="L2" s="133" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="M2" s="136" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="N2" s="117" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="O2" s="117" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="P2" s="117" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="Q2" s="9"/>
       <c r="R2" s="9"/>
       <c r="S2" s="96" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="T2" s="9"/>
       <c r="U2" s="9"/>
@@ -40837,7 +40843,7 @@
       <c r="Q4" s="9"/>
       <c r="R4" s="9"/>
       <c r="S4" s="142" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="T4" s="143"/>
       <c r="Z4" s="38"/>
@@ -40873,7 +40879,7 @@
       <c r="P5" s="145"/>
       <c r="S5" s="143"/>
       <c r="T5" s="146" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6">
@@ -40906,11 +40912,11 @@
       <c r="R6" s="9"/>
       <c r="S6" s="143"/>
       <c r="T6" s="146" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="Z6" s="89"/>
       <c r="AD6" s="39" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="7">
@@ -40940,7 +40946,7 @@
       <c r="O7" s="80"/>
       <c r="P7" s="148"/>
       <c r="AD7" s="146" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="AE7" s="143"/>
       <c r="AF7" s="143"/>
@@ -40973,11 +40979,11 @@
       <c r="O8" s="80"/>
       <c r="P8" s="148"/>
       <c r="S8" s="146" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="AA8" s="89"/>
       <c r="AD8" s="146" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
     </row>
     <row r="9">
@@ -41176,7 +41182,7 @@
       <c r="O15" s="80"/>
       <c r="P15" s="148"/>
       <c r="S15" s="39" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="16">
@@ -41289,7 +41295,7 @@
       <c r="Q19" s="9"/>
       <c r="R19" s="9"/>
       <c r="S19" s="39" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20">
@@ -41573,7 +41579,7 @@
       <c r="E27" s="9"/>
       <c r="F27" s="9"/>
       <c r="G27" s="153" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="H27" s="9"/>
       <c r="I27" s="9"/>
@@ -41658,7 +41664,7 @@
       <c r="B29" s="9"/>
       <c r="C29" s="9"/>
       <c r="D29" s="5" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="E29" s="5">
         <f>J29</f>
@@ -41680,10 +41686,10 @@
       </c>
       <c r="K29" s="9"/>
       <c r="L29" s="96" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="M29" s="96" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="O29" s="5">
         <v>1.0</v>
@@ -41783,7 +41789,7 @@
       </c>
       <c r="R31" s="9"/>
       <c r="S31" s="96" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="T31" s="9"/>
       <c r="U31" s="9"/>
@@ -41845,7 +41851,7 @@
       <c r="E33" s="9"/>
       <c r="F33" s="9"/>
       <c r="G33" s="99" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="J33" s="9"/>
       <c r="K33" s="9"/>
@@ -41859,10 +41865,10 @@
       <c r="P33" s="9"/>
       <c r="R33" s="9"/>
       <c r="T33" s="58" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="W33" s="39" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="AA33" s="38"/>
       <c r="AD33" s="9"/>
@@ -41905,7 +41911,7 @@
         <v>1626.0</v>
       </c>
       <c r="U34" s="94" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="W34" s="39">
         <v>5193.0</v>
@@ -41950,7 +41956,7 @@
         <v>4176.0</v>
       </c>
       <c r="U35" s="94" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="W35" s="39">
         <v>4863.0</v>
@@ -42048,7 +42054,7 @@
       <c r="D38" s="9"/>
       <c r="E38" s="9"/>
       <c r="F38" s="5" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="G38" s="156">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>
@@ -42250,7 +42256,7 @@
       <c r="Q45" s="9"/>
       <c r="R45" s="9"/>
       <c r="T45" s="146" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="AD45" s="9"/>
       <c r="AE45" s="9"/>
@@ -42414,7 +42420,7 @@
         <v>13</v>
       </c>
       <c r="AG49" s="7" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="50">
@@ -42579,7 +42585,7 @@
         <v>13.03594852814783</v>
       </c>
       <c r="AG52" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="53">
@@ -42640,7 +42646,7 @@
         <v>6.291840048860032</v>
       </c>
       <c r="AG53" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="54">
@@ -42701,7 +42707,7 @@
         <v>2.7243520649411117</v>
       </c>
       <c r="AG54" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="55">
@@ -42762,7 +42768,7 @@
         <v>2.1429979739456915</v>
       </c>
       <c r="AG55" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="56">
@@ -42823,7 +42829,7 @@
         <v>3.98032040346951</v>
       </c>
       <c r="AG56" s="7" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
     </row>
     <row r="57">
@@ -43046,10 +43052,10 @@
       <c r="R62" s="9"/>
       <c r="S62" s="9"/>
       <c r="U62" s="39" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="V62" s="39" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="AC62" s="9"/>
       <c r="AD62" s="9"/>
@@ -43091,7 +43097,7 @@
         <v>2165.0</v>
       </c>
       <c r="W63" s="39" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="AC63" s="9"/>
       <c r="AD63" s="9"/>
@@ -76449,146 +76455,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="39" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="9"/>
       <c r="C2" s="166" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="E2" s="167"/>
       <c r="F2" s="96" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="H2" s="167"/>
     </row>
     <row r="3">
       <c r="B3" s="116" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C3" s="168" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="D3" s="116" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="E3" s="169" t="s">
         <v>96</v>
       </c>
       <c r="F3" s="116" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="G3" s="116" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="H3" s="116" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="170" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C4" s="171" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D4" s="117" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="E4" s="172" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F4" s="173" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="G4" s="173" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H4" s="117"/>
     </row>
     <row r="5">
       <c r="B5" s="170" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="C5" s="174" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="D5" s="127"/>
       <c r="E5" s="172" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F5" s="175" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="G5" s="176" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H5" s="117"/>
     </row>
     <row r="6">
       <c r="B6" s="170" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="C6" s="171" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="D6" s="117" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="E6" s="172" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="F6" s="117" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="G6" s="117"/>
       <c r="H6" s="117"/>
     </row>
     <row r="7">
       <c r="B7" s="117" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C7" s="177" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="D7" s="117"/>
       <c r="E7" s="178" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F7" s="171" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="G7" s="117"/>
       <c r="H7" s="117" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="179" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C8" s="180" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D8" s="181"/>
       <c r="E8" s="179" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="F8" s="182" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="G8" s="183" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="H8" s="181"/>
     </row>
     <row r="9">
       <c r="B9" s="22" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="C9" s="184" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="D9" s="80"/>
       <c r="E9" s="80"/>
@@ -76598,27 +76604,27 @@
     </row>
     <row r="10">
       <c r="B10" s="22" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C10" s="147"/>
       <c r="D10" s="80"/>
       <c r="E10" s="80"/>
       <c r="F10" s="147"/>
       <c r="G10" s="173" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="H10" s="80"/>
     </row>
     <row r="11">
       <c r="B11" s="22" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="C11" s="147"/>
       <c r="D11" s="80"/>
       <c r="E11" s="80"/>
       <c r="F11" s="147"/>
       <c r="G11" s="185" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H11" s="22"/>
     </row>
@@ -76641,7 +76647,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="38" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="L1" s="10"/>
     </row>
@@ -76650,16 +76656,16 @@
     </row>
     <row r="3">
       <c r="A3" s="39" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="L3" s="10"/>
     </row>
     <row r="4">
       <c r="B4" s="39" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="G4" s="39" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="L4" s="10"/>
     </row>
@@ -76765,62 +76771,62 @@
     </row>
     <row r="11">
       <c r="A11" s="186" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="38" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="39" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="186" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="38" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="39" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F19" s="89"/>
     </row>
     <row r="20">
       <c r="B20" s="38" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C20" s="43"/>
       <c r="D20" s="43"/>
       <c r="E20" s="43"/>
       <c r="F20" s="43"/>
       <c r="G20" s="38" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="H20" s="38" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I20" s="38" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="J20" s="38" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="K20" s="38" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="38" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="G21" s="44">
         <v>2.575</v>
@@ -76828,27 +76834,27 @@
     </row>
     <row r="23">
       <c r="K23" s="38" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="39" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="H24" s="39" t="s">
         <v>170</v>
       </c>
       <c r="I24" s="39" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="K24" s="39" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="L24" s="39" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="M24" s="39" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="25">
@@ -76867,7 +76873,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="K25" s="39" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
     </row>
     <row r="26">
@@ -76878,7 +76884,7 @@
         <v>1.19</v>
       </c>
       <c r="K26" s="39" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
     </row>
     <row r="27">
@@ -76889,7 +76895,7 @@
         <v>2.19</v>
       </c>
       <c r="K27" s="39" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
     </row>
     <row r="28">
@@ -76900,7 +76906,7 @@
         <v>0.05</v>
       </c>
       <c r="K28" s="39" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
     </row>
     <row r="29">
@@ -76919,7 +76925,7 @@
         <v>6.42</v>
       </c>
       <c r="K30" s="58" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
     </row>
     <row r="31">
@@ -77064,7 +77070,7 @@
         <v>0.61</v>
       </c>
       <c r="K41" s="38" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
     </row>
     <row r="42">
@@ -77075,13 +77081,13 @@
         <v>0.69</v>
       </c>
       <c r="K42" s="39" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="L42" s="39" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="M42" s="39" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
     </row>
     <row r="43">
@@ -77213,7 +77219,7 @@
         <v>0.0</v>
       </c>
       <c r="K51" s="39" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
     </row>
     <row r="52">
@@ -77241,17 +77247,17 @@
       </c>
       <c r="K54" s="80"/>
       <c r="L54" s="187" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="M54" s="188"/>
       <c r="N54" s="85" t="s">
         <v>6</v>
       </c>
       <c r="O54" s="85" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="P54" s="85" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="R54" s="18" t="s">
         <v>106</v>
@@ -77333,7 +77339,7 @@
         <v>5.86</v>
       </c>
       <c r="R57" s="39" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="S57" s="44">
         <f>SUM(P55:P74)</f>
@@ -77348,7 +77354,7 @@
         <v>0.0</v>
       </c>
       <c r="K58" s="22" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="L58" s="189">
         <v>0.57</v>
@@ -77362,7 +77368,7 @@
         <v>0.855</v>
       </c>
       <c r="P58" s="22" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
     </row>
     <row r="59">
@@ -77409,7 +77415,7 @@
         <v>0.96</v>
       </c>
       <c r="P60" s="22" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
     </row>
     <row r="61">
@@ -77420,7 +77426,7 @@
         <v>0.02</v>
       </c>
       <c r="K61" s="22" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="L61" s="22">
         <v>0.42</v>
@@ -77492,7 +77498,7 @@
         <v>0.0</v>
       </c>
       <c r="K64" s="22" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="L64" s="22">
         <v>0.42</v>
@@ -77636,7 +77642,7 @@
         <v>0.0</v>
       </c>
       <c r="K70" s="22" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="L70" s="22">
         <v>0.66</v>

</xml_diff>

<commit_message>
DATA. Cambio modelo de FRA al tener en cuenta mas candidatos
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -268,7 +268,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="341">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="342">
   <si>
     <t>id_country</t>
   </si>
@@ -898,28 +898,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>1.68</t>
+    <t>9.08</t>
   </si>
   <si>
-    <t>10.08</t>
+    <t>0.59</t>
   </si>
   <si>
-    <t>5.20</t>
+    <t>3.90</t>
   </si>
   <si>
-    <t>9.86</t>
+    <t>7.66</t>
   </si>
   <si>
-    <t>6.71</t>
+    <t>6.37</t>
   </si>
   <si>
-    <t>9.30</t>
+    <t>5.53</t>
   </si>
   <si>
-    <t>9.47</t>
+    <t>7.41</t>
   </si>
   <si>
-    <t>9.16</t>
+    <t>7.80</t>
   </si>
   <si>
     <t>Country</t>
@@ -928,139 +928,142 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>0.53</t>
+    <t>1.30</t>
   </si>
   <si>
-    <t>0.74</t>
+    <t>1.70</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>0.85</t>
+    <t>2.00</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>0.22</t>
+    <t>3.75</t>
   </si>
   <si>
     <t>p25</t>
   </si>
   <si>
-    <t>1.26</t>
+    <t>0.19</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>0.64</t>
+    <t>5.82</t>
   </si>
   <si>
-    <t>7.33</t>
+    <t>3.00</t>
   </si>
   <si>
-    <t>7.61</t>
+    <t>6.17</t>
   </si>
   <si>
-    <t>5.07</t>
+    <t>1.03</t>
   </si>
   <si>
-    <t>7.64</t>
+    <t>5.46</t>
   </si>
   <si>
-    <t>8.25</t>
+    <t>5.43</t>
+  </si>
+  <si>
+    <t>5.89</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
   </si>
   <si>
-    <t>7.97</t>
+    <t>5.69</t>
   </si>
   <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>8.17</t>
+    <t>5.83</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
-    <t>1.55</t>
+    <t>1.11</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>9.32</t>
+    <t>6.65</t>
   </si>
   <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
-    <t>4.95</t>
+    <t>2.55</t>
   </si>
   <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>11.15</t>
+    <t>7.96</t>
   </si>
   <si>
-    <t>4.97</t>
+    <t>7.09</t>
   </si>
   <si>
-    <t>5.61</t>
+    <t>8.34</t>
   </si>
   <si>
-    <t>5.84</t>
+    <t>6.15</t>
   </si>
   <si>
-    <t>4.30</t>
+    <t>7.72</t>
   </si>
   <si>
-    <t>5.41</t>
+    <t>6.61</t>
   </si>
   <si>
-    <t>9.26</t>
+    <t>7.11</t>
   </si>
   <si>
-    <t>9.95</t>
+    <t>4.75</t>
   </si>
   <si>
-    <t>6.64</t>
+    <t>3.91</t>
   </si>
   <si>
-    <t>4.36</t>
+    <t>6.22</t>
   </si>
   <si>
-    <t>2.73</t>
+    <t>7.88</t>
   </si>
   <si>
-    <t>4.35</t>
+    <t>6.04</t>
   </si>
   <si>
-    <t>4.23</t>
+    <t>6.96</t>
   </si>
   <si>
-    <t>4.87</t>
+    <t>7.30</t>
   </si>
   <si>
-    <t>5.11</t>
+    <t>9.45</t>
   </si>
   <si>
-    <t>13.23</t>
+    <t>9.23</t>
   </si>
   <si>
-    <t>12.92</t>
+    <t>0.97</t>
   </si>
   <si>
-    <t>0.68</t>
+    <t>6.06</t>
   </si>
   <si>
-    <t>3.12</t>
+    <t>4.45</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2700,17 +2703,17 @@
         <v>45719.0</v>
       </c>
       <c r="D5" s="13">
-        <v>3960.0</v>
+        <v>3024.0</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>13</v>
       </c>
       <c r="F5" s="14"/>
       <c r="G5" s="15">
+        <v>120.0</v>
+      </c>
+      <c r="H5" s="15">
         <v>80.0</v>
-      </c>
-      <c r="H5" s="15">
-        <v>120.0</v>
       </c>
       <c r="I5" s="15">
         <v>120.0</v>
@@ -2827,21 +2830,21 @@
       </c>
       <c r="F8" s="14"/>
       <c r="G8" s="15">
-        <v>130.0</v>
+        <v>120.0</v>
       </c>
       <c r="H8" s="15">
-        <v>130.0</v>
+        <v>120.0</v>
       </c>
       <c r="I8" s="15">
-        <v>70.0</v>
+        <v>80.0</v>
       </c>
       <c r="J8" s="17">
         <f t="shared" si="1"/>
-        <v>110</v>
+        <v>106.6666667</v>
       </c>
       <c r="K8" s="24">
         <f>J8*'Data preparation'!$C$2</f>
-        <v>11</v>
+        <v>10.66666667</v>
       </c>
       <c r="L8" s="25" t="str">
         <f t="shared" si="2"/>
@@ -13521,7 +13524,7 @@
       </c>
       <c r="C3" s="96">
         <f>AVERAGE('Modelos actuales'!K4:K8)</f>
-        <v>10.2</v>
+        <v>10.13333333</v>
       </c>
       <c r="L3" s="95"/>
       <c r="P3" s="95"/>
@@ -14822,7 +14825,7 @@
       <c r="C37" s="36"/>
       <c r="D37" s="111">
         <f>AVERAGE(D39:D1775)</f>
-        <v>5.863043478</v>
+        <v>5.438913043</v>
       </c>
       <c r="G37" s="34" t="s">
         <v>35</v>
@@ -14891,7 +14894,7 @@
       </c>
       <c r="D39" s="102">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>1.68</v>
+        <v>9.08</v>
       </c>
       <c r="G39" s="34" t="s">
         <v>27</v>
@@ -14929,7 +14932,7 @@
       </c>
       <c r="D40" s="102">
         <f t="shared" si="17"/>
-        <v>10.08</v>
+        <v>0.59</v>
       </c>
       <c r="G40" s="34" t="s">
         <v>23</v>
@@ -14967,7 +14970,7 @@
       </c>
       <c r="D41" s="102">
         <f t="shared" si="17"/>
-        <v>5.2</v>
+        <v>3.9</v>
       </c>
       <c r="P41" s="100">
         <v>0.0</v>
@@ -14999,7 +15002,7 @@
       </c>
       <c r="D42" s="102">
         <f t="shared" si="17"/>
-        <v>9.86</v>
+        <v>7.66</v>
       </c>
       <c r="P42" s="100">
         <v>2.0</v>
@@ -15031,7 +15034,7 @@
       </c>
       <c r="D43" s="102">
         <f t="shared" si="17"/>
-        <v>6.71</v>
+        <v>6.37</v>
       </c>
       <c r="P43" s="100">
         <v>1.0</v>
@@ -15063,7 +15066,7 @@
       </c>
       <c r="D44" s="102">
         <f t="shared" si="17"/>
-        <v>9.3</v>
+        <v>5.53</v>
       </c>
       <c r="P44" s="100">
         <v>2.0</v>
@@ -15093,7 +15096,7 @@
       </c>
       <c r="D45" s="102">
         <f t="shared" si="17"/>
-        <v>9.47</v>
+        <v>7.41</v>
       </c>
       <c r="P45" s="100">
         <v>1.0</v>
@@ -15111,7 +15114,7 @@
       </c>
       <c r="D46" s="102">
         <f t="shared" si="17"/>
-        <v>9.16</v>
+        <v>7.8</v>
       </c>
       <c r="G46" s="115" t="s">
         <v>182</v>
@@ -15135,7 +15138,7 @@
       </c>
       <c r="D47" s="102">
         <f t="shared" si="17"/>
-        <v>0.53</v>
+        <v>1.3</v>
       </c>
       <c r="G47" s="116" t="s">
         <v>36</v>
@@ -15165,7 +15168,7 @@
       </c>
       <c r="D48" s="102">
         <f t="shared" si="17"/>
-        <v>0.74</v>
+        <v>1.7</v>
       </c>
       <c r="G48" s="116" t="s">
         <v>35</v>
@@ -15202,7 +15205,7 @@
       </c>
       <c r="D49" s="102">
         <f t="shared" si="17"/>
-        <v>0.85</v>
+        <v>2</v>
       </c>
       <c r="G49" s="116" t="s">
         <v>26</v>
@@ -15239,7 +15242,7 @@
       </c>
       <c r="D50" s="102">
         <f t="shared" si="17"/>
-        <v>0.22</v>
+        <v>3.75</v>
       </c>
       <c r="G50" s="116" t="s">
         <v>27</v>
@@ -15276,7 +15279,7 @@
       </c>
       <c r="D51" s="102">
         <f t="shared" si="17"/>
-        <v>1.26</v>
+        <v>0.19</v>
       </c>
       <c r="G51" s="116" t="s">
         <v>23</v>
@@ -15313,7 +15316,7 @@
       </c>
       <c r="D52" s="102">
         <f t="shared" si="17"/>
-        <v>0.64</v>
+        <v>5.82</v>
       </c>
       <c r="P52" s="100">
         <v>0.0</v>
@@ -15337,7 +15340,7 @@
       </c>
       <c r="D53" s="102">
         <f t="shared" si="17"/>
-        <v>7.33</v>
+        <v>3</v>
       </c>
       <c r="P53" s="100">
         <v>0.0</v>
@@ -15361,7 +15364,7 @@
       </c>
       <c r="D54" s="102">
         <f t="shared" si="17"/>
-        <v>7.61</v>
+        <v>6.17</v>
       </c>
       <c r="P54" s="100">
         <v>2.0</v>
@@ -15385,7 +15388,7 @@
       </c>
       <c r="D55" s="102">
         <f t="shared" si="17"/>
-        <v>5.07</v>
+        <v>1.03</v>
       </c>
       <c r="P55" s="100">
         <v>0.0</v>
@@ -15409,7 +15412,7 @@
       </c>
       <c r="D56" s="102">
         <f t="shared" si="17"/>
-        <v>7.64</v>
+        <v>5.46</v>
       </c>
       <c r="P56" s="100">
         <v>0.0</v>
@@ -15429,11 +15432,11 @@
     </row>
     <row r="57">
       <c r="C57" s="114" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="D57" s="102">
         <f t="shared" si="17"/>
-        <v>7.61</v>
+        <v>5.43</v>
       </c>
       <c r="P57" s="100">
         <v>2.0</v>
@@ -15453,14 +15456,14 @@
     </row>
     <row r="58">
       <c r="C58" s="114" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D58" s="102">
         <f t="shared" si="17"/>
-        <v>8.25</v>
+        <v>5.89</v>
       </c>
       <c r="G58" s="118" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H58" s="119"/>
       <c r="P58" s="100">
@@ -15481,15 +15484,15 @@
     </row>
     <row r="59">
       <c r="C59" s="114" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D59" s="102">
         <f t="shared" si="17"/>
-        <v>7.97</v>
+        <v>5.69</v>
       </c>
       <c r="G59" s="119"/>
       <c r="H59" s="120" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="P59" s="100">
         <v>0.0</v>
@@ -15509,15 +15512,15 @@
     </row>
     <row r="60">
       <c r="C60" s="114" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D60" s="102">
         <f t="shared" si="17"/>
-        <v>8.17</v>
+        <v>5.83</v>
       </c>
       <c r="G60" s="119"/>
       <c r="H60" s="120" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="P60" s="100">
         <v>2.0</v>
@@ -15537,15 +15540,15 @@
     </row>
     <row r="61">
       <c r="C61" s="114" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="D61" s="102">
         <f t="shared" si="17"/>
-        <v>1.55</v>
+        <v>1.11</v>
       </c>
       <c r="G61" s="119"/>
       <c r="H61" s="120" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="P61" s="100">
         <v>2.0</v>
@@ -15565,15 +15568,15 @@
     </row>
     <row r="62">
       <c r="C62" s="114" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D62" s="102">
         <f t="shared" si="17"/>
-        <v>9.32</v>
+        <v>6.65</v>
       </c>
       <c r="G62" s="119"/>
       <c r="H62" s="120" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P62" s="100">
         <v>1.0</v>
@@ -15593,15 +15596,15 @@
     </row>
     <row r="63">
       <c r="C63" s="114" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="D63" s="102">
         <f t="shared" si="17"/>
-        <v>4.95</v>
+        <v>2.55</v>
       </c>
       <c r="G63" s="119"/>
       <c r="H63" s="120" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P63" s="100">
         <v>0.0</v>
@@ -15615,11 +15618,11 @@
     </row>
     <row r="64">
       <c r="C64" s="114" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D64" s="102">
         <f t="shared" si="17"/>
-        <v>11.15</v>
+        <v>7.96</v>
       </c>
       <c r="P64" s="100">
         <v>1.0</v>
@@ -15633,11 +15636,11 @@
     </row>
     <row r="65">
       <c r="C65" s="114" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="D65" s="102">
         <f t="shared" si="17"/>
-        <v>4.97</v>
+        <v>7.09</v>
       </c>
       <c r="P65" s="100">
         <v>2.0</v>
@@ -15651,11 +15654,11 @@
     </row>
     <row r="66">
       <c r="C66" s="114" t="s">
-        <v>212</v>
+        <v>159</v>
       </c>
       <c r="D66" s="102">
         <f t="shared" si="17"/>
-        <v>5.61</v>
+        <v>7.91</v>
       </c>
       <c r="P66" s="100">
         <v>0.0</v>
@@ -15673,7 +15676,7 @@
       </c>
       <c r="D67" s="102">
         <f t="shared" si="17"/>
-        <v>5.84</v>
+        <v>8.34</v>
       </c>
       <c r="P67" s="100">
         <v>0.0</v>
@@ -15691,7 +15694,7 @@
       </c>
       <c r="D68" s="102">
         <f t="shared" si="17"/>
-        <v>4.3</v>
+        <v>6.15</v>
       </c>
       <c r="P68" s="100">
         <v>1.0</v>
@@ -15709,7 +15712,7 @@
       </c>
       <c r="D69" s="102">
         <f t="shared" si="17"/>
-        <v>5.41</v>
+        <v>7.72</v>
       </c>
       <c r="P69" s="100">
         <v>2.0</v>
@@ -15727,7 +15730,7 @@
       </c>
       <c r="D70" s="102">
         <f t="shared" si="17"/>
-        <v>9.26</v>
+        <v>6.61</v>
       </c>
       <c r="P70" s="100">
         <v>1.0</v>
@@ -15745,7 +15748,7 @@
       </c>
       <c r="D71" s="102">
         <f t="shared" si="17"/>
-        <v>9.95</v>
+        <v>7.11</v>
       </c>
       <c r="F71" s="121"/>
       <c r="P71" s="100">
@@ -15764,7 +15767,7 @@
       </c>
       <c r="D72" s="102">
         <f t="shared" si="17"/>
-        <v>6.64</v>
+        <v>4.75</v>
       </c>
       <c r="P72" s="100">
         <v>0.0</v>
@@ -15778,11 +15781,11 @@
     </row>
     <row r="73">
       <c r="C73" s="114" t="s">
-        <v>219</v>
+        <v>195</v>
       </c>
       <c r="D73" s="102">
         <f t="shared" si="17"/>
-        <v>4.36</v>
+        <v>6.17</v>
       </c>
       <c r="P73" s="100">
         <v>1.0</v>
@@ -15796,11 +15799,11 @@
     </row>
     <row r="74">
       <c r="C74" s="114" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D74" s="102">
         <f t="shared" si="17"/>
-        <v>2.73</v>
+        <v>3.91</v>
       </c>
       <c r="P74" s="100">
         <v>0.0</v>
@@ -15814,11 +15817,11 @@
     </row>
     <row r="75">
       <c r="C75" s="114" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D75" s="102">
         <f t="shared" si="17"/>
-        <v>4.35</v>
+        <v>6.22</v>
       </c>
       <c r="P75" s="100">
         <v>1.0</v>
@@ -15832,11 +15835,11 @@
     </row>
     <row r="76">
       <c r="C76" s="114" t="s">
-        <v>165</v>
+        <v>221</v>
       </c>
       <c r="D76" s="102">
         <f t="shared" si="17"/>
-        <v>5.56</v>
+        <v>7.88</v>
       </c>
       <c r="P76" s="100">
         <v>0.0</v>
@@ -15854,7 +15857,7 @@
       </c>
       <c r="D77" s="102">
         <f t="shared" si="17"/>
-        <v>4.23</v>
+        <v>6.04</v>
       </c>
       <c r="P77" s="100">
         <v>0.0</v>
@@ -15872,7 +15875,7 @@
       </c>
       <c r="D78" s="102">
         <f t="shared" si="17"/>
-        <v>4.87</v>
+        <v>6.96</v>
       </c>
       <c r="P78" s="100">
         <v>1.0</v>
@@ -15890,7 +15893,7 @@
       </c>
       <c r="D79" s="102">
         <f t="shared" si="17"/>
-        <v>5.11</v>
+        <v>7.3</v>
       </c>
       <c r="P79" s="100">
         <v>2.0</v>
@@ -15908,7 +15911,7 @@
       </c>
       <c r="D80" s="102">
         <f t="shared" si="17"/>
-        <v>13.23</v>
+        <v>9.45</v>
       </c>
       <c r="P80" s="100">
         <v>1.0</v>
@@ -15926,7 +15929,7 @@
       </c>
       <c r="D81" s="102">
         <f t="shared" si="17"/>
-        <v>12.92</v>
+        <v>9.23</v>
       </c>
       <c r="P81" s="100">
         <v>2.0</v>
@@ -15944,7 +15947,7 @@
       </c>
       <c r="D82" s="102">
         <f t="shared" si="17"/>
-        <v>0.68</v>
+        <v>0.97</v>
       </c>
       <c r="P82" s="100">
         <v>1.0</v>
@@ -15958,11 +15961,11 @@
     </row>
     <row r="83">
       <c r="C83" s="114" t="s">
-        <v>163</v>
+        <v>228</v>
       </c>
       <c r="D83" s="102">
         <f t="shared" si="17"/>
-        <v>4.24</v>
+        <v>6.06</v>
       </c>
       <c r="P83" s="100">
         <v>0.0</v>
@@ -15976,11 +15979,11 @@
     </row>
     <row r="84">
       <c r="C84" s="114" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D84" s="102">
         <f t="shared" si="17"/>
-        <v>3.12</v>
+        <v>4.45</v>
       </c>
       <c r="P84" s="100">
         <v>1.0</v>
@@ -39062,14 +39065,14 @@
     <row r="1">
       <c r="A1" s="126"/>
       <c r="B1" s="127" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="C1" s="128"/>
       <c r="D1" s="128"/>
       <c r="E1" s="128"/>
       <c r="F1" s="128"/>
       <c r="G1" s="129" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H1" s="128"/>
       <c r="I1" s="128"/>
@@ -39103,19 +39106,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="131" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="C2" s="132" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>170</v>
       </c>
       <c r="E2" s="132" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F2" s="133" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="G2" s="131">
         <v>1.0</v>
@@ -39127,30 +39130,30 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="132" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K2" s="134" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L2" s="132" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M2" s="135" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="N2" s="116" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="O2" s="116" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="P2" s="116" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
       <c r="S2" s="94" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
@@ -39240,7 +39243,7 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="141" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="T4" s="142"/>
       <c r="Z4" s="34"/>
@@ -39276,7 +39279,7 @@
       <c r="P5" s="144"/>
       <c r="S5" s="142"/>
       <c r="T5" s="145" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6">
@@ -39309,11 +39312,11 @@
       <c r="R6" s="7"/>
       <c r="S6" s="142"/>
       <c r="T6" s="145" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Z6" s="83"/>
       <c r="AD6" s="31" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7">
@@ -39343,7 +39346,7 @@
       <c r="O7" s="74"/>
       <c r="P7" s="147"/>
       <c r="AD7" s="145" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AE7" s="142"/>
       <c r="AF7" s="142"/>
@@ -39376,11 +39379,11 @@
       <c r="O8" s="74"/>
       <c r="P8" s="147"/>
       <c r="S8" s="145" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="AA8" s="83"/>
       <c r="AD8" s="145" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9">
@@ -39579,7 +39582,7 @@
       <c r="O15" s="74"/>
       <c r="P15" s="147"/>
       <c r="S15" s="31" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16">
@@ -39692,7 +39695,7 @@
       <c r="Q19" s="7"/>
       <c r="R19" s="7"/>
       <c r="S19" s="31" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="20">
@@ -39976,7 +39979,7 @@
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
       <c r="G27" s="152" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
@@ -40061,7 +40064,7 @@
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -40083,10 +40086,10 @@
       </c>
       <c r="K29" s="7"/>
       <c r="L29" s="94" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M29" s="94" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -40186,7 +40189,7 @@
       </c>
       <c r="R31" s="7"/>
       <c r="S31" s="94" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="T31" s="7"/>
       <c r="U31" s="7"/>
@@ -40248,7 +40251,7 @@
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
       <c r="G33" s="98" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -40262,10 +40265,10 @@
       <c r="P33" s="7"/>
       <c r="R33" s="7"/>
       <c r="T33" s="51" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="W33" s="31" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="AA33" s="34"/>
       <c r="AD33" s="7"/>
@@ -40308,7 +40311,7 @@
         <v>1626.0</v>
       </c>
       <c r="U34" s="92" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="W34" s="31">
         <v>5193.0</v>
@@ -40353,7 +40356,7 @@
         <v>4176.0</v>
       </c>
       <c r="U35" s="92" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="W35" s="31">
         <v>4863.0</v>
@@ -40451,7 +40454,7 @@
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
       <c r="F38" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="G38" s="155">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>
@@ -40653,7 +40656,7 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="T45" s="145" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="AD45" s="7"/>
       <c r="AE45" s="7"/>
@@ -40817,7 +40820,7 @@
         <v>11</v>
       </c>
       <c r="AG49" s="61" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="50">
@@ -40982,7 +40985,7 @@
         <v>13.03594852814783</v>
       </c>
       <c r="AG52" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="53">
@@ -41043,7 +41046,7 @@
         <v>6.291840048860032</v>
       </c>
       <c r="AG53" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="54">
@@ -41104,7 +41107,7 @@
         <v>2.7243520649411117</v>
       </c>
       <c r="AG54" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55">
@@ -41165,7 +41168,7 @@
         <v>2.1429979739456915</v>
       </c>
       <c r="AG55" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="56">
@@ -41226,7 +41229,7 @@
         <v>3.98032040346951</v>
       </c>
       <c r="AG56" s="61" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57">
@@ -41449,10 +41452,10 @@
       <c r="R62" s="7"/>
       <c r="S62" s="7"/>
       <c r="U62" s="31" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="V62" s="31" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AC62" s="7"/>
       <c r="AD62" s="7"/>
@@ -41494,7 +41497,7 @@
         <v>2165.0</v>
       </c>
       <c r="W63" s="31" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AC63" s="7"/>
       <c r="AD63" s="7"/>
@@ -42128,7 +42131,7 @@
       <c r="R79" s="7"/>
       <c r="S79" s="7"/>
       <c r="T79" s="94" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="U79" s="7"/>
       <c r="V79" s="7"/>
@@ -42169,7 +42172,7 @@
       <c r="R80" s="7"/>
       <c r="S80" s="7"/>
       <c r="T80" s="31" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="U80" s="18"/>
       <c r="V80" s="18"/>
@@ -74930,146 +74933,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="31" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="7"/>
       <c r="C2" s="165" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E2" s="166"/>
       <c r="F2" s="94" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="H2" s="166"/>
     </row>
     <row r="3">
       <c r="B3" s="115" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C3" s="167" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D3" s="115" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="E3" s="168" t="s">
         <v>96</v>
       </c>
       <c r="F3" s="115" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="G3" s="115" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="H3" s="115" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="169" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="C4" s="170" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D4" s="116" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E4" s="171" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F4" s="172" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="G4" s="172" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H4" s="116"/>
     </row>
     <row r="5">
       <c r="B5" s="169" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="C5" s="173" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="D5" s="126"/>
       <c r="E5" s="171" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F5" s="174" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="G5" s="175" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="H5" s="116"/>
     </row>
     <row r="6">
       <c r="B6" s="169" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C6" s="170" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="D6" s="116" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E6" s="171" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="F6" s="116" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G6" s="116"/>
       <c r="H6" s="116"/>
     </row>
     <row r="7">
       <c r="B7" s="116" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="C7" s="176" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D7" s="116"/>
       <c r="E7" s="177" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="F7" s="170" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="G7" s="116"/>
       <c r="H7" s="116" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="178" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C8" s="179" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D8" s="180"/>
       <c r="E8" s="178" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F8" s="181" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G8" s="182" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="H8" s="180"/>
     </row>
     <row r="9">
       <c r="B9" s="19" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="C9" s="183" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D9" s="74"/>
       <c r="E9" s="74"/>
@@ -75079,27 +75082,27 @@
     </row>
     <row r="10">
       <c r="B10" s="19" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="C10" s="146"/>
       <c r="D10" s="74"/>
       <c r="E10" s="74"/>
       <c r="F10" s="146"/>
       <c r="G10" s="172" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="H10" s="74"/>
     </row>
     <row r="11">
       <c r="B11" s="19" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C11" s="146"/>
       <c r="D11" s="74"/>
       <c r="E11" s="74"/>
       <c r="F11" s="146"/>
       <c r="G11" s="184" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="H11" s="19"/>
     </row>
@@ -75122,7 +75125,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="34" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L1" s="8"/>
     </row>
@@ -75131,16 +75134,16 @@
     </row>
     <row r="3">
       <c r="A3" s="31" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L3" s="8"/>
     </row>
     <row r="4">
       <c r="B4" s="31" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="G4" s="31" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="L4" s="8"/>
     </row>
@@ -75246,62 +75249,62 @@
     </row>
     <row r="11">
       <c r="A11" s="185" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="34" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="31" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="185" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="34" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="31" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="F19" s="83"/>
     </row>
     <row r="20">
       <c r="B20" s="34" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C20" s="36"/>
       <c r="D20" s="36"/>
       <c r="E20" s="36"/>
       <c r="F20" s="36"/>
       <c r="G20" s="34" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="H20" s="34" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="I20" s="34" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="J20" s="34" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="K20" s="34" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="34" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="G21" s="37">
         <v>2.575</v>
@@ -75309,27 +75312,27 @@
     </row>
     <row r="23">
       <c r="K23" s="34" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="31" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="H24" s="31" t="s">
         <v>170</v>
       </c>
       <c r="I24" s="31" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K24" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L24" s="31" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M24" s="31" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="25">
@@ -75348,7 +75351,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="K25" s="31" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
     </row>
     <row r="26">
@@ -75359,7 +75362,7 @@
         <v>1.19</v>
       </c>
       <c r="K26" s="31" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
     </row>
     <row r="27">
@@ -75370,7 +75373,7 @@
         <v>2.19</v>
       </c>
       <c r="K27" s="31" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28">
@@ -75381,7 +75384,7 @@
         <v>0.05</v>
       </c>
       <c r="K28" s="31" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
     </row>
     <row r="29">
@@ -75400,7 +75403,7 @@
         <v>6.42</v>
       </c>
       <c r="K30" s="51" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31">
@@ -75545,7 +75548,7 @@
         <v>0.61</v>
       </c>
       <c r="K41" s="34" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42">
@@ -75556,13 +75559,13 @@
         <v>0.69</v>
       </c>
       <c r="K42" s="31" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L42" s="31" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="M42" s="31" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
     </row>
     <row r="43">
@@ -75694,7 +75697,7 @@
         <v>0.0</v>
       </c>
       <c r="K51" s="31" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
     </row>
     <row r="52">
@@ -75722,17 +75725,17 @@
       </c>
       <c r="K54" s="74"/>
       <c r="L54" s="186" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="M54" s="187"/>
       <c r="N54" s="79" t="s">
         <v>5</v>
       </c>
       <c r="O54" s="79" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="P54" s="79" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="R54" s="15" t="s">
         <v>106</v>
@@ -75814,7 +75817,7 @@
         <v>5.86</v>
       </c>
       <c r="R57" s="31" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="S57" s="37">
         <f>SUM(P55:P74)</f>
@@ -75829,7 +75832,7 @@
         <v>0.0</v>
       </c>
       <c r="K58" s="19" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="L58" s="188">
         <v>0.57</v>
@@ -75843,7 +75846,7 @@
         <v>0.855</v>
       </c>
       <c r="P58" s="19" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
     </row>
     <row r="59">
@@ -75890,7 +75893,7 @@
         <v>0.96</v>
       </c>
       <c r="P60" s="19" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="61">
@@ -75901,7 +75904,7 @@
         <v>0.02</v>
       </c>
       <c r="K61" s="19" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="L61" s="19">
         <v>0.42</v>
@@ -75973,7 +75976,7 @@
         <v>0.0</v>
       </c>
       <c r="K64" s="19" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="L64" s="19">
         <v>0.42</v>
@@ -76117,7 +76120,7 @@
         <v>0.0</v>
       </c>
       <c r="K70" s="19" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="L70" s="19">
         <v>0.66</v>

</xml_diff>

<commit_message>
DATA. Reduzco m de ITA y aumento el de GER
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -268,7 +268,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="633" uniqueCount="342">
   <si>
     <t>id_country</t>
   </si>
@@ -901,28 +901,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>9.08</t>
+    <t>4.68</t>
   </si>
   <si>
-    <t>0.59</t>
+    <t>7.35</t>
   </si>
   <si>
-    <t>3.90</t>
+    <t>7.26</t>
   </si>
   <si>
-    <t>7.66</t>
+    <t>6.11</t>
   </si>
   <si>
-    <t>6.37</t>
+    <t>5.31</t>
   </si>
   <si>
-    <t>5.53</t>
+    <t>0.48</t>
   </si>
   <si>
-    <t>7.41</t>
+    <t>7.12</t>
   </si>
   <si>
-    <t>7.80</t>
+    <t>7.48</t>
   </si>
   <si>
     <t>Country</t>
@@ -931,142 +931,139 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>1.30</t>
+    <t>1.94</t>
   </si>
   <si>
-    <t>1.70</t>
+    <t>6.31</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>2.00</t>
+    <t>3.71</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>3.75</t>
-  </si>
-  <si>
     <t>p25</t>
   </si>
   <si>
-    <t>0.19</t>
+    <t>2.20</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>5.82</t>
+    <t>2.61</t>
   </si>
   <si>
-    <t>3.00</t>
+    <t>5.29</t>
   </si>
   <si>
-    <t>6.17</t>
+    <t>6.07</t>
   </si>
   <si>
-    <t>1.03</t>
+    <t>3.15</t>
   </si>
   <si>
-    <t>5.46</t>
+    <t>1.33</t>
   </si>
   <si>
-    <t>5.43</t>
+    <t>7.98</t>
   </si>
   <si>
-    <t>5.89</t>
+    <t>6.55</t>
   </si>
   <si>
     <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
   </si>
   <si>
-    <t>5.69</t>
+    <t>3.05</t>
   </si>
   <si>
     <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
-    <t>5.83</t>
+    <t>6.52</t>
   </si>
   <si>
     <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
   </si>
   <si>
-    <t>1.11</t>
+    <t>7.07</t>
   </si>
   <si>
     <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
   </si>
   <si>
-    <t>6.65</t>
+    <t>6.83</t>
   </si>
   <si>
     <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
   </si>
   <si>
-    <t>2.55</t>
+    <t>7.00</t>
   </si>
   <si>
     <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
   </si>
   <si>
-    <t>7.96</t>
+    <t>9.55</t>
   </si>
   <si>
-    <t>7.09</t>
+    <t>7.94</t>
   </si>
   <si>
-    <t>8.34</t>
+    <t>5.68</t>
   </si>
   <si>
-    <t>6.15</t>
+    <t>6.33</t>
   </si>
   <si>
-    <t>7.72</t>
+    <t>6.67</t>
   </si>
   <si>
-    <t>6.61</t>
+    <t>8.53</t>
   </si>
   <si>
-    <t>7.11</t>
+    <t>7.41</t>
   </si>
   <si>
-    <t>4.75</t>
+    <t>4.69</t>
   </si>
   <si>
-    <t>3.91</t>
+    <t>5.70</t>
   </si>
   <si>
-    <t>6.22</t>
+    <t>4.97</t>
   </si>
   <si>
-    <t>7.88</t>
+    <t>7.56</t>
   </si>
   <si>
-    <t>6.04</t>
+    <t>6.30</t>
   </si>
   <si>
-    <t>6.96</t>
+    <t>1.16</t>
   </si>
   <si>
-    <t>7.30</t>
+    <t>7.38</t>
   </si>
   <si>
-    <t>9.45</t>
+    <t>7.28</t>
   </si>
   <si>
-    <t>9.23</t>
+    <t>4.83</t>
   </si>
   <si>
-    <t>0.97</t>
+    <t>5.57</t>
   </si>
   <si>
-    <t>6.06</t>
+    <t>5.84</t>
   </si>
   <si>
-    <t>4.45</t>
+    <t>5.34</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -2747,7 +2744,7 @@
         <v>13</v>
       </c>
       <c r="F6" s="14">
-        <v>120.0</v>
+        <v>140.0</v>
       </c>
       <c r="G6" s="15"/>
       <c r="H6" s="15"/>
@@ -2758,7 +2755,7 @@
       </c>
       <c r="K6" s="24">
         <f>F6*'Data preparation'!$C$2</f>
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="L6" s="25" t="str">
         <f t="shared" si="2"/>
@@ -2783,7 +2780,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="14">
-        <v>80.0</v>
+        <v>60.0</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="15"/>
@@ -2794,7 +2791,7 @@
       </c>
       <c r="K7" s="24">
         <f>F7*'Data preparation'!$C$2</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="L7" s="25" t="str">
         <f t="shared" si="2"/>
@@ -7497,6 +7494,16 @@
   </conditionalFormatting>
   <conditionalFormatting sqref="J4:J8">
     <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFFFFFF"/>
+        <color rgb="FF57BB8A"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F4:F8">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -14811,7 +14818,7 @@
       <c r="C37" s="36"/>
       <c r="D37" s="111">
         <f>AVERAGE(D39:D1775)</f>
-        <v>5.438913043</v>
+        <v>5.637826087</v>
       </c>
       <c r="G37" s="34" t="s">
         <v>36</v>
@@ -14880,7 +14887,7 @@
       </c>
       <c r="D39" s="102">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>9.08</v>
+        <v>4.68</v>
       </c>
       <c r="G39" s="34" t="s">
         <v>28</v>
@@ -14918,7 +14925,7 @@
       </c>
       <c r="D40" s="102">
         <f t="shared" si="17"/>
-        <v>0.59</v>
+        <v>7.35</v>
       </c>
       <c r="G40" s="34" t="s">
         <v>24</v>
@@ -14956,7 +14963,7 @@
       </c>
       <c r="D41" s="102">
         <f t="shared" si="17"/>
-        <v>3.9</v>
+        <v>7.26</v>
       </c>
       <c r="P41" s="100">
         <v>0.0</v>
@@ -14988,7 +14995,7 @@
       </c>
       <c r="D42" s="102">
         <f t="shared" si="17"/>
-        <v>7.66</v>
+        <v>6.11</v>
       </c>
       <c r="P42" s="100">
         <v>2.0</v>
@@ -15020,7 +15027,7 @@
       </c>
       <c r="D43" s="102">
         <f t="shared" si="17"/>
-        <v>6.37</v>
+        <v>5.31</v>
       </c>
       <c r="P43" s="100">
         <v>1.0</v>
@@ -15052,7 +15059,7 @@
       </c>
       <c r="D44" s="102">
         <f t="shared" si="17"/>
-        <v>5.53</v>
+        <v>0.48</v>
       </c>
       <c r="P44" s="100">
         <v>2.0</v>
@@ -15082,7 +15089,7 @@
       </c>
       <c r="D45" s="102">
         <f t="shared" si="17"/>
-        <v>7.41</v>
+        <v>7.12</v>
       </c>
       <c r="P45" s="100">
         <v>1.0</v>
@@ -15100,7 +15107,7 @@
       </c>
       <c r="D46" s="102">
         <f t="shared" si="17"/>
-        <v>7.8</v>
+        <v>7.48</v>
       </c>
       <c r="G46" s="115" t="s">
         <v>183</v>
@@ -15124,7 +15131,7 @@
       </c>
       <c r="D47" s="102">
         <f t="shared" si="17"/>
-        <v>1.3</v>
+        <v>1.94</v>
       </c>
       <c r="G47" s="116" t="s">
         <v>37</v>
@@ -15154,7 +15161,7 @@
       </c>
       <c r="D48" s="102">
         <f t="shared" si="17"/>
-        <v>1.7</v>
+        <v>6.31</v>
       </c>
       <c r="G48" s="116" t="s">
         <v>36</v>
@@ -15191,7 +15198,7 @@
       </c>
       <c r="D49" s="102">
         <f t="shared" si="17"/>
-        <v>2</v>
+        <v>3.71</v>
       </c>
       <c r="G49" s="116" t="s">
         <v>27</v>
@@ -15224,11 +15231,11 @@
     </row>
     <row r="50">
       <c r="C50" s="114" t="s">
-        <v>190</v>
+        <v>178</v>
       </c>
       <c r="D50" s="102">
         <f t="shared" si="17"/>
-        <v>3.75</v>
+        <v>6.11</v>
       </c>
       <c r="G50" s="116" t="s">
         <v>28</v>
@@ -15237,7 +15244,7 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="26" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="K50" s="89">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -15261,11 +15268,11 @@
     </row>
     <row r="51">
       <c r="C51" s="114" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="D51" s="102">
         <f t="shared" si="17"/>
-        <v>0.19</v>
+        <v>2.2</v>
       </c>
       <c r="G51" s="116" t="s">
         <v>24</v>
@@ -15274,7 +15281,7 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="26" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="K51" s="89">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -15298,11 +15305,11 @@
     </row>
     <row r="52">
       <c r="C52" s="114" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="D52" s="102">
         <f t="shared" si="17"/>
-        <v>5.82</v>
+        <v>2.61</v>
       </c>
       <c r="P52" s="100">
         <v>0.0</v>
@@ -15322,11 +15329,11 @@
     </row>
     <row r="53">
       <c r="C53" s="114" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="D53" s="102">
         <f t="shared" si="17"/>
-        <v>3</v>
+        <v>5.29</v>
       </c>
       <c r="P53" s="100">
         <v>0.0</v>
@@ -15346,11 +15353,11 @@
     </row>
     <row r="54">
       <c r="C54" s="114" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="D54" s="102">
         <f t="shared" si="17"/>
-        <v>6.17</v>
+        <v>6.07</v>
       </c>
       <c r="P54" s="100">
         <v>2.0</v>
@@ -15370,11 +15377,11 @@
     </row>
     <row r="55">
       <c r="C55" s="114" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D55" s="102">
         <f t="shared" si="17"/>
-        <v>1.03</v>
+        <v>3.15</v>
       </c>
       <c r="P55" s="100">
         <v>0.0</v>
@@ -15394,11 +15401,11 @@
     </row>
     <row r="56">
       <c r="C56" s="114" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D56" s="102">
         <f t="shared" si="17"/>
-        <v>5.46</v>
+        <v>1.33</v>
       </c>
       <c r="P56" s="100">
         <v>0.0</v>
@@ -15418,11 +15425,11 @@
     </row>
     <row r="57">
       <c r="C57" s="114" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D57" s="102">
         <f t="shared" si="17"/>
-        <v>5.43</v>
+        <v>7.98</v>
       </c>
       <c r="P57" s="100">
         <v>2.0</v>
@@ -15442,14 +15449,14 @@
     </row>
     <row r="58">
       <c r="C58" s="114" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D58" s="102">
         <f t="shared" si="17"/>
-        <v>5.89</v>
+        <v>6.55</v>
       </c>
       <c r="G58" s="118" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="H58" s="119"/>
       <c r="P58" s="100">
@@ -15470,15 +15477,15 @@
     </row>
     <row r="59">
       <c r="C59" s="114" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D59" s="102">
         <f t="shared" si="17"/>
-        <v>5.69</v>
+        <v>3.05</v>
       </c>
       <c r="G59" s="119"/>
       <c r="H59" s="120" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="P59" s="100">
         <v>0.0</v>
@@ -15498,15 +15505,15 @@
     </row>
     <row r="60">
       <c r="C60" s="114" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D60" s="102">
         <f t="shared" si="17"/>
-        <v>5.83</v>
+        <v>6.52</v>
       </c>
       <c r="G60" s="119"/>
       <c r="H60" s="120" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="P60" s="100">
         <v>2.0</v>
@@ -15526,15 +15533,15 @@
     </row>
     <row r="61">
       <c r="C61" s="114" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D61" s="102">
         <f t="shared" si="17"/>
-        <v>1.11</v>
+        <v>7.07</v>
       </c>
       <c r="G61" s="119"/>
       <c r="H61" s="120" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="P61" s="100">
         <v>2.0</v>
@@ -15554,15 +15561,15 @@
     </row>
     <row r="62">
       <c r="C62" s="114" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D62" s="102">
         <f t="shared" si="17"/>
-        <v>6.65</v>
+        <v>6.83</v>
       </c>
       <c r="G62" s="119"/>
       <c r="H62" s="120" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="P62" s="100">
         <v>1.0</v>
@@ -15582,15 +15589,15 @@
     </row>
     <row r="63">
       <c r="C63" s="114" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D63" s="102">
         <f t="shared" si="17"/>
-        <v>2.55</v>
+        <v>7</v>
       </c>
       <c r="G63" s="119"/>
       <c r="H63" s="120" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="P63" s="100">
         <v>0.0</v>
@@ -15604,11 +15611,11 @@
     </row>
     <row r="64">
       <c r="C64" s="114" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D64" s="102">
         <f t="shared" si="17"/>
-        <v>7.96</v>
+        <v>9.55</v>
       </c>
       <c r="P64" s="100">
         <v>1.0</v>
@@ -15622,11 +15629,11 @@
     </row>
     <row r="65">
       <c r="C65" s="114" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D65" s="102">
         <f t="shared" si="17"/>
-        <v>7.09</v>
+        <v>7.94</v>
       </c>
       <c r="P65" s="100">
         <v>2.0</v>
@@ -15640,11 +15647,11 @@
     </row>
     <row r="66">
       <c r="C66" s="114" t="s">
-        <v>160</v>
+        <v>213</v>
       </c>
       <c r="D66" s="102">
         <f t="shared" si="17"/>
-        <v>7.91</v>
+        <v>5.68</v>
       </c>
       <c r="P66" s="100">
         <v>0.0</v>
@@ -15662,7 +15669,7 @@
       </c>
       <c r="D67" s="102">
         <f t="shared" si="17"/>
-        <v>8.34</v>
+        <v>6.33</v>
       </c>
       <c r="P67" s="100">
         <v>0.0</v>
@@ -15680,7 +15687,7 @@
       </c>
       <c r="D68" s="102">
         <f t="shared" si="17"/>
-        <v>6.15</v>
+        <v>6.67</v>
       </c>
       <c r="P68" s="100">
         <v>1.0</v>
@@ -15698,7 +15705,7 @@
       </c>
       <c r="D69" s="102">
         <f t="shared" si="17"/>
-        <v>7.72</v>
+        <v>8.53</v>
       </c>
       <c r="P69" s="100">
         <v>2.0</v>
@@ -15716,7 +15723,7 @@
       </c>
       <c r="D70" s="102">
         <f t="shared" si="17"/>
-        <v>6.61</v>
+        <v>7.41</v>
       </c>
       <c r="P70" s="100">
         <v>1.0</v>
@@ -15734,7 +15741,7 @@
       </c>
       <c r="D71" s="102">
         <f t="shared" si="17"/>
-        <v>7.11</v>
+        <v>4.69</v>
       </c>
       <c r="F71" s="121"/>
       <c r="P71" s="100">
@@ -15753,7 +15760,7 @@
       </c>
       <c r="D72" s="102">
         <f t="shared" si="17"/>
-        <v>4.75</v>
+        <v>5.7</v>
       </c>
       <c r="P72" s="100">
         <v>0.0</v>
@@ -15767,11 +15774,11 @@
     </row>
     <row r="73">
       <c r="C73" s="114" t="s">
-        <v>196</v>
+        <v>129</v>
       </c>
       <c r="D73" s="102">
         <f t="shared" si="17"/>
-        <v>6.17</v>
+        <v>4.92</v>
       </c>
       <c r="P73" s="100">
         <v>1.0</v>
@@ -15785,11 +15792,11 @@
     </row>
     <row r="74">
       <c r="C74" s="114" t="s">
-        <v>220</v>
+        <v>143</v>
       </c>
       <c r="D74" s="102">
         <f t="shared" si="17"/>
-        <v>3.91</v>
+        <v>6.18</v>
       </c>
       <c r="P74" s="100">
         <v>0.0</v>
@@ -15803,11 +15810,11 @@
     </row>
     <row r="75">
       <c r="C75" s="114" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D75" s="102">
         <f t="shared" si="17"/>
-        <v>6.22</v>
+        <v>4.97</v>
       </c>
       <c r="P75" s="100">
         <v>1.0</v>
@@ -15821,11 +15828,11 @@
     </row>
     <row r="76">
       <c r="C76" s="114" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="D76" s="102">
         <f t="shared" si="17"/>
-        <v>7.88</v>
+        <v>7.56</v>
       </c>
       <c r="P76" s="100">
         <v>0.0</v>
@@ -15839,11 +15846,11 @@
     </row>
     <row r="77">
       <c r="C77" s="114" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D77" s="102">
         <f t="shared" si="17"/>
-        <v>6.04</v>
+        <v>6.3</v>
       </c>
       <c r="P77" s="100">
         <v>0.0</v>
@@ -15857,11 +15864,11 @@
     </row>
     <row r="78">
       <c r="C78" s="114" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="D78" s="102">
         <f t="shared" si="17"/>
-        <v>6.96</v>
+        <v>1.16</v>
       </c>
       <c r="P78" s="100">
         <v>1.0</v>
@@ -15875,11 +15882,11 @@
     </row>
     <row r="79">
       <c r="C79" s="114" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="D79" s="102">
         <f t="shared" si="17"/>
-        <v>7.3</v>
+        <v>7.38</v>
       </c>
       <c r="P79" s="100">
         <v>2.0</v>
@@ -15893,11 +15900,11 @@
     </row>
     <row r="80">
       <c r="C80" s="114" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D80" s="102">
         <f t="shared" si="17"/>
-        <v>9.45</v>
+        <v>7.28</v>
       </c>
       <c r="P80" s="100">
         <v>1.0</v>
@@ -15911,11 +15918,11 @@
     </row>
     <row r="81">
       <c r="C81" s="114" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D81" s="102">
         <f t="shared" si="17"/>
-        <v>9.23</v>
+        <v>4.83</v>
       </c>
       <c r="P81" s="100">
         <v>2.0</v>
@@ -15929,11 +15936,11 @@
     </row>
     <row r="82">
       <c r="C82" s="114" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="D82" s="102">
         <f t="shared" si="17"/>
-        <v>0.97</v>
+        <v>5.57</v>
       </c>
       <c r="P82" s="100">
         <v>1.0</v>
@@ -15947,11 +15954,11 @@
     </row>
     <row r="83">
       <c r="C83" s="114" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="D83" s="102">
         <f t="shared" si="17"/>
-        <v>6.06</v>
+        <v>5.84</v>
       </c>
       <c r="P83" s="100">
         <v>0.0</v>
@@ -15965,11 +15972,11 @@
     </row>
     <row r="84">
       <c r="C84" s="114" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D84" s="102">
         <f t="shared" si="17"/>
-        <v>4.45</v>
+        <v>5.34</v>
       </c>
       <c r="P84" s="100">
         <v>1.0</v>
@@ -39051,14 +39058,14 @@
     <row r="1">
       <c r="A1" s="126"/>
       <c r="B1" s="127" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C1" s="128"/>
       <c r="D1" s="128"/>
       <c r="E1" s="128"/>
       <c r="F1" s="128"/>
       <c r="G1" s="129" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="H1" s="128"/>
       <c r="I1" s="128"/>
@@ -39092,19 +39099,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="131" t="s">
+        <v>232</v>
+      </c>
+      <c r="C2" s="132" t="s">
         <v>233</v>
-      </c>
-      <c r="C2" s="132" t="s">
-        <v>234</v>
       </c>
       <c r="D2" s="132" t="s">
         <v>171</v>
       </c>
       <c r="E2" s="132" t="s">
+        <v>234</v>
+      </c>
+      <c r="F2" s="133" t="s">
         <v>235</v>
-      </c>
-      <c r="F2" s="133" t="s">
-        <v>236</v>
       </c>
       <c r="G2" s="131">
         <v>1.0</v>
@@ -39116,30 +39123,30 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="132" t="s">
+        <v>236</v>
+      </c>
+      <c r="K2" s="134" t="s">
         <v>237</v>
       </c>
-      <c r="K2" s="134" t="s">
+      <c r="L2" s="132" t="s">
         <v>238</v>
       </c>
-      <c r="L2" s="132" t="s">
+      <c r="M2" s="135" t="s">
         <v>239</v>
       </c>
-      <c r="M2" s="135" t="s">
+      <c r="N2" s="116" t="s">
         <v>240</v>
       </c>
-      <c r="N2" s="116" t="s">
+      <c r="O2" s="116" t="s">
         <v>241</v>
       </c>
-      <c r="O2" s="116" t="s">
+      <c r="P2" s="116" t="s">
         <v>242</v>
-      </c>
-      <c r="P2" s="116" t="s">
-        <v>243</v>
       </c>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
       <c r="S2" s="94" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="T2" s="7"/>
       <c r="U2" s="7"/>
@@ -39229,7 +39236,7 @@
       <c r="Q4" s="7"/>
       <c r="R4" s="7"/>
       <c r="S4" s="141" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="T4" s="142"/>
       <c r="Z4" s="34"/>
@@ -39265,7 +39272,7 @@
       <c r="P5" s="144"/>
       <c r="S5" s="142"/>
       <c r="T5" s="145" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6">
@@ -39298,11 +39305,11 @@
       <c r="R6" s="7"/>
       <c r="S6" s="142"/>
       <c r="T6" s="145" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="Z6" s="83"/>
       <c r="AD6" s="26" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="7">
@@ -39332,7 +39339,7 @@
       <c r="O7" s="74"/>
       <c r="P7" s="147"/>
       <c r="AD7" s="145" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="AE7" s="142"/>
       <c r="AF7" s="142"/>
@@ -39365,11 +39372,11 @@
       <c r="O8" s="74"/>
       <c r="P8" s="147"/>
       <c r="S8" s="145" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="AA8" s="83"/>
       <c r="AD8" s="145" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="9">
@@ -39568,7 +39575,7 @@
       <c r="O15" s="74"/>
       <c r="P15" s="147"/>
       <c r="S15" s="26" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="16">
@@ -39681,7 +39688,7 @@
       <c r="Q19" s="7"/>
       <c r="R19" s="7"/>
       <c r="S19" s="26" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="20">
@@ -39965,7 +39972,7 @@
       <c r="E27" s="7"/>
       <c r="F27" s="7"/>
       <c r="G27" s="152" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="H27" s="7"/>
       <c r="I27" s="7"/>
@@ -40050,7 +40057,7 @@
       <c r="B29" s="7"/>
       <c r="C29" s="7"/>
       <c r="D29" s="4" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -40072,10 +40079,10 @@
       </c>
       <c r="K29" s="7"/>
       <c r="L29" s="94" t="s">
+        <v>255</v>
+      </c>
+      <c r="M29" s="94" t="s">
         <v>256</v>
-      </c>
-      <c r="M29" s="94" t="s">
-        <v>257</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -40175,7 +40182,7 @@
       </c>
       <c r="R31" s="7"/>
       <c r="S31" s="94" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="T31" s="7"/>
       <c r="U31" s="7"/>
@@ -40237,7 +40244,7 @@
       <c r="E33" s="7"/>
       <c r="F33" s="7"/>
       <c r="G33" s="98" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="J33" s="7"/>
       <c r="K33" s="7"/>
@@ -40251,10 +40258,10 @@
       <c r="P33" s="7"/>
       <c r="R33" s="7"/>
       <c r="T33" s="51" t="s">
+        <v>259</v>
+      </c>
+      <c r="W33" s="26" t="s">
         <v>260</v>
-      </c>
-      <c r="W33" s="26" t="s">
-        <v>261</v>
       </c>
       <c r="AA33" s="34"/>
       <c r="AD33" s="7"/>
@@ -40297,7 +40304,7 @@
         <v>1626.0</v>
       </c>
       <c r="U34" s="92" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="W34" s="26">
         <v>5193.0</v>
@@ -40342,7 +40349,7 @@
         <v>4176.0</v>
       </c>
       <c r="U35" s="92" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="W35" s="26">
         <v>4863.0</v>
@@ -40440,7 +40447,7 @@
       <c r="D38" s="7"/>
       <c r="E38" s="7"/>
       <c r="F38" s="4" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="G38" s="155">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>
@@ -40642,7 +40649,7 @@
       <c r="Q45" s="7"/>
       <c r="R45" s="7"/>
       <c r="T45" s="145" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="AD45" s="7"/>
       <c r="AE45" s="7"/>
@@ -40806,7 +40813,7 @@
         <v>11</v>
       </c>
       <c r="AG49" s="61" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="50">
@@ -40971,7 +40978,7 @@
         <v>13.03594852814783</v>
       </c>
       <c r="AG52" s="61" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="53">
@@ -41032,7 +41039,7 @@
         <v>6.291840048860032</v>
       </c>
       <c r="AG53" s="61" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="54">
@@ -41093,7 +41100,7 @@
         <v>2.7243520649411117</v>
       </c>
       <c r="AG54" s="61" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="55">
@@ -41154,7 +41161,7 @@
         <v>2.1429979739456915</v>
       </c>
       <c r="AG55" s="61" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="56">
@@ -41215,7 +41222,7 @@
         <v>3.98032040346951</v>
       </c>
       <c r="AG56" s="61" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57">
@@ -41438,10 +41445,10 @@
       <c r="R62" s="7"/>
       <c r="S62" s="7"/>
       <c r="U62" s="26" t="s">
+        <v>266</v>
+      </c>
+      <c r="V62" s="26" t="s">
         <v>267</v>
-      </c>
-      <c r="V62" s="26" t="s">
-        <v>268</v>
       </c>
       <c r="AC62" s="7"/>
       <c r="AD62" s="7"/>
@@ -41483,7 +41490,7 @@
         <v>2165.0</v>
       </c>
       <c r="W63" s="26" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="AC63" s="7"/>
       <c r="AD63" s="7"/>
@@ -42117,7 +42124,7 @@
       <c r="R79" s="7"/>
       <c r="S79" s="7"/>
       <c r="T79" s="94" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="U79" s="7"/>
       <c r="V79" s="7"/>
@@ -42158,7 +42165,7 @@
       <c r="R80" s="7"/>
       <c r="S80" s="7"/>
       <c r="T80" s="26" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="U80" s="18"/>
       <c r="V80" s="18"/>
@@ -74919,146 +74926,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="26" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="7"/>
       <c r="C2" s="165" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="E2" s="166"/>
       <c r="F2" s="94" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H2" s="166"/>
     </row>
     <row r="3">
       <c r="B3" s="115" t="s">
+        <v>274</v>
+      </c>
+      <c r="C3" s="167" t="s">
         <v>275</v>
       </c>
-      <c r="C3" s="167" t="s">
+      <c r="D3" s="115" t="s">
         <v>276</v>
-      </c>
-      <c r="D3" s="115" t="s">
-        <v>277</v>
       </c>
       <c r="E3" s="168" t="s">
         <v>97</v>
       </c>
       <c r="F3" s="115" t="s">
+        <v>277</v>
+      </c>
+      <c r="G3" s="115" t="s">
         <v>278</v>
       </c>
-      <c r="G3" s="115" t="s">
+      <c r="H3" s="115" t="s">
         <v>279</v>
-      </c>
-      <c r="H3" s="115" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="169" t="s">
+        <v>280</v>
+      </c>
+      <c r="C4" s="170" t="s">
         <v>281</v>
       </c>
-      <c r="C4" s="170" t="s">
+      <c r="D4" s="116" t="s">
         <v>282</v>
       </c>
-      <c r="D4" s="116" t="s">
+      <c r="E4" s="171" t="s">
         <v>283</v>
       </c>
-      <c r="E4" s="171" t="s">
+      <c r="F4" s="172" t="s">
         <v>284</v>
       </c>
-      <c r="F4" s="172" t="s">
+      <c r="G4" s="172" t="s">
         <v>285</v>
-      </c>
-      <c r="G4" s="172" t="s">
-        <v>286</v>
       </c>
       <c r="H4" s="116"/>
     </row>
     <row r="5">
       <c r="B5" s="169" t="s">
+        <v>286</v>
+      </c>
+      <c r="C5" s="173" t="s">
         <v>287</v>
-      </c>
-      <c r="C5" s="173" t="s">
-        <v>288</v>
       </c>
       <c r="D5" s="126"/>
       <c r="E5" s="171" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F5" s="174" t="s">
+        <v>288</v>
+      </c>
+      <c r="G5" s="175" t="s">
         <v>289</v>
-      </c>
-      <c r="G5" s="175" t="s">
-        <v>290</v>
       </c>
       <c r="H5" s="116"/>
     </row>
     <row r="6">
       <c r="B6" s="169" t="s">
+        <v>290</v>
+      </c>
+      <c r="C6" s="170" t="s">
+        <v>281</v>
+      </c>
+      <c r="D6" s="116" t="s">
         <v>291</v>
       </c>
-      <c r="C6" s="170" t="s">
-        <v>282</v>
-      </c>
-      <c r="D6" s="116" t="s">
-        <v>292</v>
-      </c>
       <c r="E6" s="171" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="F6" s="116" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="G6" s="116"/>
       <c r="H6" s="116"/>
     </row>
     <row r="7">
       <c r="B7" s="116" t="s">
+        <v>292</v>
+      </c>
+      <c r="C7" s="176" t="s">
         <v>293</v>
-      </c>
-      <c r="C7" s="176" t="s">
-        <v>294</v>
       </c>
       <c r="D7" s="116"/>
       <c r="E7" s="177" t="s">
+        <v>294</v>
+      </c>
+      <c r="F7" s="170" t="s">
         <v>295</v>
-      </c>
-      <c r="F7" s="170" t="s">
-        <v>296</v>
       </c>
       <c r="G7" s="116"/>
       <c r="H7" s="116" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="178" t="s">
+        <v>297</v>
+      </c>
+      <c r="C8" s="179" t="s">
         <v>298</v>
-      </c>
-      <c r="C8" s="179" t="s">
-        <v>299</v>
       </c>
       <c r="D8" s="180"/>
       <c r="E8" s="178" t="s">
+        <v>299</v>
+      </c>
+      <c r="F8" s="181" t="s">
         <v>300</v>
       </c>
-      <c r="F8" s="181" t="s">
+      <c r="G8" s="182" t="s">
         <v>301</v>
-      </c>
-      <c r="G8" s="182" t="s">
-        <v>302</v>
       </c>
       <c r="H8" s="180"/>
     </row>
     <row r="9">
       <c r="B9" s="19" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C9" s="183" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D9" s="74"/>
       <c r="E9" s="74"/>
@@ -75068,27 +75075,27 @@
     </row>
     <row r="10">
       <c r="B10" s="19" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="C10" s="146"/>
       <c r="D10" s="74"/>
       <c r="E10" s="74"/>
       <c r="F10" s="146"/>
       <c r="G10" s="172" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H10" s="74"/>
     </row>
     <row r="11">
       <c r="B11" s="19" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C11" s="146"/>
       <c r="D11" s="74"/>
       <c r="E11" s="74"/>
       <c r="F11" s="146"/>
       <c r="G11" s="184" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H11" s="19"/>
     </row>
@@ -75111,7 +75118,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="34" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="L1" s="8"/>
     </row>
@@ -75120,16 +75127,16 @@
     </row>
     <row r="3">
       <c r="A3" s="26" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="L3" s="8"/>
     </row>
     <row r="4">
       <c r="B4" s="26" t="s">
+        <v>308</v>
+      </c>
+      <c r="G4" s="26" t="s">
         <v>309</v>
-      </c>
-      <c r="G4" s="26" t="s">
-        <v>310</v>
       </c>
       <c r="L4" s="8"/>
     </row>
@@ -75235,62 +75242,62 @@
     </row>
     <row r="11">
       <c r="A11" s="185" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="34" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="26" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="185" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="34" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="26" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F19" s="83"/>
     </row>
     <row r="20">
       <c r="B20" s="34" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C20" s="36"/>
       <c r="D20" s="36"/>
       <c r="E20" s="36"/>
       <c r="F20" s="36"/>
       <c r="G20" s="34" t="s">
+        <v>317</v>
+      </c>
+      <c r="H20" s="34" t="s">
         <v>318</v>
       </c>
-      <c r="H20" s="34" t="s">
+      <c r="I20" s="34" t="s">
         <v>319</v>
       </c>
-      <c r="I20" s="34" t="s">
+      <c r="J20" s="34" t="s">
         <v>320</v>
       </c>
-      <c r="J20" s="34" t="s">
+      <c r="K20" s="34" t="s">
         <v>321</v>
-      </c>
-      <c r="K20" s="34" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="34" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="G21" s="37">
         <v>2.575</v>
@@ -75298,27 +75305,27 @@
     </row>
     <row r="23">
       <c r="K23" s="34" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="H24" s="26" t="s">
         <v>171</v>
       </c>
       <c r="I24" s="26" t="s">
+        <v>325</v>
+      </c>
+      <c r="K24" s="26" t="s">
         <v>326</v>
       </c>
-      <c r="K24" s="26" t="s">
+      <c r="L24" s="26" t="s">
         <v>327</v>
       </c>
-      <c r="L24" s="26" t="s">
+      <c r="M24" s="26" t="s">
         <v>328</v>
-      </c>
-      <c r="M24" s="26" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="25">
@@ -75337,7 +75344,7 @@
         <v>#DIV/0!</v>
       </c>
       <c r="K25" s="26" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="26">
@@ -75348,7 +75355,7 @@
         <v>1.19</v>
       </c>
       <c r="K26" s="26" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="27">
@@ -75359,7 +75366,7 @@
         <v>2.19</v>
       </c>
       <c r="K27" s="26" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28">
@@ -75370,7 +75377,7 @@
         <v>0.05</v>
       </c>
       <c r="K28" s="26" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="29">
@@ -75389,7 +75396,7 @@
         <v>6.42</v>
       </c>
       <c r="K30" s="51" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="31">
@@ -75534,7 +75541,7 @@
         <v>0.61</v>
       </c>
       <c r="K41" s="34" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="42">
@@ -75545,13 +75552,13 @@
         <v>0.69</v>
       </c>
       <c r="K42" s="26" t="s">
+        <v>326</v>
+      </c>
+      <c r="L42" s="26" t="s">
         <v>327</v>
       </c>
-      <c r="L42" s="26" t="s">
+      <c r="M42" s="26" t="s">
         <v>328</v>
-      </c>
-      <c r="M42" s="26" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="43">
@@ -75683,7 +75690,7 @@
         <v>0.0</v>
       </c>
       <c r="K51" s="26" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="52">
@@ -75711,17 +75718,17 @@
       </c>
       <c r="K54" s="74"/>
       <c r="L54" s="186" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="M54" s="187"/>
       <c r="N54" s="79" t="s">
         <v>5</v>
       </c>
       <c r="O54" s="79" t="s">
+        <v>337</v>
+      </c>
+      <c r="P54" s="79" t="s">
         <v>338</v>
-      </c>
-      <c r="P54" s="79" t="s">
-        <v>339</v>
       </c>
       <c r="R54" s="15" t="s">
         <v>107</v>
@@ -75803,7 +75810,7 @@
         <v>5.86</v>
       </c>
       <c r="R57" s="26" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="S57" s="37">
         <f>SUM(P55:P74)</f>
@@ -75818,7 +75825,7 @@
         <v>0.0</v>
       </c>
       <c r="K58" s="19" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="L58" s="188">
         <v>0.57</v>
@@ -75832,7 +75839,7 @@
         <v>0.855</v>
       </c>
       <c r="P58" s="19" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="59">
@@ -75879,7 +75886,7 @@
         <v>0.96</v>
       </c>
       <c r="P60" s="19" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="61">
@@ -75890,7 +75897,7 @@
         <v>0.02</v>
       </c>
       <c r="K61" s="19" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="L61" s="19">
         <v>0.42</v>
@@ -75962,7 +75969,7 @@
         <v>0.0</v>
       </c>
       <c r="K64" s="19" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="L64" s="19">
         <v>0.42</v>
@@ -76106,7 +76113,7 @@
         <v>0.0</v>
       </c>
       <c r="K70" s="19" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="L70" s="19">
         <v>0.66</v>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones tras cambio de modelos (priorizo mas f1_score_away y f1_score_draw que error)
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -2639,7 +2639,7 @@
         <v>45739.0</v>
       </c>
       <c r="D4" s="13">
-        <v>1071.0</v>
+        <v>1145.0</v>
       </c>
       <c r="E4" s="13" t="s">
         <v>9</v>
@@ -2668,7 +2668,7 @@
         <v>45739.0</v>
       </c>
       <c r="D5" s="13">
-        <v>918.0</v>
+        <v>1083.0</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>9</v>
@@ -2697,7 +2697,7 @@
         <v>45739.0</v>
       </c>
       <c r="D6" s="13">
-        <v>385.0</v>
+        <v>457.0</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>9</v>
@@ -2726,7 +2726,7 @@
         <v>45739.0</v>
       </c>
       <c r="D7" s="13">
-        <v>955.0</v>
+        <v>907.0</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>9</v>
@@ -2754,7 +2754,7 @@
         <v>45740.0</v>
       </c>
       <c r="D8" s="13">
-        <v>1135.0</v>
+        <v>649.0</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>9</v>

</xml_diff>

<commit_message>
DATA. Actualizo predicciones de FRA (x cambio de modelo)
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -360,7 +360,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="785" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="433">
   <si>
     <t>id_country</t>
   </si>
@@ -585,10 +585,13 @@
     <t>metricas de test aceptables</t>
   </si>
   <si>
-    <t>gran roi en test y mayor roi en assess</t>
+    <t>gran roi en test y mayor roi en assess PERO mal error y las probas de prod no me gustan</t>
   </si>
   <si>
     <t>alto roi en assess + roi aceptable en test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gran roi en test y no tan buen assess </t>
   </si>
   <si>
     <t>roi bajo</t>
@@ -1162,28 +1165,28 @@
     <t>Stake promedio</t>
   </si>
   <si>
-    <t>1.52</t>
+    <t>2.17</t>
   </si>
   <si>
-    <t>0.33</t>
+    <t>1.66</t>
   </si>
   <si>
-    <t>1.43</t>
+    <t>1.96</t>
   </si>
   <si>
-    <t>0.28</t>
+    <t>1.28</t>
   </si>
   <si>
-    <t>0.92</t>
+    <t>2.78</t>
   </si>
   <si>
-    <t>1.65</t>
+    <t>2.26</t>
   </si>
   <si>
-    <t>2.05</t>
+    <t>2.45</t>
   </si>
   <si>
-    <t>1.93</t>
+    <t>1.78</t>
   </si>
   <si>
     <t>Country</t>
@@ -1192,253 +1195,253 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>1.60</t>
+    <t>3.74</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>0.77</t>
+    <t>4.00</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>6.54</t>
+    <t>3.73</t>
   </si>
   <si>
     <t>p25</t>
   </si>
   <si>
-    <t>5.57</t>
+    <t>4.30</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
-    <t>4.51</t>
+    <t>5.93</t>
   </si>
   <si>
-    <t>0.84</t>
+    <t>3.66</t>
   </si>
   <si>
-    <t>0.82</t>
+    <t>4.11</t>
   </si>
   <si>
-    <t>5.71</t>
+    <t>5.40</t>
   </si>
   <si>
-    <t>6.89</t>
+    <t>5.97</t>
+  </si>
+  <si>
+    <t>4.34</t>
+  </si>
+  <si>
+    <t>1.81</t>
+  </si>
+  <si>
+    <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
+  </si>
+  <si>
+    <t>2.99</t>
+  </si>
+  <si>
+    <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
+  </si>
+  <si>
+    <t>4.84</t>
+  </si>
+  <si>
+    <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
+  </si>
+  <si>
+    <t>1.40</t>
+  </si>
+  <si>
+    <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
+  </si>
+  <si>
+    <t>3.34</t>
+  </si>
+  <si>
+    <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
+  </si>
+  <si>
+    <t>2.79</t>
+  </si>
+  <si>
+    <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
+  </si>
+  <si>
+    <t>5.39</t>
+  </si>
+  <si>
+    <t>7.99</t>
+  </si>
+  <si>
+    <t>7.76</t>
+  </si>
+  <si>
+    <t>5.24</t>
+  </si>
+  <si>
+    <t>7.66</t>
+  </si>
+  <si>
+    <t>5.19</t>
+  </si>
+  <si>
+    <t>3.76</t>
+  </si>
+  <si>
+    <t>4.44</t>
+  </si>
+  <si>
+    <t>4.86</t>
+  </si>
+  <si>
+    <t>3.33</t>
+  </si>
+  <si>
+    <t>4.29</t>
+  </si>
+  <si>
+    <t>4.57</t>
+  </si>
+  <si>
+    <t>4.61</t>
+  </si>
+  <si>
+    <t>3.16</t>
+  </si>
+  <si>
+    <t>1.90</t>
+  </si>
+  <si>
+    <t>2.73</t>
+  </si>
+  <si>
+    <t>3.44</t>
+  </si>
+  <si>
+    <t>1.24</t>
+  </si>
+  <si>
+    <t>2.33</t>
+  </si>
+  <si>
+    <t>2.32</t>
+  </si>
+  <si>
+    <t>2.57</t>
+  </si>
+  <si>
+    <t>2.46</t>
+  </si>
+  <si>
+    <t>7.39</t>
+  </si>
+  <si>
+    <t>6.49</t>
+  </si>
+  <si>
+    <t>10.63</t>
+  </si>
+  <si>
+    <t>7.30</t>
+  </si>
+  <si>
+    <t>6.60</t>
+  </si>
+  <si>
+    <t>1.74</t>
+  </si>
+  <si>
+    <t>1.94</t>
+  </si>
+  <si>
+    <t>1.65</t>
+  </si>
+  <si>
+    <t>3.32</t>
+  </si>
+  <si>
+    <t>1.62</t>
+  </si>
+  <si>
+    <t>1.91</t>
+  </si>
+  <si>
+    <t>1.76</t>
+  </si>
+  <si>
+    <t>1.89</t>
+  </si>
+  <si>
+    <t>1.69</t>
+  </si>
+  <si>
+    <t>6.59</t>
+  </si>
+  <si>
+    <t>3.23</t>
+  </si>
+  <si>
+    <t>2.66</t>
+  </si>
+  <si>
+    <t>0.33</t>
+  </si>
+  <si>
+    <t>1.99</t>
+  </si>
+  <si>
+    <t>2.01</t>
+  </si>
+  <si>
+    <t>3.56</t>
+  </si>
+  <si>
+    <t>1.97</t>
+  </si>
+  <si>
+    <t>2.93</t>
   </si>
   <si>
     <t>3.95</t>
   </si>
   <si>
-    <t>1.63</t>
+    <t>3.27</t>
   </si>
   <si>
-    <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
+    <t>0.36</t>
   </si>
   <si>
-    <t>2.69</t>
+    <t>0.37</t>
   </si>
   <si>
-    <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
+    <t>2.07</t>
   </si>
   <si>
-    <t>4.35</t>
+    <t>2.37</t>
   </si>
   <si>
-    <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
+    <t>3.17</t>
   </si>
   <si>
-    <t>1.26</t>
+    <t>3.47</t>
   </si>
   <si>
-    <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
+    <t>5.77</t>
   </si>
   <si>
-    <t>5.01</t>
+    <t>5.87</t>
   </si>
   <si>
-    <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
-  </si>
-  <si>
-    <t>4.18</t>
-  </si>
-  <si>
-    <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
-  </si>
-  <si>
-    <t>8.08</t>
-  </si>
-  <si>
-    <t>11.99</t>
-  </si>
-  <si>
-    <t>11.64</t>
-  </si>
-  <si>
-    <t>7.86</t>
-  </si>
-  <si>
-    <t>11.50</t>
-  </si>
-  <si>
-    <t>7.78</t>
-  </si>
-  <si>
-    <t>5.65</t>
-  </si>
-  <si>
-    <t>6.67</t>
-  </si>
-  <si>
-    <t>7.30</t>
-  </si>
-  <si>
-    <t>5.00</t>
-  </si>
-  <si>
-    <t>6.44</t>
-  </si>
-  <si>
-    <t>4.11</t>
-  </si>
-  <si>
-    <t>4.15</t>
-  </si>
-  <si>
-    <t>2.52</t>
-  </si>
-  <si>
-    <t>2.84</t>
-  </si>
-  <si>
-    <t>1.71</t>
-  </si>
-  <si>
-    <t>2.46</t>
-  </si>
-  <si>
-    <t>3.90</t>
-  </si>
-  <si>
-    <t>3.10</t>
-  </si>
-  <si>
-    <t>1.11</t>
-  </si>
-  <si>
-    <t>2.10</t>
-  </si>
-  <si>
-    <t>3.48</t>
-  </si>
-  <si>
-    <t>3.86</t>
-  </si>
-  <si>
-    <t>6.65</t>
-  </si>
-  <si>
-    <t>5.84</t>
-  </si>
-  <si>
-    <t>9.57</t>
-  </si>
-  <si>
-    <t>6.57</t>
-  </si>
-  <si>
-    <t>0.52</t>
-  </si>
-  <si>
-    <t>2.91</t>
-  </si>
-  <si>
-    <t>2.48</t>
-  </si>
-  <si>
-    <t>4.98</t>
-  </si>
-  <si>
-    <t>0.49</t>
-  </si>
-  <si>
-    <t>3.26</t>
-  </si>
-  <si>
-    <t>2.87</t>
-  </si>
-  <si>
-    <t>0.57</t>
-  </si>
-  <si>
-    <t>2.53</t>
-  </si>
-  <si>
-    <t>5.93</t>
-  </si>
-  <si>
-    <t>4.84</t>
-  </si>
-  <si>
-    <t>3.99</t>
-  </si>
-  <si>
-    <t>2.99</t>
-  </si>
-  <si>
-    <t>3.01</t>
-  </si>
-  <si>
-    <t>5.35</t>
-  </si>
-  <si>
-    <t>2.95</t>
-  </si>
-  <si>
-    <t>3.07</t>
-  </si>
-  <si>
-    <t>2.64</t>
-  </si>
-  <si>
-    <t>3.56</t>
-  </si>
-  <si>
-    <t>2.93</t>
+    <t>5.49</t>
   </si>
   <si>
     <t>2.24</t>
-  </si>
-  <si>
-    <t>0.32</t>
-  </si>
-  <si>
-    <t>1.86</t>
-  </si>
-  <si>
-    <t>2.13</t>
-  </si>
-  <si>
-    <t>2.85</t>
-  </si>
-  <si>
-    <t>5.20</t>
-  </si>
-  <si>
-    <t>5.28</t>
-  </si>
-  <si>
-    <t>4.94</t>
-  </si>
-  <si>
-    <t>1.96</t>
-  </si>
-  <si>
-    <t>2.23</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -3108,23 +3111,23 @@
         <v>45739.0</v>
       </c>
       <c r="D5" s="11">
-        <v>1134.0</v>
+        <v>1129.0</v>
       </c>
       <c r="E5" s="11" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="17">
+        <v>40.0</v>
+      </c>
+      <c r="G5" s="17">
         <v>25.0</v>
-      </c>
-      <c r="G5" s="17">
-        <v>35.0</v>
       </c>
       <c r="H5" s="17">
         <v>45.0</v>
       </c>
       <c r="I5" s="12">
         <f t="shared" si="1"/>
-        <v>35</v>
+        <v>36.66666667</v>
       </c>
     </row>
     <row r="6">
@@ -8279,7 +8282,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="48" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L1" s="6"/>
     </row>
@@ -8288,16 +8291,16 @@
     </row>
     <row r="3">
       <c r="A3" s="38" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="L3" s="6"/>
     </row>
     <row r="4">
       <c r="B4" s="38" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="G4" s="38" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="L4" s="6"/>
     </row>
@@ -8403,62 +8406,62 @@
     </row>
     <row r="11">
       <c r="A11" s="203" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="48" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="38" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="203" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="48" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="38" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="F19" s="98"/>
     </row>
     <row r="20">
       <c r="B20" s="48" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="C20" s="50"/>
       <c r="D20" s="50"/>
       <c r="E20" s="50"/>
       <c r="F20" s="50"/>
       <c r="G20" s="48" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="H20" s="48" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="I20" s="48" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="J20" s="48" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K20" s="48" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="48" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="G21" s="52">
         <v>2.575</v>
@@ -8466,27 +8469,27 @@
     </row>
     <row r="23">
       <c r="K23" s="48" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="38" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="H24" s="38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I24" s="38" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="K24" s="38" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="L24" s="38" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M24" s="38" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="25">
@@ -8505,7 +8508,7 @@
         <v>#REF!</v>
       </c>
       <c r="K25" s="38" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
     </row>
     <row r="26">
@@ -8516,7 +8519,7 @@
         <v>1.19</v>
       </c>
       <c r="K26" s="38" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
     </row>
     <row r="27">
@@ -8527,7 +8530,7 @@
         <v>2.19</v>
       </c>
       <c r="K27" s="38" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
     </row>
     <row r="28">
@@ -8538,7 +8541,7 @@
         <v>0.05</v>
       </c>
       <c r="K28" s="38" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
     </row>
     <row r="29">
@@ -8557,7 +8560,7 @@
         <v>6.42</v>
       </c>
       <c r="K30" s="68" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="31">
@@ -8574,7 +8577,7 @@
         <v>3</v>
       </c>
       <c r="M31" s="38" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="32">
@@ -8702,7 +8705,7 @@
         <v>0.61</v>
       </c>
       <c r="K41" s="48" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="42">
@@ -8713,13 +8716,13 @@
         <v>0.69</v>
       </c>
       <c r="K42" s="38" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="L42" s="38" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="M42" s="38" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
     </row>
     <row r="43">
@@ -8851,7 +8854,7 @@
         <v>0.0</v>
       </c>
       <c r="K51" s="38" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
     </row>
     <row r="52">
@@ -8879,20 +8882,20 @@
       </c>
       <c r="K54" s="90"/>
       <c r="L54" s="204" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="M54" s="205"/>
       <c r="N54" s="95" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="O54" s="95" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="P54" s="95" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="R54" s="17" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="S54" s="98">
         <v>0.15</v>
@@ -8906,7 +8909,7 @@
         <v>-0.12</v>
       </c>
       <c r="K55" s="14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="L55" s="206">
         <v>0.76</v>
@@ -8971,7 +8974,7 @@
         <v>5.86</v>
       </c>
       <c r="R57" s="38" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="S57" s="52">
         <f>SUM(P55:P74)</f>
@@ -8986,7 +8989,7 @@
         <v>0.0</v>
       </c>
       <c r="K58" s="14" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="L58" s="206">
         <v>0.57</v>
@@ -9000,7 +9003,7 @@
         <v>0.855</v>
       </c>
       <c r="P58" s="14" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
     </row>
     <row r="59">
@@ -9047,7 +9050,7 @@
         <v>0.96</v>
       </c>
       <c r="P60" s="14" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
     </row>
     <row r="61">
@@ -9058,7 +9061,7 @@
         <v>0.02</v>
       </c>
       <c r="K61" s="14" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="L61" s="14">
         <v>0.42</v>
@@ -9130,7 +9133,7 @@
         <v>0.0</v>
       </c>
       <c r="K64" s="14" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="L64" s="14">
         <v>0.42</v>
@@ -9274,7 +9277,7 @@
         <v>0.0</v>
       </c>
       <c r="K70" s="14" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="L70" s="14">
         <v>0.66</v>
@@ -13145,11 +13148,17 @@
       <c r="A33" s="41"/>
       <c r="C33" s="41"/>
       <c r="D33" s="41"/>
+      <c r="J33" s="38">
+        <v>1129.0</v>
+      </c>
+      <c r="K33" s="38" t="s">
+        <v>72</v>
+      </c>
       <c r="R33" s="38">
         <v>544.0</v>
       </c>
       <c r="S33" s="38" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34">
@@ -13161,10 +13170,10 @@
     <row r="35">
       <c r="A35" s="41"/>
       <c r="C35" s="48" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D35" s="38" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="36">
@@ -13279,14 +13288,14 @@
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="AC2:AG2"/>
+    <mergeCell ref="AI2:AL2"/>
     <mergeCell ref="AM2:AQ2"/>
-    <mergeCell ref="AI2:AL2"/>
-    <mergeCell ref="U2:X2"/>
-    <mergeCell ref="R2:T2"/>
-    <mergeCell ref="J2:L2"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:H2"/>
+    <mergeCell ref="J2:L2"/>
     <mergeCell ref="M2:P2"/>
+    <mergeCell ref="R2:T2"/>
+    <mergeCell ref="U2:X2"/>
     <mergeCell ref="Z2:AB2"/>
   </mergeCells>
   <conditionalFormatting sqref="B6:H6">
@@ -13620,13 +13629,13 @@
     </row>
     <row r="11">
       <c r="E11" s="62" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="L11" s="38" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="M11" s="55" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="N11" s="40" t="s">
         <v>21</v>
@@ -13636,10 +13645,10 @@
     </row>
     <row r="12">
       <c r="E12" s="62" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="L12" s="38" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="M12" s="55" t="s">
         <v>19</v>
@@ -13901,37 +13910,37 @@
     </row>
     <row r="24">
       <c r="C24" s="48" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25">
       <c r="C25" s="58" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26">
       <c r="C26" s="66" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27">
       <c r="C27" s="67" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28">
       <c r="C28" s="65" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="30">
       <c r="C30" s="68" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="31">
       <c r="C31" s="48" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="L31" s="48" t="s">
         <v>20</v>
@@ -15923,7 +15932,7 @@
     </row>
     <row r="63">
       <c r="C63" s="48" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="65">
@@ -15943,25 +15952,25 @@
         <v>4</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I65" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J65" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K65" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L65" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="M65" s="78" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="N65" s="79" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="66">
@@ -16226,7 +16235,7 @@
     </row>
     <row r="76">
       <c r="C76" s="48" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="77">
@@ -16246,16 +16255,16 @@
         <v>4</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I77" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J77" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K77" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="L77" s="4" t="s">
         <v>5</v>
@@ -16271,10 +16280,10 @@
         <v>8</v>
       </c>
       <c r="Q77" s="78" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="R77" s="79" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="78">
@@ -16600,7 +16609,7 @@
     </row>
     <row r="94">
       <c r="C94" s="38" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
     </row>
     <row r="96">
@@ -16620,31 +16629,31 @@
         <v>4</v>
       </c>
       <c r="H96" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="I96" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="J96" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="I96" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="J96" s="4" t="s">
-        <v>81</v>
-      </c>
       <c r="K96" s="30" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="L96" s="30" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="M96" s="30" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="N96" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="O96" s="30" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="P96" s="78" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="Q96" s="4" t="s">
         <v>5</v>
@@ -16659,7 +16668,7 @@
         <v>8</v>
       </c>
       <c r="U96" s="79" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
     <row r="97">
@@ -17074,7 +17083,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="85" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B1" s="86"/>
       <c r="C1" s="86"/>
@@ -17097,47 +17106,47 @@
     <row r="2">
       <c r="A2" s="90"/>
       <c r="B2" s="91" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C2" s="91" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D2" s="92" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E2" s="92" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F2" s="91" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G2" s="93" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H2" s="93" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I2" s="93" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J2" s="91"/>
       <c r="K2" s="91" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="L2" s="91" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="M2" s="94" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="N2" s="93" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="O2" s="93" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="P2" s="93" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="U2" s="50"/>
       <c r="V2" s="48"/>
@@ -17402,7 +17411,7 @@
     <row r="10">
       <c r="A10" s="61"/>
       <c r="E10" s="38" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O10" s="54"/>
       <c r="P10" s="61"/>
@@ -17533,7 +17542,7 @@
     <row r="18">
       <c r="A18" s="54"/>
       <c r="E18" s="38" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="O18" s="54"/>
       <c r="P18" s="54"/>
@@ -17638,7 +17647,7 @@
         <v>4</v>
       </c>
       <c r="H32" s="99" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I32" s="4" t="s">
         <v>5</v>
@@ -17653,13 +17662,13 @@
         <v>8</v>
       </c>
       <c r="M32" s="100" t="s">
+        <v>94</v>
+      </c>
+      <c r="N32" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="O32" s="101" t="s">
         <v>93</v>
-      </c>
-      <c r="N32" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="O32" s="101" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="33">
@@ -18113,13 +18122,13 @@
     </row>
     <row r="9">
       <c r="B9" s="38" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D9" s="38" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="10">
@@ -18137,7 +18146,7 @@
         <v>-0.1658536585</v>
       </c>
       <c r="F10" s="38" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11">
@@ -18155,7 +18164,7 @@
         <v>-0.15</v>
       </c>
       <c r="F11" s="38" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12">
@@ -18193,16 +18202,16 @@
     </row>
     <row r="16">
       <c r="H16" s="38" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17">
       <c r="G17" s="111"/>
       <c r="H17" s="48" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I17" s="48" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18">
@@ -18222,7 +18231,7 @@
         <v>332.0</v>
       </c>
       <c r="I18" s="42" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="19">
@@ -18239,10 +18248,10 @@
         <v>18</v>
       </c>
       <c r="H19" s="38" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="I19" s="38" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20">
@@ -18262,7 +18271,7 @@
         <v>411.0</v>
       </c>
       <c r="I20" s="38" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21">
@@ -18270,10 +18279,10 @@
         <v>20</v>
       </c>
       <c r="H21" s="38" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I21" s="38" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22">
@@ -18281,16 +18290,16 @@
         <v>21</v>
       </c>
       <c r="H22" s="38" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="I22" s="38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24">
       <c r="B24" s="8"/>
       <c r="I24" s="38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="25">
@@ -18298,7 +18307,7 @@
         <v>1</v>
       </c>
       <c r="I25" s="38" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="26">
@@ -18349,28 +18358,28 @@
         <v>530.0</v>
       </c>
       <c r="I30" s="48" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="M30" s="60"/>
       <c r="N30" s="60"/>
     </row>
     <row r="31">
       <c r="I31" s="48" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="M31" s="60"/>
       <c r="N31" s="60"/>
     </row>
     <row r="32">
       <c r="I32" s="38" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="M32" s="60"/>
       <c r="N32" s="60"/>
     </row>
     <row r="33">
       <c r="I33" s="38" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M33" s="60"/>
       <c r="N33" s="60"/>
@@ -18381,7 +18390,7 @@
     </row>
     <row r="35">
       <c r="I35" s="38" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="M35" s="60"/>
       <c r="N35" s="60"/>
@@ -18400,28 +18409,28 @@
     </row>
     <row r="39">
       <c r="I39" s="48" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="M39" s="60"/>
       <c r="N39" s="60"/>
     </row>
     <row r="40">
       <c r="I40" s="38" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M40" s="60"/>
       <c r="N40" s="60"/>
     </row>
     <row r="41">
       <c r="I41" s="38" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="M41" s="60"/>
       <c r="N41" s="60"/>
     </row>
     <row r="42">
       <c r="I42" s="68" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="M42" s="60"/>
       <c r="N42" s="60"/>
@@ -18432,7 +18441,7 @@
     </row>
     <row r="44">
       <c r="I44" s="48" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -18450,18 +18459,18 @@
   <sheetData>
     <row r="1">
       <c r="B1" s="38" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3">
       <c r="C3" s="38" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D3" s="38" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H3" s="38" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K3" s="60"/>
       <c r="L3" s="60"/>
@@ -18471,13 +18480,13 @@
         <v>17</v>
       </c>
       <c r="C4" s="48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="D4" s="48" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H4" s="38" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I4" s="113"/>
       <c r="J4" s="113"/>
@@ -18486,7 +18495,7 @@
     </row>
     <row r="5">
       <c r="B5" s="48" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C5" s="50">
         <f t="shared" ref="C5:D5" si="1">SUM(C6:C18)</f>
@@ -18501,7 +18510,7 @@
         <v>0.4077999152</v>
       </c>
       <c r="F5" s="38" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="6">
@@ -18520,7 +18529,7 @@
         <v>3.06</v>
       </c>
       <c r="H7" s="38" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8">
@@ -18539,7 +18548,7 @@
         <v>2.3</v>
       </c>
       <c r="H9" s="38" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
     </row>
     <row r="10">
@@ -18558,7 +18567,7 @@
         <v>4.18</v>
       </c>
       <c r="H11" s="38" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
     </row>
     <row r="12">
@@ -18577,7 +18586,7 @@
         <v>2.35</v>
       </c>
       <c r="H13" s="38" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="14">
@@ -18604,7 +18613,7 @@
         <v>1.37</v>
       </c>
       <c r="H16" s="38" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="17">
@@ -18628,15 +18637,15 @@
         <v>18</v>
       </c>
       <c r="C20" s="48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D20" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="21">
       <c r="B21" s="48" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C21" s="50">
         <f t="shared" ref="C21:D21" si="2">sum(C22:C34)</f>
@@ -18651,7 +18660,7 @@
         <v>0.4012276786</v>
       </c>
       <c r="F21" s="38" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
     </row>
     <row r="22">
@@ -18763,15 +18772,15 @@
         <v>19</v>
       </c>
       <c r="C37" s="48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D37" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="48" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C38" s="50">
         <f t="shared" ref="C38:D38" si="3">sum(C39:C51)</f>
@@ -18786,7 +18795,7 @@
         <v>0.03155866056</v>
       </c>
       <c r="F38" s="38" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="39">
@@ -18912,17 +18921,17 @@
         <v>20</v>
       </c>
       <c r="C54" s="48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D54" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K54" s="60"/>
       <c r="L54" s="60"/>
     </row>
     <row r="55">
       <c r="B55" s="48" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C55" s="50">
         <f>sum(C56:C69)</f>
@@ -18937,7 +18946,7 @@
         <v>0.005738332058</v>
       </c>
       <c r="F55" s="38" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="K55" s="60"/>
       <c r="L55" s="60"/>
@@ -19091,17 +19100,17 @@
         <v>21</v>
       </c>
       <c r="C71" s="48" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="D71" s="48" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="K71" s="60"/>
       <c r="L71" s="60"/>
     </row>
     <row r="72">
       <c r="B72" s="48" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C72" s="50">
         <f>sum(C73:C86)</f>
@@ -19116,7 +19125,7 @@
         <v>0.3919949174</v>
       </c>
       <c r="F72" s="38" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="K72" s="60"/>
       <c r="L72" s="60"/>
@@ -19330,7 +19339,7 @@
     <row r="2">
       <c r="A2" s="17"/>
       <c r="B2" s="114" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C2" s="17">
         <v>0.1</v>
@@ -19340,7 +19349,7 @@
     <row r="3">
       <c r="A3" s="17"/>
       <c r="B3" s="114" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C3" s="13" t="str">
         <f>AVERAGE(#REF!)</f>
@@ -19355,7 +19364,7 @@
       <c r="L4" s="20"/>
       <c r="P4" s="20"/>
       <c r="AE4" s="38" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="AF4" s="115">
         <f>CORREL(AE6:AE10000,AF6:AF10000)</f>
@@ -19365,50 +19374,50 @@
     <row r="5">
       <c r="A5" s="17"/>
       <c r="B5" s="20" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="L5" s="20" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P5" s="20" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AE5" s="38" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="AF5" s="38" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="17"/>
       <c r="B6" s="38" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="F6" s="38" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K6" s="48"/>
       <c r="L6" s="48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="N6" s="48" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P6" s="48" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="R6" s="48" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="V6" s="48" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AA6" s="38" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AB6" s="38" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AE6" s="38">
         <v>519.2</v>
@@ -19450,7 +19459,7 @@
         <v>0.5454545455</v>
       </c>
       <c r="AA7" s="38" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AB7" s="52">
         <f t="shared" ref="AB7:AB16" si="4">LEFT(REPLACE(AA7,1,1,""),FIND(",", AA7)-2)/1</f>
@@ -19466,14 +19475,14 @@
     <row r="8">
       <c r="A8" s="17"/>
       <c r="B8" s="119" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C8" s="120" t="str">
         <f t="shared" ref="C8:C17" si="5">REPLACE(B8,FIND(".",B8),1,",")*1</f>
         <v>#VALUE!</v>
       </c>
       <c r="F8" s="58" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="G8" s="120" t="str">
         <f t="shared" ref="G8:G27" si="6">REPLACE(F8,FIND(".",F8),1,",")*1</f>
@@ -19508,7 +19517,7 @@
         <v>0.5263157895</v>
       </c>
       <c r="AA8" s="38" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="AB8" s="52">
         <f t="shared" si="4"/>
@@ -19524,14 +19533,14 @@
     <row r="9">
       <c r="A9" s="17"/>
       <c r="B9" s="119" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C9" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F9" s="58" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="G9" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19545,13 +19554,13 @@
       </c>
       <c r="K9" s="17"/>
       <c r="L9" s="116" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="M9" s="116" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="N9" s="48" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="P9" s="118">
         <v>1.0</v>
@@ -19575,7 +19584,7 @@
         <v>0.25</v>
       </c>
       <c r="AA9" s="38" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AB9" s="52">
         <f t="shared" si="4"/>
@@ -19591,14 +19600,14 @@
     <row r="10">
       <c r="A10" s="17"/>
       <c r="B10" s="121" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C10" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F10" s="58" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="G10" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19635,7 +19644,7 @@
         <v>76</v>
       </c>
       <c r="AA10" s="38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AB10" s="52">
         <f t="shared" si="4"/>
@@ -19650,14 +19659,14 @@
     </row>
     <row r="11">
       <c r="B11" s="119" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C11" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F11" s="58" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="G11" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19686,7 +19695,7 @@
         <v>2.0</v>
       </c>
       <c r="AA11" s="38" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AB11" s="52">
         <f t="shared" si="4"/>
@@ -19701,14 +19710,14 @@
     </row>
     <row r="12">
       <c r="B12" s="121" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C12" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F12" s="58" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="G12" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19737,7 +19746,7 @@
         <v>1.0</v>
       </c>
       <c r="AA12" s="38" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="AB12" s="52">
         <f t="shared" si="4"/>
@@ -19752,14 +19761,14 @@
     </row>
     <row r="13">
       <c r="B13" s="119" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C13" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F13" s="58" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="G13" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19789,16 +19798,16 @@
       <c r="Q13" s="50"/>
       <c r="R13" s="90"/>
       <c r="S13" s="95" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="T13" s="95" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="U13" s="95" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AA13" s="38" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AB13" s="52">
         <f t="shared" si="4"/>
@@ -19813,14 +19822,14 @@
     </row>
     <row r="14">
       <c r="B14" s="119" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C14" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F14" s="58" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="G14" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19860,7 +19869,7 @@
         <v>11.0</v>
       </c>
       <c r="AA14" s="38" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AB14" s="52">
         <f t="shared" si="4"/>
@@ -19875,14 +19884,14 @@
     </row>
     <row r="15">
       <c r="B15" s="119" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C15" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F15" s="58" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="G15" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19922,7 +19931,7 @@
         <v>13.0</v>
       </c>
       <c r="AA15" s="38" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="AB15" s="52">
         <f t="shared" si="4"/>
@@ -19937,14 +19946,14 @@
     </row>
     <row r="16">
       <c r="B16" s="119" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C16" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F16" s="58" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G16" s="120" t="str">
         <f t="shared" si="6"/>
@@ -19984,7 +19993,7 @@
         <v>12.0</v>
       </c>
       <c r="AA16" s="38" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AB16" s="52">
         <f t="shared" si="4"/>
@@ -19999,14 +20008,14 @@
     </row>
     <row r="17">
       <c r="B17" s="119" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C17" s="120" t="str">
         <f t="shared" si="5"/>
         <v>#VALUE!</v>
       </c>
       <c r="F17" s="58" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="G17" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20034,7 +20043,7 @@
         <v>1.0</v>
       </c>
       <c r="R17" s="95" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="S17" s="123">
         <f t="shared" ref="S17:U17" si="10">SUM(S14:S16)</f>
@@ -20057,7 +20066,7 @@
     </row>
     <row r="18">
       <c r="F18" s="58" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="G18" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20094,14 +20103,14 @@
     </row>
     <row r="19">
       <c r="B19" s="48" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C19" s="52" t="str">
         <f>AVERAGE(C8:C17)</f>
         <v>#VALUE!</v>
       </c>
       <c r="F19" s="58" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="G19" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20129,7 +20138,7 @@
       <c r="T19" s="13"/>
       <c r="U19" s="13"/>
       <c r="AA19" s="38" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="AB19" s="52">
         <f>AVERAGE(AB7:AB16)</f>
@@ -20144,7 +20153,7 @@
     </row>
     <row r="20">
       <c r="F20" s="58" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="G20" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20169,7 +20178,7 @@
     </row>
     <row r="21">
       <c r="F21" s="58" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="G21" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20183,13 +20192,13 @@
       </c>
       <c r="R21" s="90"/>
       <c r="S21" s="95" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="T21" s="95" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="U21" s="95" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AE21" s="38">
         <v>146.62</v>
@@ -20201,7 +20210,7 @@
     <row r="22">
       <c r="C22" s="120"/>
       <c r="F22" s="58" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G22" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20274,7 +20283,7 @@
     </row>
     <row r="24">
       <c r="F24" s="58" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="G24" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20310,7 +20319,7 @@
     </row>
     <row r="25">
       <c r="F25" s="58" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="G25" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20323,7 +20332,7 @@
         <v>1.0</v>
       </c>
       <c r="R25" s="95" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="S25" s="123">
         <f t="shared" ref="S25:U25" si="14">SUM(S22:S24)</f>
@@ -20346,7 +20355,7 @@
     </row>
     <row r="26">
       <c r="F26" s="58" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="G26" s="120" t="str">
         <f t="shared" si="6"/>
@@ -20391,13 +20400,13 @@
         <v>1.0</v>
       </c>
       <c r="AA28" s="38" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AB28" s="38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AC28" s="38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AE28" s="38">
         <v>106.73</v>
@@ -20408,7 +20417,7 @@
     </row>
     <row r="29">
       <c r="F29" s="48" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="G29" s="52" t="str">
         <f>AVERAGE(G8:G27)</f>
@@ -20499,7 +20508,7 @@
     </row>
     <row r="32">
       <c r="B32" s="65" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="G32" s="120"/>
       <c r="P32" s="118">
@@ -20528,7 +20537,7 @@
     </row>
     <row r="33">
       <c r="B33" s="126" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="G33" s="127"/>
       <c r="P33" s="118">
@@ -20582,7 +20591,7 @@
     </row>
     <row r="35">
       <c r="H35" s="48" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="P35" s="118">
         <v>1.0</v>
@@ -20645,7 +20654,7 @@
       <c r="C37" s="50"/>
       <c r="D37" s="129">
         <f>AVERAGE(D39:D1775)</f>
-        <v>3.662637363</v>
+        <v>3.436923077</v>
       </c>
       <c r="G37" s="48" t="s">
         <v>18</v>
@@ -20710,11 +20719,11 @@
     </row>
     <row r="39">
       <c r="C39" s="131" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D39" s="120">
         <f t="shared" ref="D39:D221" si="17">IF(COUNTA(C39)=1,C39/1,"")</f>
-        <v>1.52</v>
+        <v>2.17</v>
       </c>
       <c r="G39" s="48" t="s">
         <v>20</v>
@@ -20748,11 +20757,11 @@
     </row>
     <row r="40">
       <c r="C40" s="132" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="D40" s="120">
         <f t="shared" si="17"/>
-        <v>0.33</v>
+        <v>1.66</v>
       </c>
       <c r="G40" s="48" t="s">
         <v>21</v>
@@ -20786,11 +20795,11 @@
     </row>
     <row r="41">
       <c r="C41" s="132" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="D41" s="120">
         <f t="shared" si="17"/>
-        <v>1.43</v>
+        <v>1.96</v>
       </c>
       <c r="P41" s="118">
         <v>0.0</v>
@@ -20818,11 +20827,11 @@
     </row>
     <row r="42">
       <c r="C42" s="132" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="D42" s="120">
         <f t="shared" si="17"/>
-        <v>0.28</v>
+        <v>1.28</v>
       </c>
       <c r="P42" s="118">
         <v>2.0</v>
@@ -20850,11 +20859,11 @@
     </row>
     <row r="43">
       <c r="C43" s="132" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D43" s="120">
         <f t="shared" si="17"/>
-        <v>0.92</v>
+        <v>2.78</v>
       </c>
       <c r="P43" s="118">
         <v>1.0</v>
@@ -20882,11 +20891,11 @@
     </row>
     <row r="44">
       <c r="C44" s="132" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D44" s="120">
         <f t="shared" si="17"/>
-        <v>1.65</v>
+        <v>2.26</v>
       </c>
       <c r="P44" s="118">
         <v>2.0</v>
@@ -20912,11 +20921,11 @@
     </row>
     <row r="45">
       <c r="C45" s="132" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D45" s="120">
         <f t="shared" si="17"/>
-        <v>2.05</v>
+        <v>2.45</v>
       </c>
       <c r="P45" s="118">
         <v>1.0</v>
@@ -20930,17 +20939,17 @@
     </row>
     <row r="46" ht="15.0" customHeight="1">
       <c r="C46" s="132" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D46" s="120">
         <f t="shared" si="17"/>
-        <v>1.93</v>
+        <v>1.78</v>
       </c>
       <c r="G46" s="133" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H46" s="133" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="P46" s="118">
         <v>0.0</v>
@@ -20954,11 +20963,11 @@
     </row>
     <row r="47">
       <c r="C47" s="132" t="s">
-        <v>237</v>
+        <v>204</v>
       </c>
       <c r="D47" s="120">
         <f t="shared" si="17"/>
-        <v>1.6</v>
+        <v>3.64</v>
       </c>
       <c r="G47" s="134" t="s">
         <v>17</v>
@@ -20973,7 +20982,7 @@
         <v>3</v>
       </c>
       <c r="AB47" s="38" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="AE47" s="38">
         <v>67.98</v>
@@ -20984,11 +20993,11 @@
     </row>
     <row r="48">
       <c r="C48" s="132" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="D48" s="120">
         <f t="shared" si="17"/>
-        <v>1.65</v>
+        <v>3.74</v>
       </c>
       <c r="G48" s="134" t="s">
         <v>18</v>
@@ -20997,7 +21006,7 @@
         <v>0.36678739680281</v>
       </c>
       <c r="J48" s="38" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="K48" s="110">
         <f>AVERAGE(H47:H51)</f>
@@ -21021,11 +21030,11 @@
     </row>
     <row r="49">
       <c r="C49" s="132" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D49" s="120">
         <f t="shared" si="17"/>
-        <v>0.77</v>
+        <v>4</v>
       </c>
       <c r="G49" s="134" t="s">
         <v>19</v>
@@ -21034,7 +21043,7 @@
         <v>0.142870351877935</v>
       </c>
       <c r="J49" s="38" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="K49" s="110">
         <f>MEDIAN(H47:H51)</f>
@@ -21058,11 +21067,11 @@
     </row>
     <row r="50">
       <c r="C50" s="132" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D50" s="120">
         <f t="shared" si="17"/>
-        <v>6.54</v>
+        <v>3.73</v>
       </c>
       <c r="G50" s="134" t="s">
         <v>20</v>
@@ -21071,7 +21080,7 @@
         <v>0.497437843674554</v>
       </c>
       <c r="J50" s="38" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="K50" s="110">
         <f>PERCENTILE(H47:H51,0.25)</f>
@@ -21095,11 +21104,11 @@
     </row>
     <row r="51">
       <c r="C51" s="132" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="D51" s="120">
         <f t="shared" si="17"/>
-        <v>5.57</v>
+        <v>4.3</v>
       </c>
       <c r="G51" s="134" t="s">
         <v>21</v>
@@ -21108,7 +21117,7 @@
         <v>0.247446036291655</v>
       </c>
       <c r="J51" s="38" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="K51" s="110">
         <f>PERCENTILE(H47:H51,0.75)</f>
@@ -21132,11 +21141,11 @@
     </row>
     <row r="52">
       <c r="C52" s="132" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D52" s="120">
         <f t="shared" si="17"/>
-        <v>4.51</v>
+        <v>5.93</v>
       </c>
       <c r="P52" s="118">
         <v>0.0</v>
@@ -21156,11 +21165,11 @@
     </row>
     <row r="53">
       <c r="C53" s="132" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D53" s="120">
         <f t="shared" si="17"/>
-        <v>0.84</v>
+        <v>3.66</v>
       </c>
       <c r="P53" s="118">
         <v>0.0</v>
@@ -21180,11 +21189,11 @@
     </row>
     <row r="54">
       <c r="C54" s="132" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D54" s="120">
         <f t="shared" si="17"/>
-        <v>0.82</v>
+        <v>4.11</v>
       </c>
       <c r="P54" s="118">
         <v>2.0</v>
@@ -21204,11 +21213,11 @@
     </row>
     <row r="55">
       <c r="C55" s="132" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="D55" s="120">
         <f t="shared" si="17"/>
-        <v>5.71</v>
+        <v>5.4</v>
       </c>
       <c r="P55" s="118">
         <v>0.0</v>
@@ -21228,11 +21237,11 @@
     </row>
     <row r="56">
       <c r="C56" s="132" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="D56" s="120">
         <f t="shared" si="17"/>
-        <v>6.89</v>
+        <v>5.97</v>
       </c>
       <c r="P56" s="118">
         <v>0.0</v>
@@ -21252,11 +21261,11 @@
     </row>
     <row r="57">
       <c r="C57" s="132" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D57" s="120">
         <f t="shared" si="17"/>
-        <v>3.95</v>
+        <v>4.34</v>
       </c>
       <c r="P57" s="118">
         <v>2.0</v>
@@ -21276,14 +21285,14 @@
     </row>
     <row r="58">
       <c r="C58" s="132" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D58" s="120">
         <f t="shared" si="17"/>
-        <v>1.63</v>
+        <v>1.81</v>
       </c>
       <c r="G58" s="136" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="H58" s="137"/>
       <c r="P58" s="118">
@@ -21304,15 +21313,15 @@
     </row>
     <row r="59">
       <c r="C59" s="132" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D59" s="120">
         <f t="shared" si="17"/>
-        <v>2.69</v>
+        <v>2.99</v>
       </c>
       <c r="G59" s="137"/>
       <c r="H59" s="138" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="P59" s="118">
         <v>0.0</v>
@@ -21332,15 +21341,15 @@
     </row>
     <row r="60">
       <c r="C60" s="132" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="D60" s="120">
         <f t="shared" si="17"/>
-        <v>4.35</v>
+        <v>4.84</v>
       </c>
       <c r="G60" s="137"/>
       <c r="H60" s="138" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="P60" s="118">
         <v>2.0</v>
@@ -21360,15 +21369,15 @@
     </row>
     <row r="61">
       <c r="C61" s="132" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="D61" s="120">
         <f t="shared" si="17"/>
-        <v>1.26</v>
+        <v>1.4</v>
       </c>
       <c r="G61" s="137"/>
       <c r="H61" s="138" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="P61" s="118">
         <v>2.0</v>
@@ -21388,15 +21397,15 @@
     </row>
     <row r="62">
       <c r="C62" s="132" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D62" s="120">
         <f t="shared" si="17"/>
-        <v>5.01</v>
+        <v>3.34</v>
       </c>
       <c r="G62" s="137"/>
       <c r="H62" s="138" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="P62" s="118">
         <v>1.0</v>
@@ -21416,15 +21425,15 @@
     </row>
     <row r="63">
       <c r="C63" s="132" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="D63" s="120">
         <f t="shared" si="17"/>
-        <v>4.18</v>
+        <v>2.79</v>
       </c>
       <c r="G63" s="137"/>
       <c r="H63" s="138" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="P63" s="118">
         <v>0.0</v>
@@ -21438,11 +21447,11 @@
     </row>
     <row r="64">
       <c r="C64" s="132" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D64" s="120">
         <f t="shared" si="17"/>
-        <v>8.08</v>
+        <v>5.39</v>
       </c>
       <c r="P64" s="118">
         <v>1.0</v>
@@ -21456,11 +21465,11 @@
     </row>
     <row r="65">
       <c r="C65" s="132" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D65" s="120">
         <f t="shared" si="17"/>
-        <v>11.99</v>
+        <v>7.99</v>
       </c>
       <c r="P65" s="118">
         <v>2.0</v>
@@ -21474,11 +21483,11 @@
     </row>
     <row r="66">
       <c r="C66" s="132" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D66" s="120">
         <f t="shared" si="17"/>
-        <v>11.64</v>
+        <v>7.76</v>
       </c>
       <c r="P66" s="118">
         <v>0.0</v>
@@ -21492,11 +21501,11 @@
     </row>
     <row r="67">
       <c r="C67" s="132" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D67" s="120">
         <f t="shared" si="17"/>
-        <v>7.86</v>
+        <v>5.24</v>
       </c>
       <c r="P67" s="118">
         <v>0.0</v>
@@ -21510,11 +21519,11 @@
     </row>
     <row r="68">
       <c r="C68" s="132" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D68" s="120">
         <f t="shared" si="17"/>
-        <v>11.5</v>
+        <v>7.66</v>
       </c>
       <c r="P68" s="118">
         <v>1.0</v>
@@ -21528,11 +21537,11 @@
     </row>
     <row r="69">
       <c r="C69" s="132" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="D69" s="120">
         <f t="shared" si="17"/>
-        <v>7.78</v>
+        <v>5.19</v>
       </c>
       <c r="P69" s="118">
         <v>2.0</v>
@@ -21546,11 +21555,11 @@
     </row>
     <row r="70">
       <c r="C70" s="132" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D70" s="120">
         <f t="shared" si="17"/>
-        <v>5.65</v>
+        <v>3.76</v>
       </c>
       <c r="P70" s="118">
         <v>1.0</v>
@@ -21564,11 +21573,11 @@
     </row>
     <row r="71">
       <c r="C71" s="132" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D71" s="120">
         <f t="shared" si="17"/>
-        <v>6.67</v>
+        <v>4.44</v>
       </c>
       <c r="F71" s="139"/>
       <c r="P71" s="118">
@@ -21583,11 +21592,11 @@
     </row>
     <row r="72">
       <c r="C72" s="132" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D72" s="120">
         <f t="shared" si="17"/>
-        <v>7.3</v>
+        <v>4.86</v>
       </c>
       <c r="P72" s="118">
         <v>0.0</v>
@@ -21601,11 +21610,11 @@
     </row>
     <row r="73">
       <c r="C73" s="132" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D73" s="120">
         <f t="shared" si="17"/>
-        <v>5</v>
+        <v>3.33</v>
       </c>
       <c r="P73" s="118">
         <v>1.0</v>
@@ -21619,11 +21628,11 @@
     </row>
     <row r="74">
       <c r="C74" s="132" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="D74" s="120">
         <f t="shared" si="17"/>
-        <v>6.44</v>
+        <v>4.29</v>
       </c>
       <c r="P74" s="118">
         <v>0.0</v>
@@ -21637,11 +21646,11 @@
     </row>
     <row r="75">
       <c r="C75" s="132" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="D75" s="120">
         <f t="shared" si="17"/>
-        <v>4.11</v>
+        <v>4.57</v>
       </c>
       <c r="P75" s="118">
         <v>1.0</v>
@@ -21655,11 +21664,11 @@
     </row>
     <row r="76">
       <c r="C76" s="132" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="D76" s="120">
         <f t="shared" si="17"/>
-        <v>4.15</v>
+        <v>4.61</v>
       </c>
       <c r="P76" s="118">
         <v>0.0</v>
@@ -21673,11 +21682,11 @@
     </row>
     <row r="77">
       <c r="C77" s="132" t="s">
-        <v>276</v>
+        <v>210</v>
       </c>
       <c r="D77" s="120">
         <f t="shared" si="17"/>
-        <v>2.52</v>
+        <v>2.8</v>
       </c>
       <c r="P77" s="118">
         <v>0.0</v>
@@ -21695,7 +21704,7 @@
       </c>
       <c r="D78" s="120">
         <f t="shared" si="17"/>
-        <v>2.84</v>
+        <v>3.16</v>
       </c>
       <c r="P78" s="118">
         <v>1.0</v>
@@ -21713,7 +21722,7 @@
       </c>
       <c r="D79" s="120">
         <f t="shared" si="17"/>
-        <v>1.71</v>
+        <v>1.9</v>
       </c>
       <c r="P79" s="118">
         <v>2.0</v>
@@ -21731,7 +21740,7 @@
       </c>
       <c r="D80" s="120">
         <f t="shared" si="17"/>
-        <v>2.46</v>
+        <v>2.73</v>
       </c>
       <c r="P80" s="118">
         <v>1.0</v>
@@ -21745,11 +21754,11 @@
     </row>
     <row r="81">
       <c r="C81" s="132" t="s">
-        <v>280</v>
+        <v>251</v>
       </c>
       <c r="D81" s="120">
         <f t="shared" si="17"/>
-        <v>3.9</v>
+        <v>4.34</v>
       </c>
       <c r="P81" s="118">
         <v>2.0</v>
@@ -21763,11 +21772,11 @@
     </row>
     <row r="82">
       <c r="C82" s="132" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D82" s="120">
         <f t="shared" si="17"/>
-        <v>3.1</v>
+        <v>3.44</v>
       </c>
       <c r="P82" s="118">
         <v>1.0</v>
@@ -21781,11 +21790,11 @@
     </row>
     <row r="83">
       <c r="C83" s="132" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D83" s="120">
         <f t="shared" si="17"/>
-        <v>1.11</v>
+        <v>1.24</v>
       </c>
       <c r="P83" s="118">
         <v>0.0</v>
@@ -21799,11 +21808,11 @@
     </row>
     <row r="84">
       <c r="C84" s="132" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D84" s="120">
         <f t="shared" si="17"/>
-        <v>2.1</v>
+        <v>2.33</v>
       </c>
       <c r="P84" s="118">
         <v>1.0</v>
@@ -21817,11 +21826,11 @@
     </row>
     <row r="85">
       <c r="C85" s="132" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D85" s="120">
         <f t="shared" si="17"/>
-        <v>3.48</v>
+        <v>2.32</v>
       </c>
       <c r="P85" s="118">
         <v>0.0</v>
@@ -21835,11 +21844,11 @@
     </row>
     <row r="86">
       <c r="C86" s="132" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D86" s="120">
         <f t="shared" si="17"/>
-        <v>3.86</v>
+        <v>2.57</v>
       </c>
       <c r="P86" s="118">
         <v>0.0</v>
@@ -21853,11 +21862,11 @@
     </row>
     <row r="87">
       <c r="C87" s="132" t="s">
-        <v>200</v>
+        <v>285</v>
       </c>
       <c r="D87" s="120">
         <f t="shared" si="17"/>
-        <v>3.68</v>
+        <v>2.46</v>
       </c>
       <c r="P87" s="118">
         <v>1.0</v>
@@ -21875,7 +21884,7 @@
       </c>
       <c r="D88" s="120">
         <f t="shared" si="17"/>
-        <v>6.65</v>
+        <v>7.39</v>
       </c>
       <c r="P88" s="118">
         <v>2.0</v>
@@ -21893,7 +21902,7 @@
       </c>
       <c r="D89" s="120">
         <f t="shared" si="17"/>
-        <v>5.84</v>
+        <v>6.49</v>
       </c>
       <c r="P89" s="118">
         <v>2.0</v>
@@ -21911,7 +21920,7 @@
       </c>
       <c r="D90" s="120">
         <f t="shared" si="17"/>
-        <v>9.57</v>
+        <v>10.63</v>
       </c>
       <c r="P90" s="118">
         <v>1.0</v>
@@ -21929,7 +21938,7 @@
       </c>
       <c r="D91" s="120">
         <f t="shared" si="17"/>
-        <v>6.57</v>
+        <v>7.3</v>
       </c>
       <c r="P91" s="118">
         <v>1.0</v>
@@ -21943,11 +21952,11 @@
     </row>
     <row r="92">
       <c r="C92" s="132" t="s">
-        <v>193</v>
+        <v>290</v>
       </c>
       <c r="D92" s="120">
         <f t="shared" si="17"/>
-        <v>5.94</v>
+        <v>6.6</v>
       </c>
       <c r="P92" s="118">
         <v>2.0</v>
@@ -21961,11 +21970,11 @@
     </row>
     <row r="93">
       <c r="C93" s="132" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="D93" s="120">
         <f t="shared" si="17"/>
-        <v>0.52</v>
+        <v>1.74</v>
       </c>
       <c r="P93" s="118">
         <v>0.0</v>
@@ -21979,11 +21988,11 @@
     </row>
     <row r="94">
       <c r="C94" s="132" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="D94" s="120">
         <f t="shared" si="17"/>
-        <v>2.91</v>
+        <v>1.94</v>
       </c>
       <c r="P94" s="118">
         <v>0.0</v>
@@ -21997,11 +22006,11 @@
     </row>
     <row r="95">
       <c r="C95" s="132" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="D95" s="120">
         <f t="shared" si="17"/>
-        <v>2.48</v>
+        <v>1.65</v>
       </c>
       <c r="P95" s="118">
         <v>1.0</v>
@@ -22015,11 +22024,11 @@
     </row>
     <row r="96">
       <c r="C96" s="132" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="D96" s="120">
         <f t="shared" si="17"/>
-        <v>4.98</v>
+        <v>3.32</v>
       </c>
       <c r="P96" s="118">
         <v>2.0</v>
@@ -22033,11 +22042,11 @@
     </row>
     <row r="97">
       <c r="C97" s="132" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="D97" s="120">
         <f t="shared" si="17"/>
-        <v>0.49</v>
+        <v>1.62</v>
       </c>
       <c r="P97" s="118">
         <v>0.0</v>
@@ -22051,11 +22060,11 @@
     </row>
     <row r="98">
       <c r="C98" s="132" t="s">
-        <v>295</v>
+        <v>228</v>
       </c>
       <c r="D98" s="120">
         <f t="shared" si="17"/>
-        <v>3.26</v>
+        <v>2.17</v>
       </c>
       <c r="P98" s="118">
         <v>2.0</v>
@@ -22073,7 +22082,7 @@
       </c>
       <c r="D99" s="120">
         <f t="shared" si="17"/>
-        <v>2.87</v>
+        <v>1.91</v>
       </c>
       <c r="P99" s="118">
         <v>2.0</v>
@@ -22087,11 +22096,11 @@
     </row>
     <row r="100">
       <c r="C100" s="132" t="s">
-        <v>220</v>
+        <v>297</v>
       </c>
       <c r="D100" s="120">
         <f t="shared" si="17"/>
-        <v>2.63</v>
+        <v>1.76</v>
       </c>
       <c r="P100" s="118">
         <v>2.0</v>
@@ -22105,11 +22114,11 @@
     </row>
     <row r="101">
       <c r="C101" s="132" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="D101" s="120">
         <f t="shared" si="17"/>
-        <v>0.57</v>
+        <v>1.89</v>
       </c>
       <c r="P101" s="118">
         <v>2.0</v>
@@ -22123,11 +22132,11 @@
     </row>
     <row r="102">
       <c r="C102" s="132" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="D102" s="120">
         <f t="shared" si="17"/>
-        <v>2.53</v>
+        <v>1.69</v>
       </c>
       <c r="P102" s="118">
         <v>2.0</v>
@@ -22141,11 +22150,11 @@
     </row>
     <row r="103">
       <c r="C103" s="132" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="D103" s="120">
         <f t="shared" si="17"/>
-        <v>5.93</v>
+        <v>6.59</v>
       </c>
       <c r="P103" s="118">
         <v>1.0</v>
@@ -22159,11 +22168,11 @@
     </row>
     <row r="104">
       <c r="C104" s="132" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="D104" s="120">
         <f t="shared" si="17"/>
-        <v>4.84</v>
+        <v>3.23</v>
       </c>
       <c r="N104" s="140"/>
       <c r="P104" s="118">
@@ -22178,11 +22187,11 @@
     </row>
     <row r="105">
       <c r="C105" s="132" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="D105" s="120">
         <f t="shared" si="17"/>
-        <v>3.99</v>
+        <v>2.66</v>
       </c>
       <c r="N105" s="13"/>
       <c r="P105" s="118">
@@ -22197,11 +22206,11 @@
     </row>
     <row r="106">
       <c r="C106" s="132" t="s">
-        <v>294</v>
+        <v>303</v>
       </c>
       <c r="D106" s="120">
         <f t="shared" si="17"/>
-        <v>0.49</v>
+        <v>0.33</v>
       </c>
       <c r="N106" s="13"/>
       <c r="P106" s="118">
@@ -22216,11 +22225,11 @@
     </row>
     <row r="107">
       <c r="C107" s="132" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="D107" s="120">
         <f t="shared" si="17"/>
-        <v>2.99</v>
+        <v>1.99</v>
       </c>
       <c r="N107" s="13"/>
       <c r="P107" s="118">
@@ -22235,11 +22244,11 @@
     </row>
     <row r="108">
       <c r="C108" s="132" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="D108" s="120">
         <f t="shared" si="17"/>
-        <v>3.01</v>
+        <v>2.01</v>
       </c>
       <c r="N108" s="13"/>
       <c r="P108" s="118">
@@ -22254,11 +22263,11 @@
     </row>
     <row r="109">
       <c r="C109" s="132" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="D109" s="120">
         <f t="shared" si="17"/>
-        <v>5.35</v>
+        <v>3.56</v>
       </c>
       <c r="N109" s="13"/>
       <c r="P109" s="118">
@@ -22273,11 +22282,11 @@
     </row>
     <row r="110">
       <c r="C110" s="132" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="D110" s="120">
         <f t="shared" si="17"/>
-        <v>2.95</v>
+        <v>1.97</v>
       </c>
       <c r="N110" s="13"/>
       <c r="P110" s="118">
@@ -22292,11 +22301,11 @@
     </row>
     <row r="111">
       <c r="C111" s="132" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D111" s="120">
         <f t="shared" si="17"/>
-        <v>3.07</v>
+        <v>2.93</v>
       </c>
       <c r="N111" s="13"/>
       <c r="P111" s="118">
@@ -22311,11 +22320,11 @@
     </row>
     <row r="112">
       <c r="C112" s="132" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="D112" s="120">
         <f t="shared" si="17"/>
-        <v>2.64</v>
+        <v>3.95</v>
       </c>
       <c r="P112" s="118">
         <v>1.0</v>
@@ -22329,11 +22338,11 @@
     </row>
     <row r="113">
       <c r="C113" s="132" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="D113" s="120">
         <f t="shared" si="17"/>
-        <v>3.56</v>
+        <v>3.27</v>
       </c>
       <c r="P113" s="118">
         <v>0.0</v>
@@ -22347,11 +22356,11 @@
     </row>
     <row r="114">
       <c r="C114" s="132" t="s">
-        <v>309</v>
+        <v>207</v>
       </c>
       <c r="D114" s="120">
         <f t="shared" si="17"/>
-        <v>2.93</v>
+        <v>2.71</v>
       </c>
       <c r="P114" s="118">
         <v>1.0</v>
@@ -22365,11 +22374,11 @@
     </row>
     <row r="115">
       <c r="C115" s="132" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="D115" s="120">
         <f t="shared" si="17"/>
-        <v>2.24</v>
+        <v>0.36</v>
       </c>
       <c r="P115" s="118">
         <v>1.0</v>
@@ -22383,11 +22392,11 @@
     </row>
     <row r="116">
       <c r="C116" s="132" t="s">
-        <v>228</v>
+        <v>312</v>
       </c>
       <c r="D116" s="120">
         <f t="shared" si="17"/>
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="P116" s="118">
         <v>1.0</v>
@@ -22401,11 +22410,11 @@
     </row>
     <row r="117">
       <c r="C117" s="132" t="s">
-        <v>228</v>
+        <v>311</v>
       </c>
       <c r="D117" s="120">
         <f t="shared" si="17"/>
-        <v>0.33</v>
+        <v>0.36</v>
       </c>
       <c r="P117" s="141"/>
       <c r="AE117" s="38">
@@ -22417,11 +22426,11 @@
     </row>
     <row r="118">
       <c r="C118" s="132" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="D118" s="120">
         <f t="shared" si="17"/>
-        <v>0.32</v>
+        <v>2.07</v>
       </c>
       <c r="P118" s="141"/>
       <c r="AE118" s="38">
@@ -22433,11 +22442,11 @@
     </row>
     <row r="119">
       <c r="C119" s="132" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D119" s="120">
         <f t="shared" si="17"/>
-        <v>1.86</v>
+        <v>2.37</v>
       </c>
       <c r="P119" s="141"/>
       <c r="AE119" s="38">
@@ -22449,11 +22458,11 @@
     </row>
     <row r="120">
       <c r="C120" s="132" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="D120" s="120">
         <f t="shared" si="17"/>
-        <v>2.13</v>
+        <v>3.17</v>
       </c>
       <c r="P120" s="141"/>
       <c r="AE120" s="38">
@@ -22465,11 +22474,11 @@
     </row>
     <row r="121">
       <c r="C121" s="132" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="D121" s="120">
         <f t="shared" si="17"/>
-        <v>2.85</v>
+        <v>2.07</v>
       </c>
       <c r="P121" s="141"/>
       <c r="AE121" s="38">
@@ -22481,11 +22490,11 @@
     </row>
     <row r="122">
       <c r="C122" s="132" t="s">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="D122" s="120">
         <f t="shared" si="17"/>
-        <v>1.86</v>
+        <v>3.47</v>
       </c>
       <c r="P122" s="141"/>
       <c r="AE122" s="38">
@@ -22497,11 +22506,11 @@
     </row>
     <row r="123">
       <c r="C123" s="132" t="s">
-        <v>281</v>
+        <v>317</v>
       </c>
       <c r="D123" s="120">
         <f t="shared" si="17"/>
-        <v>3.1</v>
+        <v>5.77</v>
       </c>
       <c r="P123" s="141"/>
       <c r="AE123" s="38">
@@ -22513,11 +22522,11 @@
     </row>
     <row r="124">
       <c r="C124" s="132" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D124" s="120">
         <f t="shared" si="17"/>
-        <v>5.2</v>
+        <v>5.87</v>
       </c>
       <c r="P124" s="141"/>
       <c r="AE124" s="38">
@@ -22529,11 +22538,11 @@
     </row>
     <row r="125">
       <c r="C125" s="132" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="D125" s="120">
         <f t="shared" si="17"/>
-        <v>5.28</v>
+        <v>5.49</v>
       </c>
       <c r="P125" s="141"/>
       <c r="AE125" s="38">
@@ -22545,11 +22554,11 @@
     </row>
     <row r="126">
       <c r="C126" s="132" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="D126" s="120">
         <f t="shared" si="17"/>
-        <v>4.94</v>
+        <v>2.24</v>
       </c>
       <c r="P126" s="141"/>
       <c r="AE126" s="38">
@@ -22561,11 +22570,11 @@
     </row>
     <row r="127">
       <c r="C127" s="132" t="s">
-        <v>318</v>
+        <v>282</v>
       </c>
       <c r="D127" s="120">
         <f t="shared" si="17"/>
-        <v>1.96</v>
+        <v>2.33</v>
       </c>
       <c r="P127" s="141"/>
       <c r="AE127" s="38">
@@ -22577,11 +22586,11 @@
     </row>
     <row r="128">
       <c r="C128" s="132" t="s">
-        <v>283</v>
+        <v>234</v>
       </c>
       <c r="D128" s="120">
         <f t="shared" si="17"/>
-        <v>2.1</v>
+        <v>2.45</v>
       </c>
       <c r="P128" s="141"/>
       <c r="AE128" s="38">
@@ -22593,11 +22602,11 @@
     </row>
     <row r="129">
       <c r="C129" s="132" t="s">
-        <v>319</v>
+        <v>311</v>
       </c>
       <c r="D129" s="120">
         <f t="shared" si="17"/>
-        <v>2.23</v>
+        <v>0.36</v>
       </c>
       <c r="P129" s="141"/>
       <c r="AE129" s="38">
@@ -44975,14 +44984,14 @@
     <row r="1">
       <c r="A1" s="144"/>
       <c r="B1" s="145" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C1" s="146"/>
       <c r="D1" s="146"/>
       <c r="E1" s="146"/>
       <c r="F1" s="146"/>
       <c r="G1" s="147" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="H1" s="146"/>
       <c r="I1" s="146"/>
@@ -45016,54 +45025,54 @@
         <v>3</v>
       </c>
       <c r="B2" s="149" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="C2" s="150" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="D2" s="150" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E2" s="150" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="F2" s="151" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="G2" s="149">
         <v>1.0</v>
       </c>
       <c r="H2" s="150" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I2" s="150">
         <v>2.0</v>
       </c>
       <c r="J2" s="150" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="K2" s="152" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="L2" s="150" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="M2" s="153" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="N2" s="134" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="O2" s="134" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="P2" s="134" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="Q2" s="5"/>
       <c r="R2" s="5"/>
       <c r="S2" s="114" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="T2" s="5"/>
       <c r="U2" s="5"/>
@@ -45153,7 +45162,7 @@
       <c r="Q4" s="5"/>
       <c r="R4" s="5"/>
       <c r="S4" s="159" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="T4" s="160"/>
       <c r="Z4" s="48"/>
@@ -45189,7 +45198,7 @@
       <c r="P5" s="162"/>
       <c r="S5" s="160"/>
       <c r="T5" s="163" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
     </row>
     <row r="6">
@@ -45222,11 +45231,11 @@
       <c r="R6" s="5"/>
       <c r="S6" s="160"/>
       <c r="T6" s="163" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="Z6" s="98"/>
       <c r="AD6" s="38" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
     </row>
     <row r="7">
@@ -45256,7 +45265,7 @@
       <c r="O7" s="90"/>
       <c r="P7" s="165"/>
       <c r="AD7" s="163" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="AE7" s="160"/>
       <c r="AF7" s="160"/>
@@ -45289,11 +45298,11 @@
       <c r="O8" s="90"/>
       <c r="P8" s="165"/>
       <c r="S8" s="163" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="AA8" s="98"/>
       <c r="AD8" s="163" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
     </row>
     <row r="9">
@@ -45492,7 +45501,7 @@
       <c r="O15" s="90"/>
       <c r="P15" s="165"/>
       <c r="S15" s="38" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
     </row>
     <row r="16">
@@ -45605,7 +45614,7 @@
       <c r="Q19" s="5"/>
       <c r="R19" s="5"/>
       <c r="S19" s="38" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20">
@@ -45743,7 +45752,7 @@
     </row>
     <row r="24">
       <c r="A24" s="114" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B24" s="169" t="str">
         <f t="shared" ref="B24:F24" si="4">IFERROR(AVERAGE(B3:B22),"")</f>
@@ -45889,7 +45898,7 @@
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
       <c r="G27" s="170" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="H27" s="5"/>
       <c r="I27" s="5"/>
@@ -45934,7 +45943,7 @@
         <v>1.0</v>
       </c>
       <c r="H28" s="171" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I28" s="171">
         <v>2.0</v>
@@ -45974,7 +45983,7 @@
       <c r="B29" s="5"/>
       <c r="C29" s="5"/>
       <c r="D29" s="4" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -45996,10 +46005,10 @@
       </c>
       <c r="K29" s="5"/>
       <c r="L29" s="114" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="M29" s="114" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -46099,7 +46108,7 @@
       </c>
       <c r="R31" s="5"/>
       <c r="S31" s="114" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="T31" s="5"/>
       <c r="U31" s="5"/>
@@ -46161,7 +46170,7 @@
       <c r="E33" s="5"/>
       <c r="F33" s="5"/>
       <c r="G33" s="116" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J33" s="5"/>
       <c r="K33" s="5"/>
@@ -46175,10 +46184,10 @@
       <c r="P33" s="5"/>
       <c r="R33" s="5"/>
       <c r="T33" s="68" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="W33" s="38" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="AA33" s="48"/>
       <c r="AD33" s="5"/>
@@ -46197,7 +46206,7 @@
         <v>1.0</v>
       </c>
       <c r="H34" s="174" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="I34" s="174">
         <v>2.0</v>
@@ -46221,7 +46230,7 @@
         <v>1626.0</v>
       </c>
       <c r="U34" s="42" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="W34" s="38">
         <v>5193.0</v>
@@ -46266,7 +46275,7 @@
         <v>4176.0</v>
       </c>
       <c r="U35" s="42" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="W35" s="38">
         <v>4863.0</v>
@@ -46364,7 +46373,7 @@
       <c r="D38" s="5"/>
       <c r="E38" s="5"/>
       <c r="F38" s="4" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="G38" s="173">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>
@@ -46566,7 +46575,7 @@
       <c r="Q45" s="5"/>
       <c r="R45" s="5"/>
       <c r="T45" s="163" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="AD45" s="5"/>
       <c r="AE45" s="5"/>
@@ -46703,10 +46712,10 @@
         <v>4</v>
       </c>
       <c r="X49" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="Y49" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="Z49" s="4" t="s">
         <v>5</v>
@@ -46721,16 +46730,16 @@
         <v>8</v>
       </c>
       <c r="AD49" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="AE49" s="30" t="s">
+        <v>109</v>
+      </c>
+      <c r="AF49" s="30" t="s">
         <v>93</v>
       </c>
-      <c r="AE49" s="30" t="s">
-        <v>108</v>
-      </c>
-      <c r="AF49" s="30" t="s">
-        <v>92</v>
-      </c>
       <c r="AG49" s="30" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
     </row>
     <row r="50">
@@ -46895,7 +46904,7 @@
         <v>13.03594852814783</v>
       </c>
       <c r="AG52" s="30" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="53">
@@ -46956,7 +46965,7 @@
         <v>6.291840048860032</v>
       </c>
       <c r="AG53" s="30" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="54">
@@ -47017,7 +47026,7 @@
         <v>2.7243520649411117</v>
       </c>
       <c r="AG54" s="30" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="55">
@@ -47078,7 +47087,7 @@
         <v>2.1429979739456915</v>
       </c>
       <c r="AG55" s="30" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="56">
@@ -47139,7 +47148,7 @@
         <v>3.98032040346951</v>
       </c>
       <c r="AG56" s="30" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="57">
@@ -47362,10 +47371,10 @@
       <c r="R62" s="5"/>
       <c r="S62" s="5"/>
       <c r="U62" s="38" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="V62" s="38" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="AC62" s="5"/>
       <c r="AD62" s="5"/>
@@ -47407,7 +47416,7 @@
         <v>2165.0</v>
       </c>
       <c r="W63" s="38" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="AC63" s="5"/>
       <c r="AD63" s="5"/>
@@ -48041,7 +48050,7 @@
       <c r="R79" s="5"/>
       <c r="S79" s="5"/>
       <c r="T79" s="114" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="U79" s="5"/>
       <c r="V79" s="5"/>
@@ -48082,7 +48091,7 @@
       <c r="R80" s="5"/>
       <c r="S80" s="5"/>
       <c r="T80" s="38" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="U80" s="13"/>
       <c r="V80" s="13"/>
@@ -80843,146 +80852,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="38" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="5"/>
       <c r="C2" s="182" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="E2" s="183"/>
       <c r="F2" s="114" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="H2" s="183"/>
     </row>
     <row r="3">
       <c r="B3" s="133" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C3" s="184" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D3" s="133" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="E3" s="185" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="F3" s="133" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="G3" s="133" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H3" s="133" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="186" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C4" s="187" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D4" s="134" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E4" s="188" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F4" s="189" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="G4" s="189" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H4" s="134"/>
     </row>
     <row r="5">
       <c r="B5" s="186" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C5" s="190" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="D5" s="144"/>
       <c r="E5" s="188" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F5" s="191" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="G5" s="192" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="H5" s="134"/>
     </row>
     <row r="6">
       <c r="B6" s="186" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C6" s="187" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="D6" s="134" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E6" s="188" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="F6" s="134" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="G6" s="134"/>
       <c r="H6" s="134"/>
     </row>
     <row r="7">
       <c r="B7" s="134" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C7" s="193" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D7" s="134"/>
       <c r="E7" s="194" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="F7" s="187" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="G7" s="134"/>
       <c r="H7" s="134" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="195" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C8" s="196" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D8" s="197"/>
       <c r="E8" s="195" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="F8" s="198" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="G8" s="199" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="H8" s="197"/>
     </row>
     <row r="9">
       <c r="B9" s="14" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C9" s="200" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="D9" s="90"/>
       <c r="E9" s="90"/>
@@ -80992,27 +81001,27 @@
     </row>
     <row r="10">
       <c r="B10" s="14" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C10" s="164"/>
       <c r="D10" s="90"/>
       <c r="E10" s="90"/>
       <c r="F10" s="164"/>
       <c r="G10" s="189" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="H10" s="90"/>
     </row>
     <row r="11">
       <c r="B11" s="14" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C11" s="164"/>
       <c r="D11" s="90"/>
       <c r="E11" s="90"/>
       <c r="F11" s="164"/>
       <c r="G11" s="201" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="H11" s="14"/>
     </row>

</xml_diff>

<commit_message>
DATA. Actualizo preds para eng hoy.
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -516,7 +516,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="869" uniqueCount="445">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="886" uniqueCount="461">
   <si>
     <t>id_country</t>
   </si>
@@ -1537,25 +1537,25 @@
     <t>1.39</t>
   </si>
   <si>
-    <t>0.30</t>
+    <t>1.50</t>
   </si>
   <si>
-    <t>3.88</t>
+    <t>0.46</t>
   </si>
   <si>
-    <t>2.68</t>
+    <t>0.84</t>
   </si>
   <si>
-    <t>10.34</t>
+    <t>2.83</t>
   </si>
   <si>
-    <t>3.34</t>
+    <t>1.52</t>
   </si>
   <si>
-    <t>2.81</t>
+    <t>1.94</t>
   </si>
   <si>
-    <t>0.33</t>
+    <t>1.91</t>
   </si>
   <si>
     <t>Country</t>
@@ -1564,34 +1564,97 @@
     <t>Correl ROI y Expected ROI</t>
   </si>
   <si>
-    <t>6.28</t>
+    <t>0.24</t>
   </si>
   <si>
-    <t>2.37</t>
+    <t>0.54</t>
   </si>
   <si>
     <t>mean</t>
   </si>
   <si>
-    <t>4.07</t>
+    <t>3.88</t>
   </si>
   <si>
     <t>median</t>
   </si>
   <si>
-    <t>5.16</t>
+    <t>4.22</t>
   </si>
   <si>
     <t>p25</t>
   </si>
   <si>
-    <t>0.39</t>
+    <t>4.62</t>
   </si>
   <si>
     <t>p75</t>
   </si>
   <si>
+    <t>5.77</t>
+  </si>
+  <si>
+    <t>3.56</t>
+  </si>
+  <si>
     <t>3.78</t>
+  </si>
+  <si>
+    <t>5.26</t>
+  </si>
+  <si>
+    <t>5.86</t>
+  </si>
+  <si>
+    <t>4.45</t>
+  </si>
+  <si>
+    <t>6.81</t>
+  </si>
+  <si>
+    <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
+  </si>
+  <si>
+    <t>1.35</t>
+  </si>
+  <si>
+    <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
+  </si>
+  <si>
+    <t>1.69</t>
+  </si>
+  <si>
+    <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
+  </si>
+  <si>
+    <t>0.86</t>
+  </si>
+  <si>
+    <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
+  </si>
+  <si>
+    <t>1.24</t>
+  </si>
+  <si>
+    <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
+  </si>
+  <si>
+    <t>2.38</t>
+  </si>
+  <si>
+    <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
+  </si>
+  <si>
+    <t>1.73</t>
+  </si>
+  <si>
+    <t>3.92</t>
+  </si>
+  <si>
+    <t>4.91</t>
+  </si>
+  <si>
+    <t>1.96</t>
   </si>
   <si>
     <t>2.94</t>
@@ -1612,31 +1675,16 @@
     <t>7.02</t>
   </si>
   <si>
-    <t>Gracias a las nuevas métricas de G/P sin bank en test, me di cuenta de que:</t>
-  </si>
-  <si>
     <t>9.13</t>
-  </si>
-  <si>
-    <t>La rentabilidad en ITA está en el visitante y no en el empate como creía.</t>
   </si>
   <si>
     <t>3.00</t>
   </si>
   <si>
-    <t>La rentabilidad en ENG y GER está en el empate tal como creía.</t>
-  </si>
-  <si>
-    <t>En SPA esta repartido aunque Empate saca una ventaja.</t>
-  </si>
-  <si>
     <t>1.90</t>
   </si>
   <si>
-    <t>En FRA, depende el modelo. A veces local, a veces, empate.</t>
-  </si>
-  <si>
-    <t>Si en FRA empate no rinde, no tiene sentido exigirle una buena distrib en empate… → Tiene sentido pero al parecer si importa el empate puesto que el modelo que gana se basa en empate.</t>
+    <t>0.39</t>
   </si>
   <si>
     <t>5.85</t>
@@ -1645,7 +1693,7 @@
     <t>5.70</t>
   </si>
   <si>
-    <t>0.63</t>
+    <t>3.14</t>
   </si>
   <si>
     <t>5.67</t>
@@ -1654,28 +1702,28 @@
     <t>3.55</t>
   </si>
   <si>
-    <t>3.11</t>
+    <t>2.42</t>
   </si>
   <si>
-    <t>3.05</t>
+    <t>2.64</t>
   </si>
   <si>
-    <t>5.86</t>
+    <t>3.50</t>
   </si>
   <si>
-    <t>0.37</t>
+    <t>1.99</t>
   </si>
   <si>
-    <t>2.57</t>
+    <t>2.27</t>
   </si>
   <si>
-    <t>2.28</t>
+    <t>2.55</t>
   </si>
   <si>
-    <t>2.02</t>
+    <t>1.81</t>
   </si>
   <si>
-    <t>2.22</t>
+    <t>2.16</t>
   </si>
   <si>
     <t>RENTABILIDAD</t>
@@ -3528,7 +3576,7 @@
         <v>45739.0</v>
       </c>
       <c r="D4" s="14">
-        <v>1071.0</v>
+        <v>458.0</v>
       </c>
       <c r="E4" s="14" t="s">
         <v>17</v>
@@ -3537,14 +3585,14 @@
         <v>5.0</v>
       </c>
       <c r="G4" s="24">
-        <v>9.74</v>
+        <v>12.8</v>
       </c>
       <c r="H4" s="24">
-        <v>9.74</v>
+        <v>10.79</v>
       </c>
       <c r="I4" s="24">
         <f t="shared" ref="I4:I8" si="1">AVERAGE(F4:H4)</f>
-        <v>8.16</v>
+        <v>9.53</v>
       </c>
       <c r="J4" s="25">
         <v>5.0</v>
@@ -8759,7 +8807,7 @@
     </row>
   </sheetData>
   <autoFilter ref="$A$1:$P$8"/>
-  <conditionalFormatting sqref="F4:I8">
+  <conditionalFormatting sqref="F4:H8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -8802,146 +8850,146 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="76" t="s">
-        <v>378</v>
+        <v>394</v>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="17"/>
       <c r="C2" s="5" t="s">
-        <v>379</v>
+        <v>395</v>
       </c>
       <c r="E2" s="235"/>
       <c r="F2" s="6" t="s">
-        <v>380</v>
+        <v>396</v>
       </c>
       <c r="H2" s="235"/>
     </row>
     <row r="3">
       <c r="B3" s="186" t="s">
-        <v>381</v>
+        <v>397</v>
       </c>
       <c r="C3" s="236" t="s">
-        <v>382</v>
+        <v>398</v>
       </c>
       <c r="D3" s="186" t="s">
-        <v>383</v>
+        <v>399</v>
       </c>
       <c r="E3" s="237" t="s">
         <v>212</v>
       </c>
       <c r="F3" s="186" t="s">
-        <v>384</v>
+        <v>400</v>
       </c>
       <c r="G3" s="186" t="s">
-        <v>385</v>
+        <v>401</v>
       </c>
       <c r="H3" s="186" t="s">
-        <v>386</v>
+        <v>402</v>
       </c>
     </row>
     <row r="4">
       <c r="B4" s="238" t="s">
-        <v>387</v>
+        <v>403</v>
       </c>
       <c r="C4" s="239" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="D4" s="187" t="s">
-        <v>389</v>
+        <v>405</v>
       </c>
       <c r="E4" s="240" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="F4" s="241" t="s">
-        <v>391</v>
+        <v>407</v>
       </c>
       <c r="G4" s="241" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="H4" s="187"/>
     </row>
     <row r="5">
       <c r="B5" s="238" t="s">
-        <v>393</v>
+        <v>409</v>
       </c>
       <c r="C5" s="242" t="s">
-        <v>394</v>
+        <v>410</v>
       </c>
       <c r="D5" s="197"/>
       <c r="E5" s="240" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="F5" s="243" t="s">
-        <v>395</v>
+        <v>411</v>
       </c>
       <c r="G5" s="244" t="s">
-        <v>396</v>
+        <v>412</v>
       </c>
       <c r="H5" s="187"/>
     </row>
     <row r="6">
       <c r="B6" s="238" t="s">
-        <v>397</v>
+        <v>413</v>
       </c>
       <c r="C6" s="239" t="s">
-        <v>388</v>
+        <v>404</v>
       </c>
       <c r="D6" s="187" t="s">
-        <v>398</v>
+        <v>414</v>
       </c>
       <c r="E6" s="240" t="s">
-        <v>390</v>
+        <v>406</v>
       </c>
       <c r="F6" s="187" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="G6" s="187"/>
       <c r="H6" s="187"/>
     </row>
     <row r="7">
       <c r="B7" s="187" t="s">
-        <v>399</v>
+        <v>415</v>
       </c>
       <c r="C7" s="245" t="s">
-        <v>400</v>
+        <v>416</v>
       </c>
       <c r="D7" s="187"/>
       <c r="E7" s="246" t="s">
-        <v>401</v>
+        <v>417</v>
       </c>
       <c r="F7" s="239" t="s">
-        <v>402</v>
+        <v>418</v>
       </c>
       <c r="G7" s="187"/>
       <c r="H7" s="187" t="s">
-        <v>403</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="247" t="s">
-        <v>404</v>
+        <v>420</v>
       </c>
       <c r="C8" s="248" t="s">
-        <v>405</v>
+        <v>421</v>
       </c>
       <c r="D8" s="249"/>
       <c r="E8" s="247" t="s">
-        <v>406</v>
+        <v>422</v>
       </c>
       <c r="F8" s="250" t="s">
-        <v>407</v>
+        <v>423</v>
       </c>
       <c r="G8" s="251" t="s">
-        <v>408</v>
+        <v>424</v>
       </c>
       <c r="H8" s="249"/>
     </row>
     <row r="9">
       <c r="B9" s="20" t="s">
-        <v>409</v>
+        <v>425</v>
       </c>
       <c r="C9" s="252" t="s">
-        <v>405</v>
+        <v>421</v>
       </c>
       <c r="D9" s="143"/>
       <c r="E9" s="143"/>
@@ -8951,27 +8999,27 @@
     </row>
     <row r="10">
       <c r="B10" s="20" t="s">
-        <v>410</v>
+        <v>426</v>
       </c>
       <c r="C10" s="217"/>
       <c r="D10" s="143"/>
       <c r="E10" s="143"/>
       <c r="F10" s="217"/>
       <c r="G10" s="241" t="s">
-        <v>392</v>
+        <v>408</v>
       </c>
       <c r="H10" s="143"/>
     </row>
     <row r="11">
       <c r="B11" s="20" t="s">
-        <v>411</v>
+        <v>427</v>
       </c>
       <c r="C11" s="217"/>
       <c r="D11" s="143"/>
       <c r="E11" s="143"/>
       <c r="F11" s="217"/>
       <c r="G11" s="253" t="s">
-        <v>412</v>
+        <v>428</v>
       </c>
       <c r="H11" s="20"/>
     </row>
@@ -8994,7 +9042,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="90" t="s">
-        <v>413</v>
+        <v>429</v>
       </c>
       <c r="L1" s="32"/>
     </row>
@@ -9003,16 +9051,16 @@
     </row>
     <row r="3">
       <c r="A3" s="76" t="s">
-        <v>414</v>
+        <v>430</v>
       </c>
       <c r="L3" s="32"/>
     </row>
     <row r="4">
       <c r="B4" s="76" t="s">
-        <v>415</v>
+        <v>431</v>
       </c>
       <c r="G4" s="76" t="s">
-        <v>416</v>
+        <v>432</v>
       </c>
       <c r="L4" s="32"/>
     </row>
@@ -9118,45 +9166,45 @@
     </row>
     <row r="11">
       <c r="A11" s="254" t="s">
-        <v>417</v>
+        <v>433</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="90" t="s">
-        <v>418</v>
+        <v>434</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="76" t="s">
-        <v>419</v>
+        <v>435</v>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="254" t="s">
-        <v>420</v>
+        <v>436</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="90" t="s">
-        <v>421</v>
+        <v>437</v>
       </c>
     </row>
     <row r="19">
       <c r="B19" s="76" t="s">
-        <v>422</v>
+        <v>438</v>
       </c>
       <c r="F19" s="151"/>
     </row>
     <row r="20">
       <c r="B20" s="90" t="s">
-        <v>423</v>
+        <v>439</v>
       </c>
       <c r="C20" s="105"/>
       <c r="D20" s="105"/>
       <c r="E20" s="105"/>
       <c r="F20" s="105"/>
       <c r="G20" s="90" t="s">
-        <v>424</v>
+        <v>440</v>
       </c>
       <c r="H20" s="90" t="s">
         <v>65</v>
@@ -9173,7 +9221,7 @@
     </row>
     <row r="21">
       <c r="B21" s="90" t="s">
-        <v>425</v>
+        <v>441</v>
       </c>
       <c r="G21" s="107">
         <v>2.575</v>
@@ -9181,27 +9229,27 @@
     </row>
     <row r="23">
       <c r="K23" s="90" t="s">
-        <v>426</v>
+        <v>442</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="76" t="s">
-        <v>427</v>
+        <v>443</v>
       </c>
       <c r="H24" s="76" t="s">
         <v>43</v>
       </c>
       <c r="I24" s="76" t="s">
-        <v>428</v>
+        <v>444</v>
       </c>
       <c r="K24" s="76" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="L24" s="76" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="M24" s="76" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
     </row>
     <row r="25">
@@ -9220,7 +9268,7 @@
         <v>#REF!</v>
       </c>
       <c r="K25" s="76" t="s">
-        <v>432</v>
+        <v>448</v>
       </c>
     </row>
     <row r="26">
@@ -9231,7 +9279,7 @@
         <v>1.19</v>
       </c>
       <c r="K26" s="76" t="s">
-        <v>433</v>
+        <v>449</v>
       </c>
     </row>
     <row r="27">
@@ -9242,7 +9290,7 @@
         <v>2.19</v>
       </c>
       <c r="K27" s="76" t="s">
-        <v>434</v>
+        <v>450</v>
       </c>
     </row>
     <row r="28">
@@ -9253,7 +9301,7 @@
         <v>0.05</v>
       </c>
       <c r="K28" s="76" t="s">
-        <v>435</v>
+        <v>451</v>
       </c>
     </row>
     <row r="29">
@@ -9272,7 +9320,7 @@
         <v>6.42</v>
       </c>
       <c r="K30" s="93" t="s">
-        <v>436</v>
+        <v>452</v>
       </c>
     </row>
     <row r="31">
@@ -9417,7 +9465,7 @@
         <v>0.61</v>
       </c>
       <c r="K41" s="90" t="s">
-        <v>437</v>
+        <v>453</v>
       </c>
     </row>
     <row r="42">
@@ -9428,13 +9476,13 @@
         <v>0.69</v>
       </c>
       <c r="K42" s="76" t="s">
-        <v>429</v>
+        <v>445</v>
       </c>
       <c r="L42" s="76" t="s">
-        <v>430</v>
+        <v>446</v>
       </c>
       <c r="M42" s="76" t="s">
-        <v>431</v>
+        <v>447</v>
       </c>
     </row>
     <row r="43">
@@ -9566,7 +9614,7 @@
         <v>0.0</v>
       </c>
       <c r="K51" s="76" t="s">
-        <v>438</v>
+        <v>454</v>
       </c>
     </row>
     <row r="52">
@@ -9594,17 +9642,17 @@
       </c>
       <c r="K54" s="143"/>
       <c r="L54" s="255" t="s">
-        <v>439</v>
+        <v>455</v>
       </c>
       <c r="M54" s="256"/>
       <c r="N54" s="148" t="s">
         <v>155</v>
       </c>
       <c r="O54" s="148" t="s">
-        <v>440</v>
+        <v>456</v>
       </c>
       <c r="P54" s="148" t="s">
-        <v>441</v>
+        <v>457</v>
       </c>
       <c r="R54" s="79" t="s">
         <v>222</v>
@@ -9686,7 +9734,7 @@
         <v>5.86</v>
       </c>
       <c r="R57" s="76" t="s">
-        <v>442</v>
+        <v>458</v>
       </c>
       <c r="S57" s="107">
         <f>SUM(P55:P74)</f>
@@ -9715,7 +9763,7 @@
         <v>0.855</v>
       </c>
       <c r="P58" s="20" t="s">
-        <v>443</v>
+        <v>459</v>
       </c>
     </row>
     <row r="59">
@@ -9762,7 +9810,7 @@
         <v>0.96</v>
       </c>
       <c r="P60" s="20" t="s">
-        <v>444</v>
+        <v>460</v>
       </c>
     </row>
     <row r="61">
@@ -24468,7 +24516,7 @@
       <c r="C37" s="105"/>
       <c r="D37" s="181">
         <f>AVERAGE(D39:D1775)</f>
-        <v>3.356097561</v>
+        <v>3.140689655</v>
       </c>
       <c r="G37" s="90" t="s">
         <v>34</v>
@@ -24575,7 +24623,7 @@
       </c>
       <c r="D40" s="172">
         <f t="shared" si="17"/>
-        <v>0.3</v>
+        <v>1.5</v>
       </c>
       <c r="G40" s="90" t="s">
         <v>38</v>
@@ -24613,7 +24661,7 @@
       </c>
       <c r="D41" s="172">
         <f t="shared" si="17"/>
-        <v>3.88</v>
+        <v>0.46</v>
       </c>
       <c r="P41" s="170">
         <v>0.0</v>
@@ -24645,7 +24693,7 @@
       </c>
       <c r="D42" s="172">
         <f t="shared" si="17"/>
-        <v>2.68</v>
+        <v>0.84</v>
       </c>
       <c r="P42" s="170">
         <v>2.0</v>
@@ -24677,7 +24725,7 @@
       </c>
       <c r="D43" s="172">
         <f t="shared" si="17"/>
-        <v>10.34</v>
+        <v>2.83</v>
       </c>
       <c r="P43" s="170">
         <v>1.0</v>
@@ -24709,7 +24757,7 @@
       </c>
       <c r="D44" s="172">
         <f t="shared" si="17"/>
-        <v>3.34</v>
+        <v>1.52</v>
       </c>
       <c r="P44" s="170">
         <v>2.0</v>
@@ -24739,7 +24787,7 @@
       </c>
       <c r="D45" s="172">
         <f t="shared" si="17"/>
-        <v>2.81</v>
+        <v>1.94</v>
       </c>
       <c r="P45" s="170">
         <v>1.0</v>
@@ -24757,7 +24805,7 @@
       </c>
       <c r="D46" s="172">
         <f t="shared" si="17"/>
-        <v>0.33</v>
+        <v>1.91</v>
       </c>
       <c r="G46" s="186" t="s">
         <v>297</v>
@@ -24781,7 +24829,7 @@
       </c>
       <c r="D47" s="172">
         <f t="shared" si="17"/>
-        <v>6.28</v>
+        <v>0.24</v>
       </c>
       <c r="G47" s="187" t="s">
         <v>33</v>
@@ -24811,7 +24859,7 @@
       </c>
       <c r="D48" s="172">
         <f t="shared" si="17"/>
-        <v>2.37</v>
+        <v>0.54</v>
       </c>
       <c r="G48" s="187" t="s">
         <v>34</v>
@@ -24848,7 +24896,7 @@
       </c>
       <c r="D49" s="172">
         <f t="shared" si="17"/>
-        <v>4.07</v>
+        <v>3.88</v>
       </c>
       <c r="G49" s="187" t="s">
         <v>36</v>
@@ -24885,7 +24933,7 @@
       </c>
       <c r="D50" s="172">
         <f t="shared" si="17"/>
-        <v>5.16</v>
+        <v>4.22</v>
       </c>
       <c r="G50" s="187" t="s">
         <v>37</v>
@@ -24922,7 +24970,7 @@
       </c>
       <c r="D51" s="172">
         <f t="shared" si="17"/>
-        <v>0.39</v>
+        <v>4.62</v>
       </c>
       <c r="G51" s="187" t="s">
         <v>38</v>
@@ -24959,7 +25007,7 @@
       </c>
       <c r="D52" s="172">
         <f t="shared" si="17"/>
-        <v>3.78</v>
+        <v>5.77</v>
       </c>
       <c r="P52" s="170">
         <v>0.0</v>
@@ -24983,7 +25031,7 @@
       </c>
       <c r="D53" s="172">
         <f t="shared" si="17"/>
-        <v>2.94</v>
+        <v>3.56</v>
       </c>
       <c r="P53" s="170">
         <v>0.0</v>
@@ -25007,7 +25055,7 @@
       </c>
       <c r="D54" s="172">
         <f t="shared" si="17"/>
-        <v>2.59</v>
+        <v>3.78</v>
       </c>
       <c r="P54" s="170">
         <v>2.0</v>
@@ -25031,7 +25079,7 @@
       </c>
       <c r="D55" s="172">
         <f t="shared" si="17"/>
-        <v>2.18</v>
+        <v>5.26</v>
       </c>
       <c r="P55" s="170">
         <v>0.0</v>
@@ -25055,7 +25103,7 @@
       </c>
       <c r="D56" s="172">
         <f t="shared" si="17"/>
-        <v>2.03</v>
+        <v>5.86</v>
       </c>
       <c r="P56" s="170">
         <v>0.0</v>
@@ -25079,7 +25127,7 @@
       </c>
       <c r="D57" s="172">
         <f t="shared" si="17"/>
-        <v>3.85</v>
+        <v>4.45</v>
       </c>
       <c r="P57" s="170">
         <v>2.0</v>
@@ -25103,7 +25151,7 @@
       </c>
       <c r="D58" s="172">
         <f t="shared" si="17"/>
-        <v>7.02</v>
+        <v>6.81</v>
       </c>
       <c r="G58" s="189" t="s">
         <v>315</v>
@@ -25131,7 +25179,7 @@
       </c>
       <c r="D59" s="172">
         <f t="shared" si="17"/>
-        <v>9.13</v>
+        <v>1.35</v>
       </c>
       <c r="G59" s="190"/>
       <c r="H59" s="191" t="s">
@@ -25159,7 +25207,7 @@
       </c>
       <c r="D60" s="172">
         <f t="shared" si="17"/>
-        <v>3</v>
+        <v>1.69</v>
       </c>
       <c r="G60" s="190"/>
       <c r="H60" s="191" t="s">
@@ -25183,15 +25231,15 @@
     </row>
     <row r="61">
       <c r="C61" s="185" t="s">
-        <v>269</v>
+        <v>320</v>
       </c>
       <c r="D61" s="172">
         <f t="shared" si="17"/>
-        <v>2.71</v>
+        <v>0.86</v>
       </c>
       <c r="G61" s="190"/>
       <c r="H61" s="191" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="P61" s="170">
         <v>2.0</v>
@@ -25211,15 +25259,15 @@
     </row>
     <row r="62">
       <c r="C62" s="185" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D62" s="172">
         <f t="shared" si="17"/>
-        <v>1.9</v>
+        <v>1.24</v>
       </c>
       <c r="G62" s="190"/>
       <c r="H62" s="191" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="P62" s="170">
         <v>1.0</v>
@@ -25239,15 +25287,15 @@
     </row>
     <row r="63">
       <c r="C63" s="185" t="s">
-        <v>306</v>
+        <v>324</v>
       </c>
       <c r="D63" s="172">
         <f t="shared" si="17"/>
-        <v>0.39</v>
+        <v>2.38</v>
       </c>
       <c r="G63" s="190"/>
       <c r="H63" s="191" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="P63" s="170">
         <v>0.0</v>
@@ -25261,11 +25309,11 @@
     </row>
     <row r="64">
       <c r="C64" s="185" t="s">
-        <v>241</v>
+        <v>326</v>
       </c>
       <c r="D64" s="172">
         <f t="shared" si="17"/>
-        <v>5.8</v>
+        <v>1.73</v>
       </c>
       <c r="P64" s="170">
         <v>1.0</v>
@@ -25279,11 +25327,11 @@
     </row>
     <row r="65">
       <c r="C65" s="185" t="s">
-        <v>324</v>
+        <v>253</v>
       </c>
       <c r="D65" s="172">
         <f t="shared" si="17"/>
-        <v>5.85</v>
+        <v>3.83</v>
       </c>
       <c r="P65" s="170">
         <v>2.0</v>
@@ -25297,11 +25345,11 @@
     </row>
     <row r="66">
       <c r="C66" s="185" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="D66" s="172">
         <f t="shared" si="17"/>
-        <v>5.7</v>
+        <v>3.92</v>
       </c>
       <c r="P66" s="170">
         <v>0.0</v>
@@ -25315,11 +25363,11 @@
     </row>
     <row r="67">
       <c r="C67" s="185" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="D67" s="172">
         <f t="shared" si="17"/>
-        <v>0.63</v>
+        <v>4.91</v>
       </c>
       <c r="P67" s="170">
         <v>0.0</v>
@@ -25333,11 +25381,11 @@
     </row>
     <row r="68">
       <c r="C68" s="185" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="D68" s="172">
         <f t="shared" si="17"/>
-        <v>5.67</v>
+        <v>1.96</v>
       </c>
       <c r="P68" s="170">
         <v>1.0</v>
@@ -25351,11 +25399,11 @@
     </row>
     <row r="69">
       <c r="C69" s="185" t="s">
-        <v>328</v>
+        <v>310</v>
       </c>
       <c r="D69" s="172">
         <f t="shared" si="17"/>
-        <v>3.55</v>
+        <v>3.78</v>
       </c>
       <c r="P69" s="170">
         <v>2.0</v>
@@ -25369,11 +25417,11 @@
     </row>
     <row r="70">
       <c r="C70" s="185" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
       <c r="D70" s="172">
         <f t="shared" si="17"/>
-        <v>2.03</v>
+        <v>2.94</v>
       </c>
       <c r="P70" s="170">
         <v>1.0</v>
@@ -25387,11 +25435,11 @@
     </row>
     <row r="71">
       <c r="C71" s="185" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="D71" s="172">
         <f t="shared" si="17"/>
-        <v>3.11</v>
+        <v>2.59</v>
       </c>
       <c r="F71" s="192"/>
       <c r="P71" s="170">
@@ -25406,11 +25454,11 @@
     </row>
     <row r="72">
       <c r="C72" s="185" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D72" s="172">
         <f t="shared" si="17"/>
-        <v>3.05</v>
+        <v>2.18</v>
       </c>
       <c r="P72" s="170">
         <v>0.0</v>
@@ -25424,11 +25472,11 @@
     </row>
     <row r="73">
       <c r="C73" s="185" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="D73" s="172">
         <f t="shared" si="17"/>
-        <v>5.86</v>
+        <v>2.03</v>
       </c>
       <c r="P73" s="170">
         <v>1.0</v>
@@ -25442,11 +25490,11 @@
     </row>
     <row r="74">
       <c r="C74" s="185" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="D74" s="172">
         <f t="shared" si="17"/>
-        <v>0.37</v>
+        <v>3.85</v>
       </c>
       <c r="P74" s="170">
         <v>0.0</v>
@@ -25460,11 +25508,11 @@
     </row>
     <row r="75">
       <c r="C75" s="185" t="s">
-        <v>312</v>
+        <v>335</v>
       </c>
       <c r="D75" s="172">
         <f t="shared" si="17"/>
-        <v>2.03</v>
+        <v>7.02</v>
       </c>
       <c r="P75" s="170">
         <v>1.0</v>
@@ -25478,11 +25526,11 @@
     </row>
     <row r="76">
       <c r="C76" s="185" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="D76" s="172">
         <f t="shared" si="17"/>
-        <v>2.57</v>
+        <v>9.13</v>
       </c>
       <c r="P76" s="170">
         <v>0.0</v>
@@ -25496,11 +25544,11 @@
     </row>
     <row r="77">
       <c r="C77" s="185" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="D77" s="172">
         <f t="shared" si="17"/>
-        <v>2.28</v>
+        <v>3</v>
       </c>
       <c r="P77" s="170">
         <v>0.0</v>
@@ -25514,11 +25562,11 @@
     </row>
     <row r="78">
       <c r="C78" s="185" t="s">
-        <v>335</v>
+        <v>269</v>
       </c>
       <c r="D78" s="172">
         <f t="shared" si="17"/>
-        <v>2.02</v>
+        <v>2.71</v>
       </c>
       <c r="P78" s="170">
         <v>1.0</v>
@@ -25532,11 +25580,11 @@
     </row>
     <row r="79">
       <c r="C79" s="185" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="D79" s="172">
         <f t="shared" si="17"/>
-        <v>2.22</v>
+        <v>1.9</v>
       </c>
       <c r="P79" s="170">
         <v>2.0</v>
@@ -25549,10 +25597,12 @@
       </c>
     </row>
     <row r="80">
-      <c r="C80" s="185"/>
-      <c r="D80" s="172" t="str">
+      <c r="C80" s="185" t="s">
+        <v>339</v>
+      </c>
+      <c r="D80" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>0.39</v>
       </c>
       <c r="P80" s="170">
         <v>1.0</v>
@@ -25565,10 +25615,12 @@
       </c>
     </row>
     <row r="81">
-      <c r="C81" s="185"/>
-      <c r="D81" s="172" t="str">
+      <c r="C81" s="185" t="s">
+        <v>241</v>
+      </c>
+      <c r="D81" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>5.8</v>
       </c>
       <c r="P81" s="170">
         <v>2.0</v>
@@ -25581,10 +25633,12 @@
       </c>
     </row>
     <row r="82">
-      <c r="C82" s="185"/>
-      <c r="D82" s="172" t="str">
+      <c r="C82" s="185" t="s">
+        <v>340</v>
+      </c>
+      <c r="D82" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>5.85</v>
       </c>
       <c r="P82" s="170">
         <v>1.0</v>
@@ -25597,10 +25651,12 @@
       </c>
     </row>
     <row r="83">
-      <c r="C83" s="185"/>
-      <c r="D83" s="172" t="str">
+      <c r="C83" s="185" t="s">
+        <v>341</v>
+      </c>
+      <c r="D83" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>5.7</v>
       </c>
       <c r="P83" s="170">
         <v>0.0</v>
@@ -25613,10 +25669,12 @@
       </c>
     </row>
     <row r="84">
-      <c r="C84" s="185"/>
-      <c r="D84" s="172" t="str">
+      <c r="C84" s="185" t="s">
+        <v>342</v>
+      </c>
+      <c r="D84" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>3.14</v>
       </c>
       <c r="P84" s="170">
         <v>1.0</v>
@@ -25629,10 +25687,12 @@
       </c>
     </row>
     <row r="85">
-      <c r="C85" s="185"/>
-      <c r="D85" s="172" t="str">
+      <c r="C85" s="185" t="s">
+        <v>343</v>
+      </c>
+      <c r="D85" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>5.67</v>
       </c>
       <c r="P85" s="170">
         <v>0.0</v>
@@ -25645,10 +25705,12 @@
       </c>
     </row>
     <row r="86">
-      <c r="C86" s="185"/>
-      <c r="D86" s="172" t="str">
+      <c r="C86" s="185" t="s">
+        <v>344</v>
+      </c>
+      <c r="D86" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>3.55</v>
       </c>
       <c r="P86" s="170">
         <v>0.0</v>
@@ -25661,10 +25723,12 @@
       </c>
     </row>
     <row r="87">
-      <c r="C87" s="185"/>
-      <c r="D87" s="172" t="str">
+      <c r="C87" s="185" t="s">
+        <v>345</v>
+      </c>
+      <c r="D87" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>2.42</v>
       </c>
       <c r="P87" s="170">
         <v>1.0</v>
@@ -25677,10 +25741,12 @@
       </c>
     </row>
     <row r="88">
-      <c r="C88" s="185"/>
-      <c r="D88" s="172" t="str">
+      <c r="C88" s="185" t="s">
+        <v>346</v>
+      </c>
+      <c r="D88" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>2.64</v>
       </c>
       <c r="P88" s="170">
         <v>2.0</v>
@@ -25693,10 +25759,12 @@
       </c>
     </row>
     <row r="89">
-      <c r="C89" s="185"/>
-      <c r="D89" s="172" t="str">
+      <c r="C89" s="185" t="s">
+        <v>347</v>
+      </c>
+      <c r="D89" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>3.5</v>
       </c>
       <c r="P89" s="170">
         <v>2.0</v>
@@ -25709,10 +25777,12 @@
       </c>
     </row>
     <row r="90">
-      <c r="C90" s="185"/>
-      <c r="D90" s="172" t="str">
+      <c r="C90" s="185" t="s">
+        <v>257</v>
+      </c>
+      <c r="D90" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>3.63</v>
       </c>
       <c r="P90" s="170">
         <v>1.0</v>
@@ -25725,10 +25795,12 @@
       </c>
     </row>
     <row r="91">
-      <c r="C91" s="185"/>
-      <c r="D91" s="172" t="str">
+      <c r="C91" s="185" t="s">
+        <v>348</v>
+      </c>
+      <c r="D91" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>1.99</v>
       </c>
       <c r="P91" s="170">
         <v>1.0</v>
@@ -25741,10 +25813,12 @@
       </c>
     </row>
     <row r="92">
-      <c r="C92" s="185"/>
-      <c r="D92" s="172" t="str">
+      <c r="C92" s="185" t="s">
+        <v>349</v>
+      </c>
+      <c r="D92" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>2.27</v>
       </c>
       <c r="P92" s="170">
         <v>2.0</v>
@@ -25757,10 +25831,12 @@
       </c>
     </row>
     <row r="93">
-      <c r="C93" s="185"/>
-      <c r="D93" s="172" t="str">
+      <c r="C93" s="185" t="s">
+        <v>269</v>
+      </c>
+      <c r="D93" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>2.71</v>
       </c>
       <c r="P93" s="170">
         <v>0.0</v>
@@ -25773,10 +25849,12 @@
       </c>
     </row>
     <row r="94">
-      <c r="C94" s="185"/>
-      <c r="D94" s="172" t="str">
+      <c r="C94" s="185" t="s">
+        <v>350</v>
+      </c>
+      <c r="D94" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>2.55</v>
       </c>
       <c r="P94" s="170">
         <v>0.0</v>
@@ -25789,10 +25867,12 @@
       </c>
     </row>
     <row r="95">
-      <c r="C95" s="185"/>
-      <c r="D95" s="172" t="str">
+      <c r="C95" s="185" t="s">
+        <v>351</v>
+      </c>
+      <c r="D95" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>1.81</v>
       </c>
       <c r="P95" s="170">
         <v>1.0</v>
@@ -25805,10 +25885,12 @@
       </c>
     </row>
     <row r="96">
-      <c r="C96" s="185"/>
-      <c r="D96" s="172" t="str">
+      <c r="C96" s="185" t="s">
+        <v>352</v>
+      </c>
+      <c r="D96" s="172">
         <f t="shared" si="17"/>
-        <v/>
+        <v>2.16</v>
       </c>
       <c r="P96" s="170">
         <v>2.0</v>
@@ -48698,14 +48780,14 @@
     <row r="1">
       <c r="A1" s="197"/>
       <c r="B1" s="198" t="s">
-        <v>337</v>
+        <v>353</v>
       </c>
       <c r="C1" s="199"/>
       <c r="D1" s="199"/>
       <c r="E1" s="199"/>
       <c r="F1" s="199"/>
       <c r="G1" s="200" t="s">
-        <v>338</v>
+        <v>354</v>
       </c>
       <c r="H1" s="199"/>
       <c r="I1" s="199"/>
@@ -48739,19 +48821,19 @@
         <v>3</v>
       </c>
       <c r="B2" s="202" t="s">
-        <v>339</v>
+        <v>355</v>
       </c>
       <c r="C2" s="203" t="s">
-        <v>340</v>
+        <v>356</v>
       </c>
       <c r="D2" s="203" t="s">
         <v>43</v>
       </c>
       <c r="E2" s="203" t="s">
-        <v>341</v>
+        <v>357</v>
       </c>
       <c r="F2" s="204" t="s">
-        <v>342</v>
+        <v>358</v>
       </c>
       <c r="G2" s="202">
         <v>1.0</v>
@@ -48763,30 +48845,30 @@
         <v>2.0</v>
       </c>
       <c r="J2" s="203" t="s">
-        <v>343</v>
+        <v>359</v>
       </c>
       <c r="K2" s="205" t="s">
-        <v>344</v>
+        <v>360</v>
       </c>
       <c r="L2" s="203" t="s">
-        <v>345</v>
+        <v>361</v>
       </c>
       <c r="M2" s="206" t="s">
-        <v>346</v>
+        <v>362</v>
       </c>
       <c r="N2" s="187" t="s">
-        <v>347</v>
+        <v>363</v>
       </c>
       <c r="O2" s="187" t="s">
-        <v>348</v>
+        <v>364</v>
       </c>
       <c r="P2" s="187" t="s">
-        <v>349</v>
+        <v>365</v>
       </c>
       <c r="Q2" s="17"/>
       <c r="R2" s="17"/>
       <c r="S2" s="6" t="s">
-        <v>350</v>
+        <v>366</v>
       </c>
       <c r="T2" s="17"/>
       <c r="U2" s="17"/>
@@ -48876,7 +48958,7 @@
       <c r="Q4" s="17"/>
       <c r="R4" s="17"/>
       <c r="S4" s="212" t="s">
-        <v>351</v>
+        <v>367</v>
       </c>
       <c r="T4" s="213"/>
       <c r="Z4" s="90"/>
@@ -48912,7 +48994,7 @@
       <c r="P5" s="215"/>
       <c r="S5" s="213"/>
       <c r="T5" s="216" t="s">
-        <v>352</v>
+        <v>368</v>
       </c>
     </row>
     <row r="6">
@@ -48945,11 +49027,11 @@
       <c r="R6" s="17"/>
       <c r="S6" s="213"/>
       <c r="T6" s="216" t="s">
-        <v>353</v>
+        <v>369</v>
       </c>
       <c r="Z6" s="151"/>
       <c r="AD6" s="76" t="s">
-        <v>354</v>
+        <v>370</v>
       </c>
     </row>
     <row r="7">
@@ -48979,7 +49061,7 @@
       <c r="O7" s="143"/>
       <c r="P7" s="218"/>
       <c r="AD7" s="216" t="s">
-        <v>355</v>
+        <v>371</v>
       </c>
       <c r="AE7" s="213"/>
       <c r="AF7" s="213"/>
@@ -49012,11 +49094,11 @@
       <c r="O8" s="143"/>
       <c r="P8" s="218"/>
       <c r="S8" s="216" t="s">
-        <v>356</v>
+        <v>372</v>
       </c>
       <c r="AA8" s="151"/>
       <c r="AD8" s="216" t="s">
-        <v>357</v>
+        <v>373</v>
       </c>
     </row>
     <row r="9">
@@ -49215,7 +49297,7 @@
       <c r="O15" s="143"/>
       <c r="P15" s="218"/>
       <c r="S15" s="76" t="s">
-        <v>358</v>
+        <v>374</v>
       </c>
     </row>
     <row r="16">
@@ -49328,7 +49410,7 @@
       <c r="Q19" s="17"/>
       <c r="R19" s="17"/>
       <c r="S19" s="76" t="s">
-        <v>359</v>
+        <v>375</v>
       </c>
     </row>
     <row r="20">
@@ -49612,7 +49694,7 @@
       <c r="E27" s="17"/>
       <c r="F27" s="17"/>
       <c r="G27" s="223" t="s">
-        <v>360</v>
+        <v>376</v>
       </c>
       <c r="H27" s="17"/>
       <c r="I27" s="17"/>
@@ -49697,7 +49779,7 @@
       <c r="B29" s="17"/>
       <c r="C29" s="17"/>
       <c r="D29" s="4" t="s">
-        <v>361</v>
+        <v>377</v>
       </c>
       <c r="E29" s="4">
         <f>J29</f>
@@ -49719,10 +49801,10 @@
       </c>
       <c r="K29" s="17"/>
       <c r="L29" s="6" t="s">
-        <v>362</v>
+        <v>378</v>
       </c>
       <c r="M29" s="6" t="s">
-        <v>363</v>
+        <v>379</v>
       </c>
       <c r="O29" s="4">
         <v>1.0</v>
@@ -49822,7 +49904,7 @@
       </c>
       <c r="R31" s="17"/>
       <c r="S31" s="6" t="s">
-        <v>364</v>
+        <v>380</v>
       </c>
       <c r="T31" s="17"/>
       <c r="U31" s="17"/>
@@ -49884,7 +49966,7 @@
       <c r="E33" s="17"/>
       <c r="F33" s="17"/>
       <c r="G33" s="168" t="s">
-        <v>365</v>
+        <v>381</v>
       </c>
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
@@ -49898,10 +49980,10 @@
       <c r="P33" s="17"/>
       <c r="R33" s="17"/>
       <c r="T33" s="93" t="s">
-        <v>366</v>
+        <v>382</v>
       </c>
       <c r="W33" s="76" t="s">
-        <v>367</v>
+        <v>383</v>
       </c>
       <c r="AA33" s="90"/>
       <c r="AD33" s="17"/>
@@ -49944,7 +50026,7 @@
         <v>1626.0</v>
       </c>
       <c r="U34" s="83" t="s">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="W34" s="76">
         <v>5193.0</v>
@@ -49989,7 +50071,7 @@
         <v>4176.0</v>
       </c>
       <c r="U35" s="83" t="s">
-        <v>368</v>
+        <v>384</v>
       </c>
       <c r="W35" s="76">
         <v>4863.0</v>
@@ -50087,7 +50169,7 @@
       <c r="D38" s="17"/>
       <c r="E38" s="17"/>
       <c r="F38" s="4" t="s">
-        <v>369</v>
+        <v>385</v>
       </c>
       <c r="G38" s="226">
         <f t="shared" ref="G38:I38" si="8">G30-G35</f>
@@ -50289,7 +50371,7 @@
       <c r="Q45" s="17"/>
       <c r="R45" s="17"/>
       <c r="T45" s="216" t="s">
-        <v>370</v>
+        <v>386</v>
       </c>
       <c r="AD45" s="17"/>
       <c r="AE45" s="17"/>
@@ -50453,7 +50535,7 @@
         <v>156</v>
       </c>
       <c r="AG49" s="60" t="s">
-        <v>371</v>
+        <v>387</v>
       </c>
     </row>
     <row r="50">
@@ -50618,7 +50700,7 @@
         <v>13.03594852814783</v>
       </c>
       <c r="AG52" s="60" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
     </row>
     <row r="53">
@@ -50679,7 +50761,7 @@
         <v>6.291840048860032</v>
       </c>
       <c r="AG53" s="60" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
     </row>
     <row r="54">
@@ -50740,7 +50822,7 @@
         <v>2.7243520649411117</v>
       </c>
       <c r="AG54" s="60" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
     </row>
     <row r="55">
@@ -50801,7 +50883,7 @@
         <v>2.1429979739456915</v>
       </c>
       <c r="AG55" s="60" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
     </row>
     <row r="56">
@@ -50862,7 +50944,7 @@
         <v>3.98032040346951</v>
       </c>
       <c r="AG56" s="60" t="s">
-        <v>372</v>
+        <v>388</v>
       </c>
     </row>
     <row r="57">
@@ -51085,10 +51167,10 @@
       <c r="R62" s="17"/>
       <c r="S62" s="17"/>
       <c r="U62" s="76" t="s">
-        <v>373</v>
+        <v>389</v>
       </c>
       <c r="V62" s="76" t="s">
-        <v>374</v>
+        <v>390</v>
       </c>
       <c r="AC62" s="17"/>
       <c r="AD62" s="17"/>
@@ -51130,7 +51212,7 @@
         <v>2165.0</v>
       </c>
       <c r="W63" s="76" t="s">
-        <v>375</v>
+        <v>391</v>
       </c>
       <c r="AC63" s="17"/>
       <c r="AD63" s="17"/>
@@ -51764,7 +51846,7 @@
       <c r="R79" s="17"/>
       <c r="S79" s="17"/>
       <c r="T79" s="6" t="s">
-        <v>376</v>
+        <v>392</v>
       </c>
       <c r="U79" s="17"/>
       <c r="V79" s="17"/>
@@ -51805,7 +51887,7 @@
       <c r="R80" s="17"/>
       <c r="S80" s="17"/>
       <c r="T80" s="76" t="s">
-        <v>377</v>
+        <v>393</v>
       </c>
       <c r="U80" s="21"/>
       <c r="V80" s="21"/>

</xml_diff>

<commit_message>
Valido metricas con experimento.
DE:
n_draw y expected_roi

A:
sum_aciertos_away y expected_error
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -40,16 +40,16 @@
     <t>england</t>
   </si>
   <si>
+    <t>france</t>
+  </si>
+  <si>
+    <t>XGBClassifier</t>
+  </si>
+  <si>
+    <t>germany</t>
+  </si>
+  <si>
     <t>RandomForestClassifier</t>
-  </si>
-  <si>
-    <t>france</t>
-  </si>
-  <si>
-    <t>germany</t>
-  </si>
-  <si>
-    <t>XGBClassifier</t>
   </si>
   <si>
     <t>italy</t>
@@ -71,7 +71,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -81,7 +81,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF000000"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -139,13 +145,13 @@
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -466,10 +472,10 @@
     <col min="2" max="2" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="3" max="3" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
     <col min="4" max="4" style="7" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="8" width="17.14785714285714" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
+    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="19.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -486,7 +492,7 @@
         <v>4</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="17.25">
       <c r="A2" s="4">
         <v>6</v>
       </c>
@@ -503,7 +509,7 @@
         <v>6</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="17.25">
       <c r="A3" s="4">
         <v>48</v>
       </c>
@@ -514,30 +520,30 @@
         <v>45895</v>
       </c>
       <c r="D3" s="4">
-        <v>79</v>
+        <v>23</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
+        <v>6</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="17.25">
       <c r="A4" s="4">
         <v>55</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="6">
         <v>45895</v>
       </c>
       <c r="D4" s="4">
-        <v>84</v>
+        <v>12</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
+        <v>9</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="17.25">
       <c r="A5" s="4">
         <v>59</v>
       </c>
@@ -548,13 +554,13 @@
         <v>45895</v>
       </c>
       <c r="D5" s="4">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="19.5">
+    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="17.25">
       <c r="A6" s="4">
         <v>77</v>
       </c>
@@ -565,13 +571,13 @@
         <v>45895</v>
       </c>
       <c r="D6" s="4">
-        <v>50</v>
+        <v>18</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
+        <v>6</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="17.25">
       <c r="A7" s="4">
         <v>148</v>
       </c>
@@ -582,13 +588,13 @@
         <v>45895</v>
       </c>
       <c r="D7" s="4">
-        <v>120</v>
+        <v>54</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
+        <v>6</v>
+      </c>
+    </row>
+    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="17.25">
       <c r="A8" s="4">
         <v>167</v>
       </c>

</xml_diff>

<commit_message>
Actualizo preds con nuevos modelos
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -1,40 +1,97 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Documents/GitHub/predictor-apuestas/data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAC367B-B2F2-C240-9F62-D826E8E22E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="20740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+  <si>
+    <t>id_country</t>
+  </si>
+  <si>
+    <t>country</t>
+  </si>
+  <si>
+    <t>iteration_date</t>
+  </si>
+  <si>
+    <t>n_model</t>
+  </si>
+  <si>
+    <t>model_name</t>
+  </si>
+  <si>
+    <t>argentina</t>
+  </si>
+  <si>
+    <t>LogisticRegression</t>
+  </si>
+  <si>
+    <t>england</t>
+  </si>
+  <si>
+    <t>RandomForestClassifier</t>
+  </si>
+  <si>
+    <t>france</t>
+  </si>
+  <si>
+    <t>germany</t>
+  </si>
+  <si>
+    <t>italy</t>
+  </si>
+  <si>
+    <t>spain</t>
+  </si>
+  <si>
+    <t>usa</t>
+  </si>
+  <si>
+    <t>SVC</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -49,94 +106,44 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -424,186 +431,147 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>id_country</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>country</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>iteration_date</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>n_model</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>model_name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2">
         <v>6</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>argentina</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D2" t="n">
+      <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D2">
         <v>1</v>
       </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="E2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3">
         <v>48</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>england</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D3" t="n">
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D3">
+        <v>3</v>
+      </c>
+      <c r="E3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>RandomForestClassifier</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4">
         <v>55</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>france</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D4" t="n">
-        <v>49</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="n">
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D4">
+        <v>37</v>
+      </c>
+      <c r="E4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5">
         <v>59</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>germany</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D5" t="n">
-        <v>128</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>RandomForestClassifier</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="n">
+      <c r="B5" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D5">
+        <v>31</v>
+      </c>
+      <c r="E5" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6">
         <v>77</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>italy</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D6" t="n">
-        <v>18</v>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="n">
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D6">
+        <v>2</v>
+      </c>
+      <c r="E6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7">
         <v>148</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>spain</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D7" t="n">
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D7">
         <v>54</v>
       </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>LogisticRegression</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="n">
+      <c r="E7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8">
         <v>167</v>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>usa</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="n">
-        <v>45895</v>
-      </c>
-      <c r="D8" t="n">
+      <c r="B8" t="s">
+        <v>13</v>
+      </c>
+      <c r="C8" s="2">
+        <v>45895</v>
+      </c>
+      <c r="D8">
         <v>1</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>SVC</t>
-        </is>
+      <c r="E8" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo datos y modelos
</commit_message>
<xml_diff>
--- a/data/df_best_models.xlsx
+++ b/data/df_best_models.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nachomondino/Documents/GitHub/predictor-apuestas/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFAC367B-B2F2-C240-9F62-D826E8E22E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90FE5CFF-D282-4B40-A18D-3E2234B14952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="20740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="16">
   <si>
     <t>id_country</t>
   </si>
@@ -40,19 +40,22 @@
     <t>argentina</t>
   </si>
   <si>
+    <t>RandomForestClassifier</t>
+  </si>
+  <si>
+    <t>england</t>
+  </si>
+  <si>
     <t>LogisticRegression</t>
   </si>
   <si>
-    <t>england</t>
-  </si>
-  <si>
-    <t>RandomForestClassifier</t>
-  </si>
-  <si>
     <t>france</t>
   </si>
   <si>
     <t>germany</t>
+  </si>
+  <si>
+    <t>XGBClassifier</t>
   </si>
   <si>
     <t>italy</t>
@@ -72,7 +75,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -129,7 +132,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -434,9 +437,6 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="17.6640625" bestFit="1" customWidth="1"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
@@ -469,7 +469,7 @@
         <v>1</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
@@ -483,10 +483,10 @@
         <v>45895</v>
       </c>
       <c r="D3">
-        <v>3</v>
+        <v>49</v>
       </c>
       <c r="E3" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
@@ -500,10 +500,10 @@
         <v>45895</v>
       </c>
       <c r="D4">
-        <v>37</v>
+        <v>71</v>
       </c>
       <c r="E4" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
@@ -517,10 +517,10 @@
         <v>45895</v>
       </c>
       <c r="D5">
-        <v>31</v>
+        <v>124</v>
       </c>
       <c r="E5" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
@@ -528,16 +528,16 @@
         <v>77</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C6" s="2">
         <v>45895</v>
       </c>
       <c r="D6">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E6" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -545,16 +545,16 @@
         <v>148</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C7" s="2">
         <v>45895</v>
       </c>
       <c r="D7">
-        <v>54</v>
+        <v>118</v>
       </c>
       <c r="E7" t="s">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -562,7 +562,7 @@
         <v>167</v>
       </c>
       <c r="B8" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C8" s="2">
         <v>45895</v>
@@ -571,7 +571,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>